<commit_message>
Reference workbook: channel + segment granularity for scenario-building
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
+++ b/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="C5" s="32">
-        <f>'Inputs'!$C$158</f>
+        <f>'Inputs'!$C$169</f>
         <v/>
       </c>
     </row>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="C6" s="26">
-        <f>'Inputs'!$C$158*'1. Customers'!$C$4</f>
+        <f>'Inputs'!$C$169*'1. Customers'!$C$4</f>
         <v/>
       </c>
     </row>
@@ -800,7 +800,7 @@
         </is>
       </c>
       <c r="C7" s="29">
-        <f>'Inputs'!$C$158*'1. Customers'!$E$22</f>
+        <f>'Inputs'!$C$169*'1. Customers'!$E$22</f>
         <v/>
       </c>
     </row>
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="C8" s="29">
-        <f>'Inputs'!$C$158*'1. Customers'!$E$21</f>
+        <f>'Inputs'!$C$169*'1. Customers'!$E$21</f>
         <v/>
       </c>
     </row>
@@ -822,7 +822,7 @@
         </is>
       </c>
       <c r="C9" s="29">
-        <f>'Inputs'!$C$158*'7. P&amp;L'!$C$6</f>
+        <f>'Inputs'!$C$169*'7. P&amp;L'!$C$6</f>
         <v/>
       </c>
     </row>
@@ -833,7 +833,7 @@
         </is>
       </c>
       <c r="C10" s="29">
-        <f>'Inputs'!$C$158*-'7. P&amp;L'!$C$16</f>
+        <f>'Inputs'!$C$169*-'7. P&amp;L'!$C$16</f>
         <v/>
       </c>
     </row>
@@ -890,7 +890,7 @@
         <v/>
       </c>
       <c r="D14" s="39">
-        <f>C14*'Inputs'!$C$158</f>
+        <f>C14*'Inputs'!$C$169</f>
         <v/>
       </c>
       <c r="E14" s="26">
@@ -914,7 +914,7 @@
         <v/>
       </c>
       <c r="D15" s="39">
-        <f>C15*'Inputs'!$C$158</f>
+        <f>C15*'Inputs'!$C$169</f>
         <v/>
       </c>
       <c r="E15" s="26">
@@ -938,7 +938,7 @@
         <v/>
       </c>
       <c r="D16" s="39">
-        <f>C16*'Inputs'!$C$158</f>
+        <f>C16*'Inputs'!$C$169</f>
         <v/>
       </c>
       <c r="E16" s="26">
@@ -962,7 +962,7 @@
         <v/>
       </c>
       <c r="D17" s="39">
-        <f>C17*'Inputs'!$C$158</f>
+        <f>C17*'Inputs'!$C$169</f>
         <v/>
       </c>
       <c r="E17" s="26">
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="C28" s="39">
-        <f>'3. HR &amp; Activity'!$D$38*'Inputs'!$C$158/'8. Org Structure'!$C$27</f>
+        <f>'3. HR &amp; Activity'!$D$38*'Inputs'!$C$169/'8. Org Structure'!$C$27</f>
         <v/>
       </c>
       <c r="H28" s="4" t="inlineStr">
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="C31" s="40">
-        <f>'3. HR &amp; Activity'!$D$39*'Inputs'!$C$158/'Inputs'!$C$25</f>
+        <f>'3. HR &amp; Activity'!$D$39*'Inputs'!$C$169/'Inputs'!$C$25</f>
         <v/>
       </c>
       <c r="H31" s="4" t="inlineStr">
@@ -1203,7 +1203,7 @@
         <v/>
       </c>
       <c r="D38" s="41">
-        <f>'Inputs'!$C$159</f>
+        <f>'Inputs'!$C$170</f>
         <v/>
       </c>
       <c r="E38" s="29">
@@ -1211,7 +1211,7 @@
         <v/>
       </c>
       <c r="F38" s="33">
-        <f>'Inputs'!$C$160</f>
+        <f>'Inputs'!$C$171</f>
         <v/>
       </c>
       <c r="G38" s="27">
@@ -1230,7 +1230,7 @@
         <v/>
       </c>
       <c r="D39" s="41">
-        <f>'Inputs'!$C$161</f>
+        <f>'Inputs'!$C$172</f>
         <v/>
       </c>
       <c r="E39" s="29">
@@ -1238,7 +1238,7 @@
         <v/>
       </c>
       <c r="F39" s="33">
-        <f>'Inputs'!$C$162</f>
+        <f>'Inputs'!$C$173</f>
         <v/>
       </c>
       <c r="G39" s="27">
@@ -1257,7 +1257,7 @@
         <v/>
       </c>
       <c r="D40" s="41">
-        <f>'Inputs'!$C$163</f>
+        <f>'Inputs'!$C$174</f>
         <v/>
       </c>
       <c r="E40" s="29">
@@ -1265,7 +1265,7 @@
         <v/>
       </c>
       <c r="F40" s="33">
-        <f>'Inputs'!$C$164</f>
+        <f>'Inputs'!$C$175</f>
         <v/>
       </c>
       <c r="G40" s="27">
@@ -1704,7 +1704,7 @@
         </is>
       </c>
       <c r="C70" s="29">
-        <f>'Inputs'!$C$158*'3. HR &amp; Activity'!$H$41+'8. Org Structure'!$E$38+'8. Org Structure'!$E$39+'8. Org Structure'!$E$40</f>
+        <f>'Inputs'!$C$169*'3. HR &amp; Activity'!$H$41+'8. Org Structure'!$E$38+'8. Org Structure'!$E$39+'8. Org Structure'!$E$40</f>
         <v/>
       </c>
     </row>
@@ -5670,7 +5670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E164"/>
+  <dimension ref="B1:E175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -8401,7 +8401,7 @@
     <row r="143">
       <c r="B143" s="5" t="inlineStr">
         <is>
-          <t>H. RM SALES EFFORT PER ORIGINATION (RMs are a sales force, not a service cost)</t>
+          <t>G4. SEGMENT GRANULARITY — share of each product's units held by RM-MANAGED customers</t>
         </is>
       </c>
       <c r="C143" s="6" t="inlineStr"/>
@@ -8433,151 +8433,151 @@
     <row r="145">
       <c r="B145" s="8" t="inlineStr">
         <is>
-          <t>Relative RM effort — per new term loan</t>
-        </is>
-      </c>
-      <c r="C145" s="21" t="n">
-        <v>1</v>
+          <t>Current accounts — RM-held share</t>
+        </is>
+      </c>
+      <c r="C145" s="13" t="n">
+        <v>0.15</v>
       </c>
       <c r="D145" s="4" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E145" s="10" t="inlineStr">
         <is>
-          <t>Assumption: RM cost is customer-acquisition cost, attributed per origination by relative effort</t>
+          <t>Equals pct_rm (every customer holds a BCA). Scenario dimension: shift with channel moves</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="B146" s="8" t="inlineStr">
         <is>
-          <t>Relative RM effort — per new asset finance agreement</t>
-        </is>
-      </c>
-      <c r="C146" s="21" t="n">
-        <v>0.5</v>
+          <t>Instant savings — RM-held share</t>
+        </is>
+      </c>
+      <c r="C146" s="13" t="n">
+        <v>0.2</v>
       </c>
       <c r="D146" s="4" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E146" s="10" t="inlineStr">
         <is>
-          <t>Assumption: more automated sale</t>
+          <t>Assumption — for scenario building; validate from segment data</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="B147" s="8" t="inlineStr">
         <is>
-          <t>Relative RM effort — per new invoice finance client</t>
-        </is>
-      </c>
-      <c r="C147" s="21" t="n">
-        <v>1.5</v>
+          <t>Notice &amp; fixed deposits — RM-held share</t>
+        </is>
+      </c>
+      <c r="C147" s="13" t="n">
+        <v>0.3</v>
       </c>
       <c r="D147" s="4" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E147" s="10" t="inlineStr">
         <is>
-          <t>Assumption: complex, consultative sale</t>
+          <t>Assumption</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="B148" s="8" t="inlineStr">
         <is>
-          <t>Relative RM effort — per overdraft renewal</t>
-        </is>
-      </c>
-      <c r="C148" s="23" t="n">
-        <v>0.25</v>
+          <t>Overdrafts — RM-held share</t>
+        </is>
+      </c>
+      <c r="C148" s="13" t="n">
+        <v>0.4</v>
       </c>
       <c r="D148" s="4" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E148" s="10" t="inlineStr">
         <is>
-          <t>Assumption: annual renewals; a key automation lever</t>
+          <t>Assumption</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="B149" s="8" t="inlineStr">
         <is>
-          <t>RM time — ORIGINATE (sales, attributed per origination)</t>
+          <t>Term loans — RM-held share</t>
         </is>
       </c>
       <c r="C149" s="13" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="D149" s="4" t="inlineStr">
         <is>
-          <t>% of RM time</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E149" s="10" t="inlineStr">
         <is>
-          <t>The three RM activities work as a system: stewardship generates the signals origination targets; origination builds the book stewardship protects; defence preserves the relationships that carry future originations</t>
+          <t>Consistent with rm_lend_share (RM customers are the larger borrowers)</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="B150" s="8" t="inlineStr">
         <is>
-          <t>RM time — STEWARD (credit stewardship of the covered book)</t>
+          <t>Asset finance — RM-held share</t>
         </is>
       </c>
       <c r="C150" s="13" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="D150" s="4" t="inlineStr">
         <is>
-          <t>% of RM time</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E150" s="10" t="inlineStr">
         <is>
-          <t>Attributed to lending products pro-rata covered balances; pays back through lower PDs</t>
+          <t>Assumption</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="B151" s="8" t="inlineStr">
         <is>
-          <t>RM time — DEFEND (retention at contested moments)</t>
+          <t>Invoice finance — RM-held share</t>
         </is>
       </c>
       <c r="C151" s="13" t="n">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D151" s="4" t="inlineStr">
         <is>
-          <t>% of RM time</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E151" s="10" t="inlineStr">
         <is>
-          <t>Held at centre level as tested retention spend — the three shares must sum to 100%</t>
+          <t>Assumption — consultative product</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="B152" s="8" t="inlineStr">
         <is>
-          <t>Share of lending balances held by RM-managed customers</t>
+          <t>Business cards — RM-held share</t>
         </is>
       </c>
       <c r="C152" s="13" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="D152" s="4" t="inlineStr">
         <is>
@@ -8586,18 +8586,18 @@
       </c>
       <c r="E152" s="10" t="inlineStr">
         <is>
-          <t>Assumption: RM-managed customers are the larger borrowers</t>
+          <t>Assumption</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="B153" s="8" t="inlineStr">
         <is>
-          <t>Stewardship effect: relative PD reduction on RM-covered balances</t>
-        </is>
-      </c>
-      <c r="C153" s="15" t="n">
-        <v>0.2</v>
+          <t>Payments &amp; FX users — RM-held share</t>
+        </is>
+      </c>
+      <c r="C153" s="13" t="n">
+        <v>0.4</v>
       </c>
       <c r="D153" s="4" t="inlineStr">
         <is>
@@ -8606,186 +8606,186 @@
       </c>
       <c r="E153" s="10" t="inlineStr">
         <is>
-          <t>Relationship-lending evidence: soft information and early warning lower default rates; validate against covered vs uncovered book performance</t>
+          <t>Assumption</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="B154" s="8" t="inlineStr">
-        <is>
-          <t>Defence effect: relative churn reduction among RM-managed customers</t>
-        </is>
-      </c>
-      <c r="C154" s="15" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="D154" s="4" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E154" s="10" t="inlineStr">
-        <is>
-          <t>Must be validated with holdout tests — pay only for incremental saves</t>
-        </is>
-      </c>
+      <c r="B154" s="5" t="inlineStr">
+        <is>
+          <t>H. RM SALES EFFORT PER ORIGINATION (RMs are a sales force, not a service cost)</t>
+        </is>
+      </c>
+      <c r="C154" s="6" t="inlineStr"/>
+      <c r="D154" s="6" t="inlineStr"/>
+      <c r="E154" s="6" t="inlineStr"/>
     </row>
     <row r="155">
-      <c r="B155" s="8" t="inlineStr">
-        <is>
-          <t>Expected remaining relationship life of a defended customer</t>
-        </is>
-      </c>
-      <c r="C155" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D155" s="4" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="E155" s="10" t="inlineStr">
-        <is>
-          <t>A saved customer is an annuity, not one year of contribution</t>
+      <c r="B155" s="7" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C155" s="7" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D155" s="7" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E155" s="7" t="inlineStr">
+        <is>
+          <t>Source / note</t>
         </is>
       </c>
     </row>
     <row r="156">
-      <c r="B156" s="5" t="inlineStr">
-        <is>
-          <t>I. ORGANISATION AT SCALE (drives the Org Structure tab)</t>
-        </is>
-      </c>
-      <c r="C156" s="6" t="inlineStr"/>
-      <c r="D156" s="6" t="inlineStr"/>
-      <c r="E156" s="6" t="inlineStr"/>
+      <c r="B156" s="8" t="inlineStr">
+        <is>
+          <t>Relative RM effort — per new term loan</t>
+        </is>
+      </c>
+      <c r="C156" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D156" s="4" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="E156" s="10" t="inlineStr">
+        <is>
+          <t>Assumption: RM cost is customer-acquisition cost, attributed per origination by relative effort</t>
+        </is>
+      </c>
     </row>
     <row r="157">
-      <c r="B157" s="7" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="C157" s="7" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="D157" s="7" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="E157" s="7" t="inlineStr">
-        <is>
-          <t>Source / note</t>
+      <c r="B157" s="8" t="inlineStr">
+        <is>
+          <t>Relative RM effort — per new asset finance agreement</t>
+        </is>
+      </c>
+      <c r="C157" s="21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D157" s="4" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="E157" s="10" t="inlineStr">
+        <is>
+          <t>Assumption: more automated sale</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="B158" s="8" t="inlineStr">
         <is>
-          <t>Regional business centres at scale</t>
-        </is>
-      </c>
-      <c r="C158" s="16" t="n">
-        <v>300</v>
+          <t>Relative RM effort — per new invoice finance client</t>
+        </is>
+      </c>
+      <c r="C158" s="21" t="n">
+        <v>1.5</v>
       </c>
       <c r="D158" s="4" t="inlineStr">
         <is>
-          <t>centres</t>
+          <t>index</t>
         </is>
       </c>
       <c r="E158" s="10" t="inlineStr">
         <is>
-          <t>Set for 900,000 current-account customers (300 × 3,000). Note: per-customer head-office allocations are held flat — conservative, as central costs per customer typically fall at this scale</t>
+          <t>Assumption: complex, consultative sale</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="B159" s="8" t="inlineStr">
         <is>
-          <t>Technology &amp; central ops — staff share of allocated cost</t>
-        </is>
-      </c>
-      <c r="C159" s="13" t="n">
-        <v>0.55</v>
+          <t>Relative RM effort — per overdraft renewal</t>
+        </is>
+      </c>
+      <c r="C159" s="23" t="n">
+        <v>0.25</v>
       </c>
       <c r="D159" s="4" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>index</t>
         </is>
       </c>
       <c r="E159" s="10" t="inlineStr">
         <is>
-          <t>Assumption: remainder is software licences, hosting, card scheme &amp; processing fees</t>
+          <t>Assumption: annual renewals; a key automation lever</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="B160" s="8" t="inlineStr">
         <is>
-          <t>Technology &amp; central ops — average loaded cost per FTE</t>
-        </is>
-      </c>
-      <c r="C160" s="18" t="n">
-        <v>80000</v>
+          <t>RM time — ORIGINATE (sales, attributed per origination)</t>
+        </is>
+      </c>
+      <c r="C160" s="13" t="n">
+        <v>0.5</v>
       </c>
       <c r="D160" s="4" t="inlineStr">
         <is>
-          <t>£/FTE/yr</t>
+          <t>% of RM time</t>
         </is>
       </c>
       <c r="E160" s="10" t="inlineStr">
         <is>
-          <t>Assumption: salary + on-costs (tech roles skew senior)</t>
+          <t>The three RM activities work as a system: stewardship generates the signals origination targets; origination builds the book stewardship protects; defence preserves the relationships that carry future originations</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="B161" s="8" t="inlineStr">
         <is>
-          <t>Risk, compliance &amp; audit — staff share of allocated cost</t>
+          <t>RM time — STEWARD (credit stewardship of the covered book)</t>
         </is>
       </c>
       <c r="C161" s="13" t="n">
-        <v>0.75</v>
+        <v>0.3</v>
       </c>
       <c r="D161" s="4" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% of RM time</t>
         </is>
       </c>
       <c r="E161" s="10" t="inlineStr">
         <is>
-          <t>Assumption: remainder is data, tools, professional fees</t>
+          <t>Attributed to lending products pro-rata covered balances; pays back through lower PDs</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="B162" s="8" t="inlineStr">
         <is>
-          <t>Risk, compliance &amp; audit — average loaded cost per FTE</t>
-        </is>
-      </c>
-      <c r="C162" s="18" t="n">
-        <v>75000</v>
+          <t>RM time — DEFEND (retention at contested moments)</t>
+        </is>
+      </c>
+      <c r="C162" s="13" t="n">
+        <v>0.2</v>
       </c>
       <c r="D162" s="4" t="inlineStr">
         <is>
-          <t>£/FTE/yr</t>
+          <t>% of RM time</t>
         </is>
       </c>
       <c r="E162" s="10" t="inlineStr">
         <is>
-          <t>Assumption</t>
+          <t>Held at centre level as tested retention spend — the three shares must sum to 100%</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="B163" s="8" t="inlineStr">
         <is>
-          <t>Corporate centre — staff share of allocated cost</t>
+          <t>Share of lending balances held by RM-managed customers</t>
         </is>
       </c>
       <c r="C163" s="13" t="n">
@@ -8798,25 +8798,237 @@
       </c>
       <c r="E163" s="10" t="inlineStr">
         <is>
-          <t>Assumption: remainder is brand &amp; media spend, audit &amp; professional fees, facilities</t>
+          <t>Assumption: RM-managed customers are the larger borrowers</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="B164" s="8" t="inlineStr">
         <is>
+          <t>Stewardship effect: relative PD reduction on RM-covered balances</t>
+        </is>
+      </c>
+      <c r="C164" s="15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D164" s="4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E164" s="10" t="inlineStr">
+        <is>
+          <t>Relationship-lending evidence: soft information and early warning lower default rates; validate against covered vs uncovered book performance</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="B165" s="8" t="inlineStr">
+        <is>
+          <t>Defence effect: relative churn reduction among RM-managed customers</t>
+        </is>
+      </c>
+      <c r="C165" s="15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D165" s="4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E165" s="10" t="inlineStr">
+        <is>
+          <t>Must be validated with holdout tests — pay only for incremental saves</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="B166" s="8" t="inlineStr">
+        <is>
+          <t>Expected remaining relationship life of a defended customer</t>
+        </is>
+      </c>
+      <c r="C166" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D166" s="4" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="E166" s="10" t="inlineStr">
+        <is>
+          <t>A saved customer is an annuity, not one year of contribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="B167" s="5" t="inlineStr">
+        <is>
+          <t>I. ORGANISATION AT SCALE (drives the Org Structure tab)</t>
+        </is>
+      </c>
+      <c r="C167" s="6" t="inlineStr"/>
+      <c r="D167" s="6" t="inlineStr"/>
+      <c r="E167" s="6" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="B168" s="7" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C168" s="7" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D168" s="7" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E168" s="7" t="inlineStr">
+        <is>
+          <t>Source / note</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="B169" s="8" t="inlineStr">
+        <is>
+          <t>Regional business centres at scale</t>
+        </is>
+      </c>
+      <c r="C169" s="16" t="n">
+        <v>300</v>
+      </c>
+      <c r="D169" s="4" t="inlineStr">
+        <is>
+          <t>centres</t>
+        </is>
+      </c>
+      <c r="E169" s="10" t="inlineStr">
+        <is>
+          <t>Set for 900,000 current-account customers (300 × 3,000). Note: per-customer head-office allocations are held flat — conservative, as central costs per customer typically fall at this scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="B170" s="8" t="inlineStr">
+        <is>
+          <t>Technology &amp; central ops — staff share of allocated cost</t>
+        </is>
+      </c>
+      <c r="C170" s="13" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D170" s="4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E170" s="10" t="inlineStr">
+        <is>
+          <t>Assumption: remainder is software licences, hosting, card scheme &amp; processing fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="B171" s="8" t="inlineStr">
+        <is>
+          <t>Technology &amp; central ops — average loaded cost per FTE</t>
+        </is>
+      </c>
+      <c r="C171" s="18" t="n">
+        <v>80000</v>
+      </c>
+      <c r="D171" s="4" t="inlineStr">
+        <is>
+          <t>£/FTE/yr</t>
+        </is>
+      </c>
+      <c r="E171" s="10" t="inlineStr">
+        <is>
+          <t>Assumption: salary + on-costs (tech roles skew senior)</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="B172" s="8" t="inlineStr">
+        <is>
+          <t>Risk, compliance &amp; audit — staff share of allocated cost</t>
+        </is>
+      </c>
+      <c r="C172" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D172" s="4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E172" s="10" t="inlineStr">
+        <is>
+          <t>Assumption: remainder is data, tools, professional fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="B173" s="8" t="inlineStr">
+        <is>
+          <t>Risk, compliance &amp; audit — average loaded cost per FTE</t>
+        </is>
+      </c>
+      <c r="C173" s="18" t="n">
+        <v>75000</v>
+      </c>
+      <c r="D173" s="4" t="inlineStr">
+        <is>
+          <t>£/FTE/yr</t>
+        </is>
+      </c>
+      <c r="E173" s="10" t="inlineStr">
+        <is>
+          <t>Assumption</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="B174" s="8" t="inlineStr">
+        <is>
+          <t>Corporate centre — staff share of allocated cost</t>
+        </is>
+      </c>
+      <c r="C174" s="13" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D174" s="4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E174" s="10" t="inlineStr">
+        <is>
+          <t>Assumption: remainder is brand &amp; media spend, audit &amp; professional fees, facilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="B175" s="8" t="inlineStr">
+        <is>
           <t>Corporate centre — average loaded cost per FTE</t>
         </is>
       </c>
-      <c r="C164" s="18" t="n">
+      <c r="C175" s="18" t="n">
         <v>75000</v>
       </c>
-      <c r="D164" s="4" t="inlineStr">
+      <c r="D175" s="4" t="inlineStr">
         <is>
           <t>£/FTE/yr</t>
         </is>
       </c>
-      <c r="E164" s="10" t="inlineStr">
+      <c r="E175" s="10" t="inlineStr">
         <is>
           <t>Assumption</t>
         </is>
@@ -8833,7 +9045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F25"/>
+  <dimension ref="B1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -8903,7 +9115,7 @@
         </is>
       </c>
       <c r="C7" s="26">
-        <f>'1. Customers'!$C$5*'Inputs'!$C$21*'Inputs'!$C$154</f>
+        <f>'1. Customers'!$C$5*'Inputs'!$C$21*'Inputs'!$C$165</f>
         <v/>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -8965,6 +9177,21 @@
           <t>Note</t>
         </is>
       </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>RM-held units</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Digitally-held units</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>(segment granularity — scenario dimension)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="8" t="inlineStr">
@@ -8989,6 +9216,14 @@
           <t>Credit balances held by customers</t>
         </is>
       </c>
+      <c r="G12" s="26">
+        <f>C12*'Inputs'!$C$145</f>
+        <v/>
+      </c>
+      <c r="H12" s="26">
+        <f>C12-G12</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="8" t="inlineStr">
@@ -9009,6 +9244,14 @@
         <v/>
       </c>
       <c r="F13" s="4" t="inlineStr"/>
+      <c r="G13" s="26">
+        <f>C13*'Inputs'!$C$146</f>
+        <v/>
+      </c>
+      <c r="H13" s="26">
+        <f>C13-G13</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="8" t="inlineStr">
@@ -9029,6 +9272,14 @@
         <v/>
       </c>
       <c r="F14" s="4" t="inlineStr"/>
+      <c r="G14" s="26">
+        <f>C14*'Inputs'!$C$147</f>
+        <v/>
+      </c>
+      <c r="H14" s="26">
+        <f>C14-G14</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="8" t="inlineStr">
@@ -9053,6 +9304,14 @@
           <t>Balance = limit × utilisation (drawn)</t>
         </is>
       </c>
+      <c r="G15" s="26">
+        <f>C15*'Inputs'!$C$148</f>
+        <v/>
+      </c>
+      <c r="H15" s="26">
+        <f>C15-G15</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="B16" s="8" t="inlineStr">
@@ -9073,6 +9332,14 @@
         <v/>
       </c>
       <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="26">
+        <f>C16*'Inputs'!$C$149</f>
+        <v/>
+      </c>
+      <c r="H16" s="26">
+        <f>C16-G16</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="B17" s="8" t="inlineStr">
@@ -9093,6 +9360,14 @@
         <v/>
       </c>
       <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="26">
+        <f>C17*'Inputs'!$C$150</f>
+        <v/>
+      </c>
+      <c r="H17" s="26">
+        <f>C17-G17</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="8" t="inlineStr">
@@ -9117,6 +9392,14 @@
           <t>Funds in use (advances outstanding)</t>
         </is>
       </c>
+      <c r="G18" s="26">
+        <f>C18*'Inputs'!$C$151</f>
+        <v/>
+      </c>
+      <c r="H18" s="26">
+        <f>C18-G18</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="8" t="inlineStr">
@@ -9141,6 +9424,14 @@
           <t>Avg interest-bearing balance per card</t>
         </is>
       </c>
+      <c r="G19" s="26">
+        <f>C19*'Inputs'!$C$152</f>
+        <v/>
+      </c>
+      <c r="H19" s="26">
+        <f>C19-G19</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="8" t="inlineStr">
@@ -9164,6 +9455,14 @@
         <is>
           <t>No balance product</t>
         </is>
+      </c>
+      <c r="G20" s="26">
+        <f>C20*'Inputs'!$C$153</f>
+        <v/>
+      </c>
+      <c r="H20" s="26">
+        <f>C20-G20</f>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -9857,7 +10156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:K70"/>
+  <dimension ref="B1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9997,6 +10296,11 @@
           <t>Cost high (£/yr)</t>
         </is>
       </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>Channel (scenario dimension)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="8" t="inlineStr">
@@ -10043,6 +10347,11 @@
         <f>H11*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L11" s="37" t="inlineStr">
+        <is>
+          <t>digital-amenable</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="8" t="inlineStr">
@@ -10089,6 +10398,11 @@
         <f>H12*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L12" s="37" t="inlineStr">
+        <is>
+          <t>digital-amenable</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="8" t="inlineStr">
@@ -10135,6 +10449,11 @@
         <f>H13*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L13" s="37" t="inlineStr">
+        <is>
+          <t>digital-amenable</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="8" t="inlineStr">
@@ -10181,6 +10500,11 @@
         <f>H14*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L14" s="37" t="inlineStr">
+        <is>
+          <t>digital-amenable</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="8" t="inlineStr">
@@ -10227,6 +10551,11 @@
         <f>H15*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L15" s="37" t="inlineStr">
+        <is>
+          <t>judgement</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="B16" s="8" t="inlineStr">
@@ -10273,6 +10602,11 @@
         <f>H16*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L16" s="37" t="inlineStr">
+        <is>
+          <t>judgement</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="B17" s="8" t="inlineStr">
@@ -10319,6 +10653,11 @@
         <f>H17*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L17" s="37" t="inlineStr">
+        <is>
+          <t>judgement</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="8" t="inlineStr">
@@ -10365,6 +10704,11 @@
         <f>H18*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L18" s="37" t="inlineStr">
+        <is>
+          <t>digital-amenable</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="8" t="inlineStr">
@@ -10411,6 +10755,11 @@
         <f>H19*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L19" s="37" t="inlineStr">
+        <is>
+          <t>judgement</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="8" t="inlineStr">
@@ -10457,6 +10806,11 @@
         <f>H20*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L20" s="37" t="inlineStr">
+        <is>
+          <t>judgement</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="8" t="inlineStr">
@@ -10503,6 +10857,11 @@
         <f>H21*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L21" s="37" t="inlineStr">
+        <is>
+          <t>digital-amenable</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="B22" s="8" t="inlineStr">
@@ -10549,6 +10908,11 @@
         <f>H22*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L22" s="37" t="inlineStr">
+        <is>
+          <t>digital-amenable</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="8" t="inlineStr">
@@ -10595,6 +10959,11 @@
         <f>H23*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L23" s="37" t="inlineStr">
+        <is>
+          <t>judgement</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="8" t="inlineStr">
@@ -10641,6 +11010,11 @@
         <f>H24*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L24" s="37" t="inlineStr">
+        <is>
+          <t>judgement</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="8" t="inlineStr">
@@ -10687,6 +11061,11 @@
         <f>H25*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L25" s="37" t="inlineStr">
+        <is>
+          <t>judgement</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="8" t="inlineStr">
@@ -10733,6 +11112,11 @@
         <f>H26*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L26" s="37" t="inlineStr">
+        <is>
+          <t>judgement</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="8" t="inlineStr">
@@ -10779,6 +11163,11 @@
         <f>H27*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L27" s="37" t="inlineStr">
+        <is>
+          <t>judgement</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="8" t="inlineStr">
@@ -10825,6 +11214,11 @@
         <f>H28*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L28" s="37" t="inlineStr">
+        <is>
+          <t>digital-amenable</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="8" t="inlineStr">
@@ -10871,6 +11265,11 @@
         <f>H29*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L29" s="37" t="inlineStr">
+        <is>
+          <t>digital-amenable</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="B30" s="8" t="inlineStr">
@@ -10917,6 +11316,11 @@
         <f>H30*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L30" s="37" t="inlineStr">
+        <is>
+          <t>digital-amenable</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="B31" s="8" t="inlineStr">
@@ -10963,6 +11367,11 @@
         <f>H31*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L31" s="37" t="inlineStr">
+        <is>
+          <t>judgement</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="8" t="inlineStr">
@@ -11009,6 +11418,11 @@
         <f>H32*'Inputs'!$C$117</f>
         <v/>
       </c>
+      <c r="L32" s="37" t="inlineStr">
+        <is>
+          <t>judgement</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="8" t="inlineStr">
@@ -11054,6 +11468,11 @@
       <c r="K33" s="29">
         <f>H33*'Inputs'!$C$117</f>
         <v/>
+      </c>
+      <c r="L33" s="37" t="inlineStr">
+        <is>
+          <t>judgement</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -11212,11 +11631,11 @@
         </is>
       </c>
       <c r="D46" s="41">
-        <f>'Inputs'!$C$149</f>
+        <f>'Inputs'!$C$160</f>
         <v/>
       </c>
       <c r="H46" s="29">
-        <f>'3. HR &amp; Activity'!$H$37*'Inputs'!$C$149</f>
+        <f>'3. HR &amp; Activity'!$H$37*'Inputs'!$C$160</f>
         <v/>
       </c>
     </row>
@@ -11227,11 +11646,11 @@
         </is>
       </c>
       <c r="D47" s="41">
-        <f>'Inputs'!$C$150</f>
+        <f>'Inputs'!$C$161</f>
         <v/>
       </c>
       <c r="H47" s="29">
-        <f>'3. HR &amp; Activity'!$H$37*'Inputs'!$C$150</f>
+        <f>'3. HR &amp; Activity'!$H$37*'Inputs'!$C$161</f>
         <v/>
       </c>
     </row>
@@ -11242,11 +11661,11 @@
         </is>
       </c>
       <c r="D48" s="41">
-        <f>'Inputs'!$C$151</f>
+        <f>'Inputs'!$C$162</f>
         <v/>
       </c>
       <c r="H48" s="29">
-        <f>'3. HR &amp; Activity'!$H$37*'Inputs'!$C$151</f>
+        <f>'3. HR &amp; Activity'!$H$37*'Inputs'!$C$162</f>
         <v/>
       </c>
     </row>
@@ -11307,7 +11726,7 @@
         <v/>
       </c>
       <c r="E52" s="42">
-        <f>'Inputs'!$C$145</f>
+        <f>'Inputs'!$C$156</f>
         <v/>
       </c>
       <c r="F52" s="39">
@@ -11334,7 +11753,7 @@
         <v/>
       </c>
       <c r="E53" s="42">
-        <f>'Inputs'!$C$146</f>
+        <f>'Inputs'!$C$157</f>
         <v/>
       </c>
       <c r="F53" s="39">
@@ -11361,7 +11780,7 @@
         <v/>
       </c>
       <c r="E54" s="42">
-        <f>'Inputs'!$C$147</f>
+        <f>'Inputs'!$C$158</f>
         <v/>
       </c>
       <c r="F54" s="39">
@@ -11388,7 +11807,7 @@
         <v/>
       </c>
       <c r="E55" s="42">
-        <f>'Inputs'!$C$148</f>
+        <f>'Inputs'!$C$159</f>
         <v/>
       </c>
       <c r="F55" s="39">
@@ -11572,7 +11991,7 @@
         </is>
       </c>
       <c r="G65" s="29">
-        <f>('1. Customers'!$E$15*'Inputs'!$C$75*'Inputs'!$C$76+'1. Customers'!$E$16*'Inputs'!$C$77*'Inputs'!$C$78+'1. Customers'!$E$17*'Inputs'!$C$79*'Inputs'!$C$80+'1. Customers'!$E$18*'Inputs'!$C$81*'Inputs'!$C$82)*'Inputs'!$C$153*'Inputs'!$C$152</f>
+        <f>('1. Customers'!$E$15*'Inputs'!$C$75*'Inputs'!$C$76+'1. Customers'!$E$16*'Inputs'!$C$77*'Inputs'!$C$78+'1. Customers'!$E$17*'Inputs'!$C$79*'Inputs'!$C$80+'1. Customers'!$E$18*'Inputs'!$C$81*'Inputs'!$C$82)*'Inputs'!$C$164*'Inputs'!$C$163</f>
         <v/>
       </c>
       <c r="H65" s="4" t="inlineStr">
@@ -12042,7 +12461,7 @@
         <v/>
       </c>
       <c r="E5" s="12">
-        <f>D5*(1-'Inputs'!$C$153*'Inputs'!$C$152)</f>
+        <f>D5*(1-'Inputs'!$C$164*'Inputs'!$C$163)</f>
         <v/>
       </c>
       <c r="F5" s="41">
@@ -12073,7 +12492,7 @@
         <v/>
       </c>
       <c r="E6" s="12">
-        <f>D6*(1-'Inputs'!$C$153*'Inputs'!$C$152)</f>
+        <f>D6*(1-'Inputs'!$C$164*'Inputs'!$C$163)</f>
         <v/>
       </c>
       <c r="F6" s="41">
@@ -12104,7 +12523,7 @@
         <v/>
       </c>
       <c r="E7" s="12">
-        <f>D7*(1-'Inputs'!$C$153*'Inputs'!$C$152)</f>
+        <f>D7*(1-'Inputs'!$C$164*'Inputs'!$C$163)</f>
         <v/>
       </c>
       <c r="F7" s="41">
@@ -12135,7 +12554,7 @@
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>D8*(1-'Inputs'!$C$153*'Inputs'!$C$152)</f>
+        <f>D8*(1-'Inputs'!$C$164*'Inputs'!$C$163)</f>
         <v/>
       </c>
       <c r="F8" s="41">
@@ -13422,7 +13841,7 @@
         </is>
       </c>
       <c r="C33" s="29">
-        <f>'1. Customers'!$C$7*(C27/'1. Customers'!$C$4*'Inputs'!$C$155+'Inputs'!$C$103*'3. HR &amp; Activity'!$C$7+'Inputs'!$C$132)</f>
+        <f>'1. Customers'!$C$7*(C27/'1. Customers'!$C$4*'Inputs'!$C$166+'Inputs'!$C$103*'3. HR &amp; Activity'!$C$7+'Inputs'!$C$132)</f>
         <v/>
       </c>
       <c r="D33" s="4" t="inlineStr">

</xml_diff>

<commit_message>
v1.2.1: Guide documents the period assumption (steady-state annual snapshot)
Documentation only — no formula or input changes; results identical to v1.2.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
+++ b/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B34"/>
+  <dimension ref="B1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -582,7 +582,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MODEL VERSION: v1.2 · 12 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
+          <t>MODEL VERSION: v1.2.1 · 21 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
         </is>
       </c>
     </row>
@@ -596,173 +596,215 @@
     <row r="5" ht="28" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
+          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
+          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
           <t>• v1.0 (10 Aug 2026) — first published version: 9 tabs + flow register, FTP with liquidity/behavioural terms, fraud/FSCS/change-the-bank lines, segment-pod LMUs, bridge check.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="3" t="inlineStr">
+    <row r="10">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>What this is</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="39" customHeight="1">
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="39" customHeight="1">
       <c r="B11" s="4" t="inlineStr">
         <is>
+          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="39" customHeight="1">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
           <t>• It follows the Simanis / IVE bottom-up methodology ('Running the Right Numbers'): model the last-mile operating unit, derive every cost from activity drivers (transaction intensity I and customer load L), build whole costs, and check the price/margin covers them including a competitive return on capital.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>How the tabs map to the methodology</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>• Inputs — every assumption in one place, with sources. Edit blue cells; yellow cells are the biggest levers.</t>
+    <row r="14">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>What period this models</t>
         </is>
       </c>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="26" customHeight="1">
+          <t>• One representative operating year at steady state. Balances are annual averages; rates and volumes are annual. There is no time axis, no ramp and no vintage cohorts — the model is a snapshot, not a forecast.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="52" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>• 2. Revenues — unit revenue per product: interest margins measured against internal funds transfer prices (Bank Rate for floating, + premium for term), plus fees.</t>
+          <t>• The book is stationary but not free to hold flat: customers churn (12% p.a. input) and the model costs their replacement — net new-customer onboarding hours, KYC per new customer, and RM acquisition effort are all driver-linked (Simanis: at-scale operations include 'replacement of customer churn'). Demand-generation spend (brand &amp; marketing) sits in the HQ overhead pool as a joint cost, not driver-linked to replacement volume.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>• 3. HR &amp; Activity — Step 2: every FTE derived from activity drivers (hours per onboarding, review, renewal…) — nothing is assumed as headcount.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="24" customHeight="1">
+          <t>• The capital charge (cost of equity on allocated capital) is the incumbent analogue of Simanis's start-up-cost amortisation: capital earns its required return inside the steady-state P&amp;L.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="52" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>• 4. Running Costs — the unit's direct running costs plus its share of head-office costs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>• 5. Risk &amp; Capital — Step 3: expected credit losses (PD × LGD), risk-weighted assets, allocated equity, and the required return on it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="91" customHeight="1">
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>• 6. Unit Economics — Steps 4–5: per-product unit costs and revenues on an activity-based costing basis, taken exactly as far as causality runs (the source methodology's own rule: link costs to customers and transactions 'whenever possible'). Costs with real drivers — servicing hours, RM effort per origination, staff-time-driven supervision, per-account and per-facility infrastructure — are attributed to products; genuinely joint costs (brand, exec, finance, platform build) are NOT forced into products but held as an unallocated hurdle that total contribution must clear, with a full-absorption memo showing the source doc's simple-division treatment. Product decisions should run on contribution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="26" customHeight="1">
+          <t>• Out of scope by design: transition paths. The cost and cash shape of moving between steady states — digital migration, maturity glide, behaviour-change programmes and their CAC/incentives — belongs in a scenario layer built ON TOP of this base (comparative statics between two runs of this model, plus a separate transition-cost estimate). The base model never carries scenario logic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>How the tabs map to the methodology</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
+          <t>• Inputs — every assumption in one place, with sources. Edit blue cells; yellow cells are the biggest levers.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="26" customHeight="1">
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>• 8. Org Structure — the whole-bank organisation implied by the model: front-line FTEs from activity drivers × number of centres, head-office FTEs backed out of the per-customer head-office cost allocations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="52" customHeight="1">
+          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>• 9. Flow Register — one row per flow on the operational model map: component type (CP/WP/PP/PartP), core/support/enabling, direction, digital/physical medium, the direct/administrative/managerial roles accountable, and the BIAN service domains. Ends with a BIAN completeness checklist. This is where the map, the ARM and BIAN reconcile.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Colour legend</t>
+          <t>• 2. Revenues — unit revenue per product: interest margins measured against internal funds transfer prices (Bank Rate for floating, + premium for term), plus fees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>• 3. HR &amp; Activity — Step 2: every FTE derived from activity drivers (hours per onboarding, review, renewal…) — nothing is assumed as headcount.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>• 4. Running Costs — the unit's direct running costs plus its share of head-office costs.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="26" customHeight="1">
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>• Blue = hardcoded input (edit these) · Yellow fill = key assumption / sensitivity lever · Black = formula · Green = link to another sheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>Reading the results</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="52" customHeight="1">
+          <t>• 5. Risk &amp; Capital — Step 3: expected credit losses (PD × LGD), risk-weighted assets, allocated equity, and the required return on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="91" customHeight="1">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>• 6. Unit Economics — Steps 4–5: per-product unit costs and revenues on an activity-based costing basis, taken exactly as far as causality runs (the source methodology's own rule: link costs to customers and transactions 'whenever possible'). Costs with real drivers — servicing hours, RM effort per origination, staff-time-driven supervision, per-account and per-facility infrastructure — are attributed to products; genuinely joint costs (brand, exec, finance, platform build) are NOT forced into products but held as an unallocated hurdle that total contribution must clear, with a full-absorption memo showing the source doc's simple-division treatment. Product decisions should run on contribution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="26" customHeight="1">
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="26" customHeight="1">
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>• Deposit products earn the spread between the transfer price and the rate paid; lending earns the customer rate minus the transfer price minus expected losses. Capital-heavy, labour-heavy products (term loans) can show thin or negative economic profit — consistent with the Bank of England's 2026 finding that SME lending earns the lowest product-level returns, driven by impairments and per-borrower servicing costs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="39" customHeight="1">
+          <t>• 8. Org Structure — the whole-bank organisation implied by the model: front-line FTEs from activity drivers × number of centres, head-office FTEs backed out of the per-customer head-office cost allocations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="52" customHeight="1">
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>• Use the cost-driver table on the P&amp;L tab to find leverage points, then trace them to transaction intensity (I) or customer load (L) assumptions on the Inputs tab — e.g. automating underwriting hours, raising RM portfolio size, or shifting servicing to digital.</t>
+          <t>• 9. Flow Register — one row per flow on the operational model map: component type (CP/WP/PP/PartP), core/support/enabling, direction, digital/physical medium, the direct/administrative/managerial roles accountable, and the BIAN service domains. Ends with a BIAN completeness checklist. This is where the map, the ARM and BIAN reconcile.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="3" t="inlineStr">
         <is>
+          <t>Colour legend</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1">
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>• Blue = hardcoded input (edit these) · Yellow fill = key assumption / sensitivity lever · Black = formula · Green = link to another sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Reading the results</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="52" customHeight="1">
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>• Deposit products earn the spread between the transfer price and the rate paid; lending earns the customer rate minus the transfer price minus expected losses. Capital-heavy, labour-heavy products (term loans) can show thin or negative economic profit — consistent with the Bank of England's 2026 finding that SME lending earns the lowest product-level returns, driven by impairments and per-borrower servicing costs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="39" customHeight="1">
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>• Use the cost-driver table on the P&amp;L tab to find leverage points, then trace them to transaction intensity (I) or customer load (L) assumptions on the Inputs tab — e.g. automating underwriting hours, raising RM portfolio size, or shifting servicing to digital.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
           <t>Caveats</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="39" customHeight="1">
-      <c r="B33" s="4" t="inlineStr">
+    <row r="40" ht="39" customHeight="1">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>• Benchmarks are as of August 2026 (Bank Rate 3.75%; BoE effective new SME loan rate ~6.3%; commercial interchange 1.65–1.90%; invoice finance discount base+1–3%). Items marked 'Assumption' are illustrative and should be replaced with your own data.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="65" customHeight="1">
-      <c r="B34" s="4" t="inlineStr">
+    <row r="41" ht="65" customHeight="1">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>• The FTP now carries an explicit liquidity charge (buffer × drag) and a behavioural credit for stable deposits, shown as memos on the Revenues tab; it is still a single curve, not a full behavioural-maturity model. Fraud &amp; payment losses, the FSCS levy, collateral administration &amp; recoveries, and change-the-bank spend are now modelled explicitly. Operational-risk RWA is proxied at 15% of gross income; head-office and change costs are allocated per customer.</t>
         </is>

</xml_diff>

<commit_message>
v1.3: churn replacement as an explicit costed activity
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
+++ b/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B41"/>
+  <dimension ref="B1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -582,7 +582,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MODEL VERSION: v1.2.1 · 21 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
+          <t>MODEL VERSION: v1.3 · 21 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
         </is>
       </c>
     </row>
@@ -593,218 +593,225 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="40" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
+          <t>• v1.3 (21 Aug 2026) — churn replacement is a costed activity end-to-end: new input cac_new (£240 acquisition marketing per new customer won, carved out of the corporate-centre pool — hq_oh £250→£222); driver-linked on tab 4, attributed to the current account (gateway product) on tab 6; 'value of preventing one churn' memo added to tab 6. Raising the churn input now inflates demand-generation cost, not just processing. Central PBT shifts &lt;£1k/unit (carve-out rounding).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
+          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
+          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
           <t>• v1.0 (10 Aug 2026) — first published version: 9 tabs + flow register, FTP with liquidity/behavioural terms, fraud/FSCS/change-the-bank lines, segment-pod LMUs, bridge check.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="3" t="inlineStr">
+    <row r="11">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>What this is</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="39" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="39" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
+          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="39" customHeight="1">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
           <t>• It follows the Simanis / IVE bottom-up methodology ('Running the Right Numbers'): model the last-mile operating unit, derive every cost from activity drivers (transaction intensity I and customer load L), build whole costs, and check the price/margin covers them including a competitive return on capital.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="3" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>What period this models</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="B15" s="4" t="inlineStr">
+    <row r="16" ht="26" customHeight="1">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>• One representative operating year at steady state. Balances are annual averages; rates and volumes are annual. There is no time axis, no ramp and no vintage cohorts — the model is a snapshot, not a forecast.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="52" customHeight="1">
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>• The book is stationary but not free to hold flat: customers churn (12% p.a. input) and the model costs their replacement — net new-customer onboarding hours, KYC per new customer, and RM acquisition effort are all driver-linked (Simanis: at-scale operations include 'replacement of customer churn'). Demand-generation spend (brand &amp; marketing) sits in the HQ overhead pool as a joint cost, not driver-linked to replacement volume.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="26" customHeight="1">
+    <row r="17" ht="78" customHeight="1">
       <c r="B17" s="4" t="inlineStr">
         <is>
+          <t>• The book is stationary but not free to hold flat: customers churn (12% p.a. input) and the model costs their replacement end-to-end — acquisition marketing per new customer won (cac_new, carved from the corporate-centre pool), onboarding hours, KYC per new customer and RM origination effort are all driver-linked (Simanis: at-scale operations include 'replacement of customer churn'). Only residual brand &amp; joint marketing remains pool-costed. The 'value of preventing one churn' memo on tab 6 prices retention: contribution annuity over remaining relationship life + the avoided replacement cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
           <t>• The capital charge (cost of equity on allocated capital) is the incumbent analogue of Simanis's start-up-cost amortisation: capital earns its required return inside the steady-state P&amp;L.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="52" customHeight="1">
-      <c r="B18" s="4" t="inlineStr">
+    <row r="19" ht="52" customHeight="1">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>• Out of scope by design: transition paths. The cost and cash shape of moving between steady states — digital migration, maturity glide, behaviour-change programmes and their CAC/incentives — belongs in a scenario layer built ON TOP of this base (comparative statics between two runs of this model, plus a separate transition-cost estimate). The base model never carries scenario logic.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="3" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>How the tabs map to the methodology</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="B21" s="4" t="inlineStr">
+    <row r="22" ht="24" customHeight="1">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>• Inputs — every assumption in one place, with sources. Edit blue cells; yellow cells are the biggest levers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="26" customHeight="1">
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>• 2. Revenues — unit revenue per product: interest margins measured against internal funds transfer prices (Bank Rate for floating, + premium for term), plus fees.</t>
+          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
       <c r="B24" s="4" t="inlineStr">
         <is>
+          <t>• 2. Revenues — unit revenue per product: interest margins measured against internal funds transfer prices (Bank Rate for floating, + premium for term), plus fees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
           <t>• 3. HR &amp; Activity — Step 2: every FTE derived from activity drivers (hours per onboarding, review, renewal…) — nothing is assumed as headcount.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="B25" s="4" t="inlineStr">
+    <row r="26" ht="24" customHeight="1">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>• 4. Running Costs — the unit's direct running costs plus its share of head-office costs.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="26" customHeight="1">
-      <c r="B26" s="4" t="inlineStr">
+    <row r="27" ht="26" customHeight="1">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>• 5. Risk &amp; Capital — Step 3: expected credit losses (PD × LGD), risk-weighted assets, allocated equity, and the required return on it.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="91" customHeight="1">
-      <c r="B27" s="4" t="inlineStr">
+    <row r="28" ht="91" customHeight="1">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>• 6. Unit Economics — Steps 4–5: per-product unit costs and revenues on an activity-based costing basis, taken exactly as far as causality runs (the source methodology's own rule: link costs to customers and transactions 'whenever possible'). Costs with real drivers — servicing hours, RM effort per origination, staff-time-driven supervision, per-account and per-facility infrastructure — are attributed to products; genuinely joint costs (brand, exec, finance, platform build) are NOT forced into products but held as an unallocated hurdle that total contribution must clear, with a full-absorption memo showing the source doc's simple-division treatment. Product decisions should run on contribution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="26" customHeight="1">
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1">
       <c r="B29" s="4" t="inlineStr">
         <is>
+          <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
           <t>• 8. Org Structure — the whole-bank organisation implied by the model: front-line FTEs from activity drivers × number of centres, head-office FTEs backed out of the per-customer head-office cost allocations.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="52" customHeight="1">
-      <c r="B30" s="4" t="inlineStr">
+    <row r="31" ht="52" customHeight="1">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>• 9. Flow Register — one row per flow on the operational model map: component type (CP/WP/PP/PartP), core/support/enabling, direction, digital/physical medium, the direct/administrative/managerial roles accountable, and the BIAN service domains. Ends with a BIAN completeness checklist. This is where the map, the ARM and BIAN reconcile.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="3" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>Colour legend</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="26" customHeight="1">
-      <c r="B33" s="4" t="inlineStr">
+    <row r="34" ht="26" customHeight="1">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>• Blue = hardcoded input (edit these) · Yellow fill = key assumption / sensitivity lever · Black = formula · Green = link to another sheet.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="3" t="inlineStr">
+    <row r="36">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Reading the results</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="52" customHeight="1">
-      <c r="B36" s="4" t="inlineStr">
+    <row r="37" ht="52" customHeight="1">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>• Deposit products earn the spread between the transfer price and the rate paid; lending earns the customer rate minus the transfer price minus expected losses. Capital-heavy, labour-heavy products (term loans) can show thin or negative economic profit — consistent with the Bank of England's 2026 finding that SME lending earns the lowest product-level returns, driven by impairments and per-borrower servicing costs.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="39" customHeight="1">
-      <c r="B37" s="4" t="inlineStr">
+    <row r="38" ht="39" customHeight="1">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>• Use the cost-driver table on the P&amp;L tab to find leverage points, then trace them to transaction intensity (I) or customer load (L) assumptions on the Inputs tab — e.g. automating underwriting hours, raising RM portfolio size, or shifting servicing to digital.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="B39" s="3" t="inlineStr">
+    <row r="40">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>Caveats</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="39" customHeight="1">
-      <c r="B40" s="4" t="inlineStr">
+    <row r="41" ht="39" customHeight="1">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>• Benchmarks are as of August 2026 (Bank Rate 3.75%; BoE effective new SME loan rate ~6.3%; commercial interchange 1.65–1.90%; invoice finance discount base+1–3%). Items marked 'Assumption' are illustrative and should be replaced with your own data.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="65" customHeight="1">
-      <c r="B41" s="4" t="inlineStr">
+    <row r="42" ht="65" customHeight="1">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>• The FTP now carries an explicit liquidity charge (buffer × drag) and a behavioural credit for stable deposits, shown as memos on the Revenues tab; it is still a single curve, not a full behavioural-maturity model. Fraud &amp; payment losses, the FSCS levy, collateral administration &amp; recoveries, and change-the-bank spend are now modelled explicitly. Operational-risk RWA is proxied at 15% of gross income; head-office and change costs are allocated per customer.</t>
         </is>
@@ -868,7 +875,7 @@
         </is>
       </c>
       <c r="C5" s="47">
-        <f>'Inputs'!$F$171</f>
+        <f>'Inputs'!$F$172</f>
         <v/>
       </c>
     </row>
@@ -879,7 +886,7 @@
         </is>
       </c>
       <c r="C6" s="42">
-        <f>'Inputs'!$F$171*'1. Customers'!$C$4</f>
+        <f>'Inputs'!$F$172*'1. Customers'!$C$4</f>
         <v/>
       </c>
     </row>
@@ -890,7 +897,7 @@
         </is>
       </c>
       <c r="C7" s="44">
-        <f>'Inputs'!$F$171*'1. Customers'!$E$22</f>
+        <f>'Inputs'!$F$172*'1. Customers'!$E$22</f>
         <v/>
       </c>
     </row>
@@ -901,7 +908,7 @@
         </is>
       </c>
       <c r="C8" s="44">
-        <f>'Inputs'!$F$171*'1. Customers'!$E$21</f>
+        <f>'Inputs'!$F$172*'1. Customers'!$E$21</f>
         <v/>
       </c>
     </row>
@@ -912,7 +919,7 @@
         </is>
       </c>
       <c r="C9" s="44">
-        <f>'Inputs'!$F$171*'7. P&amp;L'!$C$6</f>
+        <f>'Inputs'!$F$172*'7. P&amp;L'!$C$6</f>
         <v/>
       </c>
     </row>
@@ -923,7 +930,7 @@
         </is>
       </c>
       <c r="C10" s="44">
-        <f>'Inputs'!$F$171*-'7. P&amp;L'!$C$16</f>
+        <f>'Inputs'!$F$172*-'7. P&amp;L'!$C$16</f>
         <v/>
       </c>
     </row>
@@ -980,7 +987,7 @@
         <v/>
       </c>
       <c r="D14" s="53">
-        <f>C14*'Inputs'!$F$171</f>
+        <f>C14*'Inputs'!$F$172</f>
         <v/>
       </c>
       <c r="E14" s="42">
@@ -1004,7 +1011,7 @@
         <v/>
       </c>
       <c r="D15" s="53">
-        <f>C15*'Inputs'!$F$171</f>
+        <f>C15*'Inputs'!$F$172</f>
         <v/>
       </c>
       <c r="E15" s="42">
@@ -1028,7 +1035,7 @@
         <v/>
       </c>
       <c r="D16" s="53">
-        <f>C16*'Inputs'!$F$171</f>
+        <f>C16*'Inputs'!$F$172</f>
         <v/>
       </c>
       <c r="E16" s="42">
@@ -1052,7 +1059,7 @@
         <v/>
       </c>
       <c r="D17" s="53">
-        <f>C17*'Inputs'!$F$171</f>
+        <f>C17*'Inputs'!$F$172</f>
         <v/>
       </c>
       <c r="E17" s="42">
@@ -1177,7 +1184,7 @@
         </is>
       </c>
       <c r="C28" s="53">
-        <f>'3. HR &amp; Activity'!$D$38*'Inputs'!$F$171/'8. Org Structure'!$C$27</f>
+        <f>'3. HR &amp; Activity'!$D$38*'Inputs'!$F$172/'8. Org Structure'!$C$27</f>
         <v/>
       </c>
       <c r="H28" s="14" t="inlineStr">
@@ -1200,7 +1207,7 @@
         </is>
       </c>
       <c r="C31" s="54">
-        <f>'3. HR &amp; Activity'!$D$39*'Inputs'!$F$171/'Inputs'!$F$27</f>
+        <f>'3. HR &amp; Activity'!$D$39*'Inputs'!$F$172/'Inputs'!$F$27</f>
         <v/>
       </c>
       <c r="H31" s="14" t="inlineStr">
@@ -1293,7 +1300,7 @@
         <v/>
       </c>
       <c r="D38" s="55">
-        <f>'Inputs'!$F$172</f>
+        <f>'Inputs'!$F$173</f>
         <v/>
       </c>
       <c r="E38" s="44">
@@ -1301,7 +1308,7 @@
         <v/>
       </c>
       <c r="F38" s="48">
-        <f>'Inputs'!$F$173</f>
+        <f>'Inputs'!$F$174</f>
         <v/>
       </c>
       <c r="G38" s="22">
@@ -1320,7 +1327,7 @@
         <v/>
       </c>
       <c r="D39" s="55">
-        <f>'Inputs'!$F$174</f>
+        <f>'Inputs'!$F$175</f>
         <v/>
       </c>
       <c r="E39" s="44">
@@ -1328,7 +1335,7 @@
         <v/>
       </c>
       <c r="F39" s="48">
-        <f>'Inputs'!$F$175</f>
+        <f>'Inputs'!$F$176</f>
         <v/>
       </c>
       <c r="G39" s="22">
@@ -1347,7 +1354,7 @@
         <v/>
       </c>
       <c r="D40" s="55">
-        <f>'Inputs'!$F$176</f>
+        <f>'Inputs'!$F$177</f>
         <v/>
       </c>
       <c r="E40" s="44">
@@ -1355,7 +1362,7 @@
         <v/>
       </c>
       <c r="F40" s="48">
-        <f>'Inputs'!$F$177</f>
+        <f>'Inputs'!$F$178</f>
         <v/>
       </c>
       <c r="G40" s="22">
@@ -1617,7 +1624,7 @@
         </is>
       </c>
       <c r="C58" s="17" t="n">
-        <v>0.28</v>
+        <v>0.31</v>
       </c>
       <c r="D58" s="53">
         <f>C58*'8. Org Structure'!$G$40</f>
@@ -1635,7 +1642,7 @@
         </is>
       </c>
       <c r="C59" s="17" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="D59" s="53">
         <f>C59*'8. Org Structure'!$G$40</f>
@@ -1653,7 +1660,7 @@
         </is>
       </c>
       <c r="C60" s="17" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="D60" s="53">
         <f>C60*'8. Org Structure'!$G$40</f>
@@ -1667,11 +1674,11 @@
     <row r="61">
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>Marketing &amp; brand</t>
+          <t>Marketing &amp; brand (residual — acquisition carved out to cac_new)</t>
         </is>
       </c>
       <c r="C61" s="17" t="n">
-        <v>0.22</v>
+        <v>0.12</v>
       </c>
       <c r="D61" s="53">
         <f>C61*'8. Org Structure'!$G$40</f>
@@ -1689,7 +1696,7 @@
         </is>
       </c>
       <c r="C62" s="17" t="n">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="D62" s="53">
         <f>C62*'8. Org Structure'!$G$40</f>
@@ -1707,7 +1714,7 @@
         </is>
       </c>
       <c r="C63" s="17" t="n">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="D63" s="53">
         <f>C63*'8. Org Structure'!$G$40</f>
@@ -1725,7 +1732,7 @@
         </is>
       </c>
       <c r="C64" s="17" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="D64" s="53">
         <f>C64*'8. Org Structure'!$G$40</f>
@@ -1794,7 +1801,7 @@
         </is>
       </c>
       <c r="C70" s="44">
-        <f>'Inputs'!$F$171*'3. HR &amp; Activity'!$H$41+'8. Org Structure'!$E$38+'8. Org Structure'!$E$39+'8. Org Structure'!$E$40</f>
+        <f>'Inputs'!$F$172*'3. HR &amp; Activity'!$H$41+'8. Org Structure'!$E$38+'8. Org Structure'!$E$39+'8. Org Structure'!$E$40</f>
         <v/>
       </c>
     </row>
@@ -3925,7 +3932,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>HQ marketing &amp; brand pool (in hq_oh) + launch marketing — no activity rows; pool-costed</t>
+          <t>Churn-replacement acquisition driver-costed (cac_new × new customers won); residual brand pool (in hq_oh) pool-costed</t>
         </is>
       </c>
     </row>
@@ -4806,7 +4813,7 @@
         </is>
       </c>
       <c r="D70" s="44">
-        <f>SUMPRODUCT(('3. HR &amp; Activity'!$I$11:$I$33&lt;&gt;"")*'3. HR &amp; Activity'!$H$11:$H$33)-('4. Running Costs'!$C$24)</f>
+        <f>SUMPRODUCT(('3. HR &amp; Activity'!$I$11:$I$33&lt;&gt;"")*'3. HR &amp; Activity'!$H$11:$H$33)-('4. Running Costs'!$C$25)</f>
         <v/>
       </c>
       <c r="G70" s="14" t="inlineStr">
@@ -5077,11 +5084,11 @@
         <v/>
       </c>
       <c r="F88" s="44">
-        <f>'6. Unit Economics'!C23</f>
+        <f>'6. Unit Economics'!C24</f>
         <v/>
       </c>
       <c r="G88" s="44">
-        <f>'6. Unit Economics'!C24</f>
+        <f>'6. Unit Economics'!C25</f>
         <v/>
       </c>
     </row>
@@ -5106,11 +5113,11 @@
         <v/>
       </c>
       <c r="F89" s="44">
-        <f>'6. Unit Economics'!D23+'6. Unit Economics'!E23</f>
+        <f>'6. Unit Economics'!D24+'6. Unit Economics'!E24</f>
         <v/>
       </c>
       <c r="G89" s="44">
-        <f>'6. Unit Economics'!D24+'6. Unit Economics'!E24</f>
+        <f>'6. Unit Economics'!D25+'6. Unit Economics'!E25</f>
         <v/>
       </c>
     </row>
@@ -5135,11 +5142,11 @@
         <v/>
       </c>
       <c r="F90" s="44">
-        <f>'6. Unit Economics'!F23+'6. Unit Economics'!G23+'6. Unit Economics'!H23+'6. Unit Economics'!I23</f>
+        <f>'6. Unit Economics'!F24+'6. Unit Economics'!G24+'6. Unit Economics'!H24+'6. Unit Economics'!I24</f>
         <v/>
       </c>
       <c r="G90" s="44">
-        <f>'6. Unit Economics'!F24+'6. Unit Economics'!G24+'6. Unit Economics'!H24+'6. Unit Economics'!I24</f>
+        <f>'6. Unit Economics'!F25+'6. Unit Economics'!G25+'6. Unit Economics'!H25+'6. Unit Economics'!I25</f>
         <v/>
       </c>
     </row>
@@ -5164,11 +5171,11 @@
         <v/>
       </c>
       <c r="F91" s="44">
-        <f>'6. Unit Economics'!J23</f>
+        <f>'6. Unit Economics'!J24</f>
         <v/>
       </c>
       <c r="G91" s="44">
-        <f>'6. Unit Economics'!J24</f>
+        <f>'6. Unit Economics'!J25</f>
         <v/>
       </c>
     </row>
@@ -5193,11 +5200,11 @@
         <v/>
       </c>
       <c r="F92" s="44">
-        <f>'6. Unit Economics'!K23</f>
+        <f>'6. Unit Economics'!K24</f>
         <v/>
       </c>
       <c r="G92" s="44">
-        <f>'6. Unit Economics'!K24</f>
+        <f>'6. Unit Economics'!K25</f>
         <v/>
       </c>
     </row>
@@ -5760,7 +5767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H177"/>
+  <dimension ref="B1:H178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9426,17 +9433,17 @@
     <row r="131">
       <c r="B131" s="10" t="inlineStr">
         <is>
-          <t>Head office: finance, HR, exec, brand &amp; marketing</t>
+          <t>Head office: finance, HR, exec, brand &amp; residual (non-acquisition) marketing</t>
         </is>
       </c>
       <c r="C131" s="25" t="n">
-        <v>250</v>
+        <v>222</v>
       </c>
       <c r="D131" s="28" t="n">
-        <v>250</v>
+        <v>222</v>
       </c>
       <c r="E131" s="28" t="n">
-        <v>250</v>
+        <v>222</v>
       </c>
       <c r="F131" s="26">
         <f>CHOOSE('Inputs'!$C$4,D131,C131,E131)</f>
@@ -9449,7 +9456,7 @@
       </c>
       <c r="H131" s="5" t="inlineStr">
         <is>
-          <t>Assumption: HQ lines calibrated so cost:income ratio lands ~40–50% (specialist SME banks: OakNorth ~26%, Allica ~50%, majors' business banking 50%+)</t>
+          <t>Assumption: HQ lines calibrated so cost:income ratio lands ~40–50% (specialist SME banks: OakNorth ~26%, Allica ~50%, majors' business banking 50%+). v1.3: acquisition-directed marketing (~£28/customer/yr central) carved out into cac_new — the churn-replacement activity</t>
         </is>
       </c>
     </row>
@@ -9563,17 +9570,17 @@
     <row r="136">
       <c r="B136" s="10" t="inlineStr">
         <is>
-          <t>Payments operations &amp; processing — cost per current account</t>
-        </is>
-      </c>
-      <c r="C136" s="27" t="n">
-        <v>120</v>
+          <t>Churn replacement — acquisition marketing per new customer won</t>
+        </is>
+      </c>
+      <c r="C136" s="25" t="n">
+        <v>240</v>
       </c>
       <c r="D136" s="28" t="n">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="E136" s="28" t="n">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="F136" s="26">
         <f>CHOOSE('Inputs'!$C$4,D136,C136,E136)</f>
@@ -9581,29 +9588,29 @@
       </c>
       <c r="G136" s="14" t="inlineStr">
         <is>
-          <t>£/BCA/yr</t>
+          <t>£/new customer</t>
         </is>
       </c>
       <c r="H136" s="5" t="inlineStr">
         <is>
-          <t>Driver: current accounts (the transaction-carrying product). Attributed from the tech pool</t>
+          <t>Driver: net churn replacement (tab 1). Demand-generation spend (media, campaigns, incentives) to win the replacement relationship — carved out of the corporate-centre pool so the churn lever inflates the FULL replacement cost, not just processing. Benchmark: SME CAC £150–500/customer; BCR incentive schemes paid far more. RM origination effort (lending) and onboarding processing (KYC, setup hours) are costed separately</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="B137" s="10" t="inlineStr">
         <is>
-          <t>Core banking system — cost per account of any type</t>
+          <t>Payments operations &amp; processing — cost per current account</t>
         </is>
       </c>
       <c r="C137" s="27" t="n">
-        <v>30</v>
+        <v>120</v>
       </c>
       <c r="D137" s="28" t="n">
-        <v>30</v>
+        <v>120</v>
       </c>
       <c r="E137" s="28" t="n">
-        <v>30</v>
+        <v>120</v>
       </c>
       <c r="F137" s="26">
         <f>CHOOSE('Inputs'!$C$4,D137,C137,E137)</f>
@@ -9611,29 +9618,29 @@
       </c>
       <c r="G137" s="14" t="inlineStr">
         <is>
-          <t>£/account/yr</t>
+          <t>£/BCA/yr</t>
         </is>
       </c>
       <c r="H137" s="5" t="inlineStr">
         <is>
-          <t>Driver: accounts on the ledger. Attributed from the tech pool</t>
+          <t>Driver: current accounts (the transaction-carrying product). Attributed from the tech pool</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="B138" s="10" t="inlineStr">
         <is>
-          <t>Credit systems &amp; portfolio monitoring — cost per credit facility</t>
+          <t>Core banking system — cost per account of any type</t>
         </is>
       </c>
       <c r="C138" s="27" t="n">
-        <v>180</v>
+        <v>30</v>
       </c>
       <c r="D138" s="28" t="n">
-        <v>180</v>
+        <v>30</v>
       </c>
       <c r="E138" s="28" t="n">
-        <v>180</v>
+        <v>30</v>
       </c>
       <c r="F138" s="26">
         <f>CHOOSE('Inputs'!$C$4,D138,C138,E138)</f>
@@ -9641,273 +9648,273 @@
       </c>
       <c r="G138" s="14" t="inlineStr">
         <is>
+          <t>£/account/yr</t>
+        </is>
+      </c>
+      <c r="H138" s="5" t="inlineStr">
+        <is>
+          <t>Driver: accounts on the ledger. Attributed from the tech pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="B139" s="10" t="inlineStr">
+        <is>
+          <t>Credit systems &amp; portfolio monitoring — cost per credit facility</t>
+        </is>
+      </c>
+      <c r="C139" s="27" t="n">
+        <v>180</v>
+      </c>
+      <c r="D139" s="28" t="n">
+        <v>180</v>
+      </c>
+      <c r="E139" s="28" t="n">
+        <v>180</v>
+      </c>
+      <c r="F139" s="26">
+        <f>CHOOSE('Inputs'!$C$4,D139,C139,E139)</f>
+        <v/>
+      </c>
+      <c r="G139" s="14" t="inlineStr">
+        <is>
           <t>£/facility/yr</t>
         </is>
       </c>
-      <c r="H138" s="5" t="inlineStr">
+      <c r="H139" s="5" t="inlineStr">
         <is>
           <t>Driver: live credit facilities. Attributed from the tech pool</t>
         </is>
       </c>
     </row>
-    <row r="139">
-      <c r="B139" s="7" t="inlineStr">
+    <row r="140">
+      <c r="B140" s="7" t="inlineStr">
         <is>
           <t>G3. ADDITIONAL COSTS — FRAUD, LEVIES, CHANGE (the lines unit models often omit)</t>
         </is>
       </c>
-      <c r="C139" s="8" t="inlineStr"/>
-      <c r="D139" s="8" t="inlineStr"/>
-      <c r="E139" s="8" t="inlineStr"/>
-    </row>
-    <row r="140">
-      <c r="B140" s="9" t="inlineStr">
+      <c r="C140" s="8" t="inlineStr"/>
+      <c r="D140" s="8" t="inlineStr"/>
+      <c r="E140" s="8" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="B141" s="9" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C140" s="9" t="inlineStr">
+      <c r="C141" s="9" t="inlineStr">
         <is>
           <t>Central</t>
         </is>
       </c>
-      <c r="D140" s="9" t="inlineStr">
+      <c r="D141" s="9" t="inlineStr">
         <is>
           <t>Pessimistic</t>
         </is>
       </c>
-      <c r="E140" s="9" t="inlineStr">
+      <c r="E141" s="9" t="inlineStr">
         <is>
           <t>Optimistic</t>
         </is>
       </c>
-      <c r="F140" s="9" t="inlineStr">
+      <c r="F141" s="9" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="G140" s="9" t="inlineStr">
+      <c r="G141" s="9" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="H140" s="9" t="inlineStr">
+      <c r="H141" s="9" t="inlineStr">
         <is>
           <t>Source / note</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="B141" s="10" t="inlineStr">
-        <is>
-          <t>Fraud &amp; payment losses (incl. APP reimbursement) per current account</t>
-        </is>
-      </c>
-      <c r="C141" s="25" t="n">
-        <v>45</v>
-      </c>
-      <c r="D141" s="28" t="n">
-        <v>45</v>
-      </c>
-      <c r="E141" s="28" t="n">
-        <v>45</v>
-      </c>
-      <c r="F141" s="26">
-        <f>CHOOSE('Inputs'!$C$4,D141,C141,E141)</f>
-        <v/>
-      </c>
-      <c r="G141" s="14" t="inlineStr">
-        <is>
-          <t>£/BCA/yr</t>
-        </is>
-      </c>
-      <c r="H141" s="5" t="inlineStr">
-        <is>
-          <t>Assumption: net fraud losses incl. mandatory APP scam reimbursement (PSR rules, 2024+); driver = current accounts</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="B142" s="10" t="inlineStr">
         <is>
-          <t>FSCS deposit-protection levy</t>
-        </is>
-      </c>
-      <c r="C142" s="15" t="n">
-        <v>0.0005999999999999999</v>
-      </c>
-      <c r="D142" s="12" t="n">
-        <v>0.0005999999999999999</v>
-      </c>
-      <c r="E142" s="12" t="n">
-        <v>0.0005999999999999999</v>
-      </c>
-      <c r="F142" s="13">
+          <t>Fraud &amp; payment losses (incl. APP reimbursement) per current account</t>
+        </is>
+      </c>
+      <c r="C142" s="25" t="n">
+        <v>45</v>
+      </c>
+      <c r="D142" s="28" t="n">
+        <v>45</v>
+      </c>
+      <c r="E142" s="28" t="n">
+        <v>45</v>
+      </c>
+      <c r="F142" s="26">
         <f>CHOOSE('Inputs'!$C$4,D142,C142,E142)</f>
         <v/>
       </c>
       <c r="G142" s="14" t="inlineStr">
         <is>
-          <t>% of protected deposits</t>
+          <t>£/BCA/yr</t>
         </is>
       </c>
       <c r="H142" s="5" t="inlineStr">
         <is>
-          <t>Assumption: Financial Services Compensation Scheme levy, charged on protected deposit balances</t>
+          <t>Assumption: net fraud losses incl. mandatory APP scam reimbursement (PSR rules, 2024+); driver = current accounts</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="B143" s="10" t="inlineStr">
         <is>
-          <t>Share of deposit balances that are FSCS-protected</t>
-        </is>
-      </c>
-      <c r="C143" s="17" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D143" s="18" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E143" s="18" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="F143" s="19">
+          <t>FSCS deposit-protection levy</t>
+        </is>
+      </c>
+      <c r="C143" s="15" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="D143" s="12" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="E143" s="12" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="F143" s="13">
         <f>CHOOSE('Inputs'!$C$4,D143,C143,E143)</f>
         <v/>
       </c>
       <c r="G143" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% of protected deposits</t>
         </is>
       </c>
       <c r="H143" s="5" t="inlineStr">
         <is>
-          <t>Assumption: FSCS protects up to £85k per depositor; SME balances partly exceed the cap</t>
+          <t>Assumption: Financial Services Compensation Scheme levy, charged on protected deposit balances</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="B144" s="10" t="inlineStr">
         <is>
+          <t>Share of deposit balances that are FSCS-protected</t>
+        </is>
+      </c>
+      <c r="C144" s="17" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D144" s="18" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E144" s="18" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F144" s="19">
+        <f>CHOOSE('Inputs'!$C$4,D144,C144,E144)</f>
+        <v/>
+      </c>
+      <c r="G144" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H144" s="5" t="inlineStr">
+        <is>
+          <t>Assumption: FSCS protects up to £85k per depositor; SME balances partly exceed the cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="B145" s="10" t="inlineStr">
+        <is>
           <t>Change-the-bank / transformation spend per customer</t>
         </is>
       </c>
-      <c r="C144" s="25" t="n">
+      <c r="C145" s="25" t="n">
         <v>120</v>
       </c>
-      <c r="D144" s="28" t="n">
+      <c r="D145" s="28" t="n">
         <v>120</v>
       </c>
-      <c r="E144" s="28" t="n">
+      <c r="E145" s="28" t="n">
         <v>120</v>
       </c>
-      <c r="F144" s="26">
-        <f>CHOOSE('Inputs'!$C$4,D144,C144,E144)</f>
-        <v/>
-      </c>
-      <c r="G144" s="14" t="inlineStr">
+      <c r="F145" s="26">
+        <f>CHOOSE('Inputs'!$C$4,D145,C145,E145)</f>
+        <v/>
+      </c>
+      <c r="G145" s="14" t="inlineStr">
         <is>
           <t>£/customer/yr</t>
         </is>
       </c>
-      <c r="H144" s="5" t="inlineStr">
+      <c r="H145" s="5" t="inlineStr">
         <is>
           <t>Assumption: ongoing regulatory change + tech transformation, ~10–20% of a bank cost base; held as a portfolio hurdle, not attributed to products</t>
         </is>
       </c>
     </row>
-    <row r="145">
-      <c r="B145" s="7" t="inlineStr">
+    <row r="146">
+      <c r="B146" s="7" t="inlineStr">
         <is>
           <t>G4. SEGMENT GRANULARITY — share of each product's units held by RM-MANAGED customers</t>
         </is>
       </c>
-      <c r="C145" s="8" t="inlineStr"/>
-      <c r="D145" s="8" t="inlineStr"/>
-      <c r="E145" s="8" t="inlineStr"/>
-    </row>
-    <row r="146">
-      <c r="B146" s="9" t="inlineStr">
+      <c r="C146" s="8" t="inlineStr"/>
+      <c r="D146" s="8" t="inlineStr"/>
+      <c r="E146" s="8" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="B147" s="9" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C146" s="9" t="inlineStr">
+      <c r="C147" s="9" t="inlineStr">
         <is>
           <t>Central</t>
         </is>
       </c>
-      <c r="D146" s="9" t="inlineStr">
+      <c r="D147" s="9" t="inlineStr">
         <is>
           <t>Pessimistic</t>
         </is>
       </c>
-      <c r="E146" s="9" t="inlineStr">
+      <c r="E147" s="9" t="inlineStr">
         <is>
           <t>Optimistic</t>
         </is>
       </c>
-      <c r="F146" s="9" t="inlineStr">
+      <c r="F147" s="9" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="G146" s="9" t="inlineStr">
+      <c r="G147" s="9" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="H146" s="9" t="inlineStr">
+      <c r="H147" s="9" t="inlineStr">
         <is>
           <t>Source / note</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="B147" s="10" t="inlineStr">
-        <is>
-          <t>Current accounts — RM-held share</t>
-        </is>
-      </c>
-      <c r="C147" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D147" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E147" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F147" s="19">
-        <f>CHOOSE('Inputs'!$C$4,D147,C147,E147)</f>
-        <v/>
-      </c>
-      <c r="G147" s="14" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="H147" s="5" t="inlineStr">
-        <is>
-          <t>Equals pct_rm (every customer holds a BCA). Scenario dimension: shift with channel moves</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="B148" s="10" t="inlineStr">
         <is>
-          <t>Instant savings — RM-held share</t>
+          <t>Current accounts — RM-held share</t>
         </is>
       </c>
       <c r="C148" s="17" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="D148" s="18" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="E148" s="18" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="F148" s="19">
         <f>CHOOSE('Inputs'!$C$4,D148,C148,E148)</f>
@@ -9920,24 +9927,24 @@
       </c>
       <c r="H148" s="5" t="inlineStr">
         <is>
-          <t>Assumption — for scenario building; validate from segment data</t>
+          <t>Equals pct_rm (every customer holds a BCA). Scenario dimension: shift with channel moves</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="B149" s="10" t="inlineStr">
         <is>
-          <t>Notice &amp; fixed deposits — RM-held share</t>
+          <t>Instant savings — RM-held share</t>
         </is>
       </c>
       <c r="C149" s="17" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="D149" s="18" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="E149" s="18" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="F149" s="19">
         <f>CHOOSE('Inputs'!$C$4,D149,C149,E149)</f>
@@ -9950,24 +9957,24 @@
       </c>
       <c r="H149" s="5" t="inlineStr">
         <is>
-          <t>Assumption</t>
+          <t>Assumption — for scenario building; validate from segment data</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="B150" s="10" t="inlineStr">
         <is>
-          <t>Overdrafts — RM-held share</t>
+          <t>Notice &amp; fixed deposits — RM-held share</t>
         </is>
       </c>
       <c r="C150" s="17" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="D150" s="18" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E150" s="18" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="F150" s="19">
         <f>CHOOSE('Inputs'!$C$4,D150,C150,E150)</f>
@@ -9987,17 +9994,17 @@
     <row r="151">
       <c r="B151" s="10" t="inlineStr">
         <is>
-          <t>Term loans — RM-held share</t>
+          <t>Overdrafts — RM-held share</t>
         </is>
       </c>
       <c r="C151" s="17" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="D151" s="18" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="E151" s="18" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="F151" s="19">
         <f>CHOOSE('Inputs'!$C$4,D151,C151,E151)</f>
@@ -10010,14 +10017,14 @@
       </c>
       <c r="H151" s="5" t="inlineStr">
         <is>
-          <t>Consistent with rm_lend_share (RM customers are the larger borrowers)</t>
+          <t>Assumption</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="B152" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — RM-held share</t>
+          <t>Term loans — RM-held share</t>
         </is>
       </c>
       <c r="C152" s="17" t="n">
@@ -10040,24 +10047,24 @@
       </c>
       <c r="H152" s="5" t="inlineStr">
         <is>
-          <t>Assumption</t>
+          <t>Consistent with rm_lend_share (RM customers are the larger borrowers)</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="B153" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — RM-held share</t>
+          <t>Asset finance — RM-held share</t>
         </is>
       </c>
       <c r="C153" s="17" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="D153" s="18" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="E153" s="18" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="F153" s="19">
         <f>CHOOSE('Inputs'!$C$4,D153,C153,E153)</f>
@@ -10070,24 +10077,24 @@
       </c>
       <c r="H153" s="5" t="inlineStr">
         <is>
-          <t>Assumption — consultative product</t>
+          <t>Assumption</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="B154" s="10" t="inlineStr">
         <is>
-          <t>Business cards — RM-held share</t>
+          <t>Invoice finance — RM-held share</t>
         </is>
       </c>
       <c r="C154" s="17" t="n">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D154" s="18" t="n">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="E154" s="18" t="n">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="F154" s="19">
         <f>CHOOSE('Inputs'!$C$4,D154,C154,E154)</f>
@@ -10100,24 +10107,24 @@
       </c>
       <c r="H154" s="5" t="inlineStr">
         <is>
-          <t>Assumption</t>
+          <t>Assumption — consultative product</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="B155" s="10" t="inlineStr">
         <is>
-          <t>Payments &amp; FX users — RM-held share</t>
+          <t>Business cards — RM-held share</t>
         </is>
       </c>
       <c r="C155" s="17" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="D155" s="18" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E155" s="18" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="F155" s="19">
         <f>CHOOSE('Inputs'!$C$4,D155,C155,E155)</f>
@@ -10135,96 +10142,96 @@
       </c>
     </row>
     <row r="156">
-      <c r="B156" s="7" t="inlineStr">
+      <c r="B156" s="10" t="inlineStr">
+        <is>
+          <t>Payments &amp; FX users — RM-held share</t>
+        </is>
+      </c>
+      <c r="C156" s="17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D156" s="18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E156" s="18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F156" s="19">
+        <f>CHOOSE('Inputs'!$C$4,D156,C156,E156)</f>
+        <v/>
+      </c>
+      <c r="G156" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H156" s="5" t="inlineStr">
+        <is>
+          <t>Assumption</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="B157" s="7" t="inlineStr">
         <is>
           <t>H. RM SALES EFFORT PER ORIGINATION (RMs are a sales force, not a service cost)</t>
         </is>
       </c>
-      <c r="C156" s="8" t="inlineStr"/>
-      <c r="D156" s="8" t="inlineStr"/>
-      <c r="E156" s="8" t="inlineStr"/>
-    </row>
-    <row r="157">
-      <c r="B157" s="9" t="inlineStr">
+      <c r="C157" s="8" t="inlineStr"/>
+      <c r="D157" s="8" t="inlineStr"/>
+      <c r="E157" s="8" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="B158" s="9" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C157" s="9" t="inlineStr">
+      <c r="C158" s="9" t="inlineStr">
         <is>
           <t>Central</t>
         </is>
       </c>
-      <c r="D157" s="9" t="inlineStr">
+      <c r="D158" s="9" t="inlineStr">
         <is>
           <t>Pessimistic</t>
         </is>
       </c>
-      <c r="E157" s="9" t="inlineStr">
+      <c r="E158" s="9" t="inlineStr">
         <is>
           <t>Optimistic</t>
         </is>
       </c>
-      <c r="F157" s="9" t="inlineStr">
+      <c r="F158" s="9" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="G157" s="9" t="inlineStr">
+      <c r="G158" s="9" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="H157" s="9" t="inlineStr">
+      <c r="H158" s="9" t="inlineStr">
         <is>
           <t>Source / note</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="B158" s="10" t="inlineStr">
-        <is>
-          <t>Relative RM effort — per new term loan</t>
-        </is>
-      </c>
-      <c r="C158" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D158" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="E158" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="F158" s="37">
-        <f>CHOOSE('Inputs'!$C$4,D158,C158,E158)</f>
-        <v/>
-      </c>
-      <c r="G158" s="14" t="inlineStr">
-        <is>
-          <t>index</t>
-        </is>
-      </c>
-      <c r="H158" s="5" t="inlineStr">
-        <is>
-          <t>Assumption: RM cost is customer-acquisition cost, attributed per origination by relative effort</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="B159" s="10" t="inlineStr">
         <is>
-          <t>Relative RM effort — per new asset finance agreement</t>
+          <t>Relative RM effort — per new term loan</t>
         </is>
       </c>
       <c r="C159" s="35" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D159" s="36" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E159" s="36" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F159" s="37">
         <f>CHOOSE('Inputs'!$C$4,D159,C159,E159)</f>
@@ -10237,24 +10244,24 @@
       </c>
       <c r="H159" s="5" t="inlineStr">
         <is>
-          <t>Assumption: more automated sale</t>
+          <t>Assumption: RM cost is customer-acquisition cost, attributed per origination by relative effort</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="B160" s="10" t="inlineStr">
         <is>
-          <t>Relative RM effort — per new invoice finance client</t>
+          <t>Relative RM effort — per new asset finance agreement</t>
         </is>
       </c>
       <c r="C160" s="35" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="D160" s="36" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="E160" s="36" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="F160" s="37">
         <f>CHOOSE('Inputs'!$C$4,D160,C160,E160)</f>
@@ -10267,24 +10274,24 @@
       </c>
       <c r="H160" s="5" t="inlineStr">
         <is>
-          <t>Assumption: complex, consultative sale</t>
+          <t>Assumption: more automated sale</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="B161" s="10" t="inlineStr">
         <is>
-          <t>Relative RM effort — per overdraft renewal</t>
-        </is>
-      </c>
-      <c r="C161" s="39" t="n">
-        <v>0.25</v>
+          <t>Relative RM effort — per new invoice finance client</t>
+        </is>
+      </c>
+      <c r="C161" s="35" t="n">
+        <v>1.5</v>
       </c>
       <c r="D161" s="36" t="n">
-        <v>0.25</v>
+        <v>1.5</v>
       </c>
       <c r="E161" s="36" t="n">
-        <v>0.25</v>
+        <v>1.5</v>
       </c>
       <c r="F161" s="37">
         <f>CHOOSE('Inputs'!$C$4,D161,C161,E161)</f>
@@ -10297,54 +10304,54 @@
       </c>
       <c r="H161" s="5" t="inlineStr">
         <is>
-          <t>Assumption: annual renewals; a key automation lever</t>
+          <t>Assumption: complex, consultative sale</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="B162" s="10" t="inlineStr">
         <is>
-          <t>RM time — ORIGINATE (sales, attributed per origination)</t>
-        </is>
-      </c>
-      <c r="C162" s="17" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D162" s="18" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E162" s="18" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F162" s="19">
+          <t>Relative RM effort — per overdraft renewal</t>
+        </is>
+      </c>
+      <c r="C162" s="39" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D162" s="36" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E162" s="36" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F162" s="37">
         <f>CHOOSE('Inputs'!$C$4,D162,C162,E162)</f>
         <v/>
       </c>
       <c r="G162" s="14" t="inlineStr">
         <is>
-          <t>% of RM time</t>
+          <t>index</t>
         </is>
       </c>
       <c r="H162" s="5" t="inlineStr">
         <is>
-          <t>The three RM activities work as a system: stewardship generates the signals origination targets; origination builds the book stewardship protects; defence preserves the relationships that carry future originations</t>
+          <t>Assumption: annual renewals; a key automation lever</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="B163" s="10" t="inlineStr">
         <is>
-          <t>RM time — STEWARD (credit stewardship of the covered book)</t>
+          <t>RM time — ORIGINATE (sales, attributed per origination)</t>
         </is>
       </c>
       <c r="C163" s="17" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="D163" s="18" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="E163" s="18" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="F163" s="19">
         <f>CHOOSE('Inputs'!$C$4,D163,C163,E163)</f>
@@ -10357,24 +10364,24 @@
       </c>
       <c r="H163" s="5" t="inlineStr">
         <is>
-          <t>Attributed to lending products pro-rata covered balances; pays back through lower PDs</t>
+          <t>The three RM activities work as a system: stewardship generates the signals origination targets; origination builds the book stewardship protects; defence preserves the relationships that carry future originations</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="B164" s="10" t="inlineStr">
         <is>
-          <t>RM time — DEFEND (retention at contested moments)</t>
+          <t>RM time — STEWARD (credit stewardship of the covered book)</t>
         </is>
       </c>
       <c r="C164" s="17" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="D164" s="18" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="E164" s="18" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="F164" s="19">
         <f>CHOOSE('Inputs'!$C$4,D164,C164,E164)</f>
@@ -10387,24 +10394,24 @@
       </c>
       <c r="H164" s="5" t="inlineStr">
         <is>
-          <t>Held at centre level as tested retention spend — the three shares must sum to 100%</t>
+          <t>Attributed to lending products pro-rata covered balances; pays back through lower PDs</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="B165" s="10" t="inlineStr">
         <is>
-          <t>Share of lending balances held by RM-managed customers</t>
+          <t>RM time — DEFEND (retention at contested moments)</t>
         </is>
       </c>
       <c r="C165" s="17" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="D165" s="18" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="E165" s="18" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="F165" s="19">
         <f>CHOOSE('Inputs'!$C$4,D165,C165,E165)</f>
@@ -10412,29 +10419,29 @@
       </c>
       <c r="G165" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% of RM time</t>
         </is>
       </c>
       <c r="H165" s="5" t="inlineStr">
         <is>
-          <t>Assumption: RM-managed customers are the larger borrowers</t>
+          <t>Held at centre level as tested retention spend — the three shares must sum to 100%</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="B166" s="10" t="inlineStr">
         <is>
-          <t>Stewardship effect: relative PD reduction on RM-covered balances</t>
-        </is>
-      </c>
-      <c r="C166" s="23" t="n">
-        <v>0.2</v>
+          <t>Share of lending balances held by RM-managed customers</t>
+        </is>
+      </c>
+      <c r="C166" s="17" t="n">
+        <v>0.6</v>
       </c>
       <c r="D166" s="18" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="E166" s="18" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="F166" s="19">
         <f>CHOOSE('Inputs'!$C$4,D166,C166,E166)</f>
@@ -10447,24 +10454,24 @@
       </c>
       <c r="H166" s="5" t="inlineStr">
         <is>
-          <t>Relationship-lending evidence: soft information and early warning lower default rates; validate against covered vs uncovered book performance</t>
+          <t>Assumption: RM-managed customers are the larger borrowers</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="B167" s="10" t="inlineStr">
         <is>
-          <t>Defence effect: relative churn reduction among RM-managed customers</t>
+          <t>Stewardship effect: relative PD reduction on RM-covered balances</t>
         </is>
       </c>
       <c r="C167" s="23" t="n">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="D167" s="18" t="n">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="E167" s="18" t="n">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="F167" s="19">
         <f>CHOOSE('Inputs'!$C$4,D167,C167,E167)</f>
@@ -10477,292 +10484,322 @@
       </c>
       <c r="H167" s="5" t="inlineStr">
         <is>
-          <t>Must be validated with holdout tests — pay only for incremental saves</t>
+          <t>Relationship-lending evidence: soft information and early warning lower default rates; validate against covered vs uncovered book performance</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="B168" s="10" t="inlineStr">
         <is>
+          <t>Defence effect: relative churn reduction among RM-managed customers</t>
+        </is>
+      </c>
+      <c r="C168" s="23" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D168" s="18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E168" s="18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F168" s="19">
+        <f>CHOOSE('Inputs'!$C$4,D168,C168,E168)</f>
+        <v/>
+      </c>
+      <c r="G168" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H168" s="5" t="inlineStr">
+        <is>
+          <t>Must be validated with holdout tests — pay only for incremental saves</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="B169" s="10" t="inlineStr">
+        <is>
           <t>Expected remaining relationship life of a defended customer</t>
         </is>
       </c>
-      <c r="C168" s="20" t="n">
+      <c r="C169" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="D168" s="21" t="n">
+      <c r="D169" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="E168" s="21" t="n">
+      <c r="E169" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="F168" s="22">
-        <f>CHOOSE('Inputs'!$C$4,D168,C168,E168)</f>
-        <v/>
-      </c>
-      <c r="G168" s="14" t="inlineStr">
+      <c r="F169" s="22">
+        <f>CHOOSE('Inputs'!$C$4,D169,C169,E169)</f>
+        <v/>
+      </c>
+      <c r="G169" s="14" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="H168" s="5" t="inlineStr">
+      <c r="H169" s="5" t="inlineStr">
         <is>
           <t>A saved customer is an annuity, not one year of contribution</t>
         </is>
       </c>
     </row>
-    <row r="169">
-      <c r="B169" s="7" t="inlineStr">
+    <row r="170">
+      <c r="B170" s="7" t="inlineStr">
         <is>
           <t>I. ORGANISATION AT SCALE (drives the Org Structure tab)</t>
         </is>
       </c>
-      <c r="C169" s="8" t="inlineStr"/>
-      <c r="D169" s="8" t="inlineStr"/>
-      <c r="E169" s="8" t="inlineStr"/>
-    </row>
-    <row r="170">
-      <c r="B170" s="9" t="inlineStr">
+      <c r="C170" s="8" t="inlineStr"/>
+      <c r="D170" s="8" t="inlineStr"/>
+      <c r="E170" s="8" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="B171" s="9" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C170" s="9" t="inlineStr">
+      <c r="C171" s="9" t="inlineStr">
         <is>
           <t>Central</t>
         </is>
       </c>
-      <c r="D170" s="9" t="inlineStr">
+      <c r="D171" s="9" t="inlineStr">
         <is>
           <t>Pessimistic</t>
         </is>
       </c>
-      <c r="E170" s="9" t="inlineStr">
+      <c r="E171" s="9" t="inlineStr">
         <is>
           <t>Optimistic</t>
         </is>
       </c>
-      <c r="F170" s="9" t="inlineStr">
+      <c r="F171" s="9" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="G170" s="9" t="inlineStr">
+      <c r="G171" s="9" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="H170" s="9" t="inlineStr">
+      <c r="H171" s="9" t="inlineStr">
         <is>
           <t>Source / note</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="B171" s="10" t="inlineStr">
-        <is>
-          <t>Regional business centres at scale</t>
-        </is>
-      </c>
-      <c r="C171" s="24" t="n">
-        <v>300</v>
-      </c>
-      <c r="D171" s="21" t="n">
-        <v>300</v>
-      </c>
-      <c r="E171" s="21" t="n">
-        <v>300</v>
-      </c>
-      <c r="F171" s="22">
-        <f>CHOOSE('Inputs'!$C$4,D171,C171,E171)</f>
-        <v/>
-      </c>
-      <c r="G171" s="14" t="inlineStr">
-        <is>
-          <t>centres</t>
-        </is>
-      </c>
-      <c r="H171" s="5" t="inlineStr">
-        <is>
-          <t>Set for 900,000 current-account customers (300 × 3,000). Note: per-customer head-office allocations are held flat — conservative, as central costs per customer typically fall at this scale</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="B172" s="10" t="inlineStr">
         <is>
-          <t>Technology &amp; central ops — staff share of allocated cost</t>
-        </is>
-      </c>
-      <c r="C172" s="17" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="D172" s="18" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="E172" s="18" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F172" s="19">
+          <t>Regional business centres at scale</t>
+        </is>
+      </c>
+      <c r="C172" s="24" t="n">
+        <v>300</v>
+      </c>
+      <c r="D172" s="21" t="n">
+        <v>300</v>
+      </c>
+      <c r="E172" s="21" t="n">
+        <v>300</v>
+      </c>
+      <c r="F172" s="22">
         <f>CHOOSE('Inputs'!$C$4,D172,C172,E172)</f>
         <v/>
       </c>
       <c r="G172" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>centres</t>
         </is>
       </c>
       <c r="H172" s="5" t="inlineStr">
         <is>
-          <t>Assumption: remainder is software licences, hosting, card scheme &amp; processing fees</t>
+          <t>Set for 900,000 current-account customers (300 × 3,000). Note: per-customer head-office allocations are held flat — conservative, as central costs per customer typically fall at this scale</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="B173" s="10" t="inlineStr">
         <is>
-          <t>Technology &amp; central ops — average loaded cost per FTE</t>
-        </is>
-      </c>
-      <c r="C173" s="27" t="n">
-        <v>80000</v>
-      </c>
-      <c r="D173" s="28" t="n">
-        <v>80000</v>
-      </c>
-      <c r="E173" s="28" t="n">
-        <v>80000</v>
-      </c>
-      <c r="F173" s="26">
+          <t>Technology &amp; central ops — staff share of allocated cost</t>
+        </is>
+      </c>
+      <c r="C173" s="17" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D173" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E173" s="18" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F173" s="19">
         <f>CHOOSE('Inputs'!$C$4,D173,C173,E173)</f>
         <v/>
       </c>
       <c r="G173" s="14" t="inlineStr">
         <is>
-          <t>£/FTE/yr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="H173" s="5" t="inlineStr">
         <is>
-          <t>Assumption: salary + on-costs (tech roles skew senior)</t>
+          <t>Assumption: remainder is software licences, hosting, card scheme &amp; processing fees</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="B174" s="10" t="inlineStr">
         <is>
-          <t>Risk, compliance &amp; audit — staff share of allocated cost</t>
-        </is>
-      </c>
-      <c r="C174" s="17" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D174" s="18" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E174" s="18" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="F174" s="19">
+          <t>Technology &amp; central ops — average loaded cost per FTE</t>
+        </is>
+      </c>
+      <c r="C174" s="27" t="n">
+        <v>80000</v>
+      </c>
+      <c r="D174" s="28" t="n">
+        <v>80000</v>
+      </c>
+      <c r="E174" s="28" t="n">
+        <v>80000</v>
+      </c>
+      <c r="F174" s="26">
         <f>CHOOSE('Inputs'!$C$4,D174,C174,E174)</f>
         <v/>
       </c>
       <c r="G174" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/FTE/yr</t>
         </is>
       </c>
       <c r="H174" s="5" t="inlineStr">
         <is>
-          <t>Assumption: remainder is data, tools, professional fees</t>
+          <t>Assumption: salary + on-costs (tech roles skew senior)</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="B175" s="10" t="inlineStr">
         <is>
-          <t>Risk, compliance &amp; audit — average loaded cost per FTE</t>
-        </is>
-      </c>
-      <c r="C175" s="27" t="n">
-        <v>75000</v>
-      </c>
-      <c r="D175" s="28" t="n">
-        <v>75000</v>
-      </c>
-      <c r="E175" s="28" t="n">
-        <v>75000</v>
-      </c>
-      <c r="F175" s="26">
+          <t>Risk, compliance &amp; audit — staff share of allocated cost</t>
+        </is>
+      </c>
+      <c r="C175" s="17" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D175" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E175" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F175" s="19">
         <f>CHOOSE('Inputs'!$C$4,D175,C175,E175)</f>
         <v/>
       </c>
       <c r="G175" s="14" t="inlineStr">
         <is>
-          <t>£/FTE/yr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="H175" s="5" t="inlineStr">
         <is>
-          <t>Assumption</t>
+          <t>Assumption: remainder is data, tools, professional fees</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="B176" s="10" t="inlineStr">
         <is>
-          <t>Corporate centre — staff share of allocated cost</t>
-        </is>
-      </c>
-      <c r="C176" s="17" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D176" s="18" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E176" s="18" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="F176" s="19">
+          <t>Risk, compliance &amp; audit — average loaded cost per FTE</t>
+        </is>
+      </c>
+      <c r="C176" s="27" t="n">
+        <v>75000</v>
+      </c>
+      <c r="D176" s="28" t="n">
+        <v>75000</v>
+      </c>
+      <c r="E176" s="28" t="n">
+        <v>75000</v>
+      </c>
+      <c r="F176" s="26">
         <f>CHOOSE('Inputs'!$C$4,D176,C176,E176)</f>
         <v/>
       </c>
       <c r="G176" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/FTE/yr</t>
         </is>
       </c>
       <c r="H176" s="5" t="inlineStr">
         <is>
-          <t>Assumption: remainder is brand &amp; media spend, audit &amp; professional fees, facilities</t>
+          <t>Assumption</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="B177" s="10" t="inlineStr">
         <is>
+          <t>Corporate centre — staff share of allocated cost</t>
+        </is>
+      </c>
+      <c r="C177" s="17" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D177" s="18" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E177" s="18" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F177" s="19">
+        <f>CHOOSE('Inputs'!$C$4,D177,C177,E177)</f>
+        <v/>
+      </c>
+      <c r="G177" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="H177" s="5" t="inlineStr">
+        <is>
+          <t>Assumption: remainder is brand &amp; media spend, audit &amp; professional fees, facilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="B178" s="10" t="inlineStr">
+        <is>
           <t>Corporate centre — average loaded cost per FTE</t>
         </is>
       </c>
-      <c r="C177" s="27" t="n">
+      <c r="C178" s="27" t="n">
         <v>75000</v>
       </c>
-      <c r="D177" s="28" t="n">
+      <c r="D178" s="28" t="n">
         <v>75000</v>
       </c>
-      <c r="E177" s="28" t="n">
+      <c r="E178" s="28" t="n">
         <v>75000</v>
       </c>
-      <c r="F177" s="26">
-        <f>CHOOSE('Inputs'!$C$4,D177,C177,E177)</f>
-        <v/>
-      </c>
-      <c r="G177" s="14" t="inlineStr">
+      <c r="F178" s="26">
+        <f>CHOOSE('Inputs'!$C$4,D178,C178,E178)</f>
+        <v/>
+      </c>
+      <c r="G178" s="14" t="inlineStr">
         <is>
           <t>£/FTE/yr</t>
         </is>
       </c>
-      <c r="H177" s="5" t="inlineStr">
+      <c r="H178" s="5" t="inlineStr">
         <is>
           <t>Assumption</t>
         </is>
@@ -10849,7 +10886,7 @@
         </is>
       </c>
       <c r="C7" s="42">
-        <f>'1. Customers'!$C$5*'Inputs'!$F$23*'Inputs'!$F$167</f>
+        <f>'1. Customers'!$C$5*'Inputs'!$F$23*'Inputs'!$F$168</f>
         <v/>
       </c>
       <c r="E7" s="14" t="inlineStr">
@@ -10951,7 +10988,7 @@
         </is>
       </c>
       <c r="G12" s="42">
-        <f>C12*'Inputs'!$F$147</f>
+        <f>C12*'Inputs'!$F$148</f>
         <v/>
       </c>
       <c r="H12" s="42">
@@ -10979,7 +11016,7 @@
       </c>
       <c r="F13" s="14" t="inlineStr"/>
       <c r="G13" s="42">
-        <f>C13*'Inputs'!$F$148</f>
+        <f>C13*'Inputs'!$F$149</f>
         <v/>
       </c>
       <c r="H13" s="42">
@@ -11007,7 +11044,7 @@
       </c>
       <c r="F14" s="14" t="inlineStr"/>
       <c r="G14" s="42">
-        <f>C14*'Inputs'!$F$149</f>
+        <f>C14*'Inputs'!$F$150</f>
         <v/>
       </c>
       <c r="H14" s="42">
@@ -11039,7 +11076,7 @@
         </is>
       </c>
       <c r="G15" s="42">
-        <f>C15*'Inputs'!$F$150</f>
+        <f>C15*'Inputs'!$F$151</f>
         <v/>
       </c>
       <c r="H15" s="42">
@@ -11067,7 +11104,7 @@
       </c>
       <c r="F16" s="14" t="inlineStr"/>
       <c r="G16" s="42">
-        <f>C16*'Inputs'!$F$151</f>
+        <f>C16*'Inputs'!$F$152</f>
         <v/>
       </c>
       <c r="H16" s="42">
@@ -11095,7 +11132,7 @@
       </c>
       <c r="F17" s="14" t="inlineStr"/>
       <c r="G17" s="42">
-        <f>C17*'Inputs'!$F$152</f>
+        <f>C17*'Inputs'!$F$153</f>
         <v/>
       </c>
       <c r="H17" s="42">
@@ -11127,7 +11164,7 @@
         </is>
       </c>
       <c r="G18" s="42">
-        <f>C18*'Inputs'!$F$153</f>
+        <f>C18*'Inputs'!$F$154</f>
         <v/>
       </c>
       <c r="H18" s="42">
@@ -11159,7 +11196,7 @@
         </is>
       </c>
       <c r="G19" s="42">
-        <f>C19*'Inputs'!$F$154</f>
+        <f>C19*'Inputs'!$F$155</f>
         <v/>
       </c>
       <c r="H19" s="42">
@@ -11191,7 +11228,7 @@
         </is>
       </c>
       <c r="G20" s="42">
-        <f>C20*'Inputs'!$F$155</f>
+        <f>C20*'Inputs'!$F$156</f>
         <v/>
       </c>
       <c r="H20" s="42">
@@ -13365,11 +13402,11 @@
         </is>
       </c>
       <c r="D46" s="55">
-        <f>'Inputs'!$F$162</f>
+        <f>'Inputs'!$F$163</f>
         <v/>
       </c>
       <c r="H46" s="44">
-        <f>'3. HR &amp; Activity'!$H$37*'Inputs'!$F$162</f>
+        <f>'3. HR &amp; Activity'!$H$37*'Inputs'!$F$163</f>
         <v/>
       </c>
     </row>
@@ -13380,11 +13417,11 @@
         </is>
       </c>
       <c r="D47" s="55">
-        <f>'Inputs'!$F$163</f>
+        <f>'Inputs'!$F$164</f>
         <v/>
       </c>
       <c r="H47" s="44">
-        <f>'3. HR &amp; Activity'!$H$37*'Inputs'!$F$163</f>
+        <f>'3. HR &amp; Activity'!$H$37*'Inputs'!$F$164</f>
         <v/>
       </c>
     </row>
@@ -13395,11 +13432,11 @@
         </is>
       </c>
       <c r="D48" s="55">
-        <f>'Inputs'!$F$164</f>
+        <f>'Inputs'!$F$165</f>
         <v/>
       </c>
       <c r="H48" s="44">
-        <f>'3. HR &amp; Activity'!$H$37*'Inputs'!$F$164</f>
+        <f>'3. HR &amp; Activity'!$H$37*'Inputs'!$F$165</f>
         <v/>
       </c>
     </row>
@@ -13460,7 +13497,7 @@
         <v/>
       </c>
       <c r="E52" s="56">
-        <f>'Inputs'!$F$158</f>
+        <f>'Inputs'!$F$159</f>
         <v/>
       </c>
       <c r="F52" s="53">
@@ -13487,7 +13524,7 @@
         <v/>
       </c>
       <c r="E53" s="56">
-        <f>'Inputs'!$F$159</f>
+        <f>'Inputs'!$F$160</f>
         <v/>
       </c>
       <c r="F53" s="53">
@@ -13514,7 +13551,7 @@
         <v/>
       </c>
       <c r="E54" s="56">
-        <f>'Inputs'!$F$160</f>
+        <f>'Inputs'!$F$161</f>
         <v/>
       </c>
       <c r="F54" s="53">
@@ -13541,7 +13578,7 @@
         <v/>
       </c>
       <c r="E55" s="56">
-        <f>'Inputs'!$F$161</f>
+        <f>'Inputs'!$F$162</f>
         <v/>
       </c>
       <c r="F55" s="53">
@@ -13725,7 +13762,7 @@
         </is>
       </c>
       <c r="G65" s="44">
-        <f>('1. Customers'!$E$15*'Inputs'!$F$77*'Inputs'!$F$78+'1. Customers'!$E$16*'Inputs'!$F$79*'Inputs'!$F$80+'1. Customers'!$E$17*'Inputs'!$F$81*'Inputs'!$F$82+'1. Customers'!$E$18*'Inputs'!$F$83*'Inputs'!$F$84)*'Inputs'!$F$166*'Inputs'!$F$165</f>
+        <f>('1. Customers'!$E$15*'Inputs'!$F$77*'Inputs'!$F$78+'1. Customers'!$E$16*'Inputs'!$F$79*'Inputs'!$F$80+'1. Customers'!$E$17*'Inputs'!$F$81*'Inputs'!$F$82+'1. Customers'!$E$18*'Inputs'!$F$83*'Inputs'!$F$84)*'Inputs'!$F$167*'Inputs'!$F$166</f>
         <v/>
       </c>
       <c r="H65" s="14" t="inlineStr">
@@ -13790,7 +13827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E28"/>
+  <dimension ref="B1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -13884,7 +13921,7 @@
         </is>
       </c>
       <c r="C8" s="44">
-        <f>'Inputs'!$F$141*'1. Customers'!$C$12</f>
+        <f>'Inputs'!$F$142*'1. Customers'!$C$12</f>
         <v/>
       </c>
       <c r="E8" s="14" t="inlineStr">
@@ -13900,7 +13937,7 @@
         </is>
       </c>
       <c r="C9" s="44">
-        <f>('1. Customers'!$E$12+'1. Customers'!$E$13+'1. Customers'!$E$14)*'Inputs'!$F$143*'Inputs'!$F$142</f>
+        <f>('1. Customers'!$E$12+'1. Customers'!$E$13+'1. Customers'!$E$14)*'Inputs'!$F$144*'Inputs'!$F$143</f>
         <v/>
       </c>
       <c r="E9" s="14" t="inlineStr">
@@ -13955,7 +13992,7 @@
     <row r="15">
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Finance, HR, exec, brand &amp; marketing</t>
+          <t>Finance, HR, exec, brand &amp; residual marketing</t>
         </is>
       </c>
       <c r="C15" s="44">
@@ -13964,135 +14001,162 @@
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="40" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Churn replacement — acquisition marketing (driver: new customers won)</t>
+        </is>
+      </c>
+      <c r="C16" s="44">
+        <f>'1. Customers'!$C$8*'Inputs'!$F$136</f>
+        <v/>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>Demand generation to replace churned customers; scales with the churn input</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="40" t="inlineStr">
         <is>
           <t>TOTAL HEAD-OFFICE ALLOCATION</t>
         </is>
       </c>
-      <c r="C16" s="45">
-        <f>'4. Running Costs'!$C$13+'4. Running Costs'!$C$14+'4. Running Costs'!$C$15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="40" t="inlineStr">
-        <is>
-          <t>Change-the-bank / transformation (portfolio hurdle — no product driver)</t>
-        </is>
-      </c>
-      <c r="C18" s="58">
-        <f>'1. Customers'!$C$4*'Inputs'!$F$144</f>
-        <v/>
-      </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>Regulatory change + tech transformation; held unallocated like joint costs</t>
-        </is>
+      <c r="C17" s="45">
+        <f>'4. Running Costs'!$C$13+'4. Running Costs'!$C$14+'4. Running Costs'!$C$15+'4. Running Costs'!$C$16</f>
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="40" t="inlineStr">
         <is>
-          <t>TOTAL OPERATING COSTS (unit + HO share + change)</t>
-        </is>
-      </c>
-      <c r="C19" s="45">
-        <f>'4. Running Costs'!$C$10+'4. Running Costs'!$C$16+'4. Running Costs'!$C$18</f>
-        <v/>
+          <t>Change-the-bank / transformation (portfolio hurdle — no product driver)</t>
+        </is>
+      </c>
+      <c r="C19" s="58">
+        <f>'1. Customers'!$C$4*'Inputs'!$F$145</f>
+        <v/>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>Regulatory change + tech transformation; held unallocated like joint costs</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="40" t="inlineStr">
         <is>
+          <t>TOTAL OPERATING COSTS (unit + HO share + change)</t>
+        </is>
+      </c>
+      <c r="C20" s="45">
+        <f>'4. Running Costs'!$C$10+'4. Running Costs'!$C$17+'4. Running Costs'!$C$19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="40" t="inlineStr">
+        <is>
           <t>Operating cost per customer</t>
         </is>
       </c>
-      <c r="C20" s="26">
-        <f>'4. Running Costs'!$C$19/'1. Customers'!$C$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="7" t="inlineStr">
+      <c r="C21" s="26">
+        <f>'4. Running Costs'!$C$20/'1. Customers'!$C$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>COST ATTRIBUTION MEMO (ABC to the causality limit — see Unit Economics tab)</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr"/>
-      <c r="D22" s="8" t="inlineStr"/>
-      <c r="E22" s="8" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>RM cost (attributed to lending products as acquisition cost)</t>
-        </is>
-      </c>
-      <c r="C23" s="48">
-        <f>'3. HR &amp; Activity'!$H$37</f>
-        <v/>
-      </c>
+      <c r="C23" s="8" t="inlineStr"/>
+      <c r="D23" s="8" t="inlineStr"/>
+      <c r="E23" s="8" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Activity-driven servicing cost (analyst + service payroll)</t>
-        </is>
-      </c>
-      <c r="C24" s="44">
-        <f>'3. HR &amp; Activity'!$H$38+'3. HR &amp; Activity'!$H$39</f>
+          <t>RM cost (attributed to lending products as acquisition cost)</t>
+        </is>
+      </c>
+      <c r="C24" s="48">
+        <f>'3. HR &amp; Activity'!$H$37</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Supervision &amp; workplace pool (managers, premises, depreciation, other)</t>
+          <t>Activity-driven servicing cost (analyst + service payroll)</t>
         </is>
       </c>
       <c r="C25" s="44">
-        <f>'3. HR &amp; Activity'!$H$40+'4. Running Costs'!$C$4+'4. Running Costs'!$C$5+'4. Running Costs'!$C$6</f>
-        <v/>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>Driver: staff time — follows each product's share of servicing + RM cost</t>
-        </is>
+        <f>'3. HR &amp; Activity'!$H$38+'3. HR &amp; Activity'!$H$39</f>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Head-office tech attributed by driver (payments, core banking, credit systems)</t>
+          <t>Supervision &amp; workplace pool (managers, premises, depreciation, other)</t>
         </is>
       </c>
       <c r="C26" s="44">
-        <f>'Inputs'!$F$136*'1. Customers'!$C$12+'Inputs'!$F$137*'1. Customers'!$C$24+'Inputs'!$F$138*'1. Customers'!$C$25</f>
-        <v/>
+        <f>'3. HR &amp; Activity'!$H$40+'4. Running Costs'!$C$4+'4. Running Costs'!$C$5+'4. Running Costs'!$C$6</f>
+        <v/>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>Driver: staff time — follows each product's share of servicing + RM cost</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="10" t="inlineStr">
         <is>
+          <t>Head-office tech attributed by driver (payments, core banking, credit systems)</t>
+        </is>
+      </c>
+      <c r="C27" s="44">
+        <f>'Inputs'!$F$137*'1. Customers'!$C$12+'Inputs'!$F$138*'1. Customers'!$C$24+'Inputs'!$F$139*'1. Customers'!$C$25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="10" t="inlineStr">
+        <is>
           <t>Head-office risk attributed by driver (KYC onboarding + refresh)</t>
         </is>
       </c>
-      <c r="C27" s="44">
+      <c r="C28" s="44">
         <f>'Inputs'!$F$134*'1. Customers'!$C$8+'Inputs'!$F$135*'1. Customers'!$C$4</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="40" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Churn-replacement acquisition marketing attributed by driver (new customers won)</t>
+        </is>
+      </c>
+      <c r="C29" s="44">
+        <f>'4. Running Costs'!$C$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="40" t="inlineStr">
         <is>
           <t>UNALLOCATED JOINT COSTS (brand, exec, finance, platform build, pool remainders)</t>
         </is>
       </c>
-      <c r="C28" s="58">
-        <f>'4. Running Costs'!$C$16-'4. Running Costs'!$C$26-'4. Running Costs'!$C$27</f>
-        <v/>
-      </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="C30" s="58">
+        <f>'4. Running Costs'!$C$17-'4. Running Costs'!$C$27-'4. Running Costs'!$C$28-'4. Running Costs'!$C$29</f>
+        <v/>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
         <is>
           <t>No causal driver exists — held as a portfolio hurdle, not forced into products (source doc allocates these by simple division, not activity)</t>
         </is>
@@ -14195,7 +14259,7 @@
         <v/>
       </c>
       <c r="E5" s="16">
-        <f>D5*(1-'Inputs'!$F$166*'Inputs'!$F$165)</f>
+        <f>D5*(1-'Inputs'!$F$167*'Inputs'!$F$166)</f>
         <v/>
       </c>
       <c r="F5" s="55">
@@ -14226,7 +14290,7 @@
         <v/>
       </c>
       <c r="E6" s="16">
-        <f>D6*(1-'Inputs'!$F$166*'Inputs'!$F$165)</f>
+        <f>D6*(1-'Inputs'!$F$167*'Inputs'!$F$166)</f>
         <v/>
       </c>
       <c r="F6" s="55">
@@ -14257,7 +14321,7 @@
         <v/>
       </c>
       <c r="E7" s="16">
-        <f>D7*(1-'Inputs'!$F$166*'Inputs'!$F$165)</f>
+        <f>D7*(1-'Inputs'!$F$167*'Inputs'!$F$166)</f>
         <v/>
       </c>
       <c r="F7" s="55">
@@ -14288,7 +14352,7 @@
         <v/>
       </c>
       <c r="E8" s="16">
-        <f>D8*(1-'Inputs'!$F$166*'Inputs'!$F$165)</f>
+        <f>D8*(1-'Inputs'!$F$167*'Inputs'!$F$166)</f>
         <v/>
       </c>
       <c r="F8" s="55">
@@ -14471,7 +14535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:L42"/>
+  <dimension ref="B1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -14834,7 +14898,7 @@
         <v/>
       </c>
       <c r="L10" s="44">
-        <f>'4. Running Costs'!$C$24/L6</f>
+        <f>'4. Running Costs'!$C$25/L6</f>
         <v/>
       </c>
     </row>
@@ -14939,43 +15003,43 @@
         </is>
       </c>
       <c r="C13" s="44">
-        <f>'4. Running Costs'!$C$25*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,C5,'3. HR &amp; Activity'!$H$11:$H$33))/('4. Running Costs'!$C$24+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$12</f>
+        <f>'4. Running Costs'!$C$26*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,C5,'3. HR &amp; Activity'!$H$11:$H$33))/('4. Running Costs'!$C$25+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$12</f>
         <v/>
       </c>
       <c r="D13" s="44">
-        <f>'4. Running Costs'!$C$25*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,D5,'3. HR &amp; Activity'!$H$11:$H$33))/('4. Running Costs'!$C$24+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$13</f>
+        <f>'4. Running Costs'!$C$26*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,D5,'3. HR &amp; Activity'!$H$11:$H$33))/('4. Running Costs'!$C$25+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$13</f>
         <v/>
       </c>
       <c r="E13" s="44">
-        <f>'4. Running Costs'!$C$25*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,E5,'3. HR &amp; Activity'!$H$11:$H$33))/('4. Running Costs'!$C$24+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$14</f>
+        <f>'4. Running Costs'!$C$26*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,E5,'3. HR &amp; Activity'!$H$11:$H$33))/('4. Running Costs'!$C$25+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$14</f>
         <v/>
       </c>
       <c r="F13" s="44">
-        <f>'4. Running Costs'!$C$25*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,F5,'3. HR &amp; Activity'!$H$11:$H$33)+'3. HR &amp; Activity'!$G$55+'3. HR &amp; Activity'!$G$61)/('4. Running Costs'!$C$24+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$15</f>
+        <f>'4. Running Costs'!$C$26*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,F5,'3. HR &amp; Activity'!$H$11:$H$33)+'3. HR &amp; Activity'!$G$55+'3. HR &amp; Activity'!$G$61)/('4. Running Costs'!$C$25+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$15</f>
         <v/>
       </c>
       <c r="G13" s="44">
-        <f>'4. Running Costs'!$C$25*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,G5,'3. HR &amp; Activity'!$H$11:$H$33)+'3. HR &amp; Activity'!$G$52+'3. HR &amp; Activity'!$G$62)/('4. Running Costs'!$C$24+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$16</f>
+        <f>'4. Running Costs'!$C$26*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,G5,'3. HR &amp; Activity'!$H$11:$H$33)+'3. HR &amp; Activity'!$G$52+'3. HR &amp; Activity'!$G$62)/('4. Running Costs'!$C$25+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$16</f>
         <v/>
       </c>
       <c r="H13" s="44">
-        <f>'4. Running Costs'!$C$25*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,H5,'3. HR &amp; Activity'!$H$11:$H$33)+'3. HR &amp; Activity'!$G$53+'3. HR &amp; Activity'!$G$63)/('4. Running Costs'!$C$24+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$17</f>
+        <f>'4. Running Costs'!$C$26*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,H5,'3. HR &amp; Activity'!$H$11:$H$33)+'3. HR &amp; Activity'!$G$53+'3. HR &amp; Activity'!$G$63)/('4. Running Costs'!$C$25+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$17</f>
         <v/>
       </c>
       <c r="I13" s="44">
-        <f>'4. Running Costs'!$C$25*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,I5,'3. HR &amp; Activity'!$H$11:$H$33)+'3. HR &amp; Activity'!$G$54+'3. HR &amp; Activity'!$G$64)/('4. Running Costs'!$C$24+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$18</f>
+        <f>'4. Running Costs'!$C$26*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,I5,'3. HR &amp; Activity'!$H$11:$H$33)+'3. HR &amp; Activity'!$G$54+'3. HR &amp; Activity'!$G$64)/('4. Running Costs'!$C$25+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$18</f>
         <v/>
       </c>
       <c r="J13" s="44">
-        <f>'4. Running Costs'!$C$25*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,J5,'3. HR &amp; Activity'!$H$11:$H$33))/('4. Running Costs'!$C$24+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$19</f>
+        <f>'4. Running Costs'!$C$26*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,J5,'3. HR &amp; Activity'!$H$11:$H$33))/('4. Running Costs'!$C$25+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$19</f>
         <v/>
       </c>
       <c r="K13" s="44">
-        <f>'4. Running Costs'!$C$25*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,K5,'3. HR &amp; Activity'!$H$11:$H$33))/('4. Running Costs'!$C$24+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$20</f>
+        <f>'4. Running Costs'!$C$26*(SUMIF('3. HR &amp; Activity'!$C$11:$C$33,K5,'3. HR &amp; Activity'!$H$11:$H$33))/('4. Running Costs'!$C$25+'3. HR &amp; Activity'!$H$46+'3. HR &amp; Activity'!$H$47)/'1. Customers'!$C$20</f>
         <v/>
       </c>
       <c r="L13" s="44">
-        <f>'4. Running Costs'!$C$25/L6</f>
+        <f>'4. Running Costs'!$C$26/L6</f>
         <v/>
       </c>
     </row>
@@ -14986,35 +15050,35 @@
         </is>
       </c>
       <c r="C14" s="44">
-        <f>'Inputs'!$F$128+'Inputs'!$F$137+'Inputs'!$F$136+'Inputs'!$F$135+'Inputs'!$F$134*'1. Customers'!$C$8/'1. Customers'!$C$12</f>
+        <f>'Inputs'!$F$128+'Inputs'!$F$138+'Inputs'!$F$137+'Inputs'!$F$135+'Inputs'!$F$134*'1. Customers'!$C$8/'1. Customers'!$C$12</f>
         <v/>
       </c>
       <c r="D14" s="44">
-        <f>'Inputs'!$F$137</f>
+        <f>'Inputs'!$F$138</f>
         <v/>
       </c>
       <c r="E14" s="44">
-        <f>'Inputs'!$F$137</f>
+        <f>'Inputs'!$F$138</f>
         <v/>
       </c>
       <c r="F14" s="44">
-        <f>'Inputs'!$F$137+'Inputs'!$F$138</f>
+        <f>'Inputs'!$F$138+'Inputs'!$F$139</f>
         <v/>
       </c>
       <c r="G14" s="44">
-        <f>'Inputs'!$F$137+'Inputs'!$F$138</f>
+        <f>'Inputs'!$F$138+'Inputs'!$F$139</f>
         <v/>
       </c>
       <c r="H14" s="44">
-        <f>'Inputs'!$F$137+'Inputs'!$F$138</f>
+        <f>'Inputs'!$F$138+'Inputs'!$F$139</f>
         <v/>
       </c>
       <c r="I14" s="44">
-        <f>'Inputs'!$F$137+'Inputs'!$F$138</f>
+        <f>'Inputs'!$F$138+'Inputs'!$F$139</f>
         <v/>
       </c>
       <c r="J14" s="44">
-        <f>'Inputs'!$F$137+'Inputs'!$F$138</f>
+        <f>'Inputs'!$F$138+'Inputs'!$F$139</f>
         <v/>
       </c>
       <c r="K14" s="44">
@@ -15022,18 +15086,18 @@
         <v/>
       </c>
       <c r="L14" s="44">
-        <f>('4. Running Costs'!$C$7+'4. Running Costs'!$C$26+'4. Running Costs'!$C$27)/L6</f>
+        <f>('4. Running Costs'!$C$7+'4. Running Costs'!$C$27+'4. Running Costs'!$C$28)/L6</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Fraud &amp; payment losses per unit (driver: current accounts)</t>
+          <t>Churn-replacement acquisition per unit (driver: new customers won; gateway = current account)</t>
         </is>
       </c>
       <c r="C15" s="44">
-        <f>'Inputs'!$F$141</f>
+        <f>'Inputs'!$F$136*'1. Customers'!$C$8/'1. Customers'!$C$12</f>
         <v/>
       </c>
       <c r="D15" s="44">
@@ -15069,26 +15133,26 @@
         <v/>
       </c>
       <c r="L15" s="44">
-        <f>'4. Running Costs'!$C$8/L6</f>
+        <f>'4. Running Costs'!$C$16/L6</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>FSCS levy per unit (driver: protected deposits)</t>
+          <t>Fraud &amp; payment losses per unit (driver: current accounts)</t>
         </is>
       </c>
       <c r="C16" s="44">
-        <f>'1. Customers'!$D$12*'Inputs'!$F$143*'Inputs'!$F$142</f>
+        <f>'Inputs'!$F$142</f>
         <v/>
       </c>
       <c r="D16" s="44">
-        <f>'1. Customers'!$D$13*'Inputs'!$F$143*'Inputs'!$F$142</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="E16" s="44">
-        <f>'1. Customers'!$D$14*'Inputs'!$F$143*'Inputs'!$F$142</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="F16" s="44">
@@ -15116,363 +15180,363 @@
         <v/>
       </c>
       <c r="L16" s="44">
+        <f>'4. Running Costs'!$C$8/L6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>FSCS levy per unit (driver: protected deposits)</t>
+        </is>
+      </c>
+      <c r="C17" s="44">
+        <f>'1. Customers'!$D$12*'Inputs'!$F$144*'Inputs'!$F$143</f>
+        <v/>
+      </c>
+      <c r="D17" s="44">
+        <f>'1. Customers'!$D$13*'Inputs'!$F$144*'Inputs'!$F$143</f>
+        <v/>
+      </c>
+      <c r="E17" s="44">
+        <f>'1. Customers'!$D$14*'Inputs'!$F$144*'Inputs'!$F$143</f>
+        <v/>
+      </c>
+      <c r="F17" s="44">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="G17" s="44">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="H17" s="44">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="I17" s="44">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="J17" s="44">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="K17" s="44">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="L17" s="44">
         <f>'4. Running Costs'!$C$9/L6</f>
         <v/>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="49" t="inlineStr">
-        <is>
-          <t>ATTRIBUTABLE COST PER UNIT (EL + servicing + RM orig + RM steward + supervision + infrastructure + fraud + levies)</t>
-        </is>
-      </c>
-      <c r="C17" s="45">
-        <f>C9+C10+C11+C12+C13+C14+C15+C16</f>
-        <v/>
-      </c>
-      <c r="D17" s="45">
-        <f>D9+D10+D11+D12+D13+D14+D15+D16</f>
-        <v/>
-      </c>
-      <c r="E17" s="45">
-        <f>E9+E10+E11+E12+E13+E14+E15+E16</f>
-        <v/>
-      </c>
-      <c r="F17" s="45">
-        <f>F9+F10+F11+F12+F13+F14+F15+F16</f>
-        <v/>
-      </c>
-      <c r="G17" s="45">
-        <f>G9+G10+G11+G12+G13+G14+G15+G16</f>
-        <v/>
-      </c>
-      <c r="H17" s="45">
-        <f>H9+H10+H11+H12+H13+H14+H15+H16</f>
-        <v/>
-      </c>
-      <c r="I17" s="45">
-        <f>I9+I10+I11+I12+I13+I14+I15+I16</f>
-        <v/>
-      </c>
-      <c r="J17" s="45">
-        <f>J9+J10+J11+J12+J13+J14+J15+J16</f>
-        <v/>
-      </c>
-      <c r="K17" s="45">
-        <f>K9+K10+K11+K12+K13+K14+K15+K16</f>
-        <v/>
-      </c>
-      <c r="L17" s="45">
-        <f>L9+L10+L11+L12+L13+L14+L15+L16</f>
-        <v/>
-      </c>
-    </row>
     <row r="18">
-      <c r="B18" s="40" t="inlineStr">
+      <c r="B18" s="49" t="inlineStr">
+        <is>
+          <t>ATTRIBUTABLE COST PER UNIT (EL + servicing + RM orig + RM steward + supervision + infrastructure + churn replacement + fraud + levies)</t>
+        </is>
+      </c>
+      <c r="C18" s="45">
+        <f>C9+C10+C11+C12+C13+C14+C15+C16+C17</f>
+        <v/>
+      </c>
+      <c r="D18" s="45">
+        <f>D9+D10+D11+D12+D13+D14+D15+D16+D17</f>
+        <v/>
+      </c>
+      <c r="E18" s="45">
+        <f>E9+E10+E11+E12+E13+E14+E15+E16+E17</f>
+        <v/>
+      </c>
+      <c r="F18" s="45">
+        <f>F9+F10+F11+F12+F13+F14+F15+F16+F17</f>
+        <v/>
+      </c>
+      <c r="G18" s="45">
+        <f>G9+G10+G11+G12+G13+G14+G15+G16+G17</f>
+        <v/>
+      </c>
+      <c r="H18" s="45">
+        <f>H9+H10+H11+H12+H13+H14+H15+H16+H17</f>
+        <v/>
+      </c>
+      <c r="I18" s="45">
+        <f>I9+I10+I11+I12+I13+I14+I15+I16+I17</f>
+        <v/>
+      </c>
+      <c r="J18" s="45">
+        <f>J9+J10+J11+J12+J13+J14+J15+J16+J17</f>
+        <v/>
+      </c>
+      <c r="K18" s="45">
+        <f>K9+K10+K11+K12+K13+K14+K15+K16+K17</f>
+        <v/>
+      </c>
+      <c r="L18" s="45">
+        <f>L9+L10+L11+L12+L13+L14+L15+L16+L17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="40" t="inlineStr">
         <is>
           <t>CONTRIBUTION PER UNIT (revenue − attributable cost)</t>
         </is>
       </c>
-      <c r="C18" s="26">
-        <f>C8-C17</f>
-        <v/>
-      </c>
-      <c r="D18" s="26">
-        <f>D8-D17</f>
-        <v/>
-      </c>
-      <c r="E18" s="26">
-        <f>E8-E17</f>
-        <v/>
-      </c>
-      <c r="F18" s="26">
-        <f>F8-F17</f>
-        <v/>
-      </c>
-      <c r="G18" s="26">
-        <f>G8-G17</f>
-        <v/>
-      </c>
-      <c r="H18" s="26">
-        <f>H8-H17</f>
-        <v/>
-      </c>
-      <c r="I18" s="26">
-        <f>I8-I17</f>
-        <v/>
-      </c>
-      <c r="J18" s="26">
-        <f>J8-J17</f>
-        <v/>
-      </c>
-      <c r="K18" s="26">
-        <f>K8-K17</f>
-        <v/>
-      </c>
-      <c r="L18" s="26">
-        <f>L8-L17</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>Allocated equity per unit (credit + op-risk RWA × capital ratio)</t>
-        </is>
-      </c>
-      <c r="C19" s="44">
-        <f>'Inputs'!$F$92*C8*'Inputs'!$F$93</f>
-        <v/>
-      </c>
-      <c r="D19" s="44">
-        <f>'Inputs'!$F$92*D8*'Inputs'!$F$93</f>
-        <v/>
-      </c>
-      <c r="E19" s="44">
-        <f>'Inputs'!$F$92*E8*'Inputs'!$F$93</f>
-        <v/>
-      </c>
-      <c r="F19" s="44">
-        <f>('1. Customers'!$D$15*'Inputs'!$F$87+'Inputs'!$F$92*F8)*'Inputs'!$F$93</f>
-        <v/>
-      </c>
-      <c r="G19" s="44">
-        <f>('1. Customers'!$D$16*'Inputs'!$F$88+'Inputs'!$F$92*G8)*'Inputs'!$F$93</f>
-        <v/>
-      </c>
-      <c r="H19" s="44">
-        <f>('1. Customers'!$D$17*'Inputs'!$F$89+'Inputs'!$F$92*H8)*'Inputs'!$F$93</f>
-        <v/>
-      </c>
-      <c r="I19" s="44">
-        <f>('1. Customers'!$D$18*'Inputs'!$F$90+'Inputs'!$F$92*I8)*'Inputs'!$F$93</f>
-        <v/>
-      </c>
-      <c r="J19" s="44">
-        <f>('1. Customers'!$D$19*'Inputs'!$F$91+'Inputs'!$F$92*J8)*'Inputs'!$F$93</f>
-        <v/>
-      </c>
-      <c r="K19" s="44">
-        <f>'Inputs'!$F$92*K8*'Inputs'!$F$93</f>
+      <c r="C19" s="26">
+        <f>C8-C18</f>
+        <v/>
+      </c>
+      <c r="D19" s="26">
+        <f>D8-D18</f>
+        <v/>
+      </c>
+      <c r="E19" s="26">
+        <f>E8-E18</f>
+        <v/>
+      </c>
+      <c r="F19" s="26">
+        <f>F8-F18</f>
+        <v/>
+      </c>
+      <c r="G19" s="26">
+        <f>G8-G18</f>
+        <v/>
+      </c>
+      <c r="H19" s="26">
+        <f>H8-H18</f>
+        <v/>
+      </c>
+      <c r="I19" s="26">
+        <f>I8-I18</f>
+        <v/>
+      </c>
+      <c r="J19" s="26">
+        <f>J8-J18</f>
+        <v/>
+      </c>
+      <c r="K19" s="26">
+        <f>K8-K18</f>
+        <v/>
+      </c>
+      <c r="L19" s="26">
+        <f>L8-L18</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="10" t="inlineStr">
         <is>
+          <t>Allocated equity per unit (credit + op-risk RWA × capital ratio)</t>
+        </is>
+      </c>
+      <c r="C20" s="44">
+        <f>'Inputs'!$F$92*C8*'Inputs'!$F$93</f>
+        <v/>
+      </c>
+      <c r="D20" s="44">
+        <f>'Inputs'!$F$92*D8*'Inputs'!$F$93</f>
+        <v/>
+      </c>
+      <c r="E20" s="44">
+        <f>'Inputs'!$F$92*E8*'Inputs'!$F$93</f>
+        <v/>
+      </c>
+      <c r="F20" s="44">
+        <f>('1. Customers'!$D$15*'Inputs'!$F$87+'Inputs'!$F$92*F8)*'Inputs'!$F$93</f>
+        <v/>
+      </c>
+      <c r="G20" s="44">
+        <f>('1. Customers'!$D$16*'Inputs'!$F$88+'Inputs'!$F$92*G8)*'Inputs'!$F$93</f>
+        <v/>
+      </c>
+      <c r="H20" s="44">
+        <f>('1. Customers'!$D$17*'Inputs'!$F$89+'Inputs'!$F$92*H8)*'Inputs'!$F$93</f>
+        <v/>
+      </c>
+      <c r="I20" s="44">
+        <f>('1. Customers'!$D$18*'Inputs'!$F$90+'Inputs'!$F$92*I8)*'Inputs'!$F$93</f>
+        <v/>
+      </c>
+      <c r="J20" s="44">
+        <f>('1. Customers'!$D$19*'Inputs'!$F$91+'Inputs'!$F$92*J8)*'Inputs'!$F$93</f>
+        <v/>
+      </c>
+      <c r="K20" s="44">
+        <f>'Inputs'!$F$92*K8*'Inputs'!$F$93</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="10" t="inlineStr">
+        <is>
           <t>Net capital charge per unit (equity × (CoE − Bank Rate))</t>
         </is>
       </c>
-      <c r="C20" s="44">
-        <f>C19*('Inputs'!$F$94-'Inputs'!$F$8)</f>
-        <v/>
-      </c>
-      <c r="D20" s="44">
-        <f>D19*('Inputs'!$F$94-'Inputs'!$F$8)</f>
-        <v/>
-      </c>
-      <c r="E20" s="44">
-        <f>E19*('Inputs'!$F$94-'Inputs'!$F$8)</f>
-        <v/>
-      </c>
-      <c r="F20" s="44">
-        <f>F19*('Inputs'!$F$94-'Inputs'!$F$8)</f>
-        <v/>
-      </c>
-      <c r="G20" s="44">
-        <f>G19*('Inputs'!$F$94-'Inputs'!$F$8)</f>
-        <v/>
-      </c>
-      <c r="H20" s="44">
-        <f>H19*('Inputs'!$F$94-'Inputs'!$F$8)</f>
-        <v/>
-      </c>
-      <c r="I20" s="44">
-        <f>I19*('Inputs'!$F$94-'Inputs'!$F$8)</f>
-        <v/>
-      </c>
-      <c r="J20" s="44">
-        <f>J19*('Inputs'!$F$94-'Inputs'!$F$8)</f>
-        <v/>
-      </c>
-      <c r="K20" s="44">
-        <f>K19*('Inputs'!$F$94-'Inputs'!$F$8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="49" t="inlineStr">
+      <c r="C21" s="44">
+        <f>C20*('Inputs'!$F$94-'Inputs'!$F$8)</f>
+        <v/>
+      </c>
+      <c r="D21" s="44">
+        <f>D20*('Inputs'!$F$94-'Inputs'!$F$8)</f>
+        <v/>
+      </c>
+      <c r="E21" s="44">
+        <f>E20*('Inputs'!$F$94-'Inputs'!$F$8)</f>
+        <v/>
+      </c>
+      <c r="F21" s="44">
+        <f>F20*('Inputs'!$F$94-'Inputs'!$F$8)</f>
+        <v/>
+      </c>
+      <c r="G21" s="44">
+        <f>G20*('Inputs'!$F$94-'Inputs'!$F$8)</f>
+        <v/>
+      </c>
+      <c r="H21" s="44">
+        <f>H20*('Inputs'!$F$94-'Inputs'!$F$8)</f>
+        <v/>
+      </c>
+      <c r="I21" s="44">
+        <f>I20*('Inputs'!$F$94-'Inputs'!$F$8)</f>
+        <v/>
+      </c>
+      <c r="J21" s="44">
+        <f>J20*('Inputs'!$F$94-'Inputs'!$F$8)</f>
+        <v/>
+      </c>
+      <c r="K21" s="44">
+        <f>K20*('Inputs'!$F$94-'Inputs'!$F$8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="49" t="inlineStr">
         <is>
           <t>ECONOMIC CONTRIBUTION PER UNIT (pre-tax, before joint costs)</t>
         </is>
       </c>
-      <c r="C21" s="45">
-        <f>C18-C20</f>
-        <v/>
-      </c>
-      <c r="D21" s="45">
-        <f>D18-D20</f>
-        <v/>
-      </c>
-      <c r="E21" s="45">
-        <f>E18-E20</f>
-        <v/>
-      </c>
-      <c r="F21" s="45">
-        <f>F18-F20</f>
-        <v/>
-      </c>
-      <c r="G21" s="45">
-        <f>G18-G20</f>
-        <v/>
-      </c>
-      <c r="H21" s="45">
-        <f>H18-H20</f>
-        <v/>
-      </c>
-      <c r="I21" s="45">
-        <f>I18-I20</f>
-        <v/>
-      </c>
-      <c r="J21" s="45">
-        <f>J18-J20</f>
-        <v/>
-      </c>
-      <c r="K21" s="45">
-        <f>K18-K20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="10" t="inlineStr">
+      <c r="C22" s="45">
+        <f>C19-C21</f>
+        <v/>
+      </c>
+      <c r="D22" s="45">
+        <f>D19-D21</f>
+        <v/>
+      </c>
+      <c r="E22" s="45">
+        <f>E19-E21</f>
+        <v/>
+      </c>
+      <c r="F22" s="45">
+        <f>F19-F21</f>
+        <v/>
+      </c>
+      <c r="G22" s="45">
+        <f>G19-G21</f>
+        <v/>
+      </c>
+      <c r="H22" s="45">
+        <f>H19-H21</f>
+        <v/>
+      </c>
+      <c r="I22" s="45">
+        <f>I19-I21</f>
+        <v/>
+      </c>
+      <c r="J22" s="45">
+        <f>J19-J21</f>
+        <v/>
+      </c>
+      <c r="K22" s="45">
+        <f>K19-K21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>Economic contribution margin (% of revenue)</t>
         </is>
       </c>
-      <c r="C22" s="46">
-        <f>IF(C8=0,0,C21/C8)</f>
-        <v/>
-      </c>
-      <c r="D22" s="46">
-        <f>IF(D8=0,0,D21/D8)</f>
-        <v/>
-      </c>
-      <c r="E22" s="46">
-        <f>IF(E8=0,0,E21/E8)</f>
-        <v/>
-      </c>
-      <c r="F22" s="46">
-        <f>IF(F8=0,0,F21/F8)</f>
-        <v/>
-      </c>
-      <c r="G22" s="46">
-        <f>IF(G8=0,0,G21/G8)</f>
-        <v/>
-      </c>
-      <c r="H22" s="46">
-        <f>IF(H8=0,0,H21/H8)</f>
-        <v/>
-      </c>
-      <c r="I22" s="46">
-        <f>IF(I8=0,0,I21/I8)</f>
-        <v/>
-      </c>
-      <c r="J22" s="46">
-        <f>IF(J8=0,0,J21/J8)</f>
-        <v/>
-      </c>
-      <c r="K22" s="46">
-        <f>IF(K8=0,0,K21/K8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="40" t="inlineStr">
-        <is>
-          <t>Total contribution (£/yr)</t>
-        </is>
-      </c>
-      <c r="C23" s="26">
-        <f>C18*C6</f>
-        <v/>
-      </c>
-      <c r="D23" s="26">
-        <f>D18*D6</f>
-        <v/>
-      </c>
-      <c r="E23" s="26">
-        <f>E18*E6</f>
-        <v/>
-      </c>
-      <c r="F23" s="26">
-        <f>F18*F6</f>
-        <v/>
-      </c>
-      <c r="G23" s="26">
-        <f>G18*G6</f>
-        <v/>
-      </c>
-      <c r="H23" s="26">
-        <f>H18*H6</f>
-        <v/>
-      </c>
-      <c r="I23" s="26">
-        <f>I18*I6</f>
-        <v/>
-      </c>
-      <c r="J23" s="26">
-        <f>J18*J6</f>
-        <v/>
-      </c>
-      <c r="K23" s="26">
-        <f>K18*K6</f>
-        <v/>
-      </c>
-      <c r="L23" s="45">
-        <f>SUM(C23:K23)</f>
+      <c r="C23" s="46">
+        <f>IF(C8=0,0,C22/C8)</f>
+        <v/>
+      </c>
+      <c r="D23" s="46">
+        <f>IF(D8=0,0,D22/D8)</f>
+        <v/>
+      </c>
+      <c r="E23" s="46">
+        <f>IF(E8=0,0,E22/E8)</f>
+        <v/>
+      </c>
+      <c r="F23" s="46">
+        <f>IF(F8=0,0,F22/F8)</f>
+        <v/>
+      </c>
+      <c r="G23" s="46">
+        <f>IF(G8=0,0,G22/G8)</f>
+        <v/>
+      </c>
+      <c r="H23" s="46">
+        <f>IF(H8=0,0,H22/H8)</f>
+        <v/>
+      </c>
+      <c r="I23" s="46">
+        <f>IF(I8=0,0,I22/I8)</f>
+        <v/>
+      </c>
+      <c r="J23" s="46">
+        <f>IF(J8=0,0,J22/J8)</f>
+        <v/>
+      </c>
+      <c r="K23" s="46">
+        <f>IF(K8=0,0,K22/K8)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="40" t="inlineStr">
         <is>
-          <t>Total economic contribution (£/yr)</t>
+          <t>Total contribution (£/yr)</t>
         </is>
       </c>
       <c r="C24" s="26">
-        <f>C21*C6</f>
+        <f>C19*C6</f>
         <v/>
       </c>
       <c r="D24" s="26">
-        <f>D21*D6</f>
+        <f>D19*D6</f>
         <v/>
       </c>
       <c r="E24" s="26">
-        <f>E21*E6</f>
+        <f>E19*E6</f>
         <v/>
       </c>
       <c r="F24" s="26">
-        <f>F21*F6</f>
+        <f>F19*F6</f>
         <v/>
       </c>
       <c r="G24" s="26">
-        <f>G21*G6</f>
+        <f>G19*G6</f>
         <v/>
       </c>
       <c r="H24" s="26">
-        <f>H21*H6</f>
+        <f>H19*H6</f>
         <v/>
       </c>
       <c r="I24" s="26">
-        <f>I21*I6</f>
+        <f>I19*I6</f>
         <v/>
       </c>
       <c r="J24" s="26">
-        <f>J21*J6</f>
+        <f>J19*J6</f>
         <v/>
       </c>
       <c r="K24" s="26">
-        <f>K21*K6</f>
+        <f>K19*K6</f>
         <v/>
       </c>
       <c r="L24" s="45">
@@ -15480,253 +15544,316 @@
         <v/>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="7" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="40" t="inlineStr">
+        <is>
+          <t>Total economic contribution (£/yr)</t>
+        </is>
+      </c>
+      <c r="C25" s="26">
+        <f>C22*C6</f>
+        <v/>
+      </c>
+      <c r="D25" s="26">
+        <f>D22*D6</f>
+        <v/>
+      </c>
+      <c r="E25" s="26">
+        <f>E22*E6</f>
+        <v/>
+      </c>
+      <c r="F25" s="26">
+        <f>F22*F6</f>
+        <v/>
+      </c>
+      <c r="G25" s="26">
+        <f>G22*G6</f>
+        <v/>
+      </c>
+      <c r="H25" s="26">
+        <f>H22*H6</f>
+        <v/>
+      </c>
+      <c r="I25" s="26">
+        <f>I22*I6</f>
+        <v/>
+      </c>
+      <c r="J25" s="26">
+        <f>J22*J6</f>
+        <v/>
+      </c>
+      <c r="K25" s="26">
+        <f>K22*K6</f>
+        <v/>
+      </c>
+      <c r="L25" s="45">
+        <f>SUM(C25:K25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>BRIDGE TO THE UNIT P&amp;L</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr"/>
-      <c r="D26" s="8" t="inlineStr"/>
-      <c r="E26" s="8" t="inlineStr"/>
-      <c r="F26" s="8" t="inlineStr"/>
-      <c r="G26" s="8" t="inlineStr"/>
-      <c r="H26" s="8" t="inlineStr"/>
-      <c r="I26" s="8" t="inlineStr"/>
-      <c r="J26" s="8" t="inlineStr"/>
-      <c r="K26" s="8" t="inlineStr"/>
-      <c r="L26" s="8" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="10" t="inlineStr">
-        <is>
-          <t>Total contribution across products</t>
-        </is>
-      </c>
-      <c r="C27" s="44">
-        <f>L23</f>
-        <v/>
-      </c>
+      <c r="C27" s="8" t="inlineStr"/>
+      <c r="D27" s="8" t="inlineStr"/>
+      <c r="E27" s="8" t="inlineStr"/>
+      <c r="F27" s="8" t="inlineStr"/>
+      <c r="G27" s="8" t="inlineStr"/>
+      <c r="H27" s="8" t="inlineStr"/>
+      <c r="I27" s="8" t="inlineStr"/>
+      <c r="J27" s="8" t="inlineStr"/>
+      <c r="K27" s="8" t="inlineStr"/>
+      <c r="L27" s="8" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Less: RM defence (tested retention spend, held at centre level)</t>
+          <t>Total contribution across products</t>
         </is>
       </c>
       <c r="C28" s="44">
-        <f>-'3. HR &amp; Activity'!$H$48</f>
+        <f>L24</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Less: unallocated joint costs (no causal driver — brand, exec, finance, platform build)</t>
+          <t>Less: RM defence (tested retention spend, held at centre level)</t>
         </is>
       </c>
       <c r="C29" s="44">
-        <f>-'4. Running Costs'!$C$28</f>
+        <f>-'3. HR &amp; Activity'!$H$48</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="10" t="inlineStr">
         <is>
+          <t>Less: unallocated joint costs (no causal driver — brand, exec, finance, platform build)</t>
+        </is>
+      </c>
+      <c r="C30" s="44">
+        <f>-'4. Running Costs'!$C$30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="10" t="inlineStr">
+        <is>
           <t>Less: change-the-bank / transformation (portfolio hurdle — no product driver)</t>
         </is>
       </c>
-      <c r="C30" s="44">
-        <f>-'4. Running Costs'!$C$18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="49" t="inlineStr">
+      <c r="C31" s="44">
+        <f>-'4. Running Costs'!$C$19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="49" t="inlineStr">
         <is>
           <t>Operating profit before capital charges</t>
         </is>
       </c>
-      <c r="C31" s="45">
-        <f>C27+C28+C29+C30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>Check vs P&amp;L (income excl. equity benefit − EL − opex) — should be zero</t>
-        </is>
-      </c>
-      <c r="C32" s="44">
-        <f>C31-('2. Revenues'!$M$14-'5. Risk &amp; Capital'!$G$10-'4. Running Costs'!$C$19)</f>
-        <v/>
-      </c>
-      <c r="D32" s="14" t="inlineStr">
-        <is>
-          <t>✓ ties out</t>
-        </is>
+      <c r="C32" s="45">
+        <f>C28+C29+C30+C31</f>
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Memo — RM system payback: defence value (defended customers × contribution/customer × remaining life + avoided onboarding)</t>
+          <t>Check vs P&amp;L (income excl. equity benefit − EL − opex) — should be zero</t>
         </is>
       </c>
       <c r="C33" s="44">
-        <f>'1. Customers'!$C$7*(C27/'1. Customers'!$C$4*'Inputs'!$F$168+'Inputs'!$F$105*'3. HR &amp; Activity'!$C$7+'Inputs'!$F$134)</f>
+        <f>C32-('2. Revenues'!$M$14-'5. Risk &amp; Capital'!$G$10-'4. Running Costs'!$C$20)</f>
         <v/>
       </c>
       <c r="D33" s="14" t="inlineStr">
         <is>
-          <t>vs defence cost:</t>
-        </is>
-      </c>
-      <c r="E33" s="48">
-        <f>'3. HR &amp; Activity'!$H$48</f>
-        <v/>
+          <t>✓ ties out</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="10" t="inlineStr">
         <is>
+          <t>Memo — value of preventing ONE customer churning (contribution annuity over remaining life + avoided replacement: acquisition + onboarding + KYC)</t>
+        </is>
+      </c>
+      <c r="C34" s="26">
+        <f>C28/'1. Customers'!$C$4*'Inputs'!$F$169+'Inputs'!$F$136+'Inputs'!$F$105*'3. HR &amp; Activity'!$C$7+'Inputs'!$F$134</f>
+        <v/>
+      </c>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>£ per customer saved — the retention business case runs on this</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>Memo — RM system payback: defence value (defended customers × value of one prevented churn)</t>
+        </is>
+      </c>
+      <c r="C35" s="44">
+        <f>'1. Customers'!$C$7*(C28/'1. Customers'!$C$4*'Inputs'!$F$169+'Inputs'!$F$136+'Inputs'!$F$105*'3. HR &amp; Activity'!$C$7+'Inputs'!$F$134)</f>
+        <v/>
+      </c>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>vs defence cost:</t>
+        </is>
+      </c>
+      <c r="E35" s="48">
+        <f>'3. HR &amp; Activity'!$H$48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="10" t="inlineStr">
+        <is>
           <t>Memo — stewardship payback: expected losses avoided (tab 3) vs stewardship cost</t>
         </is>
       </c>
-      <c r="C34" s="48">
+      <c r="C36" s="48">
         <f>'3. HR &amp; Activity'!$G$65</f>
         <v/>
       </c>
-      <c r="D34" s="14" t="inlineStr">
+      <c r="D36" s="14" t="inlineStr">
         <is>
           <t>vs stewardship cost:</t>
         </is>
       </c>
-      <c r="E34" s="48">
+      <c r="E36" s="48">
         <f>'3. HR &amp; Activity'!$H$47</f>
         <v/>
       </c>
     </row>
-    <row r="36">
-      <c r="B36" s="7" t="inlineStr">
+    <row r="38">
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>MEMO — FULL ABSORPTION PER SOURCE METHODOLOGY (joint costs spread per unit, as the IFC doc divides head-office costs)</t>
         </is>
       </c>
-      <c r="C36" s="8" t="inlineStr"/>
-      <c r="D36" s="8" t="inlineStr"/>
-      <c r="E36" s="8" t="inlineStr"/>
-      <c r="F36" s="8" t="inlineStr"/>
-      <c r="G36" s="8" t="inlineStr"/>
-      <c r="H36" s="8" t="inlineStr"/>
-      <c r="I36" s="8" t="inlineStr"/>
-      <c r="J36" s="8" t="inlineStr"/>
-      <c r="K36" s="8" t="inlineStr"/>
-      <c r="L36" s="8" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="B37" s="10" t="inlineStr">
+      <c r="C38" s="8" t="inlineStr"/>
+      <c r="D38" s="8" t="inlineStr"/>
+      <c r="E38" s="8" t="inlineStr"/>
+      <c r="F38" s="8" t="inlineStr"/>
+      <c r="G38" s="8" t="inlineStr"/>
+      <c r="H38" s="8" t="inlineStr"/>
+      <c r="I38" s="8" t="inlineStr"/>
+      <c r="J38" s="8" t="inlineStr"/>
+      <c r="K38" s="8" t="inlineStr"/>
+      <c r="L38" s="8" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="10" t="inlineStr">
         <is>
           <t>Joint cost absorbed per unit (flat per-unit spread)</t>
         </is>
       </c>
-      <c r="C37" s="44">
-        <f>'4. Running Costs'!$C$28/L6</f>
-        <v/>
-      </c>
-      <c r="D37" s="44">
-        <f>'4. Running Costs'!$C$28/L6</f>
-        <v/>
-      </c>
-      <c r="E37" s="44">
-        <f>'4. Running Costs'!$C$28/L6</f>
-        <v/>
-      </c>
-      <c r="F37" s="44">
-        <f>'4. Running Costs'!$C$28/L6</f>
-        <v/>
-      </c>
-      <c r="G37" s="44">
-        <f>'4. Running Costs'!$C$28/L6</f>
-        <v/>
-      </c>
-      <c r="H37" s="44">
-        <f>'4. Running Costs'!$C$28/L6</f>
-        <v/>
-      </c>
-      <c r="I37" s="44">
-        <f>'4. Running Costs'!$C$28/L6</f>
-        <v/>
-      </c>
-      <c r="J37" s="44">
-        <f>'4. Running Costs'!$C$28/L6</f>
-        <v/>
-      </c>
-      <c r="K37" s="44">
-        <f>'4. Running Costs'!$C$28/L6</f>
-        <v/>
-      </c>
-      <c r="L37" s="44">
-        <f>'4. Running Costs'!$C$28/L6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="10" t="inlineStr">
+      <c r="C39" s="44">
+        <f>'4. Running Costs'!$C$30/L6</f>
+        <v/>
+      </c>
+      <c r="D39" s="44">
+        <f>'4. Running Costs'!$C$30/L6</f>
+        <v/>
+      </c>
+      <c r="E39" s="44">
+        <f>'4. Running Costs'!$C$30/L6</f>
+        <v/>
+      </c>
+      <c r="F39" s="44">
+        <f>'4. Running Costs'!$C$30/L6</f>
+        <v/>
+      </c>
+      <c r="G39" s="44">
+        <f>'4. Running Costs'!$C$30/L6</f>
+        <v/>
+      </c>
+      <c r="H39" s="44">
+        <f>'4. Running Costs'!$C$30/L6</f>
+        <v/>
+      </c>
+      <c r="I39" s="44">
+        <f>'4. Running Costs'!$C$30/L6</f>
+        <v/>
+      </c>
+      <c r="J39" s="44">
+        <f>'4. Running Costs'!$C$30/L6</f>
+        <v/>
+      </c>
+      <c r="K39" s="44">
+        <f>'4. Running Costs'!$C$30/L6</f>
+        <v/>
+      </c>
+      <c r="L39" s="44">
+        <f>'4. Running Costs'!$C$30/L6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="10" t="inlineStr">
         <is>
           <t>Fully-absorbed profit per unit (contribution − joint absorption)</t>
         </is>
       </c>
-      <c r="C38" s="44">
-        <f>C18-C37</f>
-        <v/>
-      </c>
-      <c r="D38" s="44">
-        <f>D18-D37</f>
-        <v/>
-      </c>
-      <c r="E38" s="44">
-        <f>E18-E37</f>
-        <v/>
-      </c>
-      <c r="F38" s="44">
-        <f>F18-F37</f>
-        <v/>
-      </c>
-      <c r="G38" s="44">
-        <f>G18-G37</f>
-        <v/>
-      </c>
-      <c r="H38" s="44">
-        <f>H18-H37</f>
-        <v/>
-      </c>
-      <c r="I38" s="44">
-        <f>I18-I37</f>
-        <v/>
-      </c>
-      <c r="J38" s="44">
-        <f>J18-J37</f>
-        <v/>
-      </c>
-      <c r="K38" s="44">
-        <f>K18-K37</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="5" t="inlineStr">
+      <c r="C40" s="44">
+        <f>C19-C39</f>
+        <v/>
+      </c>
+      <c r="D40" s="44">
+        <f>D19-D39</f>
+        <v/>
+      </c>
+      <c r="E40" s="44">
+        <f>E19-E39</f>
+        <v/>
+      </c>
+      <c r="F40" s="44">
+        <f>F19-F39</f>
+        <v/>
+      </c>
+      <c r="G40" s="44">
+        <f>G19-G39</f>
+        <v/>
+      </c>
+      <c r="H40" s="44">
+        <f>H19-H39</f>
+        <v/>
+      </c>
+      <c r="I40" s="44">
+        <f>I19-I39</f>
+        <v/>
+      </c>
+      <c r="J40" s="44">
+        <f>J19-J39</f>
+        <v/>
+      </c>
+      <c r="K40" s="44">
+        <f>K19-K39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>Cost treatment follows the source methodology's own hybrid: activity drivers wherever a causal link to customers or transactions exists ('whenever possible' — Simanis IFC Technical Doc Part II), head-office residuals without a driver held as an unallocated share rather than forced into products. Product decisions should run on CONTRIBUTION (it changes when the decision changes); the full-absorption memo shows required pricing coverage.</t>
         </is>
       </c>
     </row>
-    <row r="41"/>
-    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B40:L42"/>
+    <mergeCell ref="B42:L44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15888,7 +16015,7 @@
         </is>
       </c>
       <c r="C14" s="44">
-        <f>-'4. Running Costs'!$C$16</f>
+        <f>-'4. Running Costs'!$C$17</f>
         <v/>
       </c>
     </row>
@@ -15899,7 +16026,7 @@
         </is>
       </c>
       <c r="C15" s="44">
-        <f>-'4. Running Costs'!$C$18</f>
+        <f>-'4. Running Costs'!$C$19</f>
         <v/>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -15926,7 +16053,7 @@
         </is>
       </c>
       <c r="C17" s="44">
-        <f>'7. P&amp;L'!$C$16+'4. Running Costs'!$C$28+'3. HR &amp; Activity'!$H$48</f>
+        <f>'7. P&amp;L'!$C$16+'4. Running Costs'!$C$30+'3. HR &amp; Activity'!$H$48</f>
         <v/>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -15958,7 +16085,7 @@
         </is>
       </c>
       <c r="C19" s="44">
-        <f>-'4. Running Costs'!$C$28</f>
+        <f>-'4. Running Costs'!$C$30</f>
         <v/>
       </c>
       <c r="E19" s="5" t="inlineStr">

</xml_diff>

<commit_message>
v1.7: operational leverage — cost scale elasticity measured from published accounts
Cost per customer was flat at every scale, because every cost line scaled linearly with
its driver. Allica's accounts put the elasticity of cost against its lending book at
0.808 (2022-23) and 0.622 (2023-24).

Inputs section O adds the elasticity and its calibration point. Default 1.0 reproduces
v1.6 exactly. Tab 11 carries the out-of-sample test: the 2022-23 elasticity predicts
2024 profit before tax to within 20%.
</commit_message>
<xml_diff>
--- a/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
+++ b/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B47"/>
+  <dimension ref="B1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -606,7 +606,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MODEL VERSION: v1.6 · 22 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
+          <t>MODEL VERSION: v1.7 · 22 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
         </is>
       </c>
     </row>
@@ -620,257 +620,264 @@
     <row r="5" ht="52" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>• v1.6 (22 Aug 2026) — validation and drivers. Tab 10 ELASTICITIES: every input bumped +1% and the workbook recalculated, giving the % change in PBT, cost:income, RoE and income. Only one input has an elasticity above 1 on profit — the term loan customer rate, at +1.25; reachable market and penetration are exactly +1.00 (pure scale); nothing else exceeds 0.53. Tab 11 BACKTEST against Allica Bank FY2023 audited accounts: the revenue engine reproduces a real bank's operating income to within 8%, and the cost engine under-predicts by 7x. Diagnosis: head-office cost was modelled purely per customer, which is a scale assumption disguised as a driver. Inputs section N therefore adds a fixed component to each head-office pool, defaulting to 0 so v1.5 results are unchanged.</t>
+          <t>• v1.7 (22 Aug 2026) — operational leverage. Every cost line in the model scaled linearly with its driver, which forces a cost elasticity of exactly 1.0 and makes cost per customer flat at every scale. Allica Bank's own accounts put that elasticity at 0.808 across 2022-23 and 0.622 across 2023-24 — cost rises materially more slowly than the book. Inputs section O adds a cost scale elasticity and the customer count the per-customer rates are calibrated at; the head-office pools, the platform line and change-the-bank now scale by it. Default 1.0 reproduces v1.6 exactly. Tab 11 adds the out-of-sample test that measured it.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="52" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>• v1.5 (22 Aug 2026) — PROCESS LAYER on the Step 2 tabs. Tab 3 gains process columns M-T (process type, yield, attempts, automation, best-in-class intensity and yield, benchmark source, £ gap) and a HEAD-OFFICE PROCESS REGISTER of 22 processes already named in the tab 9 operational model but never costed. Yield inflates ATTEMPTS and never deflates outcomes — that is what stops it double-counting with the CEP layer's demand-side conversion. Head-office costs are carved OUT of the pools, so naming a process moves money from unallocated to attributed and the total never changes. New sheet 3b indexes every process to the numbers it moves, and imputes what each would have to become to hit a target cost:income. Mode OFF (default) = results identical to v1.4.</t>
+          <t>• v1.6 (22 Aug 2026) — validation and drivers. Tab 10 ELASTICITIES: every input bumped +1% and the workbook recalculated, giving the % change in PBT, cost:income, RoE and income. Only one input has an elasticity above 1 on profit — the term loan customer rate, at +1.25; reachable market and penetration are exactly +1.00 (pure scale); nothing else exceeds 0.53. Tab 11 BACKTEST against Allica Bank FY2023 audited accounts: the revenue engine reproduces a real bank's operating income to within 8%, and the cost engine under-predicts by 7x. Diagnosis: head-office cost was modelled purely per customer, which is a scale assumption disguised as a driver. Inputs section N therefore adds a fixed component to each head-office pool, defaulting to 0 so v1.5 results are unchanged.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
+          <t>• v1.5 (22 Aug 2026) — PROCESS LAYER on the Step 2 tabs. Tab 3 gains process columns M-T (process type, yield, attempts, automation, best-in-class intensity and yield, benchmark source, £ gap) and a HEAD-OFFICE PROCESS REGISTER of 22 processes already named in the tab 9 operational model but never costed. Yield inflates ATTEMPTS and never deflates outcomes — that is what stops it double-counting with the CEP layer's demand-side conversion. Head-office costs are carved OUT of the pools, so naming a process moves money from unallocated to attributed and the total never changes. New sheet 3b indexes every process to the numbers it moves, and imputes what each would have to become to hit a target cost:income. Mode OFF (default) = results identical to v1.4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="52" customHeight="1">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
           <t>• v1.4 (22 Aug 2026) — CEP DEMAND LAYER. New sheet 1b derives the nine product penetrations and the customer count instead of asserting them: penetration = (lambda*c x L) / (1 + lambda*c x L), where lambda*c = category-entry-point events x presence x conversion and L is the holding life. Little's Law run forwards; no time axis is added and the model stays a steady-state snapshot. Ships deliberately EMPTY — every event/presence/conversion cell is blank and carries the cohort query that fills it, and any unpopulated product falls back to its hardcoded penetration. Mode OFF (default) = results identical to v1.3; CALIBRATE reports the won-event rate implied by today's assumptions and changes nothing.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="B8" s="4" t="inlineStr">
+    <row r="9" ht="40" customHeight="1">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>• v1.3 (21 Aug 2026) — churn replacement is a costed activity end-to-end: new input cac_new (£240 acquisition marketing per new customer won, carved out of the corporate-centre pool — hq_oh £250→£222); driver-linked on tab 4, attributed to the current account (gateway product) on tab 6; 'value of preventing one churn' memo added to tab 6. Raising the churn input now inflates demand-generation cost, not just processing. Central PBT shifts &lt;£1k/unit (carve-out rounding).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
+          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
+          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
           <t>• v1.0 (10 Aug 2026) — first published version: 9 tabs + flow register, FTP with liquidity/behavioural terms, fraud/FSCS/change-the-bank lines, segment-pod LMUs, bridge check.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="3" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>What this is</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="39" customHeight="1">
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="39" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
         <is>
+          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="39" customHeight="1">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
           <t>• It follows the Simanis / IVE bottom-up methodology ('Running the Right Numbers'): model the last-mile operating unit, derive every cost from activity drivers (transaction intensity I and customer load L), build whole costs, and check the price/margin covers them including a competitive return on capital.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="3" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>What period this models</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="B19" s="4" t="inlineStr">
+    <row r="20" ht="26" customHeight="1">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>• One representative operating year at steady state. Balances are annual averages; rates and volumes are annual. There is no time axis, no ramp and no vintage cohorts — the model is a snapshot, not a forecast.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="78" customHeight="1">
-      <c r="B20" s="4" t="inlineStr">
+    <row r="21" ht="78" customHeight="1">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>• The book is stationary but not free to hold flat: customers churn (12% p.a. input) and the model costs their replacement end-to-end — acquisition marketing per new customer won (cac_new, carved from the corporate-centre pool), onboarding hours, KYC per new customer and RM origination effort are all driver-linked (Simanis: at-scale operations include 'replacement of customer churn'). Only residual brand &amp; joint marketing remains pool-costed. The 'value of preventing one churn' memo on tab 6 prices retention: contribution annuity over remaining relationship life + the avoided replacement cost.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="B21" s="4" t="inlineStr">
+    <row r="22" ht="26" customHeight="1">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>• The capital charge (cost of equity on allocated capital) is the incumbent analogue of Simanis's start-up-cost amortisation: capital earns its required return inside the steady-state P&amp;L.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="52" customHeight="1">
-      <c r="B22" s="4" t="inlineStr">
+    <row r="23" ht="52" customHeight="1">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>• Out of scope by design: transition paths. The cost and cash shape of moving between steady states — digital migration, maturity glide, behaviour-change programmes and their CAC/incentives — belongs in a scenario layer built ON TOP of this base (comparative statics between two runs of this model, plus a separate transition-cost estimate). The base model never carries scenario logic.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="3" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>How the tabs map to the methodology</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="B25" s="4" t="inlineStr">
+    <row r="26" ht="24" customHeight="1">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>• Inputs — every assumption in one place, with sources. Edit blue cells; yellow cells are the biggest levers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="26" customHeight="1">
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="26" customHeight="1">
       <c r="B27" s="4" t="inlineStr">
         <is>
+          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="26" customHeight="1">
+      <c r="B28" s="4" t="inlineStr">
+        <is>
           <t>• 2. Revenues — unit revenue per product: interest margins measured against internal funds transfer prices (Bank Rate for floating, + premium for term), plus fees.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="39" customHeight="1">
-      <c r="B28" s="4" t="inlineStr">
+    <row r="29" ht="39" customHeight="1">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>• 3. HR &amp; Activity — Step 2: every FTE derived from activity drivers (hours per onboarding, review, renewal…) — nothing is assumed as headcount. From v1.5 this tab is also the PROCESS REGISTER (columns M-T), with the head-office process register below it.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="26" customHeight="1">
-      <c r="B29" s="4" t="inlineStr">
+    <row r="30" ht="26" customHeight="1">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>• 1b. Demand &amp; CEPs — the demand layer (v1.4). Penetration is derived, not assumed. Mode cell on Inputs section L: OFF reproduces v1.3, CALIBRATE reports the implied event rates, LIVE derives.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="39" customHeight="1">
-      <c r="B30" s="4" t="inlineStr">
+    <row r="31" ht="39" customHeight="1">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>• 3b. Process Index — derived view, no assumptions. Every process with its flow, product, owner, the numbers it moves, its cost and its gap to best in class, plus a ranked worst-gap list and the top-down benchmark imputation. Answers 'which process do I improve to move this number?'</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="52" customHeight="1">
-      <c r="B31" s="4" t="inlineStr">
+    <row r="32" ht="52" customHeight="1">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>• 4. Running Costs — Step 2 (cont.): direct running costs plus the share of head-office costs. The attribution memo reads the tab 3 process register and reports the share of the cost base with a named process owner — the model's own assessment of how much of its cost it actually understands. What remains in UNALLOCATED JOINT COSTS is cost with no process to improve.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="26" customHeight="1">
-      <c r="B32" s="4" t="inlineStr">
+    <row r="33" ht="26" customHeight="1">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>• 5. Risk &amp; Capital — Step 3: expected credit losses (PD × LGD), risk-weighted assets, allocated equity, and the required return on it.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="91" customHeight="1">
-      <c r="B33" s="4" t="inlineStr">
+    <row r="34" ht="91" customHeight="1">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>• 6. Unit Economics — Steps 4–5: per-product unit costs and revenues on an activity-based costing basis, taken exactly as far as causality runs (the source methodology's own rule: link costs to customers and transactions 'whenever possible'). Costs with real drivers — servicing hours, RM effort per origination, staff-time-driven supervision, per-account and per-facility infrastructure — are attributed to products; genuinely joint costs (brand, exec, finance, platform build) are NOT forced into products but held as an unallocated hurdle that total contribution must clear, with a full-absorption memo showing the source doc's simple-division treatment. Product decisions should run on contribution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="26" customHeight="1">
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="26" customHeight="1">
       <c r="B35" s="4" t="inlineStr">
         <is>
+          <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="26" customHeight="1">
+      <c r="B36" s="4" t="inlineStr">
+        <is>
           <t>• 8. Org Structure — the whole-bank organisation implied by the model: front-line FTEs from activity drivers × number of centres, head-office FTEs backed out of the per-customer head-office cost allocations.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="52" customHeight="1">
-      <c r="B36" s="4" t="inlineStr">
+    <row r="37" ht="52" customHeight="1">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>• 9. Flow Register — one row per flow on the operational model map: component type (CP/WP/PP/PartP), core/support/enabling, direction, digital/physical medium, the direct/administrative/managerial roles accountable, and the BIAN service domains. Ends with a BIAN completeness checklist. This is where the map, the ARM and BIAN reconcile.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="B38" s="3" t="inlineStr">
+    <row r="39">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Colour legend</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="26" customHeight="1">
-      <c r="B39" s="4" t="inlineStr">
+    <row r="40" ht="26" customHeight="1">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>• Blue = hardcoded input (edit these) · Yellow fill = key assumption / sensitivity lever · Black = formula · Green = link to another sheet.</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="B41" s="3" t="inlineStr">
+    <row r="42">
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>Reading the results</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="52" customHeight="1">
-      <c r="B42" s="4" t="inlineStr">
+    <row r="43" ht="52" customHeight="1">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>• Deposit products earn the spread between the transfer price and the rate paid; lending earns the customer rate minus the transfer price minus expected losses. Capital-heavy, labour-heavy products (term loans) can show thin or negative economic profit — consistent with the Bank of England's 2026 finding that SME lending earns the lowest product-level returns, driven by impairments and per-borrower servicing costs.</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="39" customHeight="1">
-      <c r="B43" s="4" t="inlineStr">
+    <row r="44" ht="39" customHeight="1">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>• Use the cost-driver table on the P&amp;L tab to find leverage points, then trace them to transaction intensity (I) or customer load (L) assumptions on the Inputs tab — e.g. automating underwriting hours, raising RM portfolio size, or shifting servicing to digital.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="B45" s="3" t="inlineStr">
+    <row r="46">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>Caveats</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="39" customHeight="1">
-      <c r="B46" s="4" t="inlineStr">
+    <row r="47" ht="39" customHeight="1">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>• Benchmarks are as of August 2026 (Bank Rate 3.75%; BoE effective new SME loan rate ~6.3%; commercial interchange 1.65–1.90%; invoice finance discount base+1–3%). Items marked 'Assumption' are illustrative and should be replaced with your own data.</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="65" customHeight="1">
-      <c r="B47" s="4" t="inlineStr">
+    <row r="48" ht="65" customHeight="1">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>• The FTP now carries an explicit liquidity charge (buffer × drag) and a behavioural credit for stable deposits, shown as memos on the Revenues tab; it is still a single curve, not a full behavioural-maturity model. Fraud &amp; payment losses, the FSCS levy, collateral administration &amp; recoveries, and change-the-bank spend are now modelled explicitly. Operational-risk RWA is proxied at 15% of gross income; head-office and change costs are allocated per customer.</t>
         </is>
@@ -10085,7 +10092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F19"/>
+  <dimension ref="B1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -10291,8 +10298,165 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="40" customHeight="1">
-      <c r="B19" s="5" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>OUT-OF-SAMPLE — CALIBRATE ON 2022-23, PREDICT 2024</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr"/>
+      <c r="D19" s="8" t="inlineStr"/>
+      <c r="E19" s="8" t="inlineStr"/>
+      <c r="F19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Fitting a model to the data it was calibrated on proves nothing. The cost structure below was calibrated on two published years and then used to predict a third it never saw. Harness: backtest_allica_oos.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="45" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C21" s="45" t="inlineStr">
+        <is>
+          <t>Lending book</t>
+        </is>
+      </c>
+      <c r="D21" s="45" t="inlineStr">
+        <is>
+          <t>Operating cost</t>
+        </is>
+      </c>
+      <c r="E21" s="45" t="inlineStr">
+        <is>
+          <t>Cost / book</t>
+        </is>
+      </c>
+      <c r="F21" s="45" t="inlineStr">
+        <is>
+          <t>Elasticity vs prior year</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="42" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C22" s="46" t="n">
+        <v>1348166000</v>
+      </c>
+      <c r="D22" s="46" t="n">
+        <v>41426000</v>
+      </c>
+      <c r="E22" s="48" t="n">
+        <v>0.03072767003469899</v>
+      </c>
+      <c r="F22" s="63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="42" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C23" s="46" t="n">
+        <v>1976826000</v>
+      </c>
+      <c r="D23" s="46" t="n">
+        <v>56438000</v>
+      </c>
+      <c r="E23" s="48" t="n">
+        <v>0.02854980660918057</v>
+      </c>
+      <c r="F23" s="63" t="n">
+        <v>0.8080000000000001</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="42" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C24" s="46" t="n">
+        <v>3000000000</v>
+      </c>
+      <c r="D24" s="46" t="n">
+        <v>73148000</v>
+      </c>
+      <c r="E24" s="48" t="n">
+        <v>0.02438266666666667</v>
+      </c>
+      <c r="F24" s="63" t="n">
+        <v>0.622</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>2024 operating cost is implied — income less impairment less the published profit before tax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="B26" s="42" t="inlineStr">
+        <is>
+          <t>Predicted 2024 profit before tax</t>
+        </is>
+      </c>
+      <c r="C26" s="46" t="n">
+        <v>23993000</v>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>cost carried forward at the 0.808 elasticity measured on 2022-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="B27" s="42" t="inlineStr">
+        <is>
+          <t>Actual 2024 profit before tax</t>
+        </is>
+      </c>
+      <c r="C27" s="46" t="n">
+        <v>29900000</v>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>published</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="26" customHeight="1">
+      <c r="B28" s="42" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="C28" s="48" t="n">
+        <v>-0.198</v>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>under-predicts, because leverage steepened to 0.622 — efficiency improved faster than the prior year could have told you</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>A structural model calibrated on two years of accounts predicted the third to within 20% on profit — the residual of three larger numbers, and the hardest line to get right. Three data points and one bank: directional evidence about structure, not a validated forecast.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="40" customHeight="1">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>Source: Allica Bank Limited, Annual Report and Accounts 2023 (company number 07706156). Total operating income £86,808k; total operating expenses £56,438k; cost:income 65.0%; impairment charges £14,279k; profit before tax £16,091k; net interest margin 5.00%; loans and advances to customers £1,976,826k; colleagues at year end 496.</t>
         </is>
@@ -10309,7 +10473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H195"/>
+  <dimension ref="B1:H199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -15350,7 +15514,7 @@
     <row r="179">
       <c r="B179" s="7" t="inlineStr">
         <is>
-          <t>N. HEAD-OFFICE FIXED COST (scale generalisation, v1.6)</t>
+          <t>O. COST SCALE ELASTICITY (operational leverage, v1.7)</t>
         </is>
       </c>
       <c r="C179" s="8" t="inlineStr"/>
@@ -15388,305 +15552,292 @@
           <t>Unit</t>
         </is>
       </c>
-      <c r="H180" s="40" t="inlineStr"/>
+      <c r="H180" s="9" t="inlineStr">
+        <is>
+          <t>Source / note</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="B181" s="10" t="inlineStr">
         <is>
-          <t>Technology &amp; central operations — fixed component</t>
-        </is>
-      </c>
-      <c r="C181" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D181" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E181" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F181" s="26">
+          <t>Cost scale elasticity — d ln(cost) / d ln(customers)</t>
+        </is>
+      </c>
+      <c r="C181" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D181" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E181" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F181" s="37">
         <f>CHOOSE('Inputs'!$C$4,D181,C181,E181)</f>
         <v/>
       </c>
       <c r="G181" s="14" t="inlineStr">
         <is>
-          <t>£/yr</t>
+          <t>index</t>
         </is>
       </c>
       <c r="H181" s="5" t="inlineStr">
         <is>
-          <t>Head-office cost is otherwise modelled purely per customer, which is a scale assumption in disguise: it only holds near the modelled book size. The Allica FY2023 backtest (tab 11) showed the model under-predicting a sub-scale bank's cost base by 7x for exactly this reason. Set the fixed component to model any bank away from at-scale. Default 0 reproduces the pure per-customer behaviour of v1.5.</t>
+          <t>Every cost line in this model scales linearly with its driver, which forces an elasticity of exactly 1.0 and makes cost per customer flat at every scale. No real business behaves that way. Measured on Allica Bank's published accounts against its lending book: 0.808 across 2022-23, then 0.622 across 2023-24. Applies to the head-office pools, the platform line and change-the-bank — the lines with the least customer-specific content. Default 1.0 reproduces v1.6 exactly.</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="B182" s="10" t="inlineStr">
         <is>
-          <t>Risk, compliance &amp; audit — fixed component</t>
-        </is>
-      </c>
-      <c r="C182" s="27" t="n">
+          <t>Customer count at which the per-customer rates are calibrated</t>
+        </is>
+      </c>
+      <c r="C182" s="20" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D182" s="21" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E182" s="21" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F182" s="22">
+        <f>CHOOSE('Inputs'!$C$4,D182,C182,E182)</f>
+        <v/>
+      </c>
+      <c r="G182" s="14" t="inlineStr">
+        <is>
+          <t>customers</t>
+        </is>
+      </c>
+      <c r="H182" s="5" t="inlineStr">
+        <is>
+          <t>The elasticity pivots around this point: at this customer count the elastic form and the linear form are identical by construction. Set it to the book size the per-customer rates were derived from.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="B183" s="7" t="inlineStr">
+        <is>
+          <t>N. HEAD-OFFICE FIXED COST (scale generalisation, v1.6)</t>
+        </is>
+      </c>
+      <c r="C183" s="8" t="inlineStr"/>
+      <c r="D183" s="8" t="inlineStr"/>
+      <c r="E183" s="8" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="B184" s="9" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C184" s="9" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="D184" s="9" t="inlineStr">
+        <is>
+          <t>Pessimistic</t>
+        </is>
+      </c>
+      <c r="E184" s="9" t="inlineStr">
+        <is>
+          <t>Optimistic</t>
+        </is>
+      </c>
+      <c r="F184" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="G184" s="9" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="H184" s="40" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="B185" s="10" t="inlineStr">
+        <is>
+          <t>Technology &amp; central operations — fixed component</t>
+        </is>
+      </c>
+      <c r="C185" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="D182" s="28" t="n">
+      <c r="D185" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="E182" s="28" t="n">
+      <c r="E185" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="F182" s="26">
-        <f>CHOOSE('Inputs'!$C$4,D182,C182,E182)</f>
-        <v/>
-      </c>
-      <c r="G182" s="14" t="inlineStr">
+      <c r="F185" s="26">
+        <f>CHOOSE('Inputs'!$C$4,D185,C185,E185)</f>
+        <v/>
+      </c>
+      <c r="G185" s="14" t="inlineStr">
         <is>
           <t>£/yr</t>
         </is>
       </c>
-      <c r="H182" s="5" t="inlineStr">
-        <is>
-          <t>As above. Regulatory and compliance cost has a large irreducible floor that does not scale down with customers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="B183" s="10" t="inlineStr">
-        <is>
-          <t>Corporate centre — fixed component</t>
-        </is>
-      </c>
-      <c r="C183" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D183" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E183" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F183" s="26">
-        <f>CHOOSE('Inputs'!$C$4,D183,C183,E183)</f>
-        <v/>
-      </c>
-      <c r="G183" s="14" t="inlineStr">
-        <is>
-          <t>£/yr</t>
-        </is>
-      </c>
-      <c r="H183" s="5" t="inlineStr">
-        <is>
-          <t>As above. Platform build, brand and executive cost are the least customer-driven lines in the model.</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="B184" s="7" t="inlineStr">
-        <is>
-          <t>L. CATEGORY ENTRY POINTS (demand layer, v1.3)</t>
-        </is>
-      </c>
-      <c r="C184" s="8" t="inlineStr"/>
-      <c r="D184" s="8" t="inlineStr"/>
-      <c r="E184" s="8" t="inlineStr"/>
-    </row>
-    <row r="185">
-      <c r="B185" s="9" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="C185" s="9" t="inlineStr">
-        <is>
-          <t>Central</t>
-        </is>
-      </c>
-      <c r="D185" s="9" t="inlineStr">
-        <is>
-          <t>Pessimistic</t>
-        </is>
-      </c>
-      <c r="E185" s="9" t="inlineStr">
-        <is>
-          <t>Optimistic</t>
-        </is>
-      </c>
-      <c r="F185" s="9" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="G185" s="9" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="H185" s="9" t="inlineStr">
-        <is>
-          <t>Source / note</t>
+      <c r="H185" s="5" t="inlineStr">
+        <is>
+          <t>Head-office cost is otherwise modelled purely per customer, which is a scale assumption in disguise: it only holds near the modelled book size. The Allica FY2023 backtest (tab 11) showed the model under-predicting a sub-scale bank's cost base by 7x for exactly this reason. Set the fixed component to model any bank away from at-scale. Default 0 reproduces the pure per-customer behaviour of v1.5.</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="B186" s="10" t="inlineStr">
         <is>
-          <t>CEP layer mode (OFF · CALIBRATE · LIVE)</t>
-        </is>
-      </c>
-      <c r="C186" s="41" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="D186" s="14" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E186" s="14" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F186" s="42">
+          <t>Risk, compliance &amp; audit — fixed component</t>
+        </is>
+      </c>
+      <c r="C186" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D186" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E186" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F186" s="26">
         <f>CHOOSE('Inputs'!$C$4,D186,C186,E186)</f>
         <v/>
       </c>
       <c r="G186" s="14" t="inlineStr">
         <is>
-          <t>mode</t>
+          <t>£/yr</t>
         </is>
       </c>
       <c r="H186" s="5" t="inlineStr">
         <is>
-          <t>The CEP matrix itself is a table, not key/value pairs — it lives on sheet '1b. Demand &amp; CEPs'; edit the blue cells there. OFF = penetrations read the hardcodes below, outputs identical to v1.2. CALIBRATE = diagnostic only, reports the won-event rate implied by today's hardcodes; changes no output. LIVE = penetrations derived from the CEP matrix on 1b, falling back to the hardcode for any product whose CEP rows or holding life are unpopulated.</t>
+          <t>As above. Regulatory and compliance cost has a large irreducible floor that does not scale down with customers.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="B187" s="10" t="inlineStr">
         <is>
-          <t>Instant savings — average holding life</t>
-        </is>
-      </c>
-      <c r="C187" s="29" t="n">
+          <t>Corporate centre — fixed component</t>
+        </is>
+      </c>
+      <c r="C187" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="D187" s="30" t="n">
+      <c r="D187" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="E187" s="30" t="n">
+      <c r="E187" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="F187" s="31">
+      <c r="F187" s="26">
         <f>CHOOSE('Inputs'!$C$4,D187,C187,E187)</f>
         <v/>
       </c>
       <c r="G187" s="14" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>£/yr</t>
         </is>
       </c>
       <c r="H187" s="5" t="inlineStr">
         <is>
-          <t>REQUIRED FOR LIVE MODE — leave 0 and this product falls back to its hardcoded penetration. Cohort query: mean tenure from account-open to account-close on the savings book.</t>
+          <t>As above. Platform build, brand and executive cost are the least customer-driven lines in the model.</t>
         </is>
       </c>
     </row>
     <row r="188">
-      <c r="B188" s="10" t="inlineStr">
-        <is>
-          <t>Notice &amp; fixed — average holding life</t>
-        </is>
-      </c>
-      <c r="C188" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D188" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E188" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F188" s="31">
-        <f>CHOOSE('Inputs'!$C$4,D188,C188,E188)</f>
-        <v/>
-      </c>
-      <c r="G188" s="14" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="H188" s="5" t="inlineStr">
-        <is>
-          <t>REQUIRED FOR LIVE MODE. Cohort query: mean tenure including rollovers; a rolled deposit is one holding, not two.</t>
-        </is>
-      </c>
+      <c r="B188" s="7" t="inlineStr">
+        <is>
+          <t>L. CATEGORY ENTRY POINTS (demand layer, v1.3)</t>
+        </is>
+      </c>
+      <c r="C188" s="8" t="inlineStr"/>
+      <c r="D188" s="8" t="inlineStr"/>
+      <c r="E188" s="8" t="inlineStr"/>
     </row>
     <row r="189">
-      <c r="B189" s="10" t="inlineStr">
-        <is>
-          <t>Overdraft — average facility life</t>
-        </is>
-      </c>
-      <c r="C189" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D189" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E189" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F189" s="31">
-        <f>CHOOSE('Inputs'!$C$4,D189,C189,E189)</f>
-        <v/>
-      </c>
-      <c r="G189" s="14" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="H189" s="5" t="inlineStr">
-        <is>
-          <t>REQUIRED FOR LIVE MODE. Cohort query: mean time from facility grant to facility closed (not annual renewal).</t>
+      <c r="B189" s="9" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C189" s="9" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="D189" s="9" t="inlineStr">
+        <is>
+          <t>Pessimistic</t>
+        </is>
+      </c>
+      <c r="E189" s="9" t="inlineStr">
+        <is>
+          <t>Optimistic</t>
+        </is>
+      </c>
+      <c r="F189" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="G189" s="9" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="H189" s="9" t="inlineStr">
+        <is>
+          <t>Source / note</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="B190" s="10" t="inlineStr">
         <is>
-          <t>Business credit card — average holding life</t>
-        </is>
-      </c>
-      <c r="C190" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D190" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E190" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F190" s="31">
+          <t>CEP layer mode (OFF · CALIBRATE · LIVE)</t>
+        </is>
+      </c>
+      <c r="C190" s="41" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="D190" s="14" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E190" s="14" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F190" s="42">
         <f>CHOOSE('Inputs'!$C$4,D190,C190,E190)</f>
         <v/>
       </c>
       <c r="G190" s="14" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>mode</t>
         </is>
       </c>
       <c r="H190" s="5" t="inlineStr">
         <is>
-          <t>REQUIRED FOR LIVE MODE. Cohort query: mean tenure from card issued to account closed.</t>
+          <t>The CEP matrix itself is a table, not key/value pairs — it lives on sheet '1b. Demand &amp; CEPs'; edit the blue cells there. OFF = penetrations read the hardcodes below, outputs identical to v1.2. CALIBRATE = diagnostic only, reports the won-event rate implied by today's hardcodes; changes no output. LIVE = penetrations derived from the CEP matrix on 1b, falling back to the hardcode for any product whose CEP rows or holding life are unpopulated.</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="B191" s="10" t="inlineStr">
         <is>
-          <t>Payments &amp; FX — average active-user life</t>
+          <t>Instant savings — average holding life</t>
         </is>
       </c>
       <c r="C191" s="29" t="n">
@@ -15709,118 +15860,238 @@
       </c>
       <c r="H191" s="5" t="inlineStr">
         <is>
-          <t>REQUIRED FOR LIVE MODE. Cohort query: mean time from first international payment to 12 months' inactivity.</t>
+          <t>REQUIRED FOR LIVE MODE — leave 0 and this product falls back to its hardcoded penetration. Cohort query: mean tenure from account-open to account-close on the savings book.</t>
         </is>
       </c>
     </row>
     <row r="192">
-      <c r="B192" s="7" t="inlineStr">
-        <is>
-          <t>M. PROCESS LAYER (Step 2 performance, v1.4)</t>
-        </is>
-      </c>
-      <c r="C192" s="8" t="inlineStr"/>
-      <c r="D192" s="8" t="inlineStr"/>
-      <c r="E192" s="8" t="inlineStr"/>
+      <c r="B192" s="10" t="inlineStr">
+        <is>
+          <t>Notice &amp; fixed — average holding life</t>
+        </is>
+      </c>
+      <c r="C192" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D192" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E192" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F192" s="31">
+        <f>CHOOSE('Inputs'!$C$4,D192,C192,E192)</f>
+        <v/>
+      </c>
+      <c r="G192" s="14" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="H192" s="5" t="inlineStr">
+        <is>
+          <t>REQUIRED FOR LIVE MODE. Cohort query: mean tenure including rollovers; a rolled deposit is one holding, not two.</t>
+        </is>
+      </c>
     </row>
     <row r="193">
-      <c r="B193" s="9" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="C193" s="9" t="inlineStr">
-        <is>
-          <t>Central</t>
-        </is>
-      </c>
-      <c r="D193" s="9" t="inlineStr">
-        <is>
-          <t>Pessimistic</t>
-        </is>
-      </c>
-      <c r="E193" s="9" t="inlineStr">
-        <is>
-          <t>Optimistic</t>
-        </is>
-      </c>
-      <c r="F193" s="9" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="G193" s="9" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="H193" s="9" t="inlineStr">
-        <is>
-          <t>Source / note</t>
+      <c r="B193" s="10" t="inlineStr">
+        <is>
+          <t>Overdraft — average facility life</t>
+        </is>
+      </c>
+      <c r="C193" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D193" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E193" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F193" s="31">
+        <f>CHOOSE('Inputs'!$C$4,D193,C193,E193)</f>
+        <v/>
+      </c>
+      <c r="G193" s="14" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="H193" s="5" t="inlineStr">
+        <is>
+          <t>REQUIRED FOR LIVE MODE. Cohort query: mean time from facility grant to facility closed (not annual renewal).</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="B194" s="10" t="inlineStr">
         <is>
-          <t>Process layer mode (OFF · DIAGNOSE · LIVE)</t>
-        </is>
-      </c>
-      <c r="C194" s="41" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="D194" s="14" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E194" s="14" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="F194" s="42">
+          <t>Business credit card — average holding life</t>
+        </is>
+      </c>
+      <c r="C194" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D194" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E194" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F194" s="31">
         <f>CHOOSE('Inputs'!$C$4,D194,C194,E194)</f>
         <v/>
       </c>
       <c r="G194" s="14" t="inlineStr">
         <is>
-          <t>mode</t>
+          <t>years</t>
         </is>
       </c>
       <c r="H194" s="5" t="inlineStr">
         <is>
-          <t>OFF = yield held at 100% and no named head-office processes; outputs identical to v1.3. DIAGNOSE = reports gaps, the top-down imputation and the process-owned share; changes no output. LIVE = yields and named head-office processes in force. Yield below 100% genuinely raises cost — that is the finding, not a defect. The performance columns live on tab 3 (L-S) because Step 2 IS running costs.</t>
+          <t>REQUIRED FOR LIVE MODE. Cohort query: mean tenure from card issued to account closed.</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="B195" s="10" t="inlineStr">
         <is>
+          <t>Payments &amp; FX — average active-user life</t>
+        </is>
+      </c>
+      <c r="C195" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E195" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F195" s="31">
+        <f>CHOOSE('Inputs'!$C$4,D195,C195,E195)</f>
+        <v/>
+      </c>
+      <c r="G195" s="14" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="H195" s="5" t="inlineStr">
+        <is>
+          <t>REQUIRED FOR LIVE MODE. Cohort query: mean time from first international payment to 12 months' inactivity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="B196" s="7" t="inlineStr">
+        <is>
+          <t>M. PROCESS LAYER (Step 2 performance, v1.4)</t>
+        </is>
+      </c>
+      <c r="C196" s="8" t="inlineStr"/>
+      <c r="D196" s="8" t="inlineStr"/>
+      <c r="E196" s="8" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="B197" s="9" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C197" s="9" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="D197" s="9" t="inlineStr">
+        <is>
+          <t>Pessimistic</t>
+        </is>
+      </c>
+      <c r="E197" s="9" t="inlineStr">
+        <is>
+          <t>Optimistic</t>
+        </is>
+      </c>
+      <c r="F197" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="G197" s="9" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="H197" s="9" t="inlineStr">
+        <is>
+          <t>Source / note</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="B198" s="10" t="inlineStr">
+        <is>
+          <t>Process layer mode (OFF · DIAGNOSE · LIVE)</t>
+        </is>
+      </c>
+      <c r="C198" s="41" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="D198" s="14" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E198" s="14" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F198" s="42">
+        <f>CHOOSE('Inputs'!$C$4,D198,C198,E198)</f>
+        <v/>
+      </c>
+      <c r="G198" s="14" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="H198" s="5" t="inlineStr">
+        <is>
+          <t>OFF = yield held at 100% and no named head-office processes; outputs identical to v1.3. DIAGNOSE = reports gaps, the top-down imputation and the process-owned share; changes no output. LIVE = yields and named head-office processes in force. Yield below 100% genuinely raises cost — that is the finding, not a defect. The performance columns live on tab 3 (L-S) because Step 2 IS running costs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="B199" s="10" t="inlineStr">
+        <is>
           <t>Top-down benchmark: target cost:income ratio</t>
         </is>
       </c>
-      <c r="C195" s="23" t="n">
+      <c r="C199" s="23" t="n">
         <v>0.26</v>
       </c>
-      <c r="D195" s="18" t="n">
+      <c r="D199" s="18" t="n">
         <v>0.26</v>
       </c>
-      <c r="E195" s="18" t="n">
+      <c r="E199" s="18" t="n">
         <v>0.26</v>
       </c>
-      <c r="F195" s="19">
-        <f>CHOOSE('Inputs'!$C$4,D195,C195,E195)</f>
-        <v/>
-      </c>
-      <c r="G195" s="14" t="inlineStr">
+      <c r="F199" s="19">
+        <f>CHOOSE('Inputs'!$C$4,D199,C199,E199)</f>
+        <v/>
+      </c>
+      <c r="G199" s="14" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="H195" s="5" t="inlineStr">
+      <c r="H199" s="5" t="inlineStr">
         <is>
           <t>The only benchmark that actually exists at bank level. Specialist SME banks: OakNorth ~26%, Allica ~50%. Process-level benchmarks are not published, so DIAGNOSE imputes what each process would have to become to reach this. An imputed target is NOT evidence that anyone achieves it.</t>
         </is>
@@ -16377,7 +16648,7 @@
         </is>
       </c>
       <c r="C5" s="49">
-        <f>'Inputs'!$F$186</f>
+        <f>'Inputs'!$F$190</f>
         <v/>
       </c>
     </row>
@@ -17239,7 +17510,7 @@
         <v/>
       </c>
       <c r="E41" s="55">
-        <f>'Inputs'!$F$187</f>
+        <f>'Inputs'!$F$191</f>
         <v/>
       </c>
       <c r="F41" s="48">
@@ -17279,7 +17550,7 @@
         <v/>
       </c>
       <c r="E42" s="55">
-        <f>'Inputs'!$F$188</f>
+        <f>'Inputs'!$F$192</f>
         <v/>
       </c>
       <c r="F42" s="48">
@@ -17319,7 +17590,7 @@
         <v/>
       </c>
       <c r="E43" s="55">
-        <f>'Inputs'!$F$189</f>
+        <f>'Inputs'!$F$193</f>
         <v/>
       </c>
       <c r="F43" s="48">
@@ -17479,7 +17750,7 @@
         <v/>
       </c>
       <c r="E47" s="55">
-        <f>'Inputs'!$F$190</f>
+        <f>'Inputs'!$F$194</f>
         <v/>
       </c>
       <c r="F47" s="48">
@@ -17519,7 +17790,7 @@
         <v/>
       </c>
       <c r="E48" s="55">
-        <f>'Inputs'!$F$191</f>
+        <f>'Inputs'!$F$195</f>
         <v/>
       </c>
       <c r="F48" s="48">
@@ -18590,7 +18861,7 @@
         <v>1</v>
       </c>
       <c r="O11" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E11,IF(M11&lt;&gt;"TRANSACTIONAL",E11,IF(OR(N11="",N11&lt;=0),E11,E11/N11)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E11,IF(M11&lt;&gt;"TRANSACTIONAL",E11,IF(OR(N11="",N11&lt;=0),E11,E11/N11)))</f>
         <v/>
       </c>
       <c r="P11" s="17" t="n"/>
@@ -18658,7 +18929,7 @@
         </is>
       </c>
       <c r="O12" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E12,IF(M12&lt;&gt;"TRANSACTIONAL",E12,IF(OR(N12="",N12&lt;=0),E12,E12/N12)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E12,IF(M12&lt;&gt;"TRANSACTIONAL",E12,IF(OR(N12="",N12&lt;=0),E12,E12/N12)))</f>
         <v/>
       </c>
       <c r="P12" s="17" t="n"/>
@@ -18725,7 +18996,7 @@
         </is>
       </c>
       <c r="O13" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E13,IF(M13&lt;&gt;"TRANSACTIONAL",E13,IF(OR(N13="",N13&lt;=0),E13,E13/N13)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E13,IF(M13&lt;&gt;"TRANSACTIONAL",E13,IF(OR(N13="",N13&lt;=0),E13,E13/N13)))</f>
         <v/>
       </c>
       <c r="P13" s="17" t="n"/>
@@ -18792,7 +19063,7 @@
         </is>
       </c>
       <c r="O14" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E14,IF(M14&lt;&gt;"TRANSACTIONAL",E14,IF(OR(N14="",N14&lt;=0),E14,E14/N14)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E14,IF(M14&lt;&gt;"TRANSACTIONAL",E14,IF(OR(N14="",N14&lt;=0),E14,E14/N14)))</f>
         <v/>
       </c>
       <c r="P14" s="17" t="n"/>
@@ -18859,7 +19130,7 @@
         </is>
       </c>
       <c r="O15" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E15,IF(M15&lt;&gt;"TRANSACTIONAL",E15,IF(OR(N15="",N15&lt;=0),E15,E15/N15)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E15,IF(M15&lt;&gt;"TRANSACTIONAL",E15,IF(OR(N15="",N15&lt;=0),E15,E15/N15)))</f>
         <v/>
       </c>
       <c r="P15" s="17" t="n"/>
@@ -18929,7 +19200,7 @@
         <v>1</v>
       </c>
       <c r="O16" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E16,IF(M16&lt;&gt;"TRANSACTIONAL",E16,IF(OR(N16="",N16&lt;=0),E16,E16/N16)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E16,IF(M16&lt;&gt;"TRANSACTIONAL",E16,IF(OR(N16="",N16&lt;=0),E16,E16/N16)))</f>
         <v/>
       </c>
       <c r="P16" s="17" t="n"/>
@@ -18997,7 +19268,7 @@
         </is>
       </c>
       <c r="O17" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E17,IF(M17&lt;&gt;"TRANSACTIONAL",E17,IF(OR(N17="",N17&lt;=0),E17,E17/N17)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E17,IF(M17&lt;&gt;"TRANSACTIONAL",E17,IF(OR(N17="",N17&lt;=0),E17,E17/N17)))</f>
         <v/>
       </c>
       <c r="P17" s="17" t="n"/>
@@ -19067,7 +19338,7 @@
         <v>1</v>
       </c>
       <c r="O18" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E18,IF(M18&lt;&gt;"TRANSACTIONAL",E18,IF(OR(N18="",N18&lt;=0),E18,E18/N18)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E18,IF(M18&lt;&gt;"TRANSACTIONAL",E18,IF(OR(N18="",N18&lt;=0),E18,E18/N18)))</f>
         <v/>
       </c>
       <c r="P18" s="17" t="n"/>
@@ -19138,7 +19409,7 @@
         <v>1</v>
       </c>
       <c r="O19" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E19,IF(M19&lt;&gt;"TRANSACTIONAL",E19,IF(OR(N19="",N19&lt;=0),E19,E19/N19)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E19,IF(M19&lt;&gt;"TRANSACTIONAL",E19,IF(OR(N19="",N19&lt;=0),E19,E19/N19)))</f>
         <v/>
       </c>
       <c r="P19" s="17" t="n"/>
@@ -19206,7 +19477,7 @@
         </is>
       </c>
       <c r="O20" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E20,IF(M20&lt;&gt;"TRANSACTIONAL",E20,IF(OR(N20="",N20&lt;=0),E20,E20/N20)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E20,IF(M20&lt;&gt;"TRANSACTIONAL",E20,IF(OR(N20="",N20&lt;=0),E20,E20/N20)))</f>
         <v/>
       </c>
       <c r="P20" s="17" t="n"/>
@@ -19273,7 +19544,7 @@
         </is>
       </c>
       <c r="O21" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E21,IF(M21&lt;&gt;"TRANSACTIONAL",E21,IF(OR(N21="",N21&lt;=0),E21,E21/N21)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E21,IF(M21&lt;&gt;"TRANSACTIONAL",E21,IF(OR(N21="",N21&lt;=0),E21,E21/N21)))</f>
         <v/>
       </c>
       <c r="P21" s="17" t="n"/>
@@ -19340,7 +19611,7 @@
         </is>
       </c>
       <c r="O22" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E22,IF(M22&lt;&gt;"TRANSACTIONAL",E22,IF(OR(N22="",N22&lt;=0),E22,E22/N22)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E22,IF(M22&lt;&gt;"TRANSACTIONAL",E22,IF(OR(N22="",N22&lt;=0),E22,E22/N22)))</f>
         <v/>
       </c>
       <c r="P22" s="17" t="n"/>
@@ -19407,7 +19678,7 @@
         </is>
       </c>
       <c r="O23" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E23,IF(M23&lt;&gt;"TRANSACTIONAL",E23,IF(OR(N23="",N23&lt;=0),E23,E23/N23)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E23,IF(M23&lt;&gt;"TRANSACTIONAL",E23,IF(OR(N23="",N23&lt;=0),E23,E23/N23)))</f>
         <v/>
       </c>
       <c r="P23" s="17" t="n"/>
@@ -19474,7 +19745,7 @@
         </is>
       </c>
       <c r="O24" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E24,IF(M24&lt;&gt;"TRANSACTIONAL",E24,IF(OR(N24="",N24&lt;=0),E24,E24/N24)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E24,IF(M24&lt;&gt;"TRANSACTIONAL",E24,IF(OR(N24="",N24&lt;=0),E24,E24/N24)))</f>
         <v/>
       </c>
       <c r="P24" s="17" t="n"/>
@@ -19541,7 +19812,7 @@
         </is>
       </c>
       <c r="O25" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E25,IF(M25&lt;&gt;"TRANSACTIONAL",E25,IF(OR(N25="",N25&lt;=0),E25,E25/N25)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E25,IF(M25&lt;&gt;"TRANSACTIONAL",E25,IF(OR(N25="",N25&lt;=0),E25,E25/N25)))</f>
         <v/>
       </c>
       <c r="P25" s="17" t="n"/>
@@ -19608,7 +19879,7 @@
         </is>
       </c>
       <c r="O26" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E26,IF(M26&lt;&gt;"TRANSACTIONAL",E26,IF(OR(N26="",N26&lt;=0),E26,E26/N26)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E26,IF(M26&lt;&gt;"TRANSACTIONAL",E26,IF(OR(N26="",N26&lt;=0),E26,E26/N26)))</f>
         <v/>
       </c>
       <c r="P26" s="17" t="n"/>
@@ -19675,7 +19946,7 @@
         </is>
       </c>
       <c r="O27" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E27,IF(M27&lt;&gt;"TRANSACTIONAL",E27,IF(OR(N27="",N27&lt;=0),E27,E27/N27)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E27,IF(M27&lt;&gt;"TRANSACTIONAL",E27,IF(OR(N27="",N27&lt;=0),E27,E27/N27)))</f>
         <v/>
       </c>
       <c r="P27" s="17" t="n"/>
@@ -19742,7 +20013,7 @@
         </is>
       </c>
       <c r="O28" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E28,IF(M28&lt;&gt;"TRANSACTIONAL",E28,IF(OR(N28="",N28&lt;=0),E28,E28/N28)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E28,IF(M28&lt;&gt;"TRANSACTIONAL",E28,IF(OR(N28="",N28&lt;=0),E28,E28/N28)))</f>
         <v/>
       </c>
       <c r="P28" s="17" t="n"/>
@@ -19809,7 +20080,7 @@
         </is>
       </c>
       <c r="O29" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E29,IF(M29&lt;&gt;"TRANSACTIONAL",E29,IF(OR(N29="",N29&lt;=0),E29,E29/N29)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E29,IF(M29&lt;&gt;"TRANSACTIONAL",E29,IF(OR(N29="",N29&lt;=0),E29,E29/N29)))</f>
         <v/>
       </c>
       <c r="P29" s="17" t="n"/>
@@ -19876,7 +20147,7 @@
         </is>
       </c>
       <c r="O30" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E30,IF(M30&lt;&gt;"TRANSACTIONAL",E30,IF(OR(N30="",N30&lt;=0),E30,E30/N30)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E30,IF(M30&lt;&gt;"TRANSACTIONAL",E30,IF(OR(N30="",N30&lt;=0),E30,E30/N30)))</f>
         <v/>
       </c>
       <c r="P30" s="17" t="n"/>
@@ -19943,7 +20214,7 @@
         </is>
       </c>
       <c r="O31" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E31,IF(M31&lt;&gt;"TRANSACTIONAL",E31,IF(OR(N31="",N31&lt;=0),E31,E31/N31)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E31,IF(M31&lt;&gt;"TRANSACTIONAL",E31,IF(OR(N31="",N31&lt;=0),E31,E31/N31)))</f>
         <v/>
       </c>
       <c r="P31" s="17" t="n"/>
@@ -20010,7 +20281,7 @@
         </is>
       </c>
       <c r="O32" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E32,IF(M32&lt;&gt;"TRANSACTIONAL",E32,IF(OR(N32="",N32&lt;=0),E32,E32/N32)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E32,IF(M32&lt;&gt;"TRANSACTIONAL",E32,IF(OR(N32="",N32&lt;=0),E32,E32/N32)))</f>
         <v/>
       </c>
       <c r="P32" s="17" t="n"/>
@@ -20077,7 +20348,7 @@
         </is>
       </c>
       <c r="O33" s="44">
-        <f>IF('Inputs'!$F$194&lt;&gt;"LIVE",E33,IF(M33&lt;&gt;"TRANSACTIONAL",E33,IF(OR(N33="",N33&lt;=0),E33,E33/N33)))</f>
+        <f>IF('Inputs'!$F$198&lt;&gt;"LIVE",E33,IF(M33&lt;&gt;"TRANSACTIONAL",E33,IF(OR(N33="",N33&lt;=0),E33,E33/N33)))</f>
         <v/>
       </c>
       <c r="P33" s="17" t="n"/>
@@ -23935,7 +24206,7 @@
         </is>
       </c>
       <c r="H67" s="48">
-        <f>'Inputs'!$F$195</f>
+        <f>'Inputs'!$F$199</f>
         <v/>
       </c>
       <c r="J67" s="5" t="inlineStr">
@@ -24156,7 +24427,7 @@
         </is>
       </c>
       <c r="C7" s="46">
-        <f>'1. Customers'!$C$4*'Inputs'!$F$128</f>
+        <f>'Inputs'!$F$182*'Inputs'!$F$128*('1. Customers'!$C$4/'Inputs'!$F$182)^'Inputs'!$F$181</f>
         <v/>
       </c>
       <c r="D7" s="62" t="inlineStr">
@@ -24245,7 +24516,7 @@
         </is>
       </c>
       <c r="C13" s="46">
-        <f>'1. Customers'!$C$4*'Inputs'!$F$129+'Inputs'!$F$181</f>
+        <f>'Inputs'!$F$182*'Inputs'!$F$129*('1. Customers'!$C$4/'Inputs'!$F$182)^'Inputs'!$F$181+'Inputs'!$F$185</f>
         <v/>
       </c>
       <c r="E13" s="14" t="inlineStr">
@@ -24261,7 +24532,7 @@
         </is>
       </c>
       <c r="C14" s="46">
-        <f>'1. Customers'!$C$4*'Inputs'!$F$130+'Inputs'!$F$182</f>
+        <f>'Inputs'!$F$182*'Inputs'!$F$130*('1. Customers'!$C$4/'Inputs'!$F$182)^'Inputs'!$F$181+'Inputs'!$F$186</f>
         <v/>
       </c>
       <c r="E14" s="14" t="inlineStr">
@@ -24277,7 +24548,7 @@
         </is>
       </c>
       <c r="C15" s="46">
-        <f>'1. Customers'!$C$4*'Inputs'!$F$131+'Inputs'!$F$183</f>
+        <f>'Inputs'!$F$182*'Inputs'!$F$131*('1. Customers'!$C$4/'Inputs'!$F$182)^'Inputs'!$F$181+'Inputs'!$F$187</f>
         <v/>
       </c>
       <c r="E15" s="14" t="inlineStr">
@@ -24320,7 +24591,7 @@
         </is>
       </c>
       <c r="C19" s="68">
-        <f>'1. Customers'!$C$4*'Inputs'!$F$145</f>
+        <f>'Inputs'!$F$182*'Inputs'!$F$145*('1. Customers'!$C$4/'Inputs'!$F$182)^'Inputs'!$F$181</f>
         <v/>
       </c>
       <c r="E19" s="14" t="inlineStr">

</xml_diff>

<commit_message>
v1.8: break-even demand elasticity on tab 10
The elasticity ranking assumed nothing responds to price, which made raising any price
look accretive. Tab 10 now leads with the demand elasticity at which each price stops
paying — the card fee breaks even at 0.06, the loan rate holds to 2.91.
</commit_message>
<xml_diff>
--- a/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
+++ b/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B48"/>
+  <dimension ref="B1:B49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -606,7 +606,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MODEL VERSION: v1.7 · 22 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
+          <t>MODEL VERSION: v1.8 · 22 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
         </is>
       </c>
     </row>
@@ -620,264 +620,271 @@
     <row r="5" ht="52" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>• v1.7 (22 Aug 2026) — operational leverage. Every cost line in the model scaled linearly with its driver, which forces a cost elasticity of exactly 1.0 and makes cost per customer flat at every scale. Allica Bank's own accounts put that elasticity at 0.808 across 2022-23 and 0.622 across 2023-24 — cost rises materially more slowly than the book. Inputs section O adds a cost scale elasticity and the customer count the per-customer rates are calibrated at; the head-office pools, the platform line and change-the-bank now scale by it. Default 1.0 reproduces v1.6 exactly. Tab 11 adds the out-of-sample test that measured it.</t>
+          <t>• v1.8 (22 Aug 2026) — break-even demand elasticity on tab 10. The elasticity table ranked the term loan customer rate as the largest driver of profit at +1.25, which was an artefact: nothing in the model responds to price, so raising any price always looked accretive. Tab 10 now leads with the demand elasticity at which raising each price stops paying. The reordering matters — the card fee breaks even at 0.06 and the current-account fee at 0.13, so both are fragile to almost any customer response, while the loan rate holds to 2.91. The hidden assumption being replaced is zero, which is the least defensible value available.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="52" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>• v1.6 (22 Aug 2026) — validation and drivers. Tab 10 ELASTICITIES: every input bumped +1% and the workbook recalculated, giving the % change in PBT, cost:income, RoE and income. Only one input has an elasticity above 1 on profit — the term loan customer rate, at +1.25; reachable market and penetration are exactly +1.00 (pure scale); nothing else exceeds 0.53. Tab 11 BACKTEST against Allica Bank FY2023 audited accounts: the revenue engine reproduces a real bank's operating income to within 8%, and the cost engine under-predicts by 7x. Diagnosis: head-office cost was modelled purely per customer, which is a scale assumption disguised as a driver. Inputs section N therefore adds a fixed component to each head-office pool, defaulting to 0 so v1.5 results are unchanged.</t>
+          <t>• v1.7 (22 Aug 2026) — operational leverage. Every cost line in the model scaled linearly with its driver, which forces a cost elasticity of exactly 1.0 and makes cost per customer flat at every scale. Allica Bank's own accounts put that elasticity at 0.808 across 2022-23 and 0.622 across 2023-24 — cost rises materially more slowly than the book. Inputs section O adds a cost scale elasticity and the customer count the per-customer rates are calibrated at; the head-office pools, the platform line and change-the-bank now scale by it. Default 1.0 reproduces v1.6 exactly. Tab 11 adds the out-of-sample test that measured it.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>• v1.5 (22 Aug 2026) — PROCESS LAYER on the Step 2 tabs. Tab 3 gains process columns M-T (process type, yield, attempts, automation, best-in-class intensity and yield, benchmark source, £ gap) and a HEAD-OFFICE PROCESS REGISTER of 22 processes already named in the tab 9 operational model but never costed. Yield inflates ATTEMPTS and never deflates outcomes — that is what stops it double-counting with the CEP layer's demand-side conversion. Head-office costs are carved OUT of the pools, so naming a process moves money from unallocated to attributed and the total never changes. New sheet 3b indexes every process to the numbers it moves, and imputes what each would have to become to hit a target cost:income. Mode OFF (default) = results identical to v1.4.</t>
+          <t>• v1.6 (22 Aug 2026) — validation and drivers. Tab 10 ELASTICITIES: every input bumped +1% and the workbook recalculated, giving the % change in PBT, cost:income, RoE and income. Only one input has an elasticity above 1 on profit — the term loan customer rate, at +1.25; reachable market and penetration are exactly +1.00 (pure scale); nothing else exceeds 0.53. Tab 11 BACKTEST against Allica Bank FY2023 audited accounts: the revenue engine reproduces a real bank's operating income to within 8%, and the cost engine under-predicts by 7x. Diagnosis: head-office cost was modelled purely per customer, which is a scale assumption disguised as a driver. Inputs section N therefore adds a fixed component to each head-office pool, defaulting to 0 so v1.5 results are unchanged.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
+          <t>• v1.5 (22 Aug 2026) — PROCESS LAYER on the Step 2 tabs. Tab 3 gains process columns M-T (process type, yield, attempts, automation, best-in-class intensity and yield, benchmark source, £ gap) and a HEAD-OFFICE PROCESS REGISTER of 22 processes already named in the tab 9 operational model but never costed. Yield inflates ATTEMPTS and never deflates outcomes — that is what stops it double-counting with the CEP layer's demand-side conversion. Head-office costs are carved OUT of the pools, so naming a process moves money from unallocated to attributed and the total never changes. New sheet 3b indexes every process to the numbers it moves, and imputes what each would have to become to hit a target cost:income. Mode OFF (default) = results identical to v1.4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
           <t>• v1.4 (22 Aug 2026) — CEP DEMAND LAYER. New sheet 1b derives the nine product penetrations and the customer count instead of asserting them: penetration = (lambda*c x L) / (1 + lambda*c x L), where lambda*c = category-entry-point events x presence x conversion and L is the holding life. Little's Law run forwards; no time axis is added and the model stays a steady-state snapshot. Ships deliberately EMPTY — every event/presence/conversion cell is blank and carries the cohort query that fills it, and any unpopulated product falls back to its hardcoded penetration. Mode OFF (default) = results identical to v1.3; CALIBRATE reports the won-event rate implied by today's assumptions and changes nothing.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
+    <row r="10" ht="40" customHeight="1">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>• v1.3 (21 Aug 2026) — churn replacement is a costed activity end-to-end: new input cac_new (£240 acquisition marketing per new customer won, carved out of the corporate-centre pool — hq_oh £250→£222); driver-linked on tab 4, attributed to the current account (gateway product) on tab 6; 'value of preventing one churn' memo added to tab 6. Raising the churn input now inflates demand-generation cost, not just processing. Central PBT shifts &lt;£1k/unit (carve-out rounding).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
+          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="B13" s="4" t="inlineStr">
         <is>
+          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
           <t>• v1.0 (10 Aug 2026) — first published version: 9 tabs + flow register, FTP with liquidity/behavioural terms, fraud/FSCS/change-the-bank lines, segment-pod LMUs, bridge check.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="3" t="inlineStr">
+    <row r="16">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>What this is</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="39" customHeight="1">
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="39" customHeight="1">
       <c r="B17" s="4" t="inlineStr">
         <is>
+          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="39" customHeight="1">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
           <t>• It follows the Simanis / IVE bottom-up methodology ('Running the Right Numbers'): model the last-mile operating unit, derive every cost from activity drivers (transaction intensity I and customer load L), build whole costs, and check the price/margin covers them including a competitive return on capital.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="3" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>What period this models</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="26" customHeight="1">
-      <c r="B20" s="4" t="inlineStr">
+    <row r="21" ht="26" customHeight="1">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>• One representative operating year at steady state. Balances are annual averages; rates and volumes are annual. There is no time axis, no ramp and no vintage cohorts — the model is a snapshot, not a forecast.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="78" customHeight="1">
-      <c r="B21" s="4" t="inlineStr">
+    <row r="22" ht="78" customHeight="1">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>• The book is stationary but not free to hold flat: customers churn (12% p.a. input) and the model costs their replacement end-to-end — acquisition marketing per new customer won (cac_new, carved from the corporate-centre pool), onboarding hours, KYC per new customer and RM origination effort are all driver-linked (Simanis: at-scale operations include 'replacement of customer churn'). Only residual brand &amp; joint marketing remains pool-costed. The 'value of preventing one churn' memo on tab 6 prices retention: contribution annuity over remaining relationship life + the avoided replacement cost.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="B22" s="4" t="inlineStr">
+    <row r="23" ht="26" customHeight="1">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>• The capital charge (cost of equity on allocated capital) is the incumbent analogue of Simanis's start-up-cost amortisation: capital earns its required return inside the steady-state P&amp;L.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="52" customHeight="1">
-      <c r="B23" s="4" t="inlineStr">
+    <row r="24" ht="52" customHeight="1">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>• Out of scope by design: transition paths. The cost and cash shape of moving between steady states — digital migration, maturity glide, behaviour-change programmes and their CAC/incentives — belongs in a scenario layer built ON TOP of this base (comparative statics between two runs of this model, plus a separate transition-cost estimate). The base model never carries scenario logic.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="3" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>How the tabs map to the methodology</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="B26" s="4" t="inlineStr">
+    <row r="27" ht="24" customHeight="1">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>• Inputs — every assumption in one place, with sources. Edit blue cells; yellow cells are the biggest levers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="26" customHeight="1">
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="26" customHeight="1">
       <c r="B28" s="4" t="inlineStr">
         <is>
+          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="26" customHeight="1">
+      <c r="B29" s="4" t="inlineStr">
+        <is>
           <t>• 2. Revenues — unit revenue per product: interest margins measured against internal funds transfer prices (Bank Rate for floating, + premium for term), plus fees.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="39" customHeight="1">
-      <c r="B29" s="4" t="inlineStr">
+    <row r="30" ht="39" customHeight="1">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>• 3. HR &amp; Activity — Step 2: every FTE derived from activity drivers (hours per onboarding, review, renewal…) — nothing is assumed as headcount. From v1.5 this tab is also the PROCESS REGISTER (columns M-T), with the head-office process register below it.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="26" customHeight="1">
-      <c r="B30" s="4" t="inlineStr">
+    <row r="31" ht="26" customHeight="1">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>• 1b. Demand &amp; CEPs — the demand layer (v1.4). Penetration is derived, not assumed. Mode cell on Inputs section L: OFF reproduces v1.3, CALIBRATE reports the implied event rates, LIVE derives.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="39" customHeight="1">
-      <c r="B31" s="4" t="inlineStr">
+    <row r="32" ht="39" customHeight="1">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>• 3b. Process Index — derived view, no assumptions. Every process with its flow, product, owner, the numbers it moves, its cost and its gap to best in class, plus a ranked worst-gap list and the top-down benchmark imputation. Answers 'which process do I improve to move this number?'</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="52" customHeight="1">
-      <c r="B32" s="4" t="inlineStr">
+    <row r="33" ht="52" customHeight="1">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>• 4. Running Costs — Step 2 (cont.): direct running costs plus the share of head-office costs. The attribution memo reads the tab 3 process register and reports the share of the cost base with a named process owner — the model's own assessment of how much of its cost it actually understands. What remains in UNALLOCATED JOINT COSTS is cost with no process to improve.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="26" customHeight="1">
-      <c r="B33" s="4" t="inlineStr">
+    <row r="34" ht="26" customHeight="1">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>• 5. Risk &amp; Capital — Step 3: expected credit losses (PD × LGD), risk-weighted assets, allocated equity, and the required return on it.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="91" customHeight="1">
-      <c r="B34" s="4" t="inlineStr">
+    <row r="35" ht="91" customHeight="1">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>• 6. Unit Economics — Steps 4–5: per-product unit costs and revenues on an activity-based costing basis, taken exactly as far as causality runs (the source methodology's own rule: link costs to customers and transactions 'whenever possible'). Costs with real drivers — servicing hours, RM effort per origination, staff-time-driven supervision, per-account and per-facility infrastructure — are attributed to products; genuinely joint costs (brand, exec, finance, platform build) are NOT forced into products but held as an unallocated hurdle that total contribution must clear, with a full-absorption memo showing the source doc's simple-division treatment. Product decisions should run on contribution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="26" customHeight="1">
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="26" customHeight="1">
       <c r="B36" s="4" t="inlineStr">
         <is>
+          <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="26" customHeight="1">
+      <c r="B37" s="4" t="inlineStr">
+        <is>
           <t>• 8. Org Structure — the whole-bank organisation implied by the model: front-line FTEs from activity drivers × number of centres, head-office FTEs backed out of the per-customer head-office cost allocations.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="52" customHeight="1">
-      <c r="B37" s="4" t="inlineStr">
+    <row r="38" ht="52" customHeight="1">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>• 9. Flow Register — one row per flow on the operational model map: component type (CP/WP/PP/PartP), core/support/enabling, direction, digital/physical medium, the direct/administrative/managerial roles accountable, and the BIAN service domains. Ends with a BIAN completeness checklist. This is where the map, the ARM and BIAN reconcile.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="B39" s="3" t="inlineStr">
+    <row r="40">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>Colour legend</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="26" customHeight="1">
-      <c r="B40" s="4" t="inlineStr">
+    <row r="41" ht="26" customHeight="1">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>• Blue = hardcoded input (edit these) · Yellow fill = key assumption / sensitivity lever · Black = formula · Green = link to another sheet.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="B42" s="3" t="inlineStr">
+    <row r="43">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>Reading the results</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="52" customHeight="1">
-      <c r="B43" s="4" t="inlineStr">
+    <row r="44" ht="52" customHeight="1">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>• Deposit products earn the spread between the transfer price and the rate paid; lending earns the customer rate minus the transfer price minus expected losses. Capital-heavy, labour-heavy products (term loans) can show thin or negative economic profit — consistent with the Bank of England's 2026 finding that SME lending earns the lowest product-level returns, driven by impairments and per-borrower servicing costs.</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="39" customHeight="1">
-      <c r="B44" s="4" t="inlineStr">
+    <row r="45" ht="39" customHeight="1">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>• Use the cost-driver table on the P&amp;L tab to find leverage points, then trace them to transaction intensity (I) or customer load (L) assumptions on the Inputs tab — e.g. automating underwriting hours, raising RM portfolio size, or shifting servicing to digital.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="3" t="inlineStr">
+    <row r="47">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>Caveats</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="39" customHeight="1">
-      <c r="B47" s="4" t="inlineStr">
+    <row r="48" ht="39" customHeight="1">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>• Benchmarks are as of August 2026 (Bank Rate 3.75%; BoE effective new SME loan rate ~6.3%; commercial interchange 1.65–1.90%; invoice finance discount base+1–3%). Items marked 'Assumption' are illustrative and should be replaced with your own data.</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="65" customHeight="1">
-      <c r="B48" s="4" t="inlineStr">
+    <row r="49" ht="65" customHeight="1">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>• The FTP now carries an explicit liquidity charge (buffer × drag) and a behavioural credit for stable deposits, shown as memos on the Revenues tab; it is still a single curve, not a full behavioural-maturity model. Fraud &amp; payment losses, the FSCS levy, collateral administration &amp; recoveries, and change-the-bank spend are now modelled explicitly. Operational-risk RWA is proxied at 15% of gross income; head-office and change costs are allocated per customer.</t>
         </is>
@@ -7735,7 +7742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H91"/>
+  <dimension ref="B1:H109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -7777,779 +7784,587 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="45" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="C7" s="45" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="D7" s="45" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="E7" s="45" t="inlineStr">
-        <is>
-          <t>e(PBT)</t>
-        </is>
-      </c>
-      <c r="F7" s="45" t="inlineStr">
-        <is>
-          <t>e(Cost:income)</t>
-        </is>
-      </c>
-      <c r="G7" s="45" t="inlineStr">
-        <is>
-          <t>e(RoE)</t>
-        </is>
-      </c>
-      <c r="H7" s="45" t="inlineStr">
-        <is>
-          <t>e(Income)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Term loans — customer rate</t>
-        </is>
-      </c>
-      <c r="C8" s="63" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>% p.a.</t>
-        </is>
-      </c>
-      <c r="E8" s="71" t="n">
-        <v>1.247681048892727</v>
-      </c>
-      <c r="F8" s="71" t="n">
-        <v>-0.5920579472668667</v>
-      </c>
-      <c r="G8" s="71" t="n">
-        <v>1.148369761396499</v>
-      </c>
-      <c r="H8" s="71" t="n">
-        <v>0.5955841505629065</v>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>PRICES — AND THE DEMAND RESPONSE THAT WOULD CANCEL THEM</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr"/>
+      <c r="D7" s="8" t="inlineStr"/>
+      <c r="E7" s="8" t="inlineStr"/>
+      <c r="F7" s="8" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr"/>
+      <c r="H7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8" ht="76" customHeight="1">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>The elasticities below this section assume nothing responds to price. Raise a rate and volume does not move, so raising prices always looks accretive — the most misleading thing a model can tell anyone. This block gives, for each price, the demand elasticity at which raising it stops paying. A LOW break-even means fragile: the advice to raise that price survives only a very unresponsive customer, and the burden is on you to show they are one. None of these elasticities is known here; what the number replaces is not a measurement but a hidden assumption of zero, which is the least defensible value available. The query is the same in every case — move the price for a randomised subset and measure the volume response.</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>Reachable SMEs in region (R)</t>
-        </is>
-      </c>
-      <c r="C9" s="63" t="n">
-        <v>18750</v>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>businesses</t>
-        </is>
-      </c>
-      <c r="E9" s="71" t="n">
-        <v>1.00000000000003</v>
-      </c>
-      <c r="F9" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="71" t="n">
-        <v>1.00000000000002</v>
+      <c r="B9" s="45" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="C9" s="45" t="inlineStr">
+        <is>
+          <t>e(PBT) with no demand response</t>
+        </is>
+      </c>
+      <c r="D9" s="45" t="inlineStr">
+        <is>
+          <t>Break-even demand elasticity</t>
+        </is>
+      </c>
+      <c r="E9" s="45" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Steady-state penetration (P)</t>
-        </is>
-      </c>
-      <c r="C10" s="63" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>% of reachable</t>
-        </is>
-      </c>
-      <c r="E10" s="71" t="n">
-        <v>1.00000000000003</v>
-      </c>
-      <c r="F10" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="71" t="n">
-        <v>1.00000000000002</v>
+          <t>Card — annual card fee</t>
+        </is>
+      </c>
+      <c r="C10" s="71" t="n">
+        <v>0.006388126970350395</v>
+      </c>
+      <c r="D10" s="63" t="n">
+        <v>0.05544003490987621</v>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>fragile — only a near-inert customer makes this pay</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Business current account — penetration</t>
-        </is>
-      </c>
-      <c r="C11" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="14" t="inlineStr">
-        <is>
-          <t>% of customers</t>
-        </is>
-      </c>
-      <c r="E11" s="71" t="n">
-        <v>0.5316502207558557</v>
-      </c>
-      <c r="F11" s="71" t="n">
-        <v>-0.2263724971407025</v>
-      </c>
-      <c r="G11" s="71" t="n">
-        <v>0.4858715994436417</v>
-      </c>
-      <c r="H11" s="71" t="n">
-        <v>0.2763510458611886</v>
+          <t>BCA — monthly account fee</t>
+        </is>
+      </c>
+      <c r="C11" s="71" t="n">
+        <v>0.06787384905974791</v>
+      </c>
+      <c r="D11" s="63" t="n">
+        <v>0.1275035819127078</v>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>fragile — only a near-inert customer makes this pay</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Term loans — average balance</t>
-        </is>
-      </c>
-      <c r="C12" s="63" t="n">
-        <v>250000</v>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>£/loan</t>
-        </is>
-      </c>
-      <c r="E12" s="71" t="n">
-        <v>0.4485219355690576</v>
-      </c>
-      <c r="F12" s="71" t="n">
-        <v>-0.2508408142510311</v>
-      </c>
-      <c r="G12" s="71" t="n">
-        <v>-0.172627245775743</v>
-      </c>
-      <c r="H12" s="71" t="n">
-        <v>0.2514716076793886</v>
+          <t>Card — interest rate on revolving balances</t>
+        </is>
+      </c>
+      <c r="C12" s="71" t="n">
+        <v>0.01587050294191057</v>
+      </c>
+      <c r="D12" s="63" t="n">
+        <v>0.1376205835187992</v>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>fragile — only a near-inert customer makes this pay</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>BCA — average credit balance</t>
-        </is>
-      </c>
-      <c r="C13" s="63" t="n">
-        <v>18000</v>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>£/account</t>
-        </is>
-      </c>
-      <c r="E13" s="71" t="n">
-        <v>0.4269286171458919</v>
-      </c>
-      <c r="F13" s="71" t="n">
-        <v>-0.2009624805300439</v>
-      </c>
-      <c r="G13" s="71" t="n">
-        <v>0.3928629971036865</v>
-      </c>
-      <c r="H13" s="71" t="n">
-        <v>0.2058338824345483</v>
+          <t>Term loans — arrangement fee</t>
+        </is>
+      </c>
+      <c r="C13" s="71" t="n">
+        <v>0.07486086293356356</v>
+      </c>
+      <c r="D13" s="63" t="n">
+        <v>0.1792828253338209</v>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>fragile — only a near-inert customer makes this pay</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Term loans / commercial mortgages — penetration</t>
-        </is>
-      </c>
-      <c r="C14" s="63" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E14" s="71" t="n">
-        <v>0.4168087496628946</v>
-      </c>
-      <c r="F14" s="71" t="n">
-        <v>-0.2178158778235073</v>
-      </c>
-      <c r="G14" s="71" t="n">
-        <v>-0.2041443250685729</v>
-      </c>
-      <c r="H14" s="71" t="n">
-        <v>0.2514716076793886</v>
+          <t>Invoice finance — discount margin over base</t>
+        </is>
+      </c>
+      <c r="C14" s="71" t="n">
+        <v>0.07486086293356356</v>
+      </c>
+      <c r="D14" s="63" t="n">
+        <v>0.2515282418779798</v>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>fragile — only a near-inert customer makes this pay</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — customer yield</t>
-        </is>
-      </c>
-      <c r="C15" s="63" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-      <c r="D15" s="14" t="inlineStr">
-        <is>
-          <t>% p.a.</t>
-        </is>
-      </c>
-      <c r="E15" s="71" t="n">
-        <v>0.3619938616520847</v>
-      </c>
-      <c r="F15" s="71" t="n">
-        <v>-0.1725007356564119</v>
-      </c>
-      <c r="G15" s="71" t="n">
-        <v>0.3334124986436103</v>
-      </c>
-      <c r="H15" s="71" t="n">
-        <v>0.1727988148833219</v>
+          <t>International payment fee</t>
+        </is>
+      </c>
+      <c r="C15" s="71" t="n">
+        <v>0.06987013873799264</v>
+      </c>
+      <c r="D15" s="63" t="n">
+        <v>0.4122296676035196</v>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>fragile — only a near-inert customer makes this pay</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — average funds in use (advances)</t>
-        </is>
-      </c>
-      <c r="C16" s="63" t="n">
-        <v>150000</v>
-      </c>
-      <c r="D16" s="14" t="inlineStr">
-        <is>
-          <t>£/client</t>
-        </is>
-      </c>
-      <c r="E16" s="71" t="n">
-        <v>0.3101871844046677</v>
-      </c>
-      <c r="F16" s="71" t="n">
-        <v>-0.1543074556452041</v>
-      </c>
-      <c r="G16" s="71" t="n">
-        <v>0.209829595204097</v>
-      </c>
-      <c r="H16" s="71" t="n">
-        <v>0.1545459315400012</v>
+          <t>Overdraft — annual arrangement/renewal fee</t>
+        </is>
+      </c>
+      <c r="C16" s="71" t="n">
+        <v>0.03743043146678178</v>
+      </c>
+      <c r="D16" s="63" t="n">
+        <v>0.4581530737163218</v>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>fragile — only a near-inert customer makes this pay</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Notice &amp; fixed deposits — rate paid</t>
-        </is>
-      </c>
-      <c r="C17" s="63" t="n">
-        <v>0.041</v>
-      </c>
-      <c r="D17" s="14" t="inlineStr">
-        <is>
-          <t>% p.a.</t>
-        </is>
-      </c>
-      <c r="E17" s="71" t="n">
-        <v>-0.3069295380274881</v>
-      </c>
-      <c r="F17" s="71" t="n">
-        <v>0.1467286786560457</v>
-      </c>
-      <c r="G17" s="71" t="n">
-        <v>-0.2828446455047969</v>
-      </c>
-      <c r="H17" s="71" t="n">
-        <v>-0.1465137010384164</v>
+          <t>FX — margin on conversion volume</t>
+        </is>
+      </c>
+      <c r="C17" s="71" t="n">
+        <v>0.09981448391141808</v>
+      </c>
+      <c r="D17" s="63" t="n">
+        <v>0.5878609520414249</v>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>modest — a mildly responsive customer cancels it</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — penetration</t>
-        </is>
-      </c>
-      <c r="C18" s="63" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E18" s="71" t="n">
-        <v>0.2968754767403625</v>
-      </c>
-      <c r="F18" s="71" t="n">
-        <v>-0.1404317212375283</v>
-      </c>
-      <c r="G18" s="71" t="n">
-        <v>0.1965312055379295</v>
-      </c>
-      <c r="H18" s="71" t="n">
-        <v>0.1545459315400012</v>
+          <t>Invoice finance — service fee</t>
+        </is>
+      </c>
+      <c r="C18" s="71" t="n">
+        <v>0.2395547613874034</v>
+      </c>
+      <c r="D18" s="63" t="n">
+        <v>0.8004609263604965</v>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>modest — a mildly responsive customer cancels it</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Head office: technology &amp; central operations</t>
-        </is>
-      </c>
-      <c r="C19" s="63" t="n">
-        <v>450</v>
-      </c>
-      <c r="D19" s="14" t="inlineStr">
-        <is>
-          <t>£/customer/yr</t>
-        </is>
-      </c>
-      <c r="E19" s="71" t="n">
-        <v>-0.2965245383102628</v>
-      </c>
-      <c r="F19" s="71" t="n">
-        <v>0.3095661825398512</v>
-      </c>
-      <c r="G19" s="71" t="n">
-        <v>-0.2965245383105712</v>
-      </c>
-      <c r="H19" s="71" t="n">
-        <v>0</v>
+          <t>Overdraft — interest rate (EAR)</t>
+        </is>
+      </c>
+      <c r="C19" s="71" t="n">
+        <v>0.1094840120403367</v>
+      </c>
+      <c r="D19" s="63" t="n">
+        <v>1.328382145135671</v>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>modest — a mildly responsive customer cancels it</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Instant-access savings — rate paid</t>
-        </is>
-      </c>
-      <c r="C20" s="63" t="n">
-        <v>0.033</v>
-      </c>
-      <c r="D20" s="14" t="inlineStr">
-        <is>
-          <t>% p.a.</t>
-        </is>
-      </c>
-      <c r="E20" s="71" t="n">
-        <v>-0.2635102375261357</v>
-      </c>
-      <c r="F20" s="71" t="n">
-        <v>0.1259457965071908</v>
-      </c>
-      <c r="G20" s="71" t="n">
-        <v>-0.2428241773307234</v>
-      </c>
-      <c r="H20" s="71" t="n">
-        <v>-0.125787372598882</v>
+          <t>Asset finance — customer yield</t>
+        </is>
+      </c>
+      <c r="C20" s="71" t="n">
+        <v>0.3619938616520844</v>
+      </c>
+      <c r="D20" s="63" t="n">
+        <v>2.229914972398844</v>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>robust — needs a strongly responsive customer to destroy value</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — funded invoices as multiple of advances</t>
-        </is>
-      </c>
-      <c r="C21" s="63" t="n">
-        <v>8</v>
-      </c>
-      <c r="D21" s="14" t="inlineStr">
-        <is>
-          <t>x p.a.</t>
-        </is>
-      </c>
-      <c r="E21" s="71" t="n">
-        <v>0.2395547613874036</v>
-      </c>
-      <c r="F21" s="71" t="n">
-        <v>-0.1142215421111091</v>
-      </c>
-      <c r="G21" s="71" t="n">
-        <v>0.2206618790426836</v>
-      </c>
-      <c r="H21" s="71" t="n">
-        <v>0.1143521569080781</v>
+          <t>Term loans — customer rate</t>
+        </is>
+      </c>
+      <c r="C21" s="71" t="n">
+        <v>1.247681048892726</v>
+      </c>
+      <c r="D21" s="63" t="n">
+        <v>2.906412804688113</v>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>robust — needs a strongly responsive customer to destroy value</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — service fee</t>
-        </is>
-      </c>
-      <c r="C22" s="63" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t>% of funded invoices</t>
-        </is>
-      </c>
-      <c r="E22" s="71" t="n">
-        <v>0.2395547613874036</v>
-      </c>
-      <c r="F22" s="71" t="n">
-        <v>-0.1142215421111091</v>
-      </c>
-      <c r="G22" s="71" t="n">
-        <v>0.2206618790426836</v>
-      </c>
-      <c r="H22" s="71" t="n">
-        <v>0.1143521569080781</v>
+          <t>Instant-access savings — rate paid</t>
+        </is>
+      </c>
+      <c r="C22" s="71" t="n">
+        <v>0.2635102375261355</v>
+      </c>
+      <c r="D22" s="63" t="n">
+        <v>4.257749912948078</v>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
+          <t>robust — needs a strongly responsive customer to destroy value</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Bank of England Bank Rate</t>
-        </is>
-      </c>
-      <c r="C23" s="63" t="n">
-        <v>0.0375</v>
-      </c>
-      <c r="D23" s="14" t="inlineStr">
-        <is>
-          <t>% p.a.</t>
-        </is>
-      </c>
-      <c r="E23" s="71" t="n">
-        <v>0.1990512830997236</v>
-      </c>
-      <c r="F23" s="71" t="n">
-        <v>-0.09492750668173035</v>
-      </c>
-      <c r="G23" s="71" t="n">
-        <v>0.1931242862657616</v>
-      </c>
-      <c r="H23" s="71" t="n">
-        <v>0.09501770461968793</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>International payments &amp; FX — penetration</t>
-        </is>
-      </c>
-      <c r="C24" s="63" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D24" s="14" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E24" s="71" t="n">
-        <v>0.1687945307331029</v>
-      </c>
-      <c r="F24" s="71" t="n">
-        <v>-0.08000540090128463</v>
-      </c>
-      <c r="G24" s="71" t="n">
-        <v>0.1554207840445721</v>
-      </c>
-      <c r="H24" s="71" t="n">
-        <v>0.08099944447655529</v>
+          <t>Notice &amp; fixed deposits — rate paid</t>
+        </is>
+      </c>
+      <c r="C23" s="71" t="n">
+        <v>0.3069295380276106</v>
+      </c>
+      <c r="D23" s="63" t="n">
+        <v>42.5163639198051</v>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>robust — needs a strongly responsive customer to destroy value</t>
+        </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>Asset finance — average balance</t>
-        </is>
-      </c>
-      <c r="C25" s="63" t="n">
-        <v>80000</v>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>£/agreement</t>
-        </is>
-      </c>
-      <c r="E25" s="71" t="n">
-        <v>0.1658745747382735</v>
-      </c>
-      <c r="F25" s="71" t="n">
-        <v>-0.09273546655296665</v>
-      </c>
-      <c r="G25" s="71" t="n">
-        <v>0.008961968797843937</v>
-      </c>
-      <c r="H25" s="71" t="n">
-        <v>0.09282154504571802</v>
+      <c r="B25" s="45" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="C25" s="45" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D25" s="45" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E25" s="45" t="inlineStr">
+        <is>
+          <t>e(PBT)</t>
+        </is>
+      </c>
+      <c r="F25" s="45" t="inlineStr">
+        <is>
+          <t>e(Cost:income)</t>
+        </is>
+      </c>
+      <c r="G25" s="45" t="inlineStr">
+        <is>
+          <t>e(RoE)</t>
+        </is>
+      </c>
+      <c r="H25" s="45" t="inlineStr">
+        <is>
+          <t>e(Income)</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Head office: risk, compliance, financial crime, audit</t>
+          <t>Term loans — customer rate</t>
         </is>
       </c>
       <c r="C26" s="63" t="n">
-        <v>250</v>
+        <v>0.0625</v>
       </c>
       <c r="D26" s="14" t="inlineStr">
         <is>
-          <t>£/customer/yr</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E26" s="71" t="n">
-        <v>-0.1647358546168127</v>
+        <v>1.247681048892727</v>
       </c>
       <c r="F26" s="71" t="n">
-        <v>0.1719812125220667</v>
+        <v>-0.5920579472668667</v>
       </c>
       <c r="G26" s="71" t="n">
-        <v>-0.1647358546170901</v>
+        <v>1.148369761396499</v>
       </c>
       <c r="H26" s="71" t="n">
-        <v>0</v>
+        <v>0.5955841505629065</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — penetration</t>
+          <t>Reachable SMEs in region (R)</t>
         </is>
       </c>
       <c r="C27" s="63" t="n">
-        <v>0.08</v>
+        <v>18750</v>
       </c>
       <c r="D27" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>businesses</t>
         </is>
       </c>
       <c r="E27" s="71" t="n">
-        <v>0.1587153370028682</v>
+        <v>1.00000000000003</v>
       </c>
       <c r="F27" s="71" t="n">
-        <v>-0.08526828474335443</v>
+        <v>0</v>
       </c>
       <c r="G27" s="71" t="n">
-        <v>0.001813946205839392</v>
+        <v>0</v>
       </c>
       <c r="H27" s="71" t="n">
-        <v>0.09282154504571802</v>
+        <v>1.00000000000002</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Head office: finance, HR, exec, brand &amp; residual (non-acquisition) marketing</t>
+          <t>Steady-state penetration (P)</t>
         </is>
       </c>
       <c r="C28" s="63" t="n">
-        <v>222</v>
+        <v>0.16</v>
       </c>
       <c r="D28" s="14" t="inlineStr">
         <is>
-          <t>£/customer/yr</t>
+          <t>% of reachable</t>
         </is>
       </c>
       <c r="E28" s="71" t="n">
-        <v>-0.1462854388997297</v>
+        <v>1.00000000000003</v>
       </c>
       <c r="F28" s="71" t="n">
-        <v>0.1527193167196385</v>
+        <v>0</v>
       </c>
       <c r="G28" s="71" t="n">
-        <v>-0.1462854388999867</v>
+        <v>0</v>
       </c>
       <c r="H28" s="71" t="n">
-        <v>0</v>
+        <v>1.00000000000002</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Equity held against RWAs (CET1 target)</t>
+          <t>Business current account — penetration</t>
         </is>
       </c>
       <c r="C29" s="63" t="n">
-        <v>0.14</v>
+        <v>1</v>
       </c>
       <c r="D29" s="14" t="inlineStr">
         <is>
-          <t>% of RWA</t>
+          <t>% of customers</t>
         </is>
       </c>
       <c r="E29" s="71" t="n">
-        <v>0.1238711722148994</v>
+        <v>0.5316502207558557</v>
       </c>
       <c r="F29" s="71" t="n">
-        <v>-0.05909531843834973</v>
+        <v>-0.2263724971407025</v>
       </c>
       <c r="G29" s="71" t="n">
-        <v>-0.8674542849359645</v>
+        <v>0.4858715994436417</v>
       </c>
       <c r="H29" s="71" t="n">
-        <v>0.05913026165485447</v>
+        <v>0.2763510458611886</v>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Business credit card — penetration</t>
+          <t>Term loans — average balance</t>
         </is>
       </c>
       <c r="C30" s="63" t="n">
-        <v>0.3</v>
+        <v>250000</v>
       </c>
       <c r="D30" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/loan</t>
         </is>
       </c>
       <c r="E30" s="71" t="n">
-        <v>0.115162001627308</v>
+        <v>0.4485219355690576</v>
       </c>
       <c r="F30" s="71" t="n">
-        <v>-0.05450341134971946</v>
+        <v>-0.2508408142510311</v>
       </c>
       <c r="G30" s="71" t="n">
-        <v>0.1025383467743691</v>
+        <v>-0.172627245775743</v>
       </c>
       <c r="H30" s="71" t="n">
-        <v>0.05762391571351869</v>
+        <v>0.2514716076793886</v>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — interest rate (EAR)</t>
+          <t>BCA — average credit balance</t>
         </is>
       </c>
       <c r="C31" s="63" t="n">
-        <v>0.0975</v>
+        <v>18000</v>
       </c>
       <c r="D31" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/account</t>
         </is>
       </c>
       <c r="E31" s="71" t="n">
-        <v>0.1094840120404391</v>
+        <v>0.4269286171458919</v>
       </c>
       <c r="F31" s="71" t="n">
-        <v>-0.05223520978052387</v>
+        <v>-0.2009624805300439</v>
       </c>
       <c r="G31" s="71" t="n">
-        <v>0.1008596961142311</v>
+        <v>0.3928629971036865</v>
       </c>
       <c r="H31" s="71" t="n">
-        <v>0.05226250921193411</v>
+        <v>0.2058338824345483</v>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>Card — average monthly spend</t>
+          <t>Term loans / commercial mortgages — penetration</t>
         </is>
       </c>
       <c r="C32" s="63" t="n">
-        <v>2500</v>
+        <v>0.12</v>
       </c>
       <c r="D32" s="14" t="inlineStr">
         <is>
-          <t>£/card/month</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E32" s="71" t="n">
-        <v>0.1018107735896629</v>
+        <v>0.4168087496628946</v>
       </c>
       <c r="F32" s="71" t="n">
-        <v>-0.04857605888322602</v>
+        <v>-0.2178158778235073</v>
       </c>
       <c r="G32" s="71" t="n">
-        <v>0.09379146319211618</v>
+        <v>-0.2041443250685729</v>
       </c>
       <c r="H32" s="71" t="n">
-        <v>0.04859966668594098</v>
+        <v>0.2514716076793886</v>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Card — commercial interchange earned</t>
+          <t>Asset finance — customer yield</t>
         </is>
       </c>
       <c r="C33" s="63" t="n">
-        <v>0.017</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="D33" s="14" t="inlineStr">
         <is>
-          <t>% of spend</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E33" s="71" t="n">
-        <v>0.1018107735896629</v>
+        <v>0.3619938616520847</v>
       </c>
       <c r="F33" s="71" t="n">
-        <v>-0.04857605888322602</v>
+        <v>-0.1725007356564119</v>
       </c>
       <c r="G33" s="71" t="n">
-        <v>0.09379146319211618</v>
+        <v>0.3334124986436103</v>
       </c>
       <c r="H33" s="71" t="n">
-        <v>0.04859966668594098</v>
+        <v>0.1727988148833219</v>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Term funding premium over Bank Rate</t>
+          <t>Invoice finance — average funds in use (advances)</t>
         </is>
       </c>
       <c r="C34" s="63" t="n">
-        <v>0.006</v>
+        <v>150000</v>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/client</t>
         </is>
       </c>
       <c r="E34" s="71" t="n">
-        <v>-0.1004133708148834</v>
+        <v>0.3101871844046677</v>
       </c>
       <c r="F34" s="71" t="n">
-        <v>0.04795559880866109</v>
+        <v>-0.1543074556452041</v>
       </c>
       <c r="G34" s="71" t="n">
-        <v>-0.09251885130815904</v>
+        <v>0.209829595204097</v>
       </c>
       <c r="H34" s="71" t="n">
-        <v>-0.04793261243730116</v>
+        <v>0.1545459315400012</v>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Behavioural term credit for stable non-maturing deposits</t>
+          <t>Notice &amp; fixed deposits — rate paid</t>
         </is>
       </c>
       <c r="C35" s="63" t="n">
-        <v>0.005</v>
+        <v>0.041</v>
       </c>
       <c r="D35" s="14" t="inlineStr">
         <is>
@@ -8557,188 +8372,188 @@
         </is>
       </c>
       <c r="E35" s="71" t="n">
-        <v>0.09981448391141816</v>
+        <v>-0.3069295380274881</v>
       </c>
       <c r="F35" s="71" t="n">
-        <v>-0.04762404074601882</v>
+        <v>0.1467286786560457</v>
       </c>
       <c r="G35" s="71" t="n">
-        <v>0.09195255933441075</v>
+        <v>-0.2828446455047969</v>
       </c>
       <c r="H35" s="71" t="n">
-        <v>0.04764673204503252</v>
+        <v>-0.1465137010384164</v>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>FX — average annual conversion volume</t>
+          <t>Invoice finance — penetration</t>
         </is>
       </c>
       <c r="C36" s="63" t="n">
-        <v>100000</v>
+        <v>0.03</v>
       </c>
       <c r="D36" s="14" t="inlineStr">
         <is>
-          <t>£/user/yr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E36" s="71" t="n">
-        <v>0.09981448391141816</v>
+        <v>0.2968754767403625</v>
       </c>
       <c r="F36" s="71" t="n">
-        <v>-0.04762404074601882</v>
+        <v>-0.1404317212375283</v>
       </c>
       <c r="G36" s="71" t="n">
-        <v>0.09195255933441075</v>
+        <v>0.1965312055379295</v>
       </c>
       <c r="H36" s="71" t="n">
-        <v>0.04764673204503252</v>
+        <v>0.1545459315400012</v>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>FX — margin on conversion volume</t>
+          <t>Head office: technology &amp; central operations</t>
         </is>
       </c>
       <c r="C37" s="63" t="n">
-        <v>0.0075</v>
+        <v>450</v>
       </c>
       <c r="D37" s="14" t="inlineStr">
         <is>
-          <t>% of volume</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E37" s="71" t="n">
-        <v>0.09981448391141816</v>
+        <v>-0.2965245383102628</v>
       </c>
       <c r="F37" s="71" t="n">
-        <v>-0.04762404074601882</v>
+        <v>0.3095661825398512</v>
       </c>
       <c r="G37" s="71" t="n">
-        <v>0.09195255933441075</v>
+        <v>-0.2965245383105712</v>
       </c>
       <c r="H37" s="71" t="n">
-        <v>0.04764673204503252</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — average limit</t>
+          <t>Instant-access savings — rate paid</t>
         </is>
       </c>
       <c r="C38" s="63" t="n">
-        <v>15000</v>
+        <v>0.033</v>
       </c>
       <c r="D38" s="14" t="inlineStr">
         <is>
-          <t>£/facility</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E38" s="71" t="n">
-        <v>0.09519058528012668</v>
+        <v>-0.2635102375261357</v>
       </c>
       <c r="F38" s="71" t="n">
-        <v>-0.05209194641982378</v>
+        <v>0.1259457965071908</v>
       </c>
       <c r="G38" s="71" t="n">
-        <v>0.051574506124141</v>
+        <v>-0.2428241773307234</v>
       </c>
       <c r="H38" s="71" t="n">
-        <v>0.05211909627141639</v>
+        <v>-0.125787372598882</v>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Productive hours per FTE per month</t>
+          <t>Invoice finance — funded invoices as multiple of advances</t>
         </is>
       </c>
       <c r="C39" s="63" t="n">
-        <v>147</v>
+        <v>8</v>
       </c>
       <c r="D39" s="14" t="inlineStr">
         <is>
-          <t>hours</t>
+          <t>x p.a.</t>
         </is>
       </c>
       <c r="E39" s="71" t="n">
-        <v>0.09121190632452875</v>
+        <v>0.2395547613874036</v>
       </c>
       <c r="F39" s="71" t="n">
-        <v>-0.09522355823886089</v>
+        <v>-0.1142215421111091</v>
       </c>
       <c r="G39" s="71" t="n">
-        <v>0.09121190632435788</v>
+        <v>0.2206618790426836</v>
       </c>
       <c r="H39" s="71" t="n">
-        <v>0</v>
+        <v>0.1143521569080781</v>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — penetration</t>
+          <t>Invoice finance — service fee</t>
         </is>
       </c>
       <c r="C40" s="63" t="n">
-        <v>0.25</v>
+        <v>0.01</v>
       </c>
       <c r="D40" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% of funded invoices</t>
         </is>
       </c>
       <c r="E40" s="71" t="n">
-        <v>0.08132422312990931</v>
+        <v>0.2395547613874036</v>
       </c>
       <c r="F40" s="71" t="n">
-        <v>-0.0376232594615131</v>
+        <v>-0.1142215421111091</v>
       </c>
       <c r="G40" s="71" t="n">
-        <v>0.0377141861854879</v>
+        <v>0.2206618790426836</v>
       </c>
       <c r="H40" s="71" t="n">
-        <v>0.05211909627141639</v>
+        <v>0.1143521569080781</v>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Customers per relationship manager (L)</t>
+          <t>Bank of England Bank Rate</t>
         </is>
       </c>
       <c r="C41" s="63" t="n">
-        <v>120</v>
+        <v>0.0375</v>
       </c>
       <c r="D41" s="14" t="inlineStr">
         <is>
-          <t>customers</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E41" s="71" t="n">
-        <v>0.08107710567534358</v>
+        <v>0.1990512830997236</v>
       </c>
       <c r="F41" s="71" t="n">
-        <v>-0.08464301213748615</v>
+        <v>-0.09492750668173035</v>
       </c>
       <c r="G41" s="71" t="n">
-        <v>0.08107710567522457</v>
+        <v>0.1931242862657616</v>
       </c>
       <c r="H41" s="71" t="n">
-        <v>0</v>
+        <v>0.09501770461968793</v>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Share of customers that are relationship-managed</t>
+          <t>International payments &amp; FX — penetration</t>
         </is>
       </c>
       <c r="C42" s="63" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
@@ -8746,53 +8561,53 @@
         </is>
       </c>
       <c r="E42" s="71" t="n">
-        <v>-0.08092587948856705</v>
+        <v>0.1687945307331029</v>
       </c>
       <c r="F42" s="71" t="n">
-        <v>0.08448513477060619</v>
+        <v>-0.08000540090128463</v>
       </c>
       <c r="G42" s="71" t="n">
-        <v>-0.08092587948885854</v>
+        <v>0.1554207840445721</v>
       </c>
       <c r="H42" s="71" t="n">
-        <v>0</v>
+        <v>0.08099944447655529</v>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>BCA — net transaction &amp; cash-handling income</t>
+          <t>Asset finance — average balance</t>
         </is>
       </c>
       <c r="C43" s="63" t="n">
-        <v>120</v>
+        <v>80000</v>
       </c>
       <c r="D43" s="14" t="inlineStr">
         <is>
-          <t>£/account/yr</t>
+          <t>£/agreement</t>
         </is>
       </c>
       <c r="E43" s="71" t="n">
-        <v>0.07985158712913452</v>
+        <v>0.1658745747382735</v>
       </c>
       <c r="F43" s="71" t="n">
-        <v>-0.03810286182134639</v>
+        <v>-0.09273546655296665</v>
       </c>
       <c r="G43" s="71" t="n">
-        <v>0.07356320301076685</v>
+        <v>0.008961968797843937</v>
       </c>
       <c r="H43" s="71" t="n">
-        <v>0.03811738563602602</v>
+        <v>0.09282154504571802</v>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>Change-the-bank / transformation spend per customer</t>
+          <t>Head office: risk, compliance, financial crime, audit</t>
         </is>
       </c>
       <c r="C44" s="63" t="n">
-        <v>120</v>
+        <v>250</v>
       </c>
       <c r="D44" s="14" t="inlineStr">
         <is>
@@ -8800,13 +8615,13 @@
         </is>
       </c>
       <c r="E44" s="71" t="n">
-        <v>-0.07907321021607008</v>
+        <v>-0.1647358546168127</v>
       </c>
       <c r="F44" s="71" t="n">
-        <v>0.08255098201058327</v>
+        <v>0.1719812125220667</v>
       </c>
       <c r="G44" s="71" t="n">
-        <v>-0.0790732102163739</v>
+        <v>-0.1647358546170901</v>
       </c>
       <c r="H44" s="71" t="n">
         <v>0</v>
@@ -8815,52 +8630,52 @@
     <row r="45">
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>Term loans — probability of default</t>
+          <t>Asset finance — penetration</t>
         </is>
       </c>
       <c r="C45" s="63" t="n">
-        <v>0.018</v>
+        <v>0.08</v>
       </c>
       <c r="D45" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E45" s="71" t="n">
-        <v>-0.07828247811390938</v>
+        <v>0.1587153370028682</v>
       </c>
       <c r="F45" s="71" t="n">
-        <v>0</v>
+        <v>-0.08526828474335443</v>
       </c>
       <c r="G45" s="71" t="n">
-        <v>-0.07828247811415756</v>
+        <v>0.001813946205839392</v>
       </c>
       <c r="H45" s="71" t="n">
-        <v>0</v>
+        <v>0.09282154504571802</v>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>Term loans — loss given default</t>
+          <t>Head office: finance, HR, exec, brand &amp; residual (non-acquisition) marketing</t>
         </is>
       </c>
       <c r="C46" s="63" t="n">
-        <v>0.25</v>
+        <v>222</v>
       </c>
       <c r="D46" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E46" s="71" t="n">
-        <v>-0.07828247811390938</v>
+        <v>-0.1462854388997297</v>
       </c>
       <c r="F46" s="71" t="n">
-        <v>0</v>
+        <v>0.1527193167196385</v>
       </c>
       <c r="G46" s="71" t="n">
-        <v>-0.07828247811415756</v>
+        <v>-0.1462854388999867</v>
       </c>
       <c r="H46" s="71" t="n">
         <v>0</v>
@@ -8869,349 +8684,349 @@
     <row r="47">
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>Term loans — arrangement fee</t>
+          <t>Equity held against RWAs (CET1 target)</t>
         </is>
       </c>
       <c r="C47" s="63" t="n">
-        <v>0.015</v>
+        <v>0.14</v>
       </c>
       <c r="D47" s="14" t="inlineStr">
         <is>
-          <t>% of loan</t>
+          <t>% of RWA</t>
         </is>
       </c>
       <c r="E47" s="71" t="n">
-        <v>0.07486086293356362</v>
+        <v>0.1238711722148994</v>
       </c>
       <c r="F47" s="71" t="n">
-        <v>-0.03572228365829964</v>
+        <v>-0.05909531843834973</v>
       </c>
       <c r="G47" s="71" t="n">
-        <v>0.0689657736584007</v>
+        <v>-0.8674542849359645</v>
       </c>
       <c r="H47" s="71" t="n">
-        <v>0.03573504903377439</v>
+        <v>0.05913026165485447</v>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — discount margin over base</t>
+          <t>Business credit card — penetration</t>
         </is>
       </c>
       <c r="C48" s="63" t="n">
-        <v>0.025</v>
+        <v>0.3</v>
       </c>
       <c r="D48" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E48" s="71" t="n">
-        <v>0.07486086293356362</v>
+        <v>0.115162001627308</v>
       </c>
       <c r="F48" s="71" t="n">
-        <v>-0.03572228365829964</v>
+        <v>-0.05450341134971946</v>
       </c>
       <c r="G48" s="71" t="n">
-        <v>0.0689657736584007</v>
+        <v>0.1025383467743691</v>
       </c>
       <c r="H48" s="71" t="n">
-        <v>0.03573504903377439</v>
+        <v>0.05762391571351869</v>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Term loans — risk weight</t>
+          <t>Overdraft — interest rate (EAR)</t>
         </is>
       </c>
       <c r="C49" s="63" t="n">
-        <v>0.7</v>
+        <v>0.0975</v>
       </c>
       <c r="D49" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E49" s="71" t="n">
-        <v>0.07264851188601439</v>
+        <v>0.1094840120404391</v>
       </c>
       <c r="F49" s="71" t="n">
-        <v>-0.03466695472918382</v>
+        <v>-0.05223520978052387</v>
       </c>
       <c r="G49" s="71" t="n">
-        <v>-0.5108399059911144</v>
+        <v>0.1008596961142311</v>
       </c>
       <c r="H49" s="71" t="n">
-        <v>0.03467897687449064</v>
+        <v>0.05226250921193411</v>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>International payments — number per user per year</t>
+          <t>Card — average monthly spend</t>
         </is>
       </c>
       <c r="C50" s="63" t="n">
-        <v>30</v>
+        <v>2500</v>
       </c>
       <c r="D50" s="14" t="inlineStr">
         <is>
-          <t>payments</t>
+          <t>£/card/month</t>
         </is>
       </c>
       <c r="E50" s="71" t="n">
-        <v>0.06987013873799271</v>
+        <v>0.1018107735896629</v>
       </c>
       <c r="F50" s="71" t="n">
-        <v>-0.03334159210622355</v>
+        <v>-0.04857605888322602</v>
       </c>
       <c r="G50" s="71" t="n">
-        <v>0.06436830819666425</v>
+        <v>0.09379146319211618</v>
       </c>
       <c r="H50" s="71" t="n">
-        <v>0.03335271243152277</v>
+        <v>0.04859966668594098</v>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>International payment fee</t>
+          <t>Card — commercial interchange earned</t>
         </is>
       </c>
       <c r="C51" s="63" t="n">
-        <v>17.5</v>
+        <v>0.017</v>
       </c>
       <c r="D51" s="14" t="inlineStr">
         <is>
-          <t>£/payment</t>
+          <t>% of spend</t>
         </is>
       </c>
       <c r="E51" s="71" t="n">
-        <v>0.06987013873799271</v>
+        <v>0.1018107735896629</v>
       </c>
       <c r="F51" s="71" t="n">
-        <v>-0.03334159210622355</v>
+        <v>-0.04857605888322602</v>
       </c>
       <c r="G51" s="71" t="n">
-        <v>0.06436830819666425</v>
+        <v>0.09379146319211618</v>
       </c>
       <c r="H51" s="71" t="n">
-        <v>0.03335271243152277</v>
+        <v>0.04859966668594098</v>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>BCA — monthly account fee</t>
+          <t>Term funding premium over Bank Rate</t>
         </is>
       </c>
       <c r="C52" s="63" t="n">
-        <v>8.5</v>
+        <v>0.006</v>
       </c>
       <c r="D52" s="14" t="inlineStr">
         <is>
-          <t>£/month</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E52" s="71" t="n">
-        <v>0.06787384905976844</v>
+        <v>-0.1004133708148834</v>
       </c>
       <c r="F52" s="71" t="n">
-        <v>-0.03238928373466862</v>
+        <v>0.04795559880866109</v>
       </c>
       <c r="G52" s="71" t="n">
-        <v>0.06252931190123294</v>
+        <v>-0.09251885130815904</v>
       </c>
       <c r="H52" s="71" t="n">
-        <v>0.03239977779061431</v>
+        <v>-0.04793261243730116</v>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>Relationship manager — salary</t>
+          <t>Behavioural term credit for stable non-maturing deposits</t>
         </is>
       </c>
       <c r="C53" s="63" t="n">
-        <v>65000</v>
+        <v>0.005</v>
       </c>
       <c r="D53" s="14" t="inlineStr">
         <is>
-          <t>£/yr</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E53" s="71" t="n">
-        <v>-0.06464852694618542</v>
+        <v>0.09981448391141816</v>
       </c>
       <c r="F53" s="71" t="n">
-        <v>0.06749187708921207</v>
+        <v>-0.04762404074601882</v>
       </c>
       <c r="G53" s="71" t="n">
-        <v>-0.06464852694648321</v>
+        <v>0.09195255933441075</v>
       </c>
       <c r="H53" s="71" t="n">
-        <v>0</v>
+        <v>0.04764673204503252</v>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>Instant-access savings — average balance</t>
+          <t>FX — average annual conversion volume</t>
         </is>
       </c>
       <c r="C54" s="63" t="n">
-        <v>30000</v>
+        <v>100000</v>
       </c>
       <c r="D54" s="14" t="inlineStr">
         <is>
-          <t>£/account</t>
+          <t>£/user/yr</t>
         </is>
       </c>
       <c r="E54" s="71" t="n">
-        <v>0.06103463413552909</v>
+        <v>0.09981448391141816</v>
       </c>
       <c r="F54" s="71" t="n">
-        <v>-0.02751368315916409</v>
+        <v>-0.04762404074601882</v>
       </c>
       <c r="G54" s="71" t="n">
-        <v>0.05600480950303754</v>
+        <v>0.09195255933441075</v>
       </c>
       <c r="H54" s="71" t="n">
-        <v>0.03049390850881691</v>
+        <v>0.04764673204503252</v>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>Term loans — average life</t>
+          <t>FX — margin on conversion volume</t>
         </is>
       </c>
       <c r="C55" s="63" t="n">
-        <v>4</v>
+        <v>0.0075</v>
       </c>
       <c r="D55" s="14" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>% of volume</t>
         </is>
       </c>
       <c r="E55" s="71" t="n">
-        <v>-0.0605521133221927</v>
+        <v>0.09981448391141816</v>
       </c>
       <c r="F55" s="71" t="n">
-        <v>0.02122446956929888</v>
+        <v>-0.04762404074601882</v>
       </c>
       <c r="G55" s="71" t="n">
-        <v>-0.05472260563925134</v>
+        <v>0.09195255933441075</v>
       </c>
       <c r="H55" s="71" t="n">
-        <v>-0.03538123666704555</v>
+        <v>0.04764673204503252</v>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>BCA — credit interest paid</t>
+          <t>Overdraft — average limit</t>
         </is>
       </c>
       <c r="C56" s="63" t="n">
-        <v>0.005</v>
+        <v>15000</v>
       </c>
       <c r="D56" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/facility</t>
         </is>
       </c>
       <c r="E56" s="71" t="n">
-        <v>-0.0598886903468509</v>
+        <v>0.09519058528012668</v>
       </c>
       <c r="F56" s="71" t="n">
-        <v>0.02859621432394117</v>
+        <v>-0.05209194641982378</v>
       </c>
       <c r="G56" s="71" t="n">
-        <v>-0.05517846962304982</v>
+        <v>0.051574506124141</v>
       </c>
       <c r="H56" s="71" t="n">
-        <v>-0.02858803922701951</v>
+        <v>0.05211909627141639</v>
       </c>
     </row>
     <row r="57">
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>Instant-access savings — penetration</t>
+          <t>Productive hours per FTE per month</t>
         </is>
       </c>
       <c r="C57" s="63" t="n">
-        <v>0.4</v>
+        <v>147</v>
       </c>
       <c r="D57" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>hours</t>
         </is>
       </c>
       <c r="E57" s="71" t="n">
-        <v>0.0592544503026677</v>
+        <v>0.09121190632452875</v>
       </c>
       <c r="F57" s="71" t="n">
-        <v>-0.02565577041929928</v>
+        <v>-0.09522355823886089</v>
       </c>
       <c r="G57" s="71" t="n">
-        <v>0.05422471515567431</v>
+        <v>0.09121190632435788</v>
       </c>
       <c r="H57" s="71" t="n">
-        <v>0.03049390850881691</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — average utilisation</t>
+          <t>Overdraft — penetration</t>
         </is>
       </c>
       <c r="C58" s="63" t="n">
-        <v>0.45</v>
+        <v>0.25</v>
       </c>
       <c r="D58" s="14" t="inlineStr">
         <is>
-          <t>% of limit</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E58" s="71" t="n">
-        <v>0.05776015381344716</v>
+        <v>0.08132422312990931</v>
       </c>
       <c r="F58" s="71" t="n">
-        <v>-0.03423984406982809</v>
+        <v>-0.0376232594615131</v>
       </c>
       <c r="G58" s="71" t="n">
-        <v>0.01710511817772802</v>
+        <v>0.0377141861854879</v>
       </c>
       <c r="H58" s="71" t="n">
-        <v>0.03425157175458779</v>
+        <v>0.05211909627141639</v>
       </c>
     </row>
     <row r="59">
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>Credit analyst / underwriter — salary</t>
+          <t>Customers per relationship manager (L)</t>
         </is>
       </c>
       <c r="C59" s="63" t="n">
-        <v>55000</v>
+        <v>120</v>
       </c>
       <c r="D59" s="14" t="inlineStr">
         <is>
-          <t>£/yr</t>
+          <t>customers</t>
         </is>
       </c>
       <c r="E59" s="71" t="n">
-        <v>-0.05171141124509487</v>
+        <v>0.08107710567534358</v>
       </c>
       <c r="F59" s="71" t="n">
-        <v>0.05398576544161963</v>
+        <v>-0.08464301213748615</v>
       </c>
       <c r="G59" s="71" t="n">
-        <v>-0.05171141124499209</v>
+        <v>0.08107710567522457</v>
       </c>
       <c r="H59" s="71" t="n">
         <v>0</v>
@@ -9220,7 +9035,7 @@
     <row r="60">
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>Liquidity buffer held against deposits (LCR / HQLA)</t>
+          <t>Share of customers that are relationship-managed</t>
         </is>
       </c>
       <c r="C60" s="63" t="n">
@@ -9228,57 +9043,57 @@
       </c>
       <c r="D60" s="14" t="inlineStr">
         <is>
-          <t>% of deposits</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E60" s="71" t="n">
-        <v>-0.04117347461329634</v>
+        <v>-0.08092587948856705</v>
       </c>
       <c r="F60" s="71" t="n">
-        <v>0.01965814063393465</v>
+        <v>0.08448513477060619</v>
       </c>
       <c r="G60" s="71" t="n">
-        <v>-0.03793463915464931</v>
+        <v>-0.08092587948885854</v>
       </c>
       <c r="H60" s="71" t="n">
-        <v>-0.01965427696859545</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>Yield give-up on the liquidity buffer vs Bank Rate</t>
+          <t>BCA — net transaction &amp; cash-handling income</t>
         </is>
       </c>
       <c r="C61" s="63" t="n">
-        <v>0.01</v>
+        <v>120</v>
       </c>
       <c r="D61" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/account/yr</t>
         </is>
       </c>
       <c r="E61" s="71" t="n">
-        <v>-0.04117347461329634</v>
+        <v>0.07985158712913452</v>
       </c>
       <c r="F61" s="71" t="n">
-        <v>0.01965814063393465</v>
+        <v>-0.03810286182134639</v>
       </c>
       <c r="G61" s="71" t="n">
-        <v>-0.03793463915464931</v>
+        <v>0.07356320301076685</v>
       </c>
       <c r="H61" s="71" t="n">
-        <v>-0.01965427696859545</v>
+        <v>0.03811738563602602</v>
       </c>
     </row>
     <row r="62">
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Unit-level platform &amp; processing cost</t>
+          <t>Change-the-bank / transformation spend per customer</t>
         </is>
       </c>
       <c r="C62" s="63" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="D62" s="14" t="inlineStr">
         <is>
@@ -9286,13 +9101,13 @@
         </is>
       </c>
       <c r="E62" s="71" t="n">
-        <v>-0.03953660510803504</v>
+        <v>-0.07907321021607008</v>
       </c>
       <c r="F62" s="71" t="n">
-        <v>0.0412754910054009</v>
+        <v>0.08255098201058327</v>
       </c>
       <c r="G62" s="71" t="n">
-        <v>-0.03953660510795137</v>
+        <v>-0.0790732102163739</v>
       </c>
       <c r="H62" s="71" t="n">
         <v>0</v>
@@ -9301,52 +9116,52 @@
     <row r="63">
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — annual arrangement/renewal fee</t>
+          <t>Term loans — probability of default</t>
         </is>
       </c>
       <c r="C63" s="63" t="n">
-        <v>0.015</v>
+        <v>0.018</v>
       </c>
       <c r="D63" s="14" t="inlineStr">
         <is>
-          <t>% of limit</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E63" s="71" t="n">
-        <v>0.03743043146690454</v>
+        <v>-0.07828247811390938</v>
       </c>
       <c r="F63" s="71" t="n">
-        <v>-0.01786433260297001</v>
+        <v>0</v>
       </c>
       <c r="G63" s="71" t="n">
-        <v>0.03448390249733824</v>
+        <v>-0.07828247811415756</v>
       </c>
       <c r="H63" s="71" t="n">
-        <v>0.01786752451694579</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>Fraud &amp; payment losses (incl. APP reimbursement) per current account</t>
+          <t>Term loans — loss given default</t>
         </is>
       </c>
       <c r="C64" s="63" t="n">
-        <v>45</v>
+        <v>0.25</v>
       </c>
       <c r="D64" s="14" t="inlineStr">
         <is>
-          <t>£/BCA/yr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E64" s="71" t="n">
-        <v>-0.02965245383102628</v>
+        <v>-0.07828247811390938</v>
       </c>
       <c r="F64" s="71" t="n">
-        <v>0.03095661825405067</v>
+        <v>0</v>
       </c>
       <c r="G64" s="71" t="n">
-        <v>-0.02965245383120229</v>
+        <v>-0.07828247811415756</v>
       </c>
       <c r="H64" s="71" t="n">
         <v>0</v>
@@ -9355,281 +9170,281 @@
     <row r="65">
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — probability of default</t>
+          <t>Term loans — arrangement fee</t>
         </is>
       </c>
       <c r="C65" s="63" t="n">
-        <v>0.022</v>
+        <v>0.015</v>
       </c>
       <c r="D65" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>% of loan</t>
         </is>
       </c>
       <c r="E65" s="71" t="n">
-        <v>-0.02857600386260983</v>
+        <v>0.07486086293356362</v>
       </c>
       <c r="F65" s="71" t="n">
-        <v>0</v>
+        <v>-0.03572228365829964</v>
       </c>
       <c r="G65" s="71" t="n">
-        <v>-0.02857600386254362</v>
+        <v>0.0689657736584007</v>
       </c>
       <c r="H65" s="71" t="n">
-        <v>0</v>
+        <v>0.03573504903377439</v>
       </c>
     </row>
     <row r="66">
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — loss given default</t>
+          <t>Invoice finance — discount margin over base</t>
         </is>
       </c>
       <c r="C66" s="63" t="n">
-        <v>0.35</v>
+        <v>0.025</v>
       </c>
       <c r="D66" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E66" s="71" t="n">
-        <v>-0.02857600386260983</v>
+        <v>0.07486086293356362</v>
       </c>
       <c r="F66" s="71" t="n">
-        <v>0</v>
+        <v>-0.03572228365829964</v>
       </c>
       <c r="G66" s="71" t="n">
-        <v>-0.02857600386254362</v>
+        <v>0.0689657736584007</v>
       </c>
       <c r="H66" s="71" t="n">
-        <v>0</v>
+        <v>0.03573504903377439</v>
       </c>
     </row>
     <row r="67">
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>Management span (staff per manager)</t>
+          <t>Term loans — risk weight</t>
         </is>
       </c>
       <c r="C67" s="63" t="n">
-        <v>8</v>
+        <v>0.7</v>
       </c>
       <c r="D67" s="14" t="inlineStr">
         <is>
-          <t>staff</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E67" s="71" t="n">
-        <v>0.02728475739292511</v>
+        <v>0.07264851188601439</v>
       </c>
       <c r="F67" s="71" t="n">
-        <v>-0.0284847865736678</v>
+        <v>-0.03466695472918382</v>
       </c>
       <c r="G67" s="71" t="n">
-        <v>0.02728475739261982</v>
+        <v>-0.5108399059911144</v>
       </c>
       <c r="H67" s="71" t="n">
-        <v>0</v>
+        <v>0.03467897687449064</v>
       </c>
     </row>
     <row r="68">
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>Team manager — salary</t>
+          <t>International payments — number per user per year</t>
         </is>
       </c>
       <c r="C68" s="63" t="n">
-        <v>85000</v>
+        <v>30</v>
       </c>
       <c r="D68" s="14" t="inlineStr">
         <is>
-          <t>£/yr</t>
+          <t>payments</t>
         </is>
       </c>
       <c r="E68" s="71" t="n">
-        <v>-0.0257511658564655</v>
+        <v>0.06987013873799271</v>
       </c>
       <c r="F68" s="71" t="n">
-        <v>0.02688374512136233</v>
+        <v>-0.03334159210622355</v>
       </c>
       <c r="G68" s="71" t="n">
-        <v>-0.02575116585676012</v>
+        <v>0.06436830819666425</v>
       </c>
       <c r="H68" s="71" t="n">
-        <v>0</v>
+        <v>0.03335271243152277</v>
       </c>
     </row>
     <row r="69">
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>Annual customer churn (replaced at steady state)</t>
+          <t>International payment fee</t>
         </is>
       </c>
       <c r="C69" s="63" t="n">
-        <v>0.12</v>
+        <v>17.5</v>
       </c>
       <c r="D69" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/payment</t>
         </is>
       </c>
       <c r="E69" s="71" t="n">
-        <v>-0.02469126258220576</v>
+        <v>0.06987013873799271</v>
       </c>
       <c r="F69" s="71" t="n">
-        <v>0.02577722553153486</v>
+        <v>-0.03334159210622355</v>
       </c>
       <c r="G69" s="71" t="n">
-        <v>-0.02469126258230462</v>
+        <v>0.06436830819666425</v>
       </c>
       <c r="H69" s="71" t="n">
-        <v>0</v>
+        <v>0.03335271243152277</v>
       </c>
     </row>
     <row r="70">
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>Employment on-costs (NI, pension, benefits)</t>
+          <t>BCA — monthly account fee</t>
         </is>
       </c>
       <c r="C70" s="63" t="n">
-        <v>0.15</v>
+        <v>8.5</v>
       </c>
       <c r="D70" s="14" t="inlineStr">
         <is>
-          <t>% of salary</t>
+          <t>£/month</t>
         </is>
       </c>
       <c r="E70" s="71" t="n">
-        <v>-0.02057660219051082</v>
+        <v>0.06787384905976844</v>
       </c>
       <c r="F70" s="71" t="n">
-        <v>0.02148159550679803</v>
+        <v>-0.03238928373466862</v>
       </c>
       <c r="G70" s="71" t="n">
-        <v>-0.02057660219063057</v>
+        <v>0.06252931190123294</v>
       </c>
       <c r="H70" s="71" t="n">
-        <v>0</v>
+        <v>0.03239977779061431</v>
       </c>
     </row>
     <row r="71">
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>Operational-risk RWA multiple of gross income</t>
+          <t>Relationship manager — salary</t>
         </is>
       </c>
       <c r="C71" s="63" t="n">
-        <v>1.875</v>
+        <v>65000</v>
       </c>
       <c r="D71" s="14" t="inlineStr">
         <is>
-          <t>x revenue</t>
+          <t>£/yr</t>
         </is>
       </c>
       <c r="E71" s="71" t="n">
-        <v>0.01940217969118421</v>
+        <v>-0.06464852694618542</v>
       </c>
       <c r="F71" s="71" t="n">
-        <v>-0.009260828777932256</v>
+        <v>0.06749187708921207</v>
       </c>
       <c r="G71" s="71" t="n">
-        <v>-0.1370151321223097</v>
+        <v>-0.06464852694648321</v>
       </c>
       <c r="H71" s="71" t="n">
-        <v>0.009261686486871161</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>Share of lending balances held by RM-managed customers</t>
+          <t>Instant-access savings — average balance</t>
         </is>
       </c>
       <c r="C72" s="63" t="n">
-        <v>0.6</v>
+        <v>30000</v>
       </c>
       <c r="D72" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/account</t>
         </is>
       </c>
       <c r="E72" s="71" t="n">
-        <v>0.01833005970171241</v>
+        <v>0.06103463413552909</v>
       </c>
       <c r="F72" s="71" t="n">
-        <v>0</v>
+        <v>-0.02751368315916409</v>
       </c>
       <c r="G72" s="71" t="n">
-        <v>0.0183300597013768</v>
+        <v>0.05600480950303754</v>
       </c>
       <c r="H72" s="71" t="n">
-        <v>0</v>
+        <v>0.03049390850881691</v>
       </c>
     </row>
     <row r="73">
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>Stewardship effect: relative PD reduction on RM-covered balances</t>
+          <t>Term loans — average life</t>
         </is>
       </c>
       <c r="C73" s="63" t="n">
-        <v>0.2</v>
+        <v>4</v>
       </c>
       <c r="D73" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>years</t>
         </is>
       </c>
       <c r="E73" s="71" t="n">
-        <v>0.01833005970171241</v>
+        <v>-0.0605521133221927</v>
       </c>
       <c r="F73" s="71" t="n">
-        <v>0</v>
+        <v>0.02122446956929888</v>
       </c>
       <c r="G73" s="71" t="n">
-        <v>0.0183300597013768</v>
+        <v>-0.05472260563925134</v>
       </c>
       <c r="H73" s="71" t="n">
-        <v>0</v>
+        <v>-0.03538123666704555</v>
       </c>
     </row>
     <row r="74">
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>Churn replacement — acquisition marketing per new customer won</t>
+          <t>BCA — credit interest paid</t>
         </is>
       </c>
       <c r="C74" s="63" t="n">
-        <v>240</v>
+        <v>0.005</v>
       </c>
       <c r="D74" s="14" t="inlineStr">
         <is>
-          <t>£/new customer</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E74" s="71" t="n">
-        <v>-0.01826591155990401</v>
+        <v>-0.0598886903468509</v>
       </c>
       <c r="F74" s="71" t="n">
-        <v>0.01906927684454543</v>
+        <v>0.02859621432394117</v>
       </c>
       <c r="G74" s="71" t="n">
-        <v>-0.01826591156004862</v>
+        <v>-0.05517846962304982</v>
       </c>
       <c r="H74" s="71" t="n">
-        <v>0</v>
+        <v>-0.02858803922701951</v>
       </c>
     </row>
     <row r="75">
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — risk weight</t>
+          <t>Instant-access savings — penetration</t>
         </is>
       </c>
       <c r="C75" s="63" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="D75" s="14" t="inlineStr">
         <is>
@@ -9637,53 +9452,53 @@
         </is>
       </c>
       <c r="E75" s="71" t="n">
-        <v>0.01771239908840788</v>
+        <v>0.0592544503026677</v>
       </c>
       <c r="F75" s="71" t="n">
-        <v>-0.008454350017280498</v>
+        <v>-0.02565577041929928</v>
       </c>
       <c r="G75" s="71" t="n">
-        <v>-0.125099206722287</v>
+        <v>0.05422471515567431</v>
       </c>
       <c r="H75" s="71" t="n">
-        <v>0.008455064837974957</v>
+        <v>0.03049390850881691</v>
       </c>
     </row>
     <row r="76">
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t>Card — interest rate on revolving balances</t>
+          <t>Overdraft — average utilisation</t>
         </is>
       </c>
       <c r="C76" s="63" t="n">
-        <v>0.159</v>
+        <v>0.45</v>
       </c>
       <c r="D76" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>% of limit</t>
         </is>
       </c>
       <c r="E76" s="71" t="n">
-        <v>0.01587050294203331</v>
+        <v>0.05776015381344716</v>
       </c>
       <c r="F76" s="71" t="n">
-        <v>-0.007575256506550518</v>
+        <v>-0.03423984406982809</v>
       </c>
       <c r="G76" s="71" t="n">
-        <v>0.01462142272077909</v>
+        <v>0.01710511817772802</v>
       </c>
       <c r="H76" s="71" t="n">
-        <v>0.007575830395216416</v>
+        <v>0.03425157175458779</v>
       </c>
     </row>
     <row r="77">
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>Service &amp; operations staff — salary</t>
+          <t>Credit analyst / underwriter — salary</t>
         </is>
       </c>
       <c r="C77" s="63" t="n">
-        <v>32000</v>
+        <v>55000</v>
       </c>
       <c r="D77" s="14" t="inlineStr">
         <is>
@@ -9691,13 +9506,13 @@
         </is>
       </c>
       <c r="E77" s="71" t="n">
-        <v>-0.01564284608034933</v>
+        <v>-0.05171141124509487</v>
       </c>
       <c r="F77" s="71" t="n">
-        <v>0.01633084456626305</v>
+        <v>0.05398576544161963</v>
       </c>
       <c r="G77" s="71" t="n">
-        <v>-0.01564284608081514</v>
+        <v>-0.05171141124499209</v>
       </c>
       <c r="H77" s="71" t="n">
         <v>0</v>
@@ -9706,79 +9521,79 @@
     <row r="78">
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — probability of default</t>
+          <t>Liquidity buffer held against deposits (LCR / HQLA)</t>
         </is>
       </c>
       <c r="C78" s="63" t="n">
-        <v>0.026</v>
+        <v>0.15</v>
       </c>
       <c r="D78" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>% of deposits</t>
         </is>
       </c>
       <c r="E78" s="71" t="n">
-        <v>-0.01399299296284985</v>
+        <v>-0.04117347461329634</v>
       </c>
       <c r="F78" s="71" t="n">
-        <v>0</v>
+        <v>0.01965814063393465</v>
       </c>
       <c r="G78" s="71" t="n">
-        <v>-0.01399299296281295</v>
+        <v>-0.03793463915464931</v>
       </c>
       <c r="H78" s="71" t="n">
-        <v>0</v>
+        <v>-0.01965427696859545</v>
       </c>
     </row>
     <row r="79">
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — loss given default</t>
+          <t>Yield give-up on the liquidity buffer vs Bank Rate</t>
         </is>
       </c>
       <c r="C79" s="63" t="n">
-        <v>0.55</v>
+        <v>0.01</v>
       </c>
       <c r="D79" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E79" s="71" t="n">
-        <v>-0.01399299296284985</v>
+        <v>-0.04117347461329634</v>
       </c>
       <c r="F79" s="71" t="n">
-        <v>0</v>
+        <v>0.01965814063393465</v>
       </c>
       <c r="G79" s="71" t="n">
-        <v>-0.01399299296281295</v>
+        <v>-0.03793463915464931</v>
       </c>
       <c r="H79" s="71" t="n">
-        <v>0</v>
+        <v>-0.01965427696859545</v>
       </c>
     </row>
     <row r="80">
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t>Term loan underwriting &amp; completion</t>
+          <t>Unit-level platform &amp; processing cost</t>
         </is>
       </c>
       <c r="C80" s="63" t="n">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="D80" s="14" t="inlineStr">
         <is>
-          <t>hrs/new loan</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E80" s="71" t="n">
-        <v>-0.01370322847785298</v>
+        <v>-0.03953660510803504</v>
       </c>
       <c r="F80" s="71" t="n">
-        <v>0.01430591934339043</v>
+        <v>0.0412754910054009</v>
       </c>
       <c r="G80" s="71" t="n">
-        <v>-0.0137032284779602</v>
+        <v>-0.03953660510795137</v>
       </c>
       <c r="H80" s="71" t="n">
         <v>0</v>
@@ -9787,52 +9602,52 @@
     <row r="81">
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — probability of default</t>
+          <t>Overdraft — annual arrangement/renewal fee</t>
         </is>
       </c>
       <c r="C81" s="63" t="n">
-        <v>0.026</v>
+        <v>0.015</v>
       </c>
       <c r="D81" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>% of limit</t>
         </is>
       </c>
       <c r="E81" s="71" t="n">
-        <v>-0.01356896287307272</v>
+        <v>0.03743043146690454</v>
       </c>
       <c r="F81" s="71" t="n">
-        <v>0</v>
+        <v>-0.01786433260297001</v>
       </c>
       <c r="G81" s="71" t="n">
-        <v>-0.01356896287333288</v>
+        <v>0.03448390249733824</v>
       </c>
       <c r="H81" s="71" t="n">
-        <v>0</v>
+        <v>0.01786752451694579</v>
       </c>
     </row>
     <row r="82">
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — loss given default</t>
+          <t>Fraud &amp; payment losses (incl. APP reimbursement) per current account</t>
         </is>
       </c>
       <c r="C82" s="63" t="n">
-        <v>0.2</v>
+        <v>45</v>
       </c>
       <c r="D82" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/BCA/yr</t>
         </is>
       </c>
       <c r="E82" s="71" t="n">
-        <v>-0.01356896287307272</v>
+        <v>-0.02965245383102628</v>
       </c>
       <c r="F82" s="71" t="n">
-        <v>0</v>
+        <v>0.03095661825405067</v>
       </c>
       <c r="G82" s="71" t="n">
-        <v>-0.01356896287333288</v>
+        <v>-0.02965245383120229</v>
       </c>
       <c r="H82" s="71" t="n">
         <v>0</v>
@@ -9841,25 +9656,25 @@
     <row r="83">
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t>Premises &amp; facilities per unit FTE</t>
+          <t>Asset finance — probability of default</t>
         </is>
       </c>
       <c r="C83" s="63" t="n">
-        <v>6000</v>
+        <v>0.022</v>
       </c>
       <c r="D83" s="14" t="inlineStr">
         <is>
-          <t>£/FTE/yr</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E83" s="71" t="n">
-        <v>-0.01354829332592148</v>
+        <v>-0.02857600386260983</v>
       </c>
       <c r="F83" s="71" t="n">
-        <v>0.01414416988493427</v>
+        <v>0</v>
       </c>
       <c r="G83" s="71" t="n">
-        <v>-0.01354829332627234</v>
+        <v>-0.02857600386254362</v>
       </c>
       <c r="H83" s="71" t="n">
         <v>0</v>
@@ -9868,25 +9683,25 @@
     <row r="84">
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t>BCA servicing (queries, payments support)</t>
+          <t>Asset finance — loss given default</t>
         </is>
       </c>
       <c r="C84" s="63" t="n">
-        <v>0.6</v>
+        <v>0.35</v>
       </c>
       <c r="D84" s="14" t="inlineStr">
         <is>
-          <t>hrs/account/yr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E84" s="71" t="n">
-        <v>-0.01335137874766737</v>
+        <v>-0.02857600386260983</v>
       </c>
       <c r="F84" s="71" t="n">
-        <v>0.01393859467455354</v>
+        <v>0</v>
       </c>
       <c r="G84" s="71" t="n">
-        <v>-0.01335137874769045</v>
+        <v>-0.02857600386254362</v>
       </c>
       <c r="H84" s="71" t="n">
         <v>0</v>
@@ -9895,25 +9710,25 @@
     <row r="85">
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t>Overdraft annual review &amp; renewal</t>
+          <t>Management span (staff per manager)</t>
         </is>
       </c>
       <c r="C85" s="63" t="n">
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="D85" s="14" t="inlineStr">
         <is>
-          <t>hrs/facility/yr</t>
+          <t>staff</t>
         </is>
       </c>
       <c r="E85" s="71" t="n">
-        <v>-0.01223502542667563</v>
+        <v>0.02728475739292511</v>
       </c>
       <c r="F85" s="71" t="n">
-        <v>0.01277314227084876</v>
+        <v>-0.0284847865736678</v>
       </c>
       <c r="G85" s="71" t="n">
-        <v>-0.01223502542703396</v>
+        <v>0.02728475739261982</v>
       </c>
       <c r="H85" s="71" t="n">
         <v>0</v>
@@ -9922,25 +9737,25 @@
     <row r="86">
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t>Term loan annual review</t>
+          <t>Team manager — salary</t>
         </is>
       </c>
       <c r="C86" s="63" t="n">
-        <v>3</v>
+        <v>85000</v>
       </c>
       <c r="D86" s="14" t="inlineStr">
         <is>
-          <t>hrs/loan/yr</t>
+          <t>£/yr</t>
         </is>
       </c>
       <c r="E86" s="71" t="n">
-        <v>-0.01174562440962334</v>
+        <v>-0.0257511658564655</v>
       </c>
       <c r="F86" s="71" t="n">
-        <v>0.01226221658007843</v>
+        <v>0.02688374512136233</v>
       </c>
       <c r="G86" s="71" t="n">
-        <v>-0.01174562440975294</v>
+        <v>-0.02575116585676012</v>
       </c>
       <c r="H86" s="71" t="n">
         <v>0</v>
@@ -9949,25 +9764,25 @@
     <row r="87">
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t>FSCS deposit-protection levy</t>
+          <t>Annual customer churn (replaced at steady state)</t>
         </is>
       </c>
       <c r="C87" s="63" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.12</v>
       </c>
       <c r="D87" s="14" t="inlineStr">
         <is>
-          <t>% of protected deposits</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E87" s="71" t="n">
-        <v>-0.009785309764238673</v>
+        <v>-0.02469126258220576</v>
       </c>
       <c r="F87" s="71" t="n">
-        <v>0.01021568402375696</v>
+        <v>0.02577722553153486</v>
       </c>
       <c r="G87" s="71" t="n">
-        <v>-0.009785309764105748</v>
+        <v>-0.02469126258230462</v>
       </c>
       <c r="H87" s="71" t="n">
         <v>0</v>
@@ -9976,25 +9791,25 @@
     <row r="88">
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t>Share of deposit balances that are FSCS-protected</t>
+          <t>Employment on-costs (NI, pension, benefits)</t>
         </is>
       </c>
       <c r="C88" s="63" t="n">
-        <v>0.6</v>
+        <v>0.15</v>
       </c>
       <c r="D88" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% of salary</t>
         </is>
       </c>
       <c r="E88" s="71" t="n">
-        <v>-0.009785309764238673</v>
+        <v>-0.02057660219051082</v>
       </c>
       <c r="F88" s="71" t="n">
-        <v>0.01021568402375696</v>
+        <v>0.02148159550679803</v>
       </c>
       <c r="G88" s="71" t="n">
-        <v>-0.009785309764105748</v>
+        <v>-0.02057660219063057</v>
       </c>
       <c r="H88" s="71" t="n">
         <v>0</v>
@@ -10003,65 +9818,65 @@
     <row r="89">
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — risk weight</t>
+          <t>Operational-risk RWA multiple of gross income</t>
         </is>
       </c>
       <c r="C89" s="63" t="n">
-        <v>0.6</v>
+        <v>1.875</v>
       </c>
       <c r="D89" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>x revenue</t>
         </is>
       </c>
       <c r="E89" s="71" t="n">
-        <v>0.009340522956773279</v>
+        <v>0.01940217969118421</v>
       </c>
       <c r="F89" s="71" t="n">
-        <v>-0.00445852680457372</v>
+        <v>-0.009260828777932256</v>
       </c>
       <c r="G89" s="71" t="n">
-        <v>-0.06601483744602295</v>
+        <v>-0.1370151321223097</v>
       </c>
       <c r="H89" s="71" t="n">
-        <v>0.004458725598148796</v>
+        <v>0.009261686486871161</v>
       </c>
     </row>
     <row r="90">
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — risk weight</t>
+          <t>Share of lending balances held by RM-managed customers</t>
         </is>
       </c>
       <c r="C90" s="63" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="D90" s="14" t="inlineStr">
         <is>
-          <t>% of drawn</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E90" s="71" t="n">
-        <v>0.004378370135987474</v>
+        <v>0.01833005970171241</v>
       </c>
       <c r="F90" s="71" t="n">
-        <v>-0.002089983942857775</v>
+        <v>0</v>
       </c>
       <c r="G90" s="71" t="n">
-        <v>-0.03095684670595658</v>
+        <v>0.0183300597013768</v>
       </c>
       <c r="H90" s="71" t="n">
-        <v>0.002090027624132248</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91">
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t>Tax rate (corporation tax + bank surcharge)</t>
+          <t>Stewardship effect: relative PD reduction on RM-covered balances</t>
         </is>
       </c>
       <c r="C91" s="63" t="n">
-        <v>0.28</v>
+        <v>0.2</v>
       </c>
       <c r="D91" s="14" t="inlineStr">
         <is>
@@ -10069,15 +9884,501 @@
         </is>
       </c>
       <c r="E91" s="71" t="n">
-        <v>0</v>
+        <v>0.01833005970171241</v>
       </c>
       <c r="F91" s="71" t="n">
         <v>0</v>
       </c>
       <c r="G91" s="71" t="n">
+        <v>0.0183300597013768</v>
+      </c>
+      <c r="H91" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="10" t="inlineStr">
+        <is>
+          <t>Churn replacement — acquisition marketing per new customer won</t>
+        </is>
+      </c>
+      <c r="C92" s="63" t="n">
+        <v>240</v>
+      </c>
+      <c r="D92" s="14" t="inlineStr">
+        <is>
+          <t>£/new customer</t>
+        </is>
+      </c>
+      <c r="E92" s="71" t="n">
+        <v>-0.01826591155990401</v>
+      </c>
+      <c r="F92" s="71" t="n">
+        <v>0.01906927684454543</v>
+      </c>
+      <c r="G92" s="71" t="n">
+        <v>-0.01826591156004862</v>
+      </c>
+      <c r="H92" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" s="10" t="inlineStr">
+        <is>
+          <t>Asset finance — risk weight</t>
+        </is>
+      </c>
+      <c r="C93" s="63" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D93" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E93" s="71" t="n">
+        <v>0.01771239908840788</v>
+      </c>
+      <c r="F93" s="71" t="n">
+        <v>-0.008454350017280498</v>
+      </c>
+      <c r="G93" s="71" t="n">
+        <v>-0.125099206722287</v>
+      </c>
+      <c r="H93" s="71" t="n">
+        <v>0.008455064837974957</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="B94" s="10" t="inlineStr">
+        <is>
+          <t>Card — interest rate on revolving balances</t>
+        </is>
+      </c>
+      <c r="C94" s="63" t="n">
+        <v>0.159</v>
+      </c>
+      <c r="D94" s="14" t="inlineStr">
+        <is>
+          <t>% p.a.</t>
+        </is>
+      </c>
+      <c r="E94" s="71" t="n">
+        <v>0.01587050294203331</v>
+      </c>
+      <c r="F94" s="71" t="n">
+        <v>-0.007575256506550518</v>
+      </c>
+      <c r="G94" s="71" t="n">
+        <v>0.01462142272077909</v>
+      </c>
+      <c r="H94" s="71" t="n">
+        <v>0.007575830395216416</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="B95" s="10" t="inlineStr">
+        <is>
+          <t>Service &amp; operations staff — salary</t>
+        </is>
+      </c>
+      <c r="C95" s="63" t="n">
+        <v>32000</v>
+      </c>
+      <c r="D95" s="14" t="inlineStr">
+        <is>
+          <t>£/yr</t>
+        </is>
+      </c>
+      <c r="E95" s="71" t="n">
+        <v>-0.01564284608034933</v>
+      </c>
+      <c r="F95" s="71" t="n">
+        <v>0.01633084456626305</v>
+      </c>
+      <c r="G95" s="71" t="n">
+        <v>-0.01564284608081514</v>
+      </c>
+      <c r="H95" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" s="10" t="inlineStr">
+        <is>
+          <t>Overdraft — probability of default</t>
+        </is>
+      </c>
+      <c r="C96" s="63" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="D96" s="14" t="inlineStr">
+        <is>
+          <t>% p.a.</t>
+        </is>
+      </c>
+      <c r="E96" s="71" t="n">
+        <v>-0.01399299296284985</v>
+      </c>
+      <c r="F96" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G96" s="71" t="n">
+        <v>-0.01399299296281295</v>
+      </c>
+      <c r="H96" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" s="10" t="inlineStr">
+        <is>
+          <t>Overdraft — loss given default</t>
+        </is>
+      </c>
+      <c r="C97" s="63" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D97" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E97" s="71" t="n">
+        <v>-0.01399299296284985</v>
+      </c>
+      <c r="F97" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G97" s="71" t="n">
+        <v>-0.01399299296281295</v>
+      </c>
+      <c r="H97" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="B98" s="10" t="inlineStr">
+        <is>
+          <t>Term loan underwriting &amp; completion</t>
+        </is>
+      </c>
+      <c r="C98" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="D98" s="14" t="inlineStr">
+        <is>
+          <t>hrs/new loan</t>
+        </is>
+      </c>
+      <c r="E98" s="71" t="n">
+        <v>-0.01370322847785298</v>
+      </c>
+      <c r="F98" s="71" t="n">
+        <v>0.01430591934339043</v>
+      </c>
+      <c r="G98" s="71" t="n">
+        <v>-0.0137032284779602</v>
+      </c>
+      <c r="H98" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" s="10" t="inlineStr">
+        <is>
+          <t>Invoice finance — probability of default</t>
+        </is>
+      </c>
+      <c r="C99" s="63" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="D99" s="14" t="inlineStr">
+        <is>
+          <t>% p.a.</t>
+        </is>
+      </c>
+      <c r="E99" s="71" t="n">
+        <v>-0.01356896287307272</v>
+      </c>
+      <c r="F99" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" s="71" t="n">
+        <v>-0.01356896287333288</v>
+      </c>
+      <c r="H99" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" s="10" t="inlineStr">
+        <is>
+          <t>Invoice finance — loss given default</t>
+        </is>
+      </c>
+      <c r="C100" s="63" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D100" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E100" s="71" t="n">
+        <v>-0.01356896287307272</v>
+      </c>
+      <c r="F100" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100" s="71" t="n">
+        <v>-0.01356896287333288</v>
+      </c>
+      <c r="H100" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" s="10" t="inlineStr">
+        <is>
+          <t>Premises &amp; facilities per unit FTE</t>
+        </is>
+      </c>
+      <c r="C101" s="63" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D101" s="14" t="inlineStr">
+        <is>
+          <t>£/FTE/yr</t>
+        </is>
+      </c>
+      <c r="E101" s="71" t="n">
+        <v>-0.01354829332592148</v>
+      </c>
+      <c r="F101" s="71" t="n">
+        <v>0.01414416988493427</v>
+      </c>
+      <c r="G101" s="71" t="n">
+        <v>-0.01354829332627234</v>
+      </c>
+      <c r="H101" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="B102" s="10" t="inlineStr">
+        <is>
+          <t>BCA servicing (queries, payments support)</t>
+        </is>
+      </c>
+      <c r="C102" s="63" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D102" s="14" t="inlineStr">
+        <is>
+          <t>hrs/account/yr</t>
+        </is>
+      </c>
+      <c r="E102" s="71" t="n">
+        <v>-0.01335137874766737</v>
+      </c>
+      <c r="F102" s="71" t="n">
+        <v>0.01393859467455354</v>
+      </c>
+      <c r="G102" s="71" t="n">
+        <v>-0.01335137874769045</v>
+      </c>
+      <c r="H102" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="B103" s="10" t="inlineStr">
+        <is>
+          <t>Overdraft annual review &amp; renewal</t>
+        </is>
+      </c>
+      <c r="C103" s="63" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D103" s="14" t="inlineStr">
+        <is>
+          <t>hrs/facility/yr</t>
+        </is>
+      </c>
+      <c r="E103" s="71" t="n">
+        <v>-0.01223502542667563</v>
+      </c>
+      <c r="F103" s="71" t="n">
+        <v>0.01277314227084876</v>
+      </c>
+      <c r="G103" s="71" t="n">
+        <v>-0.01223502542703396</v>
+      </c>
+      <c r="H103" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="B104" s="10" t="inlineStr">
+        <is>
+          <t>Term loan annual review</t>
+        </is>
+      </c>
+      <c r="C104" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="D104" s="14" t="inlineStr">
+        <is>
+          <t>hrs/loan/yr</t>
+        </is>
+      </c>
+      <c r="E104" s="71" t="n">
+        <v>-0.01174562440962334</v>
+      </c>
+      <c r="F104" s="71" t="n">
+        <v>0.01226221658007843</v>
+      </c>
+      <c r="G104" s="71" t="n">
+        <v>-0.01174562440975294</v>
+      </c>
+      <c r="H104" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="B105" s="10" t="inlineStr">
+        <is>
+          <t>FSCS deposit-protection levy</t>
+        </is>
+      </c>
+      <c r="C105" s="63" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="D105" s="14" t="inlineStr">
+        <is>
+          <t>% of protected deposits</t>
+        </is>
+      </c>
+      <c r="E105" s="71" t="n">
+        <v>-0.009785309764238673</v>
+      </c>
+      <c r="F105" s="71" t="n">
+        <v>0.01021568402375696</v>
+      </c>
+      <c r="G105" s="71" t="n">
+        <v>-0.009785309764105748</v>
+      </c>
+      <c r="H105" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" s="10" t="inlineStr">
+        <is>
+          <t>Share of deposit balances that are FSCS-protected</t>
+        </is>
+      </c>
+      <c r="C106" s="63" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D106" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E106" s="71" t="n">
+        <v>-0.009785309764238673</v>
+      </c>
+      <c r="F106" s="71" t="n">
+        <v>0.01021568402375696</v>
+      </c>
+      <c r="G106" s="71" t="n">
+        <v>-0.009785309764105748</v>
+      </c>
+      <c r="H106" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" s="10" t="inlineStr">
+        <is>
+          <t>Invoice finance — risk weight</t>
+        </is>
+      </c>
+      <c r="C107" s="63" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D107" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E107" s="71" t="n">
+        <v>0.009340522956773279</v>
+      </c>
+      <c r="F107" s="71" t="n">
+        <v>-0.00445852680457372</v>
+      </c>
+      <c r="G107" s="71" t="n">
+        <v>-0.06601483744602295</v>
+      </c>
+      <c r="H107" s="71" t="n">
+        <v>0.004458725598148796</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" s="10" t="inlineStr">
+        <is>
+          <t>Overdraft — risk weight</t>
+        </is>
+      </c>
+      <c r="C108" s="63" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D108" s="14" t="inlineStr">
+        <is>
+          <t>% of drawn</t>
+        </is>
+      </c>
+      <c r="E108" s="71" t="n">
+        <v>0.004378370135987474</v>
+      </c>
+      <c r="F108" s="71" t="n">
+        <v>-0.002089983942857775</v>
+      </c>
+      <c r="G108" s="71" t="n">
+        <v>-0.03095684670595658</v>
+      </c>
+      <c r="H108" s="71" t="n">
+        <v>0.002090027624132248</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" s="10" t="inlineStr">
+        <is>
+          <t>Tax rate (corporation tax + bank surcharge)</t>
+        </is>
+      </c>
+      <c r="C109" s="63" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="D109" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E109" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="F109" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G109" s="71" t="n">
         <v>-0.388888888889195</v>
       </c>
-      <c r="H91" s="71" t="n">
+      <c r="H109" s="71" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
v1.9: competitive response on tab 10
Every scenario assumed rivals stand still. A firm with share s moving alone faces
roughly the industry elasticity divided by s; in concert it faces only the industry
elasticity. Penetration here IS market share (16%), so moving alone multiplies the
demand response by 6.25x.

Tab 10 inverts every break-even into the industry elasticity the move survives in each
regime. The term loan rate survives 2.91 in concert and 0.47 alone.
</commit_message>
<xml_diff>
--- a/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
+++ b/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B49"/>
+  <dimension ref="B1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -606,7 +606,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MODEL VERSION: v1.8 · 22 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
+          <t>MODEL VERSION: v1.9 · 22 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
         </is>
       </c>
     </row>
@@ -620,271 +620,278 @@
     <row r="5" ht="52" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>• v1.8 (22 Aug 2026) — break-even demand elasticity on tab 10. The elasticity table ranked the term loan customer rate as the largest driver of profit at +1.25, which was an artefact: nothing in the model responds to price, so raising any price always looked accretive. Tab 10 now leads with the demand elasticity at which raising each price stops paying. The reordering matters — the card fee breaks even at 0.06 and the current-account fee at 0.13, so both are fragile to almost any customer response, while the loan rate holds to 2.91. The hidden assumption being replaced is zero, which is the least defensible value available.</t>
+          <t>• v1.9 (22 Aug 2026) — competitive response. Every scenario assumed rivals stand still, which flatters both directions at once: raising a price looks safer than it is, and cutting one looks better than it is. A firm with market share s moving alone faces roughly the industry elasticity divided by s; moving in concert it faces only the industry elasticity. This model's penetration IS market share (16%), so moving alone multiplies the demand response by 6.25x. Tab 10 now inverts every break-even into the industry elasticity the move survives in each regime. The headline lever moves with it: raising the term loan rate survives an industry elasticity of 2.91 in concert but only 0.47 alone — marginal rather than comfortable.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="52" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>• v1.7 (22 Aug 2026) — operational leverage. Every cost line in the model scaled linearly with its driver, which forces a cost elasticity of exactly 1.0 and makes cost per customer flat at every scale. Allica Bank's own accounts put that elasticity at 0.808 across 2022-23 and 0.622 across 2023-24 — cost rises materially more slowly than the book. Inputs section O adds a cost scale elasticity and the customer count the per-customer rates are calibrated at; the head-office pools, the platform line and change-the-bank now scale by it. Default 1.0 reproduces v1.6 exactly. Tab 11 adds the out-of-sample test that measured it.</t>
+          <t>• v1.8 (22 Aug 2026) — break-even demand elasticity on tab 10. The elasticity table ranked the term loan customer rate as the largest driver of profit at +1.25, which was an artefact: nothing in the model responds to price, so raising any price always looked accretive. Tab 10 now leads with the demand elasticity at which raising each price stops paying. The reordering matters — the card fee breaks even at 0.06 and the current-account fee at 0.13, so both are fragile to almost any customer response, while the loan rate holds to 2.91. The hidden assumption being replaced is zero, which is the least defensible value available.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>• v1.6 (22 Aug 2026) — validation and drivers. Tab 10 ELASTICITIES: every input bumped +1% and the workbook recalculated, giving the % change in PBT, cost:income, RoE and income. Only one input has an elasticity above 1 on profit — the term loan customer rate, at +1.25; reachable market and penetration are exactly +1.00 (pure scale); nothing else exceeds 0.53. Tab 11 BACKTEST against Allica Bank FY2023 audited accounts: the revenue engine reproduces a real bank's operating income to within 8%, and the cost engine under-predicts by 7x. Diagnosis: head-office cost was modelled purely per customer, which is a scale assumption disguised as a driver. Inputs section N therefore adds a fixed component to each head-office pool, defaulting to 0 so v1.5 results are unchanged.</t>
+          <t>• v1.7 (22 Aug 2026) — operational leverage. Every cost line in the model scaled linearly with its driver, which forces a cost elasticity of exactly 1.0 and makes cost per customer flat at every scale. Allica Bank's own accounts put that elasticity at 0.808 across 2022-23 and 0.622 across 2023-24 — cost rises materially more slowly than the book. Inputs section O adds a cost scale elasticity and the customer count the per-customer rates are calibrated at; the head-office pools, the platform line and change-the-bank now scale by it. Default 1.0 reproduces v1.6 exactly. Tab 11 adds the out-of-sample test that measured it.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>• v1.5 (22 Aug 2026) — PROCESS LAYER on the Step 2 tabs. Tab 3 gains process columns M-T (process type, yield, attempts, automation, best-in-class intensity and yield, benchmark source, £ gap) and a HEAD-OFFICE PROCESS REGISTER of 22 processes already named in the tab 9 operational model but never costed. Yield inflates ATTEMPTS and never deflates outcomes — that is what stops it double-counting with the CEP layer's demand-side conversion. Head-office costs are carved OUT of the pools, so naming a process moves money from unallocated to attributed and the total never changes. New sheet 3b indexes every process to the numbers it moves, and imputes what each would have to become to hit a target cost:income. Mode OFF (default) = results identical to v1.4.</t>
+          <t>• v1.6 (22 Aug 2026) — validation and drivers. Tab 10 ELASTICITIES: every input bumped +1% and the workbook recalculated, giving the % change in PBT, cost:income, RoE and income. Only one input has an elasticity above 1 on profit — the term loan customer rate, at +1.25; reachable market and penetration are exactly +1.00 (pure scale); nothing else exceeds 0.53. Tab 11 BACKTEST against Allica Bank FY2023 audited accounts: the revenue engine reproduces a real bank's operating income to within 8%, and the cost engine under-predicts by 7x. Diagnosis: head-office cost was modelled purely per customer, which is a scale assumption disguised as a driver. Inputs section N therefore adds a fixed component to each head-office pool, defaulting to 0 so v1.5 results are unchanged.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="52" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
+          <t>• v1.5 (22 Aug 2026) — PROCESS LAYER on the Step 2 tabs. Tab 3 gains process columns M-T (process type, yield, attempts, automation, best-in-class intensity and yield, benchmark source, £ gap) and a HEAD-OFFICE PROCESS REGISTER of 22 processes already named in the tab 9 operational model but never costed. Yield inflates ATTEMPTS and never deflates outcomes — that is what stops it double-counting with the CEP layer's demand-side conversion. Head-office costs are carved OUT of the pools, so naming a process moves money from unallocated to attributed and the total never changes. New sheet 3b indexes every process to the numbers it moves, and imputes what each would have to become to hit a target cost:income. Mode OFF (default) = results identical to v1.4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
           <t>• v1.4 (22 Aug 2026) — CEP DEMAND LAYER. New sheet 1b derives the nine product penetrations and the customer count instead of asserting them: penetration = (lambda*c x L) / (1 + lambda*c x L), where lambda*c = category-entry-point events x presence x conversion and L is the holding life. Little's Law run forwards; no time axis is added and the model stays a steady-state snapshot. Ships deliberately EMPTY — every event/presence/conversion cell is blank and carries the cohort query that fills it, and any unpopulated product falls back to its hardcoded penetration. Mode OFF (default) = results identical to v1.3; CALIBRATE reports the won-event rate implied by today's assumptions and changes nothing.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="40" customHeight="1">
-      <c r="B10" s="4" t="inlineStr">
+    <row r="11" ht="40" customHeight="1">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>• v1.3 (21 Aug 2026) — churn replacement is a costed activity end-to-end: new input cac_new (£240 acquisition marketing per new customer won, carved out of the corporate-centre pool — hq_oh £250→£222); driver-linked on tab 4, attributed to the current account (gateway product) on tab 6; 'value of preventing one churn' memo added to tab 6. Raising the churn input now inflates demand-generation cost, not just processing. Central PBT shifts &lt;£1k/unit (carve-out rounding).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
+          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
           <t>• v1.0 (10 Aug 2026) — first published version: 9 tabs + flow register, FTP with liquidity/behavioural terms, fraud/FSCS/change-the-bank lines, segment-pod LMUs, bridge check.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="3" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>What this is</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="39" customHeight="1">
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="39" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
         <is>
+          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="39" customHeight="1">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
           <t>• It follows the Simanis / IVE bottom-up methodology ('Running the Right Numbers'): model the last-mile operating unit, derive every cost from activity drivers (transaction intensity I and customer load L), build whole costs, and check the price/margin covers them including a competitive return on capital.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="3" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>What period this models</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="B21" s="4" t="inlineStr">
+    <row r="22" ht="26" customHeight="1">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>• One representative operating year at steady state. Balances are annual averages; rates and volumes are annual. There is no time axis, no ramp and no vintage cohorts — the model is a snapshot, not a forecast.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="78" customHeight="1">
-      <c r="B22" s="4" t="inlineStr">
+    <row r="23" ht="78" customHeight="1">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>• The book is stationary but not free to hold flat: customers churn (12% p.a. input) and the model costs their replacement end-to-end — acquisition marketing per new customer won (cac_new, carved from the corporate-centre pool), onboarding hours, KYC per new customer and RM origination effort are all driver-linked (Simanis: at-scale operations include 'replacement of customer churn'). Only residual brand &amp; joint marketing remains pool-costed. The 'value of preventing one churn' memo on tab 6 prices retention: contribution annuity over remaining relationship life + the avoided replacement cost.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="26" customHeight="1">
-      <c r="B23" s="4" t="inlineStr">
+    <row r="24" ht="26" customHeight="1">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>• The capital charge (cost of equity on allocated capital) is the incumbent analogue of Simanis's start-up-cost amortisation: capital earns its required return inside the steady-state P&amp;L.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="52" customHeight="1">
-      <c r="B24" s="4" t="inlineStr">
+    <row r="25" ht="52" customHeight="1">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>• Out of scope by design: transition paths. The cost and cash shape of moving between steady states — digital migration, maturity glide, behaviour-change programmes and their CAC/incentives — belongs in a scenario layer built ON TOP of this base (comparative statics between two runs of this model, plus a separate transition-cost estimate). The base model never carries scenario logic.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="3" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>How the tabs map to the methodology</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="B27" s="4" t="inlineStr">
+    <row r="28" ht="24" customHeight="1">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>• Inputs — every assumption in one place, with sources. Edit blue cells; yellow cells are the biggest levers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="26" customHeight="1">
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1">
       <c r="B29" s="4" t="inlineStr">
         <is>
+          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
           <t>• 2. Revenues — unit revenue per product: interest margins measured against internal funds transfer prices (Bank Rate for floating, + premium for term), plus fees.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="39" customHeight="1">
-      <c r="B30" s="4" t="inlineStr">
+    <row r="31" ht="39" customHeight="1">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>• 3. HR &amp; Activity — Step 2: every FTE derived from activity drivers (hours per onboarding, review, renewal…) — nothing is assumed as headcount. From v1.5 this tab is also the PROCESS REGISTER (columns M-T), with the head-office process register below it.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="26" customHeight="1">
-      <c r="B31" s="4" t="inlineStr">
+    <row r="32" ht="26" customHeight="1">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>• 1b. Demand &amp; CEPs — the demand layer (v1.4). Penetration is derived, not assumed. Mode cell on Inputs section L: OFF reproduces v1.3, CALIBRATE reports the implied event rates, LIVE derives.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="39" customHeight="1">
-      <c r="B32" s="4" t="inlineStr">
+    <row r="33" ht="39" customHeight="1">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>• 3b. Process Index — derived view, no assumptions. Every process with its flow, product, owner, the numbers it moves, its cost and its gap to best in class, plus a ranked worst-gap list and the top-down benchmark imputation. Answers 'which process do I improve to move this number?'</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="52" customHeight="1">
-      <c r="B33" s="4" t="inlineStr">
+    <row r="34" ht="52" customHeight="1">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>• 4. Running Costs — Step 2 (cont.): direct running costs plus the share of head-office costs. The attribution memo reads the tab 3 process register and reports the share of the cost base with a named process owner — the model's own assessment of how much of its cost it actually understands. What remains in UNALLOCATED JOINT COSTS is cost with no process to improve.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="26" customHeight="1">
-      <c r="B34" s="4" t="inlineStr">
+    <row r="35" ht="26" customHeight="1">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>• 5. Risk &amp; Capital — Step 3: expected credit losses (PD × LGD), risk-weighted assets, allocated equity, and the required return on it.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="91" customHeight="1">
-      <c r="B35" s="4" t="inlineStr">
+    <row r="36" ht="91" customHeight="1">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>• 6. Unit Economics — Steps 4–5: per-product unit costs and revenues on an activity-based costing basis, taken exactly as far as causality runs (the source methodology's own rule: link costs to customers and transactions 'whenever possible'). Costs with real drivers — servicing hours, RM effort per origination, staff-time-driven supervision, per-account and per-facility infrastructure — are attributed to products; genuinely joint costs (brand, exec, finance, platform build) are NOT forced into products but held as an unallocated hurdle that total contribution must clear, with a full-absorption memo showing the source doc's simple-division treatment. Product decisions should run on contribution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="26" customHeight="1">
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="26" customHeight="1">
       <c r="B37" s="4" t="inlineStr">
         <is>
+          <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="26" customHeight="1">
+      <c r="B38" s="4" t="inlineStr">
+        <is>
           <t>• 8. Org Structure — the whole-bank organisation implied by the model: front-line FTEs from activity drivers × number of centres, head-office FTEs backed out of the per-customer head-office cost allocations.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="52" customHeight="1">
-      <c r="B38" s="4" t="inlineStr">
+    <row r="39" ht="52" customHeight="1">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>• 9. Flow Register — one row per flow on the operational model map: component type (CP/WP/PP/PartP), core/support/enabling, direction, digital/physical medium, the direct/administrative/managerial roles accountable, and the BIAN service domains. Ends with a BIAN completeness checklist. This is where the map, the ARM and BIAN reconcile.</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="B40" s="3" t="inlineStr">
+    <row r="41">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>Colour legend</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="26" customHeight="1">
-      <c r="B41" s="4" t="inlineStr">
+    <row r="42" ht="26" customHeight="1">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>• Blue = hardcoded input (edit these) · Yellow fill = key assumption / sensitivity lever · Black = formula · Green = link to another sheet.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="3" t="inlineStr">
+    <row r="44">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>Reading the results</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="52" customHeight="1">
-      <c r="B44" s="4" t="inlineStr">
+    <row r="45" ht="52" customHeight="1">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>• Deposit products earn the spread between the transfer price and the rate paid; lending earns the customer rate minus the transfer price minus expected losses. Capital-heavy, labour-heavy products (term loans) can show thin or negative economic profit — consistent with the Bank of England's 2026 finding that SME lending earns the lowest product-level returns, driven by impairments and per-borrower servicing costs.</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="39" customHeight="1">
-      <c r="B45" s="4" t="inlineStr">
+    <row r="46" ht="39" customHeight="1">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>• Use the cost-driver table on the P&amp;L tab to find leverage points, then trace them to transaction intensity (I) or customer load (L) assumptions on the Inputs tab — e.g. automating underwriting hours, raising RM portfolio size, or shifting servicing to digital.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="B47" s="3" t="inlineStr">
+    <row r="48">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>Caveats</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="39" customHeight="1">
-      <c r="B48" s="4" t="inlineStr">
+    <row r="49" ht="39" customHeight="1">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>• Benchmarks are as of August 2026 (Bank Rate 3.75%; BoE effective new SME loan rate ~6.3%; commercial interchange 1.65–1.90%; invoice finance discount base+1–3%). Items marked 'Assumption' are illustrative and should be replaced with your own data.</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="65" customHeight="1">
-      <c r="B49" s="4" t="inlineStr">
+    <row r="50" ht="65" customHeight="1">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>• The FTP now carries an explicit liquidity charge (buffer × drag) and a behavioural credit for stable deposits, shown as memos on the Revenues tab; it is still a single curve, not a full behavioural-maturity model. Fraud &amp; payment losses, the FSCS levy, collateral administration &amp; recoveries, and change-the-bank spend are now modelled explicitly. Operational-risk RWA is proxied at 15% of gross income; head-office and change costs are allocated per customer.</t>
         </is>
@@ -7742,7 +7749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H109"/>
+  <dimension ref="B1:H112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -7803,59 +7810,66 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="45" t="inlineStr">
+    <row r="9" ht="58" customHeight="1">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Break-even is of the EFFECTIVE elasticity the bank faces. What the bank faces depends on whether rivals follow. A firm with market share s that moves alone faces roughly e_industry / s, because customers can go next door; if the whole industry moves together it faces only e_industry. This model's penetration IS market share — 16% of the national SME market — so moving alone multiplies the demand response by 1/s. The last two columns invert the break-even into the INDUSTRY elasticity each move survives, in each regime.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="B10" s="45" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="C9" s="45" t="inlineStr">
-        <is>
-          <t>e(PBT) with no demand response</t>
-        </is>
-      </c>
-      <c r="D9" s="45" t="inlineStr">
-        <is>
-          <t>Break-even demand elasticity</t>
-        </is>
-      </c>
-      <c r="E9" s="45" t="inlineStr">
+      <c r="C10" s="45" t="inlineStr">
+        <is>
+          <t>e(PBT), no response</t>
+        </is>
+      </c>
+      <c r="D10" s="45" t="inlineStr">
+        <is>
+          <t>Break-even (effective)</t>
+        </is>
+      </c>
+      <c r="E10" s="45" t="inlineStr">
+        <is>
+          <t>Survives industry e up to — MOVING ALONE</t>
+        </is>
+      </c>
+      <c r="F10" s="45" t="inlineStr">
+        <is>
+          <t>Survives industry e up to — IN CONCERT</t>
+        </is>
+      </c>
+      <c r="G10" s="45" t="inlineStr">
         <is>
           <t>Reading</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Card — annual card fee</t>
-        </is>
-      </c>
-      <c r="C10" s="71" t="n">
-        <v>0.006388126970350395</v>
-      </c>
-      <c r="D10" s="63" t="n">
-        <v>0.05544003490987621</v>
-      </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>fragile — only a near-inert customer makes this pay</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>BCA — monthly account fee</t>
+          <t>Card — annual card fee</t>
         </is>
       </c>
       <c r="C11" s="71" t="n">
-        <v>0.06787384905974791</v>
+        <v>0.006388126970350395</v>
       </c>
       <c r="D11" s="63" t="n">
-        <v>0.1275035819127078</v>
-      </c>
-      <c r="E11" s="14" t="inlineStr">
+        <v>0.05544003490987621</v>
+      </c>
+      <c r="E11" s="63">
+        <f>D11*'Inputs'!$F$22</f>
+        <v/>
+      </c>
+      <c r="F11" s="63">
+        <f>D11</f>
+        <v/>
+      </c>
+      <c r="G11" s="14" t="inlineStr">
         <is>
           <t>fragile — only a near-inert customer makes this pay</t>
         </is>
@@ -7864,16 +7878,24 @@
     <row r="12">
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Card — interest rate on revolving balances</t>
+          <t>BCA — monthly account fee</t>
         </is>
       </c>
       <c r="C12" s="71" t="n">
-        <v>0.01587050294191057</v>
+        <v>0.06787384905974791</v>
       </c>
       <c r="D12" s="63" t="n">
-        <v>0.1376205835187992</v>
-      </c>
-      <c r="E12" s="14" t="inlineStr">
+        <v>0.1275035819127078</v>
+      </c>
+      <c r="E12" s="63">
+        <f>D12*'Inputs'!$F$22</f>
+        <v/>
+      </c>
+      <c r="F12" s="63">
+        <f>D12</f>
+        <v/>
+      </c>
+      <c r="G12" s="14" t="inlineStr">
         <is>
           <t>fragile — only a near-inert customer makes this pay</t>
         </is>
@@ -7882,16 +7904,24 @@
     <row r="13">
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Term loans — arrangement fee</t>
+          <t>Card — interest rate on revolving balances</t>
         </is>
       </c>
       <c r="C13" s="71" t="n">
-        <v>0.07486086293356356</v>
+        <v>0.01587050294191057</v>
       </c>
       <c r="D13" s="63" t="n">
-        <v>0.1792828253338209</v>
-      </c>
-      <c r="E13" s="14" t="inlineStr">
+        <v>0.1376205835187992</v>
+      </c>
+      <c r="E13" s="63">
+        <f>D13*'Inputs'!$F$22</f>
+        <v/>
+      </c>
+      <c r="F13" s="63">
+        <f>D13</f>
+        <v/>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
         <is>
           <t>fragile — only a near-inert customer makes this pay</t>
         </is>
@@ -7900,16 +7930,24 @@
     <row r="14">
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — discount margin over base</t>
+          <t>Term loans — arrangement fee</t>
         </is>
       </c>
       <c r="C14" s="71" t="n">
         <v>0.07486086293356356</v>
       </c>
       <c r="D14" s="63" t="n">
-        <v>0.2515282418779798</v>
-      </c>
-      <c r="E14" s="14" t="inlineStr">
+        <v>0.1792828253338209</v>
+      </c>
+      <c r="E14" s="63">
+        <f>D14*'Inputs'!$F$22</f>
+        <v/>
+      </c>
+      <c r="F14" s="63">
+        <f>D14</f>
+        <v/>
+      </c>
+      <c r="G14" s="14" t="inlineStr">
         <is>
           <t>fragile — only a near-inert customer makes this pay</t>
         </is>
@@ -7918,16 +7956,24 @@
     <row r="15">
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>International payment fee</t>
+          <t>Invoice finance — discount margin over base</t>
         </is>
       </c>
       <c r="C15" s="71" t="n">
-        <v>0.06987013873799264</v>
+        <v>0.07486086293356356</v>
       </c>
       <c r="D15" s="63" t="n">
-        <v>0.4122296676035196</v>
-      </c>
-      <c r="E15" s="14" t="inlineStr">
+        <v>0.2515282418779798</v>
+      </c>
+      <c r="E15" s="63">
+        <f>D15*'Inputs'!$F$22</f>
+        <v/>
+      </c>
+      <c r="F15" s="63">
+        <f>D15</f>
+        <v/>
+      </c>
+      <c r="G15" s="14" t="inlineStr">
         <is>
           <t>fragile — only a near-inert customer makes this pay</t>
         </is>
@@ -7936,16 +7982,24 @@
     <row r="16">
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — annual arrangement/renewal fee</t>
+          <t>International payment fee</t>
         </is>
       </c>
       <c r="C16" s="71" t="n">
-        <v>0.03743043146678178</v>
+        <v>0.06987013873799264</v>
       </c>
       <c r="D16" s="63" t="n">
-        <v>0.4581530737163218</v>
-      </c>
-      <c r="E16" s="14" t="inlineStr">
+        <v>0.4122296676035196</v>
+      </c>
+      <c r="E16" s="63">
+        <f>D16*'Inputs'!$F$22</f>
+        <v/>
+      </c>
+      <c r="F16" s="63">
+        <f>D16</f>
+        <v/>
+      </c>
+      <c r="G16" s="14" t="inlineStr">
         <is>
           <t>fragile — only a near-inert customer makes this pay</t>
         </is>
@@ -7954,34 +8008,50 @@
     <row r="17">
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>FX — margin on conversion volume</t>
+          <t>Overdraft — annual arrangement/renewal fee</t>
         </is>
       </c>
       <c r="C17" s="71" t="n">
-        <v>0.09981448391141808</v>
+        <v>0.03743043146678178</v>
       </c>
       <c r="D17" s="63" t="n">
-        <v>0.5878609520414249</v>
-      </c>
-      <c r="E17" s="14" t="inlineStr">
-        <is>
-          <t>modest — a mildly responsive customer cancels it</t>
+        <v>0.4581530737163218</v>
+      </c>
+      <c r="E17" s="63">
+        <f>D17*'Inputs'!$F$22</f>
+        <v/>
+      </c>
+      <c r="F17" s="63">
+        <f>D17</f>
+        <v/>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>fragile — only a near-inert customer makes this pay</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — service fee</t>
+          <t>FX — margin on conversion volume</t>
         </is>
       </c>
       <c r="C18" s="71" t="n">
-        <v>0.2395547613874034</v>
+        <v>0.09981448391141808</v>
       </c>
       <c r="D18" s="63" t="n">
-        <v>0.8004609263604965</v>
-      </c>
-      <c r="E18" s="14" t="inlineStr">
+        <v>0.5878609520414249</v>
+      </c>
+      <c r="E18" s="63">
+        <f>D18*'Inputs'!$F$22</f>
+        <v/>
+      </c>
+      <c r="F18" s="63">
+        <f>D18</f>
+        <v/>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
         <is>
           <t>modest — a mildly responsive customer cancels it</t>
         </is>
@@ -7990,16 +8060,24 @@
     <row r="19">
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — interest rate (EAR)</t>
+          <t>Invoice finance — service fee</t>
         </is>
       </c>
       <c r="C19" s="71" t="n">
-        <v>0.1094840120403367</v>
+        <v>0.2395547613874034</v>
       </c>
       <c r="D19" s="63" t="n">
-        <v>1.328382145135671</v>
-      </c>
-      <c r="E19" s="14" t="inlineStr">
+        <v>0.8004609263604965</v>
+      </c>
+      <c r="E19" s="63">
+        <f>D19*'Inputs'!$F$22</f>
+        <v/>
+      </c>
+      <c r="F19" s="63">
+        <f>D19</f>
+        <v/>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
         <is>
           <t>modest — a mildly responsive customer cancels it</t>
         </is>
@@ -8008,34 +8086,50 @@
     <row r="20">
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — customer yield</t>
+          <t>Overdraft — interest rate (EAR)</t>
         </is>
       </c>
       <c r="C20" s="71" t="n">
-        <v>0.3619938616520844</v>
+        <v>0.1094840120403367</v>
       </c>
       <c r="D20" s="63" t="n">
-        <v>2.229914972398844</v>
-      </c>
-      <c r="E20" s="14" t="inlineStr">
-        <is>
-          <t>robust — needs a strongly responsive customer to destroy value</t>
+        <v>1.328382145135671</v>
+      </c>
+      <c r="E20" s="63">
+        <f>D20*'Inputs'!$F$22</f>
+        <v/>
+      </c>
+      <c r="F20" s="63">
+        <f>D20</f>
+        <v/>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>modest — a mildly responsive customer cancels it</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Term loans — customer rate</t>
+          <t>Asset finance — customer yield</t>
         </is>
       </c>
       <c r="C21" s="71" t="n">
-        <v>1.247681048892726</v>
+        <v>0.3619938616520844</v>
       </c>
       <c r="D21" s="63" t="n">
-        <v>2.906412804688113</v>
-      </c>
-      <c r="E21" s="14" t="inlineStr">
+        <v>2.229914972398844</v>
+      </c>
+      <c r="E21" s="63">
+        <f>D21*'Inputs'!$F$22</f>
+        <v/>
+      </c>
+      <c r="F21" s="63">
+        <f>D21</f>
+        <v/>
+      </c>
+      <c r="G21" s="14" t="inlineStr">
         <is>
           <t>robust — needs a strongly responsive customer to destroy value</t>
         </is>
@@ -8044,16 +8138,24 @@
     <row r="22">
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Instant-access savings — rate paid</t>
+          <t>Term loans — customer rate</t>
         </is>
       </c>
       <c r="C22" s="71" t="n">
-        <v>0.2635102375261355</v>
+        <v>1.247681048892726</v>
       </c>
       <c r="D22" s="63" t="n">
-        <v>4.257749912948078</v>
-      </c>
-      <c r="E22" s="14" t="inlineStr">
+        <v>2.906412804688113</v>
+      </c>
+      <c r="E22" s="63">
+        <f>D22*'Inputs'!$F$22</f>
+        <v/>
+      </c>
+      <c r="F22" s="63">
+        <f>D22</f>
+        <v/>
+      </c>
+      <c r="G22" s="14" t="inlineStr">
         <is>
           <t>robust — needs a strongly responsive customer to destroy value</t>
         </is>
@@ -8062,390 +8164,350 @@
     <row r="23">
       <c r="B23" s="10" t="inlineStr">
         <is>
+          <t>Instant-access savings — rate paid</t>
+        </is>
+      </c>
+      <c r="C23" s="71" t="n">
+        <v>0.2635102375261355</v>
+      </c>
+      <c r="D23" s="63" t="n">
+        <v>4.257749912948078</v>
+      </c>
+      <c r="E23" s="63">
+        <f>D23*'Inputs'!$F$22</f>
+        <v/>
+      </c>
+      <c r="F23" s="63">
+        <f>D23</f>
+        <v/>
+      </c>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>robust — needs a strongly responsive customer to destroy value</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="10" t="inlineStr">
+        <is>
           <t>Notice &amp; fixed deposits — rate paid</t>
         </is>
       </c>
-      <c r="C23" s="71" t="n">
+      <c r="C24" s="71" t="n">
         <v>0.3069295380276106</v>
       </c>
-      <c r="D23" s="63" t="n">
+      <c r="D24" s="63" t="n">
         <v>42.5163639198051</v>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E24" s="63">
+        <f>D24*'Inputs'!$F$22</f>
+        <v/>
+      </c>
+      <c r="F24" s="63">
+        <f>D24</f>
+        <v/>
+      </c>
+      <c r="G24" s="14" t="inlineStr">
         <is>
           <t>robust — needs a strongly responsive customer to destroy value</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="45" t="inlineStr">
+    <row r="26" ht="62" customHeight="1">
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>A cut is the mirror image: cut alone and share moves, so the cut can pay; cut and get matched and volume responds only at the industry elasticity, because nobody's relative price changed — you keep your share and give away the margin. For the term loan rate the band between 0.47 and 2.91 is where the answer depends entirely on whether rivals follow. The same move creates value in one regime and destroys it in the other, and no amount of internal analysis resolves that. SME banking is concentrated with observable prices, which is the textbook setting for high match rates: the prior should be that rivals follow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="45" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="C25" s="45" t="inlineStr">
+      <c r="C28" s="45" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="D25" s="45" t="inlineStr">
+      <c r="D28" s="45" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="E25" s="45" t="inlineStr">
+      <c r="E28" s="45" t="inlineStr">
         <is>
           <t>e(PBT)</t>
         </is>
       </c>
-      <c r="F25" s="45" t="inlineStr">
+      <c r="F28" s="45" t="inlineStr">
         <is>
           <t>e(Cost:income)</t>
         </is>
       </c>
-      <c r="G25" s="45" t="inlineStr">
+      <c r="G28" s="45" t="inlineStr">
         <is>
           <t>e(RoE)</t>
         </is>
       </c>
-      <c r="H25" s="45" t="inlineStr">
+      <c r="H28" s="45" t="inlineStr">
         <is>
           <t>e(Income)</t>
         </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t>Term loans — customer rate</t>
-        </is>
-      </c>
-      <c r="C26" s="63" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="D26" s="14" t="inlineStr">
-        <is>
-          <t>% p.a.</t>
-        </is>
-      </c>
-      <c r="E26" s="71" t="n">
-        <v>1.247681048892727</v>
-      </c>
-      <c r="F26" s="71" t="n">
-        <v>-0.5920579472668667</v>
-      </c>
-      <c r="G26" s="71" t="n">
-        <v>1.148369761396499</v>
-      </c>
-      <c r="H26" s="71" t="n">
-        <v>0.5955841505629065</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="10" t="inlineStr">
-        <is>
-          <t>Reachable SMEs in region (R)</t>
-        </is>
-      </c>
-      <c r="C27" s="63" t="n">
-        <v>18750</v>
-      </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>businesses</t>
-        </is>
-      </c>
-      <c r="E27" s="71" t="n">
-        <v>1.00000000000003</v>
-      </c>
-      <c r="F27" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="71" t="n">
-        <v>1.00000000000002</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="10" t="inlineStr">
-        <is>
-          <t>Steady-state penetration (P)</t>
-        </is>
-      </c>
-      <c r="C28" s="63" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="D28" s="14" t="inlineStr">
-        <is>
-          <t>% of reachable</t>
-        </is>
-      </c>
-      <c r="E28" s="71" t="n">
-        <v>1.00000000000003</v>
-      </c>
-      <c r="F28" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="71" t="n">
-        <v>1.00000000000002</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Business current account — penetration</t>
+          <t>Term loans — customer rate</t>
         </is>
       </c>
       <c r="C29" s="63" t="n">
-        <v>1</v>
+        <v>0.0625</v>
       </c>
       <c r="D29" s="14" t="inlineStr">
         <is>
-          <t>% of customers</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E29" s="71" t="n">
-        <v>0.5316502207558557</v>
+        <v>1.247681048892727</v>
       </c>
       <c r="F29" s="71" t="n">
-        <v>-0.2263724971407025</v>
+        <v>-0.5920579472668667</v>
       </c>
       <c r="G29" s="71" t="n">
-        <v>0.4858715994436417</v>
+        <v>1.148369761396499</v>
       </c>
       <c r="H29" s="71" t="n">
-        <v>0.2763510458611886</v>
+        <v>0.5955841505629065</v>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Term loans — average balance</t>
+          <t>Reachable SMEs in region (R)</t>
         </is>
       </c>
       <c r="C30" s="63" t="n">
-        <v>250000</v>
+        <v>18750</v>
       </c>
       <c r="D30" s="14" t="inlineStr">
         <is>
-          <t>£/loan</t>
+          <t>businesses</t>
         </is>
       </c>
       <c r="E30" s="71" t="n">
-        <v>0.4485219355690576</v>
+        <v>1.00000000000003</v>
       </c>
       <c r="F30" s="71" t="n">
-        <v>-0.2508408142510311</v>
+        <v>0</v>
       </c>
       <c r="G30" s="71" t="n">
-        <v>-0.172627245775743</v>
+        <v>0</v>
       </c>
       <c r="H30" s="71" t="n">
-        <v>0.2514716076793886</v>
+        <v>1.00000000000002</v>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>BCA — average credit balance</t>
+          <t>Steady-state penetration (P)</t>
         </is>
       </c>
       <c r="C31" s="63" t="n">
-        <v>18000</v>
+        <v>0.16</v>
       </c>
       <c r="D31" s="14" t="inlineStr">
         <is>
-          <t>£/account</t>
+          <t>% of reachable</t>
         </is>
       </c>
       <c r="E31" s="71" t="n">
-        <v>0.4269286171458919</v>
+        <v>1.00000000000003</v>
       </c>
       <c r="F31" s="71" t="n">
-        <v>-0.2009624805300439</v>
+        <v>0</v>
       </c>
       <c r="G31" s="71" t="n">
-        <v>0.3928629971036865</v>
+        <v>0</v>
       </c>
       <c r="H31" s="71" t="n">
-        <v>0.2058338824345483</v>
+        <v>1.00000000000002</v>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>Term loans / commercial mortgages — penetration</t>
+          <t>Business current account — penetration</t>
         </is>
       </c>
       <c r="C32" s="63" t="n">
-        <v>0.12</v>
+        <v>1</v>
       </c>
       <c r="D32" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% of customers</t>
         </is>
       </c>
       <c r="E32" s="71" t="n">
-        <v>0.4168087496628946</v>
+        <v>0.5316502207558557</v>
       </c>
       <c r="F32" s="71" t="n">
-        <v>-0.2178158778235073</v>
+        <v>-0.2263724971407025</v>
       </c>
       <c r="G32" s="71" t="n">
-        <v>-0.2041443250685729</v>
+        <v>0.4858715994436417</v>
       </c>
       <c r="H32" s="71" t="n">
-        <v>0.2514716076793886</v>
+        <v>0.2763510458611886</v>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — customer yield</t>
+          <t>Term loans — average balance</t>
         </is>
       </c>
       <c r="C33" s="63" t="n">
-        <v>0.08500000000000001</v>
+        <v>250000</v>
       </c>
       <c r="D33" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/loan</t>
         </is>
       </c>
       <c r="E33" s="71" t="n">
-        <v>0.3619938616520847</v>
+        <v>0.4485219355690576</v>
       </c>
       <c r="F33" s="71" t="n">
-        <v>-0.1725007356564119</v>
+        <v>-0.2508408142510311</v>
       </c>
       <c r="G33" s="71" t="n">
-        <v>0.3334124986436103</v>
+        <v>-0.172627245775743</v>
       </c>
       <c r="H33" s="71" t="n">
-        <v>0.1727988148833219</v>
+        <v>0.2514716076793886</v>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — average funds in use (advances)</t>
+          <t>BCA — average credit balance</t>
         </is>
       </c>
       <c r="C34" s="63" t="n">
-        <v>150000</v>
+        <v>18000</v>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>£/client</t>
+          <t>£/account</t>
         </is>
       </c>
       <c r="E34" s="71" t="n">
-        <v>0.3101871844046677</v>
+        <v>0.4269286171458919</v>
       </c>
       <c r="F34" s="71" t="n">
-        <v>-0.1543074556452041</v>
+        <v>-0.2009624805300439</v>
       </c>
       <c r="G34" s="71" t="n">
-        <v>0.209829595204097</v>
+        <v>0.3928629971036865</v>
       </c>
       <c r="H34" s="71" t="n">
-        <v>0.1545459315400012</v>
+        <v>0.2058338824345483</v>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Notice &amp; fixed deposits — rate paid</t>
+          <t>Term loans / commercial mortgages — penetration</t>
         </is>
       </c>
       <c r="C35" s="63" t="n">
-        <v>0.041</v>
+        <v>0.12</v>
       </c>
       <c r="D35" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E35" s="71" t="n">
-        <v>-0.3069295380274881</v>
+        <v>0.4168087496628946</v>
       </c>
       <c r="F35" s="71" t="n">
-        <v>0.1467286786560457</v>
+        <v>-0.2178158778235073</v>
       </c>
       <c r="G35" s="71" t="n">
-        <v>-0.2828446455047969</v>
+        <v>-0.2041443250685729</v>
       </c>
       <c r="H35" s="71" t="n">
-        <v>-0.1465137010384164</v>
+        <v>0.2514716076793886</v>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — penetration</t>
+          <t>Asset finance — customer yield</t>
         </is>
       </c>
       <c r="C36" s="63" t="n">
-        <v>0.03</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="D36" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E36" s="71" t="n">
-        <v>0.2968754767403625</v>
+        <v>0.3619938616520847</v>
       </c>
       <c r="F36" s="71" t="n">
-        <v>-0.1404317212375283</v>
+        <v>-0.1725007356564119</v>
       </c>
       <c r="G36" s="71" t="n">
-        <v>0.1965312055379295</v>
+        <v>0.3334124986436103</v>
       </c>
       <c r="H36" s="71" t="n">
-        <v>0.1545459315400012</v>
+        <v>0.1727988148833219</v>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Head office: technology &amp; central operations</t>
+          <t>Invoice finance — average funds in use (advances)</t>
         </is>
       </c>
       <c r="C37" s="63" t="n">
-        <v>450</v>
+        <v>150000</v>
       </c>
       <c r="D37" s="14" t="inlineStr">
         <is>
-          <t>£/customer/yr</t>
+          <t>£/client</t>
         </is>
       </c>
       <c r="E37" s="71" t="n">
-        <v>-0.2965245383102628</v>
+        <v>0.3101871844046677</v>
       </c>
       <c r="F37" s="71" t="n">
-        <v>0.3095661825398512</v>
+        <v>-0.1543074556452041</v>
       </c>
       <c r="G37" s="71" t="n">
-        <v>-0.2965245383105712</v>
+        <v>0.209829595204097</v>
       </c>
       <c r="H37" s="71" t="n">
-        <v>0</v>
+        <v>0.1545459315400012</v>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Instant-access savings — rate paid</t>
+          <t>Notice &amp; fixed deposits — rate paid</t>
         </is>
       </c>
       <c r="C38" s="63" t="n">
-        <v>0.033</v>
+        <v>0.041</v>
       </c>
       <c r="D38" s="14" t="inlineStr">
         <is>
@@ -8453,80 +8515,80 @@
         </is>
       </c>
       <c r="E38" s="71" t="n">
-        <v>-0.2635102375261357</v>
+        <v>-0.3069295380274881</v>
       </c>
       <c r="F38" s="71" t="n">
-        <v>0.1259457965071908</v>
+        <v>0.1467286786560457</v>
       </c>
       <c r="G38" s="71" t="n">
-        <v>-0.2428241773307234</v>
+        <v>-0.2828446455047969</v>
       </c>
       <c r="H38" s="71" t="n">
-        <v>-0.125787372598882</v>
+        <v>-0.1465137010384164</v>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — funded invoices as multiple of advances</t>
+          <t>Invoice finance — penetration</t>
         </is>
       </c>
       <c r="C39" s="63" t="n">
-        <v>8</v>
+        <v>0.03</v>
       </c>
       <c r="D39" s="14" t="inlineStr">
         <is>
-          <t>x p.a.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E39" s="71" t="n">
-        <v>0.2395547613874036</v>
+        <v>0.2968754767403625</v>
       </c>
       <c r="F39" s="71" t="n">
-        <v>-0.1142215421111091</v>
+        <v>-0.1404317212375283</v>
       </c>
       <c r="G39" s="71" t="n">
-        <v>0.2206618790426836</v>
+        <v>0.1965312055379295</v>
       </c>
       <c r="H39" s="71" t="n">
-        <v>0.1143521569080781</v>
+        <v>0.1545459315400012</v>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — service fee</t>
+          <t>Head office: technology &amp; central operations</t>
         </is>
       </c>
       <c r="C40" s="63" t="n">
-        <v>0.01</v>
+        <v>450</v>
       </c>
       <c r="D40" s="14" t="inlineStr">
         <is>
-          <t>% of funded invoices</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E40" s="71" t="n">
-        <v>0.2395547613874036</v>
+        <v>-0.2965245383102628</v>
       </c>
       <c r="F40" s="71" t="n">
-        <v>-0.1142215421111091</v>
+        <v>0.3095661825398512</v>
       </c>
       <c r="G40" s="71" t="n">
-        <v>0.2206618790426836</v>
+        <v>-0.2965245383105712</v>
       </c>
       <c r="H40" s="71" t="n">
-        <v>0.1143521569080781</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Bank of England Bank Rate</t>
+          <t>Instant-access savings — rate paid</t>
         </is>
       </c>
       <c r="C41" s="63" t="n">
-        <v>0.0375</v>
+        <v>0.033</v>
       </c>
       <c r="D41" s="14" t="inlineStr">
         <is>
@@ -8534,107 +8596,107 @@
         </is>
       </c>
       <c r="E41" s="71" t="n">
-        <v>0.1990512830997236</v>
+        <v>-0.2635102375261357</v>
       </c>
       <c r="F41" s="71" t="n">
-        <v>-0.09492750668173035</v>
+        <v>0.1259457965071908</v>
       </c>
       <c r="G41" s="71" t="n">
-        <v>0.1931242862657616</v>
+        <v>-0.2428241773307234</v>
       </c>
       <c r="H41" s="71" t="n">
-        <v>0.09501770461968793</v>
+        <v>-0.125787372598882</v>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>International payments &amp; FX — penetration</t>
+          <t>Invoice finance — funded invoices as multiple of advances</t>
         </is>
       </c>
       <c r="C42" s="63" t="n">
-        <v>0.2</v>
+        <v>8</v>
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>x p.a.</t>
         </is>
       </c>
       <c r="E42" s="71" t="n">
-        <v>0.1687945307331029</v>
+        <v>0.2395547613874036</v>
       </c>
       <c r="F42" s="71" t="n">
-        <v>-0.08000540090128463</v>
+        <v>-0.1142215421111091</v>
       </c>
       <c r="G42" s="71" t="n">
-        <v>0.1554207840445721</v>
+        <v>0.2206618790426836</v>
       </c>
       <c r="H42" s="71" t="n">
-        <v>0.08099944447655529</v>
+        <v>0.1143521569080781</v>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — average balance</t>
+          <t>Invoice finance — service fee</t>
         </is>
       </c>
       <c r="C43" s="63" t="n">
-        <v>80000</v>
+        <v>0.01</v>
       </c>
       <c r="D43" s="14" t="inlineStr">
         <is>
-          <t>£/agreement</t>
+          <t>% of funded invoices</t>
         </is>
       </c>
       <c r="E43" s="71" t="n">
-        <v>0.1658745747382735</v>
+        <v>0.2395547613874036</v>
       </c>
       <c r="F43" s="71" t="n">
-        <v>-0.09273546655296665</v>
+        <v>-0.1142215421111091</v>
       </c>
       <c r="G43" s="71" t="n">
-        <v>0.008961968797843937</v>
+        <v>0.2206618790426836</v>
       </c>
       <c r="H43" s="71" t="n">
-        <v>0.09282154504571802</v>
+        <v>0.1143521569080781</v>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>Head office: risk, compliance, financial crime, audit</t>
+          <t>Bank of England Bank Rate</t>
         </is>
       </c>
       <c r="C44" s="63" t="n">
-        <v>250</v>
+        <v>0.0375</v>
       </c>
       <c r="D44" s="14" t="inlineStr">
         <is>
-          <t>£/customer/yr</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E44" s="71" t="n">
-        <v>-0.1647358546168127</v>
+        <v>0.1990512830997236</v>
       </c>
       <c r="F44" s="71" t="n">
-        <v>0.1719812125220667</v>
+        <v>-0.09492750668173035</v>
       </c>
       <c r="G44" s="71" t="n">
-        <v>-0.1647358546170901</v>
+        <v>0.1931242862657616</v>
       </c>
       <c r="H44" s="71" t="n">
-        <v>0</v>
+        <v>0.09501770461968793</v>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — penetration</t>
+          <t>International payments &amp; FX — penetration</t>
         </is>
       </c>
       <c r="C45" s="63" t="n">
-        <v>0.08</v>
+        <v>0.2</v>
       </c>
       <c r="D45" s="14" t="inlineStr">
         <is>
@@ -8642,80 +8704,80 @@
         </is>
       </c>
       <c r="E45" s="71" t="n">
-        <v>0.1587153370028682</v>
+        <v>0.1687945307331029</v>
       </c>
       <c r="F45" s="71" t="n">
-        <v>-0.08526828474335443</v>
+        <v>-0.08000540090128463</v>
       </c>
       <c r="G45" s="71" t="n">
-        <v>0.001813946205839392</v>
+        <v>0.1554207840445721</v>
       </c>
       <c r="H45" s="71" t="n">
-        <v>0.09282154504571802</v>
+        <v>0.08099944447655529</v>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>Head office: finance, HR, exec, brand &amp; residual (non-acquisition) marketing</t>
+          <t>Asset finance — average balance</t>
         </is>
       </c>
       <c r="C46" s="63" t="n">
-        <v>222</v>
+        <v>80000</v>
       </c>
       <c r="D46" s="14" t="inlineStr">
         <is>
-          <t>£/customer/yr</t>
+          <t>£/agreement</t>
         </is>
       </c>
       <c r="E46" s="71" t="n">
-        <v>-0.1462854388997297</v>
+        <v>0.1658745747382735</v>
       </c>
       <c r="F46" s="71" t="n">
-        <v>0.1527193167196385</v>
+        <v>-0.09273546655296665</v>
       </c>
       <c r="G46" s="71" t="n">
-        <v>-0.1462854388999867</v>
+        <v>0.008961968797843937</v>
       </c>
       <c r="H46" s="71" t="n">
-        <v>0</v>
+        <v>0.09282154504571802</v>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>Equity held against RWAs (CET1 target)</t>
+          <t>Head office: risk, compliance, financial crime, audit</t>
         </is>
       </c>
       <c r="C47" s="63" t="n">
-        <v>0.14</v>
+        <v>250</v>
       </c>
       <c r="D47" s="14" t="inlineStr">
         <is>
-          <t>% of RWA</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E47" s="71" t="n">
-        <v>0.1238711722148994</v>
+        <v>-0.1647358546168127</v>
       </c>
       <c r="F47" s="71" t="n">
-        <v>-0.05909531843834973</v>
+        <v>0.1719812125220667</v>
       </c>
       <c r="G47" s="71" t="n">
-        <v>-0.8674542849359645</v>
+        <v>-0.1647358546170901</v>
       </c>
       <c r="H47" s="71" t="n">
-        <v>0.05913026165485447</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Business credit card — penetration</t>
+          <t>Asset finance — penetration</t>
         </is>
       </c>
       <c r="C48" s="63" t="n">
-        <v>0.3</v>
+        <v>0.08</v>
       </c>
       <c r="D48" s="14" t="inlineStr">
         <is>
@@ -8723,107 +8785,107 @@
         </is>
       </c>
       <c r="E48" s="71" t="n">
-        <v>0.115162001627308</v>
+        <v>0.1587153370028682</v>
       </c>
       <c r="F48" s="71" t="n">
-        <v>-0.05450341134971946</v>
+        <v>-0.08526828474335443</v>
       </c>
       <c r="G48" s="71" t="n">
-        <v>0.1025383467743691</v>
+        <v>0.001813946205839392</v>
       </c>
       <c r="H48" s="71" t="n">
-        <v>0.05762391571351869</v>
+        <v>0.09282154504571802</v>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — interest rate (EAR)</t>
+          <t>Head office: finance, HR, exec, brand &amp; residual (non-acquisition) marketing</t>
         </is>
       </c>
       <c r="C49" s="63" t="n">
-        <v>0.0975</v>
+        <v>222</v>
       </c>
       <c r="D49" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E49" s="71" t="n">
-        <v>0.1094840120404391</v>
+        <v>-0.1462854388997297</v>
       </c>
       <c r="F49" s="71" t="n">
-        <v>-0.05223520978052387</v>
+        <v>0.1527193167196385</v>
       </c>
       <c r="G49" s="71" t="n">
-        <v>0.1008596961142311</v>
+        <v>-0.1462854388999867</v>
       </c>
       <c r="H49" s="71" t="n">
-        <v>0.05226250921193411</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>Card — average monthly spend</t>
+          <t>Equity held against RWAs (CET1 target)</t>
         </is>
       </c>
       <c r="C50" s="63" t="n">
-        <v>2500</v>
+        <v>0.14</v>
       </c>
       <c r="D50" s="14" t="inlineStr">
         <is>
-          <t>£/card/month</t>
+          <t>% of RWA</t>
         </is>
       </c>
       <c r="E50" s="71" t="n">
-        <v>0.1018107735896629</v>
+        <v>0.1238711722148994</v>
       </c>
       <c r="F50" s="71" t="n">
-        <v>-0.04857605888322602</v>
+        <v>-0.05909531843834973</v>
       </c>
       <c r="G50" s="71" t="n">
-        <v>0.09379146319211618</v>
+        <v>-0.8674542849359645</v>
       </c>
       <c r="H50" s="71" t="n">
-        <v>0.04859966668594098</v>
+        <v>0.05913026165485447</v>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>Card — commercial interchange earned</t>
+          <t>Business credit card — penetration</t>
         </is>
       </c>
       <c r="C51" s="63" t="n">
-        <v>0.017</v>
+        <v>0.3</v>
       </c>
       <c r="D51" s="14" t="inlineStr">
         <is>
-          <t>% of spend</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E51" s="71" t="n">
-        <v>0.1018107735896629</v>
+        <v>0.115162001627308</v>
       </c>
       <c r="F51" s="71" t="n">
-        <v>-0.04857605888322602</v>
+        <v>-0.05450341134971946</v>
       </c>
       <c r="G51" s="71" t="n">
-        <v>0.09379146319211618</v>
+        <v>0.1025383467743691</v>
       </c>
       <c r="H51" s="71" t="n">
-        <v>0.04859966668594098</v>
+        <v>0.05762391571351869</v>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>Term funding premium over Bank Rate</t>
+          <t>Overdraft — interest rate (EAR)</t>
         </is>
       </c>
       <c r="C52" s="63" t="n">
-        <v>0.006</v>
+        <v>0.0975</v>
       </c>
       <c r="D52" s="14" t="inlineStr">
         <is>
@@ -8831,229 +8893,229 @@
         </is>
       </c>
       <c r="E52" s="71" t="n">
-        <v>-0.1004133708148834</v>
+        <v>0.1094840120404391</v>
       </c>
       <c r="F52" s="71" t="n">
-        <v>0.04795559880866109</v>
+        <v>-0.05223520978052387</v>
       </c>
       <c r="G52" s="71" t="n">
-        <v>-0.09251885130815904</v>
+        <v>0.1008596961142311</v>
       </c>
       <c r="H52" s="71" t="n">
-        <v>-0.04793261243730116</v>
+        <v>0.05226250921193411</v>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>Behavioural term credit for stable non-maturing deposits</t>
+          <t>Card — average monthly spend</t>
         </is>
       </c>
       <c r="C53" s="63" t="n">
-        <v>0.005</v>
+        <v>2500</v>
       </c>
       <c r="D53" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/card/month</t>
         </is>
       </c>
       <c r="E53" s="71" t="n">
-        <v>0.09981448391141816</v>
+        <v>0.1018107735896629</v>
       </c>
       <c r="F53" s="71" t="n">
-        <v>-0.04762404074601882</v>
+        <v>-0.04857605888322602</v>
       </c>
       <c r="G53" s="71" t="n">
-        <v>0.09195255933441075</v>
+        <v>0.09379146319211618</v>
       </c>
       <c r="H53" s="71" t="n">
-        <v>0.04764673204503252</v>
+        <v>0.04859966668594098</v>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>FX — average annual conversion volume</t>
+          <t>Card — commercial interchange earned</t>
         </is>
       </c>
       <c r="C54" s="63" t="n">
-        <v>100000</v>
+        <v>0.017</v>
       </c>
       <c r="D54" s="14" t="inlineStr">
         <is>
-          <t>£/user/yr</t>
+          <t>% of spend</t>
         </is>
       </c>
       <c r="E54" s="71" t="n">
-        <v>0.09981448391141816</v>
+        <v>0.1018107735896629</v>
       </c>
       <c r="F54" s="71" t="n">
-        <v>-0.04762404074601882</v>
+        <v>-0.04857605888322602</v>
       </c>
       <c r="G54" s="71" t="n">
-        <v>0.09195255933441075</v>
+        <v>0.09379146319211618</v>
       </c>
       <c r="H54" s="71" t="n">
-        <v>0.04764673204503252</v>
+        <v>0.04859966668594098</v>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>FX — margin on conversion volume</t>
+          <t>Term funding premium over Bank Rate</t>
         </is>
       </c>
       <c r="C55" s="63" t="n">
-        <v>0.0075</v>
+        <v>0.006</v>
       </c>
       <c r="D55" s="14" t="inlineStr">
         <is>
-          <t>% of volume</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E55" s="71" t="n">
-        <v>0.09981448391141816</v>
+        <v>-0.1004133708148834</v>
       </c>
       <c r="F55" s="71" t="n">
-        <v>-0.04762404074601882</v>
+        <v>0.04795559880866109</v>
       </c>
       <c r="G55" s="71" t="n">
-        <v>0.09195255933441075</v>
+        <v>-0.09251885130815904</v>
       </c>
       <c r="H55" s="71" t="n">
-        <v>0.04764673204503252</v>
+        <v>-0.04793261243730116</v>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — average limit</t>
+          <t>Behavioural term credit for stable non-maturing deposits</t>
         </is>
       </c>
       <c r="C56" s="63" t="n">
-        <v>15000</v>
+        <v>0.005</v>
       </c>
       <c r="D56" s="14" t="inlineStr">
         <is>
-          <t>£/facility</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E56" s="71" t="n">
-        <v>0.09519058528012668</v>
+        <v>0.09981448391141816</v>
       </c>
       <c r="F56" s="71" t="n">
-        <v>-0.05209194641982378</v>
+        <v>-0.04762404074601882</v>
       </c>
       <c r="G56" s="71" t="n">
-        <v>0.051574506124141</v>
+        <v>0.09195255933441075</v>
       </c>
       <c r="H56" s="71" t="n">
-        <v>0.05211909627141639</v>
+        <v>0.04764673204503252</v>
       </c>
     </row>
     <row r="57">
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>Productive hours per FTE per month</t>
+          <t>FX — average annual conversion volume</t>
         </is>
       </c>
       <c r="C57" s="63" t="n">
-        <v>147</v>
+        <v>100000</v>
       </c>
       <c r="D57" s="14" t="inlineStr">
         <is>
-          <t>hours</t>
+          <t>£/user/yr</t>
         </is>
       </c>
       <c r="E57" s="71" t="n">
-        <v>0.09121190632452875</v>
+        <v>0.09981448391141816</v>
       </c>
       <c r="F57" s="71" t="n">
-        <v>-0.09522355823886089</v>
+        <v>-0.04762404074601882</v>
       </c>
       <c r="G57" s="71" t="n">
-        <v>0.09121190632435788</v>
+        <v>0.09195255933441075</v>
       </c>
       <c r="H57" s="71" t="n">
-        <v>0</v>
+        <v>0.04764673204503252</v>
       </c>
     </row>
     <row r="58">
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — penetration</t>
+          <t>FX — margin on conversion volume</t>
         </is>
       </c>
       <c r="C58" s="63" t="n">
-        <v>0.25</v>
+        <v>0.0075</v>
       </c>
       <c r="D58" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% of volume</t>
         </is>
       </c>
       <c r="E58" s="71" t="n">
-        <v>0.08132422312990931</v>
+        <v>0.09981448391141816</v>
       </c>
       <c r="F58" s="71" t="n">
-        <v>-0.0376232594615131</v>
+        <v>-0.04762404074601882</v>
       </c>
       <c r="G58" s="71" t="n">
-        <v>0.0377141861854879</v>
+        <v>0.09195255933441075</v>
       </c>
       <c r="H58" s="71" t="n">
-        <v>0.05211909627141639</v>
+        <v>0.04764673204503252</v>
       </c>
     </row>
     <row r="59">
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>Customers per relationship manager (L)</t>
+          <t>Overdraft — average limit</t>
         </is>
       </c>
       <c r="C59" s="63" t="n">
-        <v>120</v>
+        <v>15000</v>
       </c>
       <c r="D59" s="14" t="inlineStr">
         <is>
-          <t>customers</t>
+          <t>£/facility</t>
         </is>
       </c>
       <c r="E59" s="71" t="n">
-        <v>0.08107710567534358</v>
+        <v>0.09519058528012668</v>
       </c>
       <c r="F59" s="71" t="n">
-        <v>-0.08464301213748615</v>
+        <v>-0.05209194641982378</v>
       </c>
       <c r="G59" s="71" t="n">
-        <v>0.08107710567522457</v>
+        <v>0.051574506124141</v>
       </c>
       <c r="H59" s="71" t="n">
-        <v>0</v>
+        <v>0.05211909627141639</v>
       </c>
     </row>
     <row r="60">
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>Share of customers that are relationship-managed</t>
+          <t>Productive hours per FTE per month</t>
         </is>
       </c>
       <c r="C60" s="63" t="n">
-        <v>0.15</v>
+        <v>147</v>
       </c>
       <c r="D60" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>hours</t>
         </is>
       </c>
       <c r="E60" s="71" t="n">
-        <v>-0.08092587948856705</v>
+        <v>0.09121190632452875</v>
       </c>
       <c r="F60" s="71" t="n">
-        <v>0.08448513477060619</v>
+        <v>-0.09522355823886089</v>
       </c>
       <c r="G60" s="71" t="n">
-        <v>-0.08092587948885854</v>
+        <v>0.09121190632435788</v>
       </c>
       <c r="H60" s="71" t="n">
         <v>0</v>
@@ -9062,34 +9124,34 @@
     <row r="61">
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>BCA — net transaction &amp; cash-handling income</t>
+          <t>Overdraft — penetration</t>
         </is>
       </c>
       <c r="C61" s="63" t="n">
-        <v>120</v>
+        <v>0.25</v>
       </c>
       <c r="D61" s="14" t="inlineStr">
         <is>
-          <t>£/account/yr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E61" s="71" t="n">
-        <v>0.07985158712913452</v>
+        <v>0.08132422312990931</v>
       </c>
       <c r="F61" s="71" t="n">
-        <v>-0.03810286182134639</v>
+        <v>-0.0376232594615131</v>
       </c>
       <c r="G61" s="71" t="n">
-        <v>0.07356320301076685</v>
+        <v>0.0377141861854879</v>
       </c>
       <c r="H61" s="71" t="n">
-        <v>0.03811738563602602</v>
+        <v>0.05211909627141639</v>
       </c>
     </row>
     <row r="62">
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Change-the-bank / transformation spend per customer</t>
+          <t>Customers per relationship manager (L)</t>
         </is>
       </c>
       <c r="C62" s="63" t="n">
@@ -9097,17 +9159,17 @@
       </c>
       <c r="D62" s="14" t="inlineStr">
         <is>
-          <t>£/customer/yr</t>
+          <t>customers</t>
         </is>
       </c>
       <c r="E62" s="71" t="n">
-        <v>-0.07907321021607008</v>
+        <v>0.08107710567534358</v>
       </c>
       <c r="F62" s="71" t="n">
-        <v>0.08255098201058327</v>
+        <v>-0.08464301213748615</v>
       </c>
       <c r="G62" s="71" t="n">
-        <v>-0.0790732102163739</v>
+        <v>0.08107710567522457</v>
       </c>
       <c r="H62" s="71" t="n">
         <v>0</v>
@@ -9116,25 +9178,25 @@
     <row r="63">
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>Term loans — probability of default</t>
+          <t>Share of customers that are relationship-managed</t>
         </is>
       </c>
       <c r="C63" s="63" t="n">
-        <v>0.018</v>
+        <v>0.15</v>
       </c>
       <c r="D63" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E63" s="71" t="n">
-        <v>-0.07828247811390938</v>
+        <v>-0.08092587948856705</v>
       </c>
       <c r="F63" s="71" t="n">
-        <v>0</v>
+        <v>0.08448513477060619</v>
       </c>
       <c r="G63" s="71" t="n">
-        <v>-0.07828247811415756</v>
+        <v>-0.08092587948885854</v>
       </c>
       <c r="H63" s="71" t="n">
         <v>0</v>
@@ -9143,65 +9205,65 @@
     <row r="64">
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>Term loans — loss given default</t>
+          <t>BCA — net transaction &amp; cash-handling income</t>
         </is>
       </c>
       <c r="C64" s="63" t="n">
-        <v>0.25</v>
+        <v>120</v>
       </c>
       <c r="D64" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/account/yr</t>
         </is>
       </c>
       <c r="E64" s="71" t="n">
-        <v>-0.07828247811390938</v>
+        <v>0.07985158712913452</v>
       </c>
       <c r="F64" s="71" t="n">
-        <v>0</v>
+        <v>-0.03810286182134639</v>
       </c>
       <c r="G64" s="71" t="n">
-        <v>-0.07828247811415756</v>
+        <v>0.07356320301076685</v>
       </c>
       <c r="H64" s="71" t="n">
-        <v>0</v>
+        <v>0.03811738563602602</v>
       </c>
     </row>
     <row r="65">
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>Term loans — arrangement fee</t>
+          <t>Change-the-bank / transformation spend per customer</t>
         </is>
       </c>
       <c r="C65" s="63" t="n">
-        <v>0.015</v>
+        <v>120</v>
       </c>
       <c r="D65" s="14" t="inlineStr">
         <is>
-          <t>% of loan</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E65" s="71" t="n">
-        <v>0.07486086293356362</v>
+        <v>-0.07907321021607008</v>
       </c>
       <c r="F65" s="71" t="n">
-        <v>-0.03572228365829964</v>
+        <v>0.08255098201058327</v>
       </c>
       <c r="G65" s="71" t="n">
-        <v>0.0689657736584007</v>
+        <v>-0.0790732102163739</v>
       </c>
       <c r="H65" s="71" t="n">
-        <v>0.03573504903377439</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — discount margin over base</t>
+          <t>Term loans — probability of default</t>
         </is>
       </c>
       <c r="C66" s="63" t="n">
-        <v>0.025</v>
+        <v>0.018</v>
       </c>
       <c r="D66" s="14" t="inlineStr">
         <is>
@@ -9209,26 +9271,26 @@
         </is>
       </c>
       <c r="E66" s="71" t="n">
-        <v>0.07486086293356362</v>
+        <v>-0.07828247811390938</v>
       </c>
       <c r="F66" s="71" t="n">
-        <v>-0.03572228365829964</v>
+        <v>0</v>
       </c>
       <c r="G66" s="71" t="n">
-        <v>0.0689657736584007</v>
+        <v>-0.07828247811415756</v>
       </c>
       <c r="H66" s="71" t="n">
-        <v>0.03573504903377439</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>Term loans — risk weight</t>
+          <t>Term loans — loss given default</t>
         </is>
       </c>
       <c r="C67" s="63" t="n">
-        <v>0.7</v>
+        <v>0.25</v>
       </c>
       <c r="D67" s="14" t="inlineStr">
         <is>
@@ -9236,229 +9298,229 @@
         </is>
       </c>
       <c r="E67" s="71" t="n">
-        <v>0.07264851188601439</v>
+        <v>-0.07828247811390938</v>
       </c>
       <c r="F67" s="71" t="n">
-        <v>-0.03466695472918382</v>
+        <v>0</v>
       </c>
       <c r="G67" s="71" t="n">
-        <v>-0.5108399059911144</v>
+        <v>-0.07828247811415756</v>
       </c>
       <c r="H67" s="71" t="n">
-        <v>0.03467897687449064</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>International payments — number per user per year</t>
+          <t>Term loans — arrangement fee</t>
         </is>
       </c>
       <c r="C68" s="63" t="n">
-        <v>30</v>
+        <v>0.015</v>
       </c>
       <c r="D68" s="14" t="inlineStr">
         <is>
-          <t>payments</t>
+          <t>% of loan</t>
         </is>
       </c>
       <c r="E68" s="71" t="n">
-        <v>0.06987013873799271</v>
+        <v>0.07486086293356362</v>
       </c>
       <c r="F68" s="71" t="n">
-        <v>-0.03334159210622355</v>
+        <v>-0.03572228365829964</v>
       </c>
       <c r="G68" s="71" t="n">
-        <v>0.06436830819666425</v>
+        <v>0.0689657736584007</v>
       </c>
       <c r="H68" s="71" t="n">
-        <v>0.03335271243152277</v>
+        <v>0.03573504903377439</v>
       </c>
     </row>
     <row r="69">
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>International payment fee</t>
+          <t>Invoice finance — discount margin over base</t>
         </is>
       </c>
       <c r="C69" s="63" t="n">
-        <v>17.5</v>
+        <v>0.025</v>
       </c>
       <c r="D69" s="14" t="inlineStr">
         <is>
-          <t>£/payment</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E69" s="71" t="n">
-        <v>0.06987013873799271</v>
+        <v>0.07486086293356362</v>
       </c>
       <c r="F69" s="71" t="n">
-        <v>-0.03334159210622355</v>
+        <v>-0.03572228365829964</v>
       </c>
       <c r="G69" s="71" t="n">
-        <v>0.06436830819666425</v>
+        <v>0.0689657736584007</v>
       </c>
       <c r="H69" s="71" t="n">
-        <v>0.03335271243152277</v>
+        <v>0.03573504903377439</v>
       </c>
     </row>
     <row r="70">
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>BCA — monthly account fee</t>
+          <t>Term loans — risk weight</t>
         </is>
       </c>
       <c r="C70" s="63" t="n">
-        <v>8.5</v>
+        <v>0.7</v>
       </c>
       <c r="D70" s="14" t="inlineStr">
         <is>
-          <t>£/month</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E70" s="71" t="n">
-        <v>0.06787384905976844</v>
+        <v>0.07264851188601439</v>
       </c>
       <c r="F70" s="71" t="n">
-        <v>-0.03238928373466862</v>
+        <v>-0.03466695472918382</v>
       </c>
       <c r="G70" s="71" t="n">
-        <v>0.06252931190123294</v>
+        <v>-0.5108399059911144</v>
       </c>
       <c r="H70" s="71" t="n">
-        <v>0.03239977779061431</v>
+        <v>0.03467897687449064</v>
       </c>
     </row>
     <row r="71">
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>Relationship manager — salary</t>
+          <t>International payments — number per user per year</t>
         </is>
       </c>
       <c r="C71" s="63" t="n">
-        <v>65000</v>
+        <v>30</v>
       </c>
       <c r="D71" s="14" t="inlineStr">
         <is>
-          <t>£/yr</t>
+          <t>payments</t>
         </is>
       </c>
       <c r="E71" s="71" t="n">
-        <v>-0.06464852694618542</v>
+        <v>0.06987013873799271</v>
       </c>
       <c r="F71" s="71" t="n">
-        <v>0.06749187708921207</v>
+        <v>-0.03334159210622355</v>
       </c>
       <c r="G71" s="71" t="n">
-        <v>-0.06464852694648321</v>
+        <v>0.06436830819666425</v>
       </c>
       <c r="H71" s="71" t="n">
-        <v>0</v>
+        <v>0.03335271243152277</v>
       </c>
     </row>
     <row r="72">
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>Instant-access savings — average balance</t>
+          <t>International payment fee</t>
         </is>
       </c>
       <c r="C72" s="63" t="n">
-        <v>30000</v>
+        <v>17.5</v>
       </c>
       <c r="D72" s="14" t="inlineStr">
         <is>
-          <t>£/account</t>
+          <t>£/payment</t>
         </is>
       </c>
       <c r="E72" s="71" t="n">
-        <v>0.06103463413552909</v>
+        <v>0.06987013873799271</v>
       </c>
       <c r="F72" s="71" t="n">
-        <v>-0.02751368315916409</v>
+        <v>-0.03334159210622355</v>
       </c>
       <c r="G72" s="71" t="n">
-        <v>0.05600480950303754</v>
+        <v>0.06436830819666425</v>
       </c>
       <c r="H72" s="71" t="n">
-        <v>0.03049390850881691</v>
+        <v>0.03335271243152277</v>
       </c>
     </row>
     <row r="73">
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>Term loans — average life</t>
+          <t>BCA — monthly account fee</t>
         </is>
       </c>
       <c r="C73" s="63" t="n">
-        <v>4</v>
+        <v>8.5</v>
       </c>
       <c r="D73" s="14" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>£/month</t>
         </is>
       </c>
       <c r="E73" s="71" t="n">
-        <v>-0.0605521133221927</v>
+        <v>0.06787384905976844</v>
       </c>
       <c r="F73" s="71" t="n">
-        <v>0.02122446956929888</v>
+        <v>-0.03238928373466862</v>
       </c>
       <c r="G73" s="71" t="n">
-        <v>-0.05472260563925134</v>
+        <v>0.06252931190123294</v>
       </c>
       <c r="H73" s="71" t="n">
-        <v>-0.03538123666704555</v>
+        <v>0.03239977779061431</v>
       </c>
     </row>
     <row r="74">
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>BCA — credit interest paid</t>
+          <t>Relationship manager — salary</t>
         </is>
       </c>
       <c r="C74" s="63" t="n">
-        <v>0.005</v>
+        <v>65000</v>
       </c>
       <c r="D74" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/yr</t>
         </is>
       </c>
       <c r="E74" s="71" t="n">
-        <v>-0.0598886903468509</v>
+        <v>-0.06464852694618542</v>
       </c>
       <c r="F74" s="71" t="n">
-        <v>0.02859621432394117</v>
+        <v>0.06749187708921207</v>
       </c>
       <c r="G74" s="71" t="n">
-        <v>-0.05517846962304982</v>
+        <v>-0.06464852694648321</v>
       </c>
       <c r="H74" s="71" t="n">
-        <v>-0.02858803922701951</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>Instant-access savings — penetration</t>
+          <t>Instant-access savings — average balance</t>
         </is>
       </c>
       <c r="C75" s="63" t="n">
-        <v>0.4</v>
+        <v>30000</v>
       </c>
       <c r="D75" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/account</t>
         </is>
       </c>
       <c r="E75" s="71" t="n">
-        <v>0.0592544503026677</v>
+        <v>0.06103463413552909</v>
       </c>
       <c r="F75" s="71" t="n">
-        <v>-0.02565577041929928</v>
+        <v>-0.02751368315916409</v>
       </c>
       <c r="G75" s="71" t="n">
-        <v>0.05422471515567431</v>
+        <v>0.05600480950303754</v>
       </c>
       <c r="H75" s="71" t="n">
         <v>0.03049390850881691</v>
@@ -9467,133 +9529,133 @@
     <row r="76">
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — average utilisation</t>
+          <t>Term loans — average life</t>
         </is>
       </c>
       <c r="C76" s="63" t="n">
-        <v>0.45</v>
+        <v>4</v>
       </c>
       <c r="D76" s="14" t="inlineStr">
         <is>
-          <t>% of limit</t>
+          <t>years</t>
         </is>
       </c>
       <c r="E76" s="71" t="n">
-        <v>0.05776015381344716</v>
+        <v>-0.0605521133221927</v>
       </c>
       <c r="F76" s="71" t="n">
-        <v>-0.03423984406982809</v>
+        <v>0.02122446956929888</v>
       </c>
       <c r="G76" s="71" t="n">
-        <v>0.01710511817772802</v>
+        <v>-0.05472260563925134</v>
       </c>
       <c r="H76" s="71" t="n">
-        <v>0.03425157175458779</v>
+        <v>-0.03538123666704555</v>
       </c>
     </row>
     <row r="77">
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>Credit analyst / underwriter — salary</t>
+          <t>BCA — credit interest paid</t>
         </is>
       </c>
       <c r="C77" s="63" t="n">
-        <v>55000</v>
+        <v>0.005</v>
       </c>
       <c r="D77" s="14" t="inlineStr">
         <is>
-          <t>£/yr</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E77" s="71" t="n">
-        <v>-0.05171141124509487</v>
+        <v>-0.0598886903468509</v>
       </c>
       <c r="F77" s="71" t="n">
-        <v>0.05398576544161963</v>
+        <v>0.02859621432394117</v>
       </c>
       <c r="G77" s="71" t="n">
-        <v>-0.05171141124499209</v>
+        <v>-0.05517846962304982</v>
       </c>
       <c r="H77" s="71" t="n">
-        <v>0</v>
+        <v>-0.02858803922701951</v>
       </c>
     </row>
     <row r="78">
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t>Liquidity buffer held against deposits (LCR / HQLA)</t>
+          <t>Instant-access savings — penetration</t>
         </is>
       </c>
       <c r="C78" s="63" t="n">
-        <v>0.15</v>
+        <v>0.4</v>
       </c>
       <c r="D78" s="14" t="inlineStr">
         <is>
-          <t>% of deposits</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E78" s="71" t="n">
-        <v>-0.04117347461329634</v>
+        <v>0.0592544503026677</v>
       </c>
       <c r="F78" s="71" t="n">
-        <v>0.01965814063393465</v>
+        <v>-0.02565577041929928</v>
       </c>
       <c r="G78" s="71" t="n">
-        <v>-0.03793463915464931</v>
+        <v>0.05422471515567431</v>
       </c>
       <c r="H78" s="71" t="n">
-        <v>-0.01965427696859545</v>
+        <v>0.03049390850881691</v>
       </c>
     </row>
     <row r="79">
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t>Yield give-up on the liquidity buffer vs Bank Rate</t>
+          <t>Overdraft — average utilisation</t>
         </is>
       </c>
       <c r="C79" s="63" t="n">
-        <v>0.01</v>
+        <v>0.45</v>
       </c>
       <c r="D79" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>% of limit</t>
         </is>
       </c>
       <c r="E79" s="71" t="n">
-        <v>-0.04117347461329634</v>
+        <v>0.05776015381344716</v>
       </c>
       <c r="F79" s="71" t="n">
-        <v>0.01965814063393465</v>
+        <v>-0.03423984406982809</v>
       </c>
       <c r="G79" s="71" t="n">
-        <v>-0.03793463915464931</v>
+        <v>0.01710511817772802</v>
       </c>
       <c r="H79" s="71" t="n">
-        <v>-0.01965427696859545</v>
+        <v>0.03425157175458779</v>
       </c>
     </row>
     <row r="80">
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t>Unit-level platform &amp; processing cost</t>
+          <t>Credit analyst / underwriter — salary</t>
         </is>
       </c>
       <c r="C80" s="63" t="n">
-        <v>60</v>
+        <v>55000</v>
       </c>
       <c r="D80" s="14" t="inlineStr">
         <is>
-          <t>£/customer/yr</t>
+          <t>£/yr</t>
         </is>
       </c>
       <c r="E80" s="71" t="n">
-        <v>-0.03953660510803504</v>
+        <v>-0.05171141124509487</v>
       </c>
       <c r="F80" s="71" t="n">
-        <v>0.0412754910054009</v>
+        <v>0.05398576544161963</v>
       </c>
       <c r="G80" s="71" t="n">
-        <v>-0.03953660510795137</v>
+        <v>-0.05171141124499209</v>
       </c>
       <c r="H80" s="71" t="n">
         <v>0</v>
@@ -9602,79 +9664,79 @@
     <row r="81">
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — annual arrangement/renewal fee</t>
+          <t>Liquidity buffer held against deposits (LCR / HQLA)</t>
         </is>
       </c>
       <c r="C81" s="63" t="n">
-        <v>0.015</v>
+        <v>0.15</v>
       </c>
       <c r="D81" s="14" t="inlineStr">
         <is>
-          <t>% of limit</t>
+          <t>% of deposits</t>
         </is>
       </c>
       <c r="E81" s="71" t="n">
-        <v>0.03743043146690454</v>
+        <v>-0.04117347461329634</v>
       </c>
       <c r="F81" s="71" t="n">
-        <v>-0.01786433260297001</v>
+        <v>0.01965814063393465</v>
       </c>
       <c r="G81" s="71" t="n">
-        <v>0.03448390249733824</v>
+        <v>-0.03793463915464931</v>
       </c>
       <c r="H81" s="71" t="n">
-        <v>0.01786752451694579</v>
+        <v>-0.01965427696859545</v>
       </c>
     </row>
     <row r="82">
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t>Fraud &amp; payment losses (incl. APP reimbursement) per current account</t>
+          <t>Yield give-up on the liquidity buffer vs Bank Rate</t>
         </is>
       </c>
       <c r="C82" s="63" t="n">
-        <v>45</v>
+        <v>0.01</v>
       </c>
       <c r="D82" s="14" t="inlineStr">
         <is>
-          <t>£/BCA/yr</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E82" s="71" t="n">
-        <v>-0.02965245383102628</v>
+        <v>-0.04117347461329634</v>
       </c>
       <c r="F82" s="71" t="n">
-        <v>0.03095661825405067</v>
+        <v>0.01965814063393465</v>
       </c>
       <c r="G82" s="71" t="n">
-        <v>-0.02965245383120229</v>
+        <v>-0.03793463915464931</v>
       </c>
       <c r="H82" s="71" t="n">
-        <v>0</v>
+        <v>-0.01965427696859545</v>
       </c>
     </row>
     <row r="83">
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — probability of default</t>
+          <t>Unit-level platform &amp; processing cost</t>
         </is>
       </c>
       <c r="C83" s="63" t="n">
-        <v>0.022</v>
+        <v>60</v>
       </c>
       <c r="D83" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E83" s="71" t="n">
-        <v>-0.02857600386260983</v>
+        <v>-0.03953660510803504</v>
       </c>
       <c r="F83" s="71" t="n">
-        <v>0</v>
+        <v>0.0412754910054009</v>
       </c>
       <c r="G83" s="71" t="n">
-        <v>-0.02857600386254362</v>
+        <v>-0.03953660510795137</v>
       </c>
       <c r="H83" s="71" t="n">
         <v>0</v>
@@ -9683,52 +9745,52 @@
     <row r="84">
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — loss given default</t>
+          <t>Overdraft — annual arrangement/renewal fee</t>
         </is>
       </c>
       <c r="C84" s="63" t="n">
-        <v>0.35</v>
+        <v>0.015</v>
       </c>
       <c r="D84" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% of limit</t>
         </is>
       </c>
       <c r="E84" s="71" t="n">
-        <v>-0.02857600386260983</v>
+        <v>0.03743043146690454</v>
       </c>
       <c r="F84" s="71" t="n">
-        <v>0</v>
+        <v>-0.01786433260297001</v>
       </c>
       <c r="G84" s="71" t="n">
-        <v>-0.02857600386254362</v>
+        <v>0.03448390249733824</v>
       </c>
       <c r="H84" s="71" t="n">
-        <v>0</v>
+        <v>0.01786752451694579</v>
       </c>
     </row>
     <row r="85">
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t>Management span (staff per manager)</t>
+          <t>Fraud &amp; payment losses (incl. APP reimbursement) per current account</t>
         </is>
       </c>
       <c r="C85" s="63" t="n">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="D85" s="14" t="inlineStr">
         <is>
-          <t>staff</t>
+          <t>£/BCA/yr</t>
         </is>
       </c>
       <c r="E85" s="71" t="n">
-        <v>0.02728475739292511</v>
+        <v>-0.02965245383102628</v>
       </c>
       <c r="F85" s="71" t="n">
-        <v>-0.0284847865736678</v>
+        <v>0.03095661825405067</v>
       </c>
       <c r="G85" s="71" t="n">
-        <v>0.02728475739261982</v>
+        <v>-0.02965245383120229</v>
       </c>
       <c r="H85" s="71" t="n">
         <v>0</v>
@@ -9737,25 +9799,25 @@
     <row r="86">
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t>Team manager — salary</t>
+          <t>Asset finance — probability of default</t>
         </is>
       </c>
       <c r="C86" s="63" t="n">
-        <v>85000</v>
+        <v>0.022</v>
       </c>
       <c r="D86" s="14" t="inlineStr">
         <is>
-          <t>£/yr</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E86" s="71" t="n">
-        <v>-0.0257511658564655</v>
+        <v>-0.02857600386260983</v>
       </c>
       <c r="F86" s="71" t="n">
-        <v>0.02688374512136233</v>
+        <v>0</v>
       </c>
       <c r="G86" s="71" t="n">
-        <v>-0.02575116585676012</v>
+        <v>-0.02857600386254362</v>
       </c>
       <c r="H86" s="71" t="n">
         <v>0</v>
@@ -9764,25 +9826,25 @@
     <row r="87">
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t>Annual customer churn (replaced at steady state)</t>
+          <t>Asset finance — loss given default</t>
         </is>
       </c>
       <c r="C87" s="63" t="n">
-        <v>0.12</v>
+        <v>0.35</v>
       </c>
       <c r="D87" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E87" s="71" t="n">
-        <v>-0.02469126258220576</v>
+        <v>-0.02857600386260983</v>
       </c>
       <c r="F87" s="71" t="n">
-        <v>0.02577722553153486</v>
+        <v>0</v>
       </c>
       <c r="G87" s="71" t="n">
-        <v>-0.02469126258230462</v>
+        <v>-0.02857600386254362</v>
       </c>
       <c r="H87" s="71" t="n">
         <v>0</v>
@@ -9791,25 +9853,25 @@
     <row r="88">
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t>Employment on-costs (NI, pension, benefits)</t>
+          <t>Management span (staff per manager)</t>
         </is>
       </c>
       <c r="C88" s="63" t="n">
-        <v>0.15</v>
+        <v>8</v>
       </c>
       <c r="D88" s="14" t="inlineStr">
         <is>
-          <t>% of salary</t>
+          <t>staff</t>
         </is>
       </c>
       <c r="E88" s="71" t="n">
-        <v>-0.02057660219051082</v>
+        <v>0.02728475739292511</v>
       </c>
       <c r="F88" s="71" t="n">
-        <v>0.02148159550679803</v>
+        <v>-0.0284847865736678</v>
       </c>
       <c r="G88" s="71" t="n">
-        <v>-0.02057660219063057</v>
+        <v>0.02728475739261982</v>
       </c>
       <c r="H88" s="71" t="n">
         <v>0</v>
@@ -9818,52 +9880,52 @@
     <row r="89">
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t>Operational-risk RWA multiple of gross income</t>
+          <t>Team manager — salary</t>
         </is>
       </c>
       <c r="C89" s="63" t="n">
-        <v>1.875</v>
+        <v>85000</v>
       </c>
       <c r="D89" s="14" t="inlineStr">
         <is>
-          <t>x revenue</t>
+          <t>£/yr</t>
         </is>
       </c>
       <c r="E89" s="71" t="n">
-        <v>0.01940217969118421</v>
+        <v>-0.0257511658564655</v>
       </c>
       <c r="F89" s="71" t="n">
-        <v>-0.009260828777932256</v>
+        <v>0.02688374512136233</v>
       </c>
       <c r="G89" s="71" t="n">
-        <v>-0.1370151321223097</v>
+        <v>-0.02575116585676012</v>
       </c>
       <c r="H89" s="71" t="n">
-        <v>0.009261686486871161</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90">
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t>Share of lending balances held by RM-managed customers</t>
+          <t>Annual customer churn (replaced at steady state)</t>
         </is>
       </c>
       <c r="C90" s="63" t="n">
-        <v>0.6</v>
+        <v>0.12</v>
       </c>
       <c r="D90" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E90" s="71" t="n">
-        <v>0.01833005970171241</v>
+        <v>-0.02469126258220576</v>
       </c>
       <c r="F90" s="71" t="n">
-        <v>0</v>
+        <v>0.02577722553153486</v>
       </c>
       <c r="G90" s="71" t="n">
-        <v>0.0183300597013768</v>
+        <v>-0.02469126258230462</v>
       </c>
       <c r="H90" s="71" t="n">
         <v>0</v>
@@ -9872,25 +9934,25 @@
     <row r="91">
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t>Stewardship effect: relative PD reduction on RM-covered balances</t>
+          <t>Employment on-costs (NI, pension, benefits)</t>
         </is>
       </c>
       <c r="C91" s="63" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="D91" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% of salary</t>
         </is>
       </c>
       <c r="E91" s="71" t="n">
-        <v>0.01833005970171241</v>
+        <v>-0.02057660219051082</v>
       </c>
       <c r="F91" s="71" t="n">
-        <v>0</v>
+        <v>0.02148159550679803</v>
       </c>
       <c r="G91" s="71" t="n">
-        <v>0.0183300597013768</v>
+        <v>-0.02057660219063057</v>
       </c>
       <c r="H91" s="71" t="n">
         <v>0</v>
@@ -9899,38 +9961,38 @@
     <row r="92">
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t>Churn replacement — acquisition marketing per new customer won</t>
+          <t>Operational-risk RWA multiple of gross income</t>
         </is>
       </c>
       <c r="C92" s="63" t="n">
-        <v>240</v>
+        <v>1.875</v>
       </c>
       <c r="D92" s="14" t="inlineStr">
         <is>
-          <t>£/new customer</t>
+          <t>x revenue</t>
         </is>
       </c>
       <c r="E92" s="71" t="n">
-        <v>-0.01826591155990401</v>
+        <v>0.01940217969118421</v>
       </c>
       <c r="F92" s="71" t="n">
-        <v>0.01906927684454543</v>
+        <v>-0.009260828777932256</v>
       </c>
       <c r="G92" s="71" t="n">
-        <v>-0.01826591156004862</v>
+        <v>-0.1370151321223097</v>
       </c>
       <c r="H92" s="71" t="n">
-        <v>0</v>
+        <v>0.009261686486871161</v>
       </c>
     </row>
     <row r="93">
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — risk weight</t>
+          <t>Share of lending balances held by RM-managed customers</t>
         </is>
       </c>
       <c r="C93" s="63" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="D93" s="14" t="inlineStr">
         <is>
@@ -9938,67 +10000,67 @@
         </is>
       </c>
       <c r="E93" s="71" t="n">
-        <v>0.01771239908840788</v>
+        <v>0.01833005970171241</v>
       </c>
       <c r="F93" s="71" t="n">
-        <v>-0.008454350017280498</v>
+        <v>0</v>
       </c>
       <c r="G93" s="71" t="n">
-        <v>-0.125099206722287</v>
+        <v>0.0183300597013768</v>
       </c>
       <c r="H93" s="71" t="n">
-        <v>0.008455064837974957</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t>Card — interest rate on revolving balances</t>
+          <t>Stewardship effect: relative PD reduction on RM-covered balances</t>
         </is>
       </c>
       <c r="C94" s="63" t="n">
-        <v>0.159</v>
+        <v>0.2</v>
       </c>
       <c r="D94" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E94" s="71" t="n">
-        <v>0.01587050294203331</v>
+        <v>0.01833005970171241</v>
       </c>
       <c r="F94" s="71" t="n">
-        <v>-0.007575256506550518</v>
+        <v>0</v>
       </c>
       <c r="G94" s="71" t="n">
-        <v>0.01462142272077909</v>
+        <v>0.0183300597013768</v>
       </c>
       <c r="H94" s="71" t="n">
-        <v>0.007575830395216416</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95">
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t>Service &amp; operations staff — salary</t>
+          <t>Churn replacement — acquisition marketing per new customer won</t>
         </is>
       </c>
       <c r="C95" s="63" t="n">
-        <v>32000</v>
+        <v>240</v>
       </c>
       <c r="D95" s="14" t="inlineStr">
         <is>
-          <t>£/yr</t>
+          <t>£/new customer</t>
         </is>
       </c>
       <c r="E95" s="71" t="n">
-        <v>-0.01564284608034933</v>
+        <v>-0.01826591155990401</v>
       </c>
       <c r="F95" s="71" t="n">
-        <v>0.01633084456626305</v>
+        <v>0.01906927684454543</v>
       </c>
       <c r="G95" s="71" t="n">
-        <v>-0.01564284608081514</v>
+        <v>-0.01826591156004862</v>
       </c>
       <c r="H95" s="71" t="n">
         <v>0</v>
@@ -10007,79 +10069,79 @@
     <row r="96">
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — probability of default</t>
+          <t>Asset finance — risk weight</t>
         </is>
       </c>
       <c r="C96" s="63" t="n">
-        <v>0.026</v>
+        <v>0.8</v>
       </c>
       <c r="D96" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E96" s="71" t="n">
-        <v>-0.01399299296284985</v>
+        <v>0.01771239908840788</v>
       </c>
       <c r="F96" s="71" t="n">
-        <v>0</v>
+        <v>-0.008454350017280498</v>
       </c>
       <c r="G96" s="71" t="n">
-        <v>-0.01399299296281295</v>
+        <v>-0.125099206722287</v>
       </c>
       <c r="H96" s="71" t="n">
-        <v>0</v>
+        <v>0.008455064837974957</v>
       </c>
     </row>
     <row r="97">
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — loss given default</t>
+          <t>Card — interest rate on revolving balances</t>
         </is>
       </c>
       <c r="C97" s="63" t="n">
-        <v>0.55</v>
+        <v>0.159</v>
       </c>
       <c r="D97" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E97" s="71" t="n">
-        <v>-0.01399299296284985</v>
+        <v>0.01587050294203331</v>
       </c>
       <c r="F97" s="71" t="n">
-        <v>0</v>
+        <v>-0.007575256506550518</v>
       </c>
       <c r="G97" s="71" t="n">
-        <v>-0.01399299296281295</v>
+        <v>0.01462142272077909</v>
       </c>
       <c r="H97" s="71" t="n">
-        <v>0</v>
+        <v>0.007575830395216416</v>
       </c>
     </row>
     <row r="98">
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t>Term loan underwriting &amp; completion</t>
+          <t>Service &amp; operations staff — salary</t>
         </is>
       </c>
       <c r="C98" s="63" t="n">
-        <v>14</v>
+        <v>32000</v>
       </c>
       <c r="D98" s="14" t="inlineStr">
         <is>
-          <t>hrs/new loan</t>
+          <t>£/yr</t>
         </is>
       </c>
       <c r="E98" s="71" t="n">
-        <v>-0.01370322847785298</v>
+        <v>-0.01564284608034933</v>
       </c>
       <c r="F98" s="71" t="n">
-        <v>0.01430591934339043</v>
+        <v>0.01633084456626305</v>
       </c>
       <c r="G98" s="71" t="n">
-        <v>-0.0137032284779602</v>
+        <v>-0.01564284608081514</v>
       </c>
       <c r="H98" s="71" t="n">
         <v>0</v>
@@ -10088,7 +10150,7 @@
     <row r="99">
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — probability of default</t>
+          <t>Overdraft — probability of default</t>
         </is>
       </c>
       <c r="C99" s="63" t="n">
@@ -10100,13 +10162,13 @@
         </is>
       </c>
       <c r="E99" s="71" t="n">
-        <v>-0.01356896287307272</v>
+        <v>-0.01399299296284985</v>
       </c>
       <c r="F99" s="71" t="n">
         <v>0</v>
       </c>
       <c r="G99" s="71" t="n">
-        <v>-0.01356896287333288</v>
+        <v>-0.01399299296281295</v>
       </c>
       <c r="H99" s="71" t="n">
         <v>0</v>
@@ -10115,11 +10177,11 @@
     <row r="100">
       <c r="B100" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — loss given default</t>
+          <t>Overdraft — loss given default</t>
         </is>
       </c>
       <c r="C100" s="63" t="n">
-        <v>0.2</v>
+        <v>0.55</v>
       </c>
       <c r="D100" s="14" t="inlineStr">
         <is>
@@ -10127,13 +10189,13 @@
         </is>
       </c>
       <c r="E100" s="71" t="n">
-        <v>-0.01356896287307272</v>
+        <v>-0.01399299296284985</v>
       </c>
       <c r="F100" s="71" t="n">
         <v>0</v>
       </c>
       <c r="G100" s="71" t="n">
-        <v>-0.01356896287333288</v>
+        <v>-0.01399299296281295</v>
       </c>
       <c r="H100" s="71" t="n">
         <v>0</v>
@@ -10142,25 +10204,25 @@
     <row r="101">
       <c r="B101" s="10" t="inlineStr">
         <is>
-          <t>Premises &amp; facilities per unit FTE</t>
+          <t>Term loan underwriting &amp; completion</t>
         </is>
       </c>
       <c r="C101" s="63" t="n">
-        <v>6000</v>
+        <v>14</v>
       </c>
       <c r="D101" s="14" t="inlineStr">
         <is>
-          <t>£/FTE/yr</t>
+          <t>hrs/new loan</t>
         </is>
       </c>
       <c r="E101" s="71" t="n">
-        <v>-0.01354829332592148</v>
+        <v>-0.01370322847785298</v>
       </c>
       <c r="F101" s="71" t="n">
-        <v>0.01414416988493427</v>
+        <v>0.01430591934339043</v>
       </c>
       <c r="G101" s="71" t="n">
-        <v>-0.01354829332627234</v>
+        <v>-0.0137032284779602</v>
       </c>
       <c r="H101" s="71" t="n">
         <v>0</v>
@@ -10169,25 +10231,25 @@
     <row r="102">
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t>BCA servicing (queries, payments support)</t>
+          <t>Invoice finance — probability of default</t>
         </is>
       </c>
       <c r="C102" s="63" t="n">
-        <v>0.6</v>
+        <v>0.026</v>
       </c>
       <c r="D102" s="14" t="inlineStr">
         <is>
-          <t>hrs/account/yr</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E102" s="71" t="n">
-        <v>-0.01335137874766737</v>
+        <v>-0.01356896287307272</v>
       </c>
       <c r="F102" s="71" t="n">
-        <v>0.01393859467455354</v>
+        <v>0</v>
       </c>
       <c r="G102" s="71" t="n">
-        <v>-0.01335137874769045</v>
+        <v>-0.01356896287333288</v>
       </c>
       <c r="H102" s="71" t="n">
         <v>0</v>
@@ -10196,25 +10258,25 @@
     <row r="103">
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t>Overdraft annual review &amp; renewal</t>
+          <t>Invoice finance — loss given default</t>
         </is>
       </c>
       <c r="C103" s="63" t="n">
-        <v>1.5</v>
+        <v>0.2</v>
       </c>
       <c r="D103" s="14" t="inlineStr">
         <is>
-          <t>hrs/facility/yr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E103" s="71" t="n">
-        <v>-0.01223502542667563</v>
+        <v>-0.01356896287307272</v>
       </c>
       <c r="F103" s="71" t="n">
-        <v>0.01277314227084876</v>
+        <v>0</v>
       </c>
       <c r="G103" s="71" t="n">
-        <v>-0.01223502542703396</v>
+        <v>-0.01356896287333288</v>
       </c>
       <c r="H103" s="71" t="n">
         <v>0</v>
@@ -10223,25 +10285,25 @@
     <row r="104">
       <c r="B104" s="10" t="inlineStr">
         <is>
-          <t>Term loan annual review</t>
+          <t>Premises &amp; facilities per unit FTE</t>
         </is>
       </c>
       <c r="C104" s="63" t="n">
-        <v>3</v>
+        <v>6000</v>
       </c>
       <c r="D104" s="14" t="inlineStr">
         <is>
-          <t>hrs/loan/yr</t>
+          <t>£/FTE/yr</t>
         </is>
       </c>
       <c r="E104" s="71" t="n">
-        <v>-0.01174562440962334</v>
+        <v>-0.01354829332592148</v>
       </c>
       <c r="F104" s="71" t="n">
-        <v>0.01226221658007843</v>
+        <v>0.01414416988493427</v>
       </c>
       <c r="G104" s="71" t="n">
-        <v>-0.01174562440975294</v>
+        <v>-0.01354829332627234</v>
       </c>
       <c r="H104" s="71" t="n">
         <v>0</v>
@@ -10250,25 +10312,25 @@
     <row r="105">
       <c r="B105" s="10" t="inlineStr">
         <is>
-          <t>FSCS deposit-protection levy</t>
+          <t>BCA servicing (queries, payments support)</t>
         </is>
       </c>
       <c r="C105" s="63" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.6</v>
       </c>
       <c r="D105" s="14" t="inlineStr">
         <is>
-          <t>% of protected deposits</t>
+          <t>hrs/account/yr</t>
         </is>
       </c>
       <c r="E105" s="71" t="n">
-        <v>-0.009785309764238673</v>
+        <v>-0.01335137874766737</v>
       </c>
       <c r="F105" s="71" t="n">
-        <v>0.01021568402375696</v>
+        <v>0.01393859467455354</v>
       </c>
       <c r="G105" s="71" t="n">
-        <v>-0.009785309764105748</v>
+        <v>-0.01335137874769045</v>
       </c>
       <c r="H105" s="71" t="n">
         <v>0</v>
@@ -10277,25 +10339,25 @@
     <row r="106">
       <c r="B106" s="10" t="inlineStr">
         <is>
-          <t>Share of deposit balances that are FSCS-protected</t>
+          <t>Overdraft annual review &amp; renewal</t>
         </is>
       </c>
       <c r="C106" s="63" t="n">
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="D106" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>hrs/facility/yr</t>
         </is>
       </c>
       <c r="E106" s="71" t="n">
-        <v>-0.009785309764238673</v>
+        <v>-0.01223502542667563</v>
       </c>
       <c r="F106" s="71" t="n">
-        <v>0.01021568402375696</v>
+        <v>0.01277314227084876</v>
       </c>
       <c r="G106" s="71" t="n">
-        <v>-0.009785309764105748</v>
+        <v>-0.01223502542703396</v>
       </c>
       <c r="H106" s="71" t="n">
         <v>0</v>
@@ -10304,81 +10366,162 @@
     <row r="107">
       <c r="B107" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — risk weight</t>
+          <t>Term loan annual review</t>
         </is>
       </c>
       <c r="C107" s="63" t="n">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="D107" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>hrs/loan/yr</t>
         </is>
       </c>
       <c r="E107" s="71" t="n">
-        <v>0.009340522956773279</v>
+        <v>-0.01174562440962334</v>
       </c>
       <c r="F107" s="71" t="n">
-        <v>-0.00445852680457372</v>
+        <v>0.01226221658007843</v>
       </c>
       <c r="G107" s="71" t="n">
-        <v>-0.06601483744602295</v>
+        <v>-0.01174562440975294</v>
       </c>
       <c r="H107" s="71" t="n">
-        <v>0.004458725598148796</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108">
       <c r="B108" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — risk weight</t>
+          <t>FSCS deposit-protection levy</t>
         </is>
       </c>
       <c r="C108" s="63" t="n">
-        <v>0.75</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="D108" s="14" t="inlineStr">
         <is>
-          <t>% of drawn</t>
+          <t>% of protected deposits</t>
         </is>
       </c>
       <c r="E108" s="71" t="n">
-        <v>0.004378370135987474</v>
+        <v>-0.009785309764238673</v>
       </c>
       <c r="F108" s="71" t="n">
-        <v>-0.002089983942857775</v>
+        <v>0.01021568402375696</v>
       </c>
       <c r="G108" s="71" t="n">
-        <v>-0.03095684670595658</v>
+        <v>-0.009785309764105748</v>
       </c>
       <c r="H108" s="71" t="n">
-        <v>0.002090027624132248</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109">
       <c r="B109" s="10" t="inlineStr">
         <is>
+          <t>Share of deposit balances that are FSCS-protected</t>
+        </is>
+      </c>
+      <c r="C109" s="63" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D109" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E109" s="71" t="n">
+        <v>-0.009785309764238673</v>
+      </c>
+      <c r="F109" s="71" t="n">
+        <v>0.01021568402375696</v>
+      </c>
+      <c r="G109" s="71" t="n">
+        <v>-0.009785309764105748</v>
+      </c>
+      <c r="H109" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" s="10" t="inlineStr">
+        <is>
+          <t>Invoice finance — risk weight</t>
+        </is>
+      </c>
+      <c r="C110" s="63" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D110" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E110" s="71" t="n">
+        <v>0.009340522956773279</v>
+      </c>
+      <c r="F110" s="71" t="n">
+        <v>-0.00445852680457372</v>
+      </c>
+      <c r="G110" s="71" t="n">
+        <v>-0.06601483744602295</v>
+      </c>
+      <c r="H110" s="71" t="n">
+        <v>0.004458725598148796</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="B111" s="10" t="inlineStr">
+        <is>
+          <t>Overdraft — risk weight</t>
+        </is>
+      </c>
+      <c r="C111" s="63" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D111" s="14" t="inlineStr">
+        <is>
+          <t>% of drawn</t>
+        </is>
+      </c>
+      <c r="E111" s="71" t="n">
+        <v>0.004378370135987474</v>
+      </c>
+      <c r="F111" s="71" t="n">
+        <v>-0.002089983942857775</v>
+      </c>
+      <c r="G111" s="71" t="n">
+        <v>-0.03095684670595658</v>
+      </c>
+      <c r="H111" s="71" t="n">
+        <v>0.002090027624132248</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" s="10" t="inlineStr">
+        <is>
           <t>Tax rate (corporation tax + bank surcharge)</t>
         </is>
       </c>
-      <c r="C109" s="63" t="n">
+      <c r="C112" s="63" t="n">
         <v>0.28</v>
       </c>
-      <c r="D109" s="14" t="inlineStr">
+      <c r="D112" s="14" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E109" s="71" t="n">
+      <c r="E112" s="71" t="n">
         <v>0</v>
       </c>
-      <c r="F109" s="71" t="n">
+      <c r="F112" s="71" t="n">
         <v>0</v>
       </c>
-      <c r="G109" s="71" t="n">
+      <c r="G112" s="71" t="n">
         <v>-0.388888888889195</v>
       </c>
-      <c r="H109" s="71" t="n">
+      <c r="H112" s="71" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
v2.0: trajectory tab — the ramp from nothing to steady state
Peak funding £8.3m, payback year 7, NPV at 12% about -£106k. The snapshot reports only
the final year and calls the business comfortably good. A profitable steady state is not
the same thing as a worthwhile investment.
</commit_message>
<xml_diff>
--- a/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
+++ b/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
@@ -22,6 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. Flow Register" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. Elasticities" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. Backtest" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12. Trajectory" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -589,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B50"/>
+  <dimension ref="B1:B52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -606,7 +607,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MODEL VERSION: v1.9 · 22 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
+          <t>MODEL VERSION: v2.0 · 22 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
         </is>
       </c>
     </row>
@@ -620,278 +621,292 @@
     <row r="5" ht="52" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>• v1.9 (22 Aug 2026) — competitive response. Every scenario assumed rivals stand still, which flatters both directions at once: raising a price looks safer than it is, and cutting one looks better than it is. A firm with market share s moving alone faces roughly the industry elasticity divided by s; moving in concert it faces only the industry elasticity. This model's penetration IS market share (16%), so moving alone multiplies the demand response by 6.25x. Tab 10 now inverts every break-even into the industry elasticity the move survives in each regime. The headline lever moves with it: raising the term loan rate survives an industry elasticity of 2.91 in concert but only 0.47 alone — marginal rather than comfortable.</t>
+          <t>• v2.0 (22 Aug 2026) — trajectory. Every other tab describes a steady state; tab 12 describes getting there. Time stays OUT of the base model deliberately — the steady-state identities are what let the whole chain work without a forecast — so the trajectory runs the same model at a series of maturity states and reads the result as a cash flow. Building one regional centre from nothing needs £8.3m of funding at its deepest point, repays in year seven, and has an NPV at the model's own 12% cost of equity of about MINUS £106,000. The snapshot alone reports only the final year and calls the business comfortably good. Both are true: a profitable steady state is not the same thing as a worthwhile investment.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="52" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>• v1.8 (22 Aug 2026) — break-even demand elasticity on tab 10. The elasticity table ranked the term loan customer rate as the largest driver of profit at +1.25, which was an artefact: nothing in the model responds to price, so raising any price always looked accretive. Tab 10 now leads with the demand elasticity at which raising each price stops paying. The reordering matters — the card fee breaks even at 0.06 and the current-account fee at 0.13, so both are fragile to almost any customer response, while the loan rate holds to 2.91. The hidden assumption being replaced is zero, which is the least defensible value available.</t>
+          <t>• v1.9 (22 Aug 2026) — competitive response. Every scenario assumed rivals stand still, which flatters both directions at once: raising a price looks safer than it is, and cutting one looks better than it is. A firm with market share s moving alone faces roughly the industry elasticity divided by s; moving in concert it faces only the industry elasticity. This model's penetration IS market share (16%), so moving alone multiplies the demand response by 6.25x. Tab 10 now inverts every break-even into the industry elasticity the move survives in each regime. The headline lever moves with it: raising the term loan rate survives an industry elasticity of 2.91 in concert but only 0.47 alone — marginal rather than comfortable.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>• v1.7 (22 Aug 2026) — operational leverage. Every cost line in the model scaled linearly with its driver, which forces a cost elasticity of exactly 1.0 and makes cost per customer flat at every scale. Allica Bank's own accounts put that elasticity at 0.808 across 2022-23 and 0.622 across 2023-24 — cost rises materially more slowly than the book. Inputs section O adds a cost scale elasticity and the customer count the per-customer rates are calibrated at; the head-office pools, the platform line and change-the-bank now scale by it. Default 1.0 reproduces v1.6 exactly. Tab 11 adds the out-of-sample test that measured it.</t>
+          <t>• v1.8 (22 Aug 2026) — break-even demand elasticity on tab 10. The elasticity table ranked the term loan customer rate as the largest driver of profit at +1.25, which was an artefact: nothing in the model responds to price, so raising any price always looked accretive. Tab 10 now leads with the demand elasticity at which raising each price stops paying. The reordering matters — the card fee breaks even at 0.06 and the current-account fee at 0.13, so both are fragile to almost any customer response, while the loan rate holds to 2.91. The hidden assumption being replaced is zero, which is the least defensible value available.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>• v1.6 (22 Aug 2026) — validation and drivers. Tab 10 ELASTICITIES: every input bumped +1% and the workbook recalculated, giving the % change in PBT, cost:income, RoE and income. Only one input has an elasticity above 1 on profit — the term loan customer rate, at +1.25; reachable market and penetration are exactly +1.00 (pure scale); nothing else exceeds 0.53. Tab 11 BACKTEST against Allica Bank FY2023 audited accounts: the revenue engine reproduces a real bank's operating income to within 8%, and the cost engine under-predicts by 7x. Diagnosis: head-office cost was modelled purely per customer, which is a scale assumption disguised as a driver. Inputs section N therefore adds a fixed component to each head-office pool, defaulting to 0 so v1.5 results are unchanged.</t>
+          <t>• v1.7 (22 Aug 2026) — operational leverage. Every cost line in the model scaled linearly with its driver, which forces a cost elasticity of exactly 1.0 and makes cost per customer flat at every scale. Allica Bank's own accounts put that elasticity at 0.808 across 2022-23 and 0.622 across 2023-24 — cost rises materially more slowly than the book. Inputs section O adds a cost scale elasticity and the customer count the per-customer rates are calibrated at; the head-office pools, the platform line and change-the-bank now scale by it. Default 1.0 reproduces v1.6 exactly. Tab 11 adds the out-of-sample test that measured it.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="52" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>• v1.5 (22 Aug 2026) — PROCESS LAYER on the Step 2 tabs. Tab 3 gains process columns M-T (process type, yield, attempts, automation, best-in-class intensity and yield, benchmark source, £ gap) and a HEAD-OFFICE PROCESS REGISTER of 22 processes already named in the tab 9 operational model but never costed. Yield inflates ATTEMPTS and never deflates outcomes — that is what stops it double-counting with the CEP layer's demand-side conversion. Head-office costs are carved OUT of the pools, so naming a process moves money from unallocated to attributed and the total never changes. New sheet 3b indexes every process to the numbers it moves, and imputes what each would have to become to hit a target cost:income. Mode OFF (default) = results identical to v1.4.</t>
+          <t>• v1.6 (22 Aug 2026) — validation and drivers. Tab 10 ELASTICITIES: every input bumped +1% and the workbook recalculated, giving the % change in PBT, cost:income, RoE and income. Only one input has an elasticity above 1 on profit — the term loan customer rate, at +1.25; reachable market and penetration are exactly +1.00 (pure scale); nothing else exceeds 0.53. Tab 11 BACKTEST against Allica Bank FY2023 audited accounts: the revenue engine reproduces a real bank's operating income to within 8%, and the cost engine under-predicts by 7x. Diagnosis: head-office cost was modelled purely per customer, which is a scale assumption disguised as a driver. Inputs section N therefore adds a fixed component to each head-office pool, defaulting to 0 so v1.5 results are unchanged.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="52" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
+          <t>• v1.5 (22 Aug 2026) — PROCESS LAYER on the Step 2 tabs. Tab 3 gains process columns M-T (process type, yield, attempts, automation, best-in-class intensity and yield, benchmark source, £ gap) and a HEAD-OFFICE PROCESS REGISTER of 22 processes already named in the tab 9 operational model but never costed. Yield inflates ATTEMPTS and never deflates outcomes — that is what stops it double-counting with the CEP layer's demand-side conversion. Head-office costs are carved OUT of the pools, so naming a process moves money from unallocated to attributed and the total never changes. New sheet 3b indexes every process to the numbers it moves, and imputes what each would have to become to hit a target cost:income. Mode OFF (default) = results identical to v1.4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
           <t>• v1.4 (22 Aug 2026) — CEP DEMAND LAYER. New sheet 1b derives the nine product penetrations and the customer count instead of asserting them: penetration = (lambda*c x L) / (1 + lambda*c x L), where lambda*c = category-entry-point events x presence x conversion and L is the holding life. Little's Law run forwards; no time axis is added and the model stays a steady-state snapshot. Ships deliberately EMPTY — every event/presence/conversion cell is blank and carries the cohort query that fills it, and any unpopulated product falls back to its hardcoded penetration. Mode OFF (default) = results identical to v1.3; CALIBRATE reports the won-event rate implied by today's assumptions and changes nothing.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
+    <row r="12" ht="40" customHeight="1">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>• v1.3 (21 Aug 2026) — churn replacement is a costed activity end-to-end: new input cac_new (£240 acquisition marketing per new customer won, carved out of the corporate-centre pool — hq_oh £250→£222); driver-linked on tab 4, attributed to the current account (gateway product) on tab 6; 'value of preventing one churn' memo added to tab 6. Raising the churn input now inflates demand-generation cost, not just processing. Central PBT shifts &lt;£1k/unit (carve-out rounding).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
+          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="B15" s="4" t="inlineStr">
         <is>
+          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
           <t>• v1.0 (10 Aug 2026) — first published version: 9 tabs + flow register, FTP with liquidity/behavioural terms, fraud/FSCS/change-the-bank lines, segment-pod LMUs, bridge check.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="3" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>What this is</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="39" customHeight="1">
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="39" customHeight="1">
       <c r="B19" s="4" t="inlineStr">
         <is>
+          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="39" customHeight="1">
+      <c r="B20" s="4" t="inlineStr">
+        <is>
           <t>• It follows the Simanis / IVE bottom-up methodology ('Running the Right Numbers'): model the last-mile operating unit, derive every cost from activity drivers (transaction intensity I and customer load L), build whole costs, and check the price/margin covers them including a competitive return on capital.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="3" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>What period this models</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="B22" s="4" t="inlineStr">
+    <row r="23" ht="26" customHeight="1">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>• One representative operating year at steady state. Balances are annual averages; rates and volumes are annual. There is no time axis, no ramp and no vintage cohorts — the model is a snapshot, not a forecast.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="78" customHeight="1">
-      <c r="B23" s="4" t="inlineStr">
+    <row r="24" ht="78" customHeight="1">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>• The book is stationary but not free to hold flat: customers churn (12% p.a. input) and the model costs their replacement end-to-end — acquisition marketing per new customer won (cac_new, carved from the corporate-centre pool), onboarding hours, KYC per new customer and RM origination effort are all driver-linked (Simanis: at-scale operations include 'replacement of customer churn'). Only residual brand &amp; joint marketing remains pool-costed. The 'value of preventing one churn' memo on tab 6 prices retention: contribution annuity over remaining relationship life + the avoided replacement cost.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="26" customHeight="1">
-      <c r="B24" s="4" t="inlineStr">
+    <row r="25" ht="26" customHeight="1">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>• The capital charge (cost of equity on allocated capital) is the incumbent analogue of Simanis's start-up-cost amortisation: capital earns its required return inside the steady-state P&amp;L.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="52" customHeight="1">
-      <c r="B25" s="4" t="inlineStr">
+    <row r="26" ht="52" customHeight="1">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>• Out of scope by design: transition paths. The cost and cash shape of moving between steady states — digital migration, maturity glide, behaviour-change programmes and their CAC/incentives — belongs in a scenario layer built ON TOP of this base (comparative statics between two runs of this model, plus a separate transition-cost estimate). The base model never carries scenario logic.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="3" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>How the tabs map to the methodology</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="B28" s="4" t="inlineStr">
+    <row r="29" ht="24" customHeight="1">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>• Inputs — every assumption in one place, with sources. Edit blue cells; yellow cells are the biggest levers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="26" customHeight="1">
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="26" customHeight="1">
       <c r="B30" s="4" t="inlineStr">
         <is>
+          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="26" customHeight="1">
+      <c r="B31" s="4" t="inlineStr">
+        <is>
           <t>• 2. Revenues — unit revenue per product: interest margins measured against internal funds transfer prices (Bank Rate for floating, + premium for term), plus fees.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="39" customHeight="1">
-      <c r="B31" s="4" t="inlineStr">
+    <row r="32" ht="39" customHeight="1">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>• 3. HR &amp; Activity — Step 2: every FTE derived from activity drivers (hours per onboarding, review, renewal…) — nothing is assumed as headcount. From v1.5 this tab is also the PROCESS REGISTER (columns M-T), with the head-office process register below it.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="26" customHeight="1">
-      <c r="B32" s="4" t="inlineStr">
+    <row r="33" ht="26" customHeight="1">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>• 1b. Demand &amp; CEPs — the demand layer (v1.4). Penetration is derived, not assumed. Mode cell on Inputs section L: OFF reproduces v1.3, CALIBRATE reports the implied event rates, LIVE derives.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="39" customHeight="1">
-      <c r="B33" s="4" t="inlineStr">
+    <row r="34" ht="26" customHeight="1">
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>• 12. Trajectory — the ramp from nothing to steady state: cash flow, peak funding, payback and NPV. Time lives here and nowhere else, as a wrapper around the snapshot rather than inside it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="39" customHeight="1">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>• 3b. Process Index — derived view, no assumptions. Every process with its flow, product, owner, the numbers it moves, its cost and its gap to best in class, plus a ranked worst-gap list and the top-down benchmark imputation. Answers 'which process do I improve to move this number?'</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="52" customHeight="1">
-      <c r="B34" s="4" t="inlineStr">
+    <row r="36" ht="52" customHeight="1">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>• 4. Running Costs — Step 2 (cont.): direct running costs plus the share of head-office costs. The attribution memo reads the tab 3 process register and reports the share of the cost base with a named process owner — the model's own assessment of how much of its cost it actually understands. What remains in UNALLOCATED JOINT COSTS is cost with no process to improve.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="26" customHeight="1">
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>• 5. Risk &amp; Capital — Step 3: expected credit losses (PD × LGD), risk-weighted assets, allocated equity, and the required return on it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="91" customHeight="1">
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>• 6. Unit Economics — Steps 4–5: per-product unit costs and revenues on an activity-based costing basis, taken exactly as far as causality runs (the source methodology's own rule: link costs to customers and transactions 'whenever possible'). Costs with real drivers — servicing hours, RM effort per origination, staff-time-driven supervision, per-account and per-facility infrastructure — are attributed to products; genuinely joint costs (brand, exec, finance, platform build) are NOT forced into products but held as an unallocated hurdle that total contribution must clear, with a full-absorption memo showing the source doc's simple-division treatment. Product decisions should run on contribution.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="26" customHeight="1">
       <c r="B37" s="4" t="inlineStr">
         <is>
+          <t>• 5. Risk &amp; Capital — Step 3: expected credit losses (PD × LGD), risk-weighted assets, allocated equity, and the required return on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="91" customHeight="1">
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>• 6. Unit Economics — Steps 4–5: per-product unit costs and revenues on an activity-based costing basis, taken exactly as far as causality runs (the source methodology's own rule: link costs to customers and transactions 'whenever possible'). Costs with real drivers — servicing hours, RM effort per origination, staff-time-driven supervision, per-account and per-facility infrastructure — are attributed to products; genuinely joint costs (brand, exec, finance, platform build) are NOT forced into products but held as an unallocated hurdle that total contribution must clear, with a full-absorption memo showing the source doc's simple-division treatment. Product decisions should run on contribution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="26" customHeight="1">
+      <c r="B39" s="4" t="inlineStr">
+        <is>
           <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="26" customHeight="1">
-      <c r="B38" s="4" t="inlineStr">
+    <row r="40" ht="26" customHeight="1">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>• 8. Org Structure — the whole-bank organisation implied by the model: front-line FTEs from activity drivers × number of centres, head-office FTEs backed out of the per-customer head-office cost allocations.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="52" customHeight="1">
-      <c r="B39" s="4" t="inlineStr">
+    <row r="41" ht="52" customHeight="1">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>• 9. Flow Register — one row per flow on the operational model map: component type (CP/WP/PP/PartP), core/support/enabling, direction, digital/physical medium, the direct/administrative/managerial roles accountable, and the BIAN service domains. Ends with a BIAN completeness checklist. This is where the map, the ARM and BIAN reconcile.</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="B41" s="3" t="inlineStr">
+    <row r="43">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>Colour legend</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="26" customHeight="1">
-      <c r="B42" s="4" t="inlineStr">
+    <row r="44" ht="26" customHeight="1">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>• Blue = hardcoded input (edit these) · Yellow fill = key assumption / sensitivity lever · Black = formula · Green = link to another sheet.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="3" t="inlineStr">
+    <row r="46">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>Reading the results</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="52" customHeight="1">
-      <c r="B45" s="4" t="inlineStr">
+    <row r="47" ht="52" customHeight="1">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>• Deposit products earn the spread between the transfer price and the rate paid; lending earns the customer rate minus the transfer price minus expected losses. Capital-heavy, labour-heavy products (term loans) can show thin or negative economic profit — consistent with the Bank of England's 2026 finding that SME lending earns the lowest product-level returns, driven by impairments and per-borrower servicing costs.</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="39" customHeight="1">
-      <c r="B46" s="4" t="inlineStr">
+    <row r="48" ht="39" customHeight="1">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>• Use the cost-driver table on the P&amp;L tab to find leverage points, then trace them to transaction intensity (I) or customer load (L) assumptions on the Inputs tab — e.g. automating underwriting hours, raising RM portfolio size, or shifting servicing to digital.</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="B48" s="3" t="inlineStr">
+    <row r="50">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Caveats</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="39" customHeight="1">
-      <c r="B49" s="4" t="inlineStr">
+    <row r="51" ht="39" customHeight="1">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>• Benchmarks are as of August 2026 (Bank Rate 3.75%; BoE effective new SME loan rate ~6.3%; commercial interchange 1.65–1.90%; invoice finance discount base+1–3%). Items marked 'Assumption' are illustrative and should be replaced with your own data.</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="65" customHeight="1">
-      <c r="B50" s="4" t="inlineStr">
+    <row r="52" ht="65" customHeight="1">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t>• The FTP now carries an explicit liquidity charge (buffer × drag) and a behavioural credit for stable deposits, shown as memos on the Revenues tab; it is still a single curve, not a full behavioural-maturity model. Fraud &amp; payment losses, the FSCS levy, collateral administration &amp; recoveries, and change-the-bank spend are now modelled explicitly. Operational-risk RWA is proxied at 15% of gross income; head-office and change costs are allocated per customer.</t>
         </is>
@@ -10903,6 +10918,426 @@
       <c r="B31" s="5" t="inlineStr">
         <is>
           <t>Source: Allica Bank Limited, Annual Report and Accounts 2023 (company number 07706156). Total operating income £86,808k; total operating expenses £56,438k; cost:income 65.0%; impairment charges £14,279k; profit before tax £16,091k; net interest margin 5.00%; loans and advances to customers £1,976,826k; colleagues at year end 496.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:J26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>TRAJECTORY — WHAT IT TAKES TO BUILD THIS FROM NOTHING</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Every other tab in this workbook describes a steady state. This one describes getting there. Time is deliberately NOT in the base model: at steady state a stock and a rate are the same statement, which is what makes the whole identity chain work without a forecast. So the trajectory runs the SAME model at a series of maturity states and reads the results as a cash flow — a wrapper around the snapshot, never inside it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>This matters because every new business starts sub-scale, where fixed cost dominates and unit economics look nothing like the steady state. That is the region the Allica backtest showed this model could not previously represent at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="42" t="inlineStr">
+        <is>
+          <t>One regional business centre, built from nothing — 8-year ramp to steady state, cost scale elasticity 0.808</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Build cost £6.0m in year 1 and £3.0m in year 2. Discount rate 12% — the model's own cost of equity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="45" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C7" s="45" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="D7" s="45" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="E7" s="45" t="inlineStr">
+        <is>
+          <t>Operating cost</t>
+        </is>
+      </c>
+      <c r="F7" s="45" t="inlineStr">
+        <is>
+          <t>Profit before tax</t>
+        </is>
+      </c>
+      <c r="G7" s="45" t="inlineStr">
+        <is>
+          <t>Cash flow</t>
+        </is>
+      </c>
+      <c r="H7" s="45" t="inlineStr">
+        <is>
+          <t>Cumulative cash</t>
+        </is>
+      </c>
+      <c r="I7" s="45" t="inlineStr">
+        <is>
+          <t>Cost / customer</t>
+        </is>
+      </c>
+      <c r="J7" s="45" t="inlineStr">
+        <is>
+          <t>Cost:income</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="44" t="n">
+        <v>301.171875</v>
+      </c>
+      <c r="D8" s="46" t="n">
+        <v>957473.4381271362</v>
+      </c>
+      <c r="E8" s="46" t="n">
+        <v>621931.4444624339</v>
+      </c>
+      <c r="F8" s="46" t="n">
+        <v>272918.9040553273</v>
+      </c>
+      <c r="G8" s="46" t="n">
+        <v>-5803498.389080164</v>
+      </c>
+      <c r="H8" s="46" t="n">
+        <v>-5803498.389080164</v>
+      </c>
+      <c r="I8" s="46" t="n">
+        <v>2065.038259174878</v>
+      </c>
+      <c r="J8" s="48" t="n">
+        <v>0.6495547758264308</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="44" t="n">
+        <v>620.625</v>
+      </c>
+      <c r="D9" s="46" t="n">
+        <v>1973065.886506348</v>
+      </c>
+      <c r="E9" s="46" t="n">
+        <v>1143780.437777619</v>
+      </c>
+      <c r="F9" s="46" t="n">
+        <v>700238.0236037285</v>
+      </c>
+      <c r="G9" s="46" t="n">
+        <v>-2495828.623005316</v>
+      </c>
+      <c r="H9" s="46" t="n">
+        <v>-8299327.01208548</v>
+      </c>
+      <c r="I9" s="46" t="n">
+        <v>1842.949345865247</v>
+      </c>
+      <c r="J9" s="48" t="n">
+        <v>0.579697031710826</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="44" t="n">
+        <v>1072.265625</v>
+      </c>
+      <c r="D10" s="46" t="n">
+        <v>3408903.485939026</v>
+      </c>
+      <c r="E10" s="46" t="n">
+        <v>1816763.121417706</v>
+      </c>
+      <c r="F10" s="46" t="n">
+        <v>1369182.671943195</v>
+      </c>
+      <c r="G10" s="46" t="n">
+        <v>985811.5237991003</v>
+      </c>
+      <c r="H10" s="46" t="n">
+        <v>-7313515.48828638</v>
+      </c>
+      <c r="I10" s="46" t="n">
+        <v>1694.321891012506</v>
+      </c>
+      <c r="J10" s="48" t="n">
+        <v>0.5329464823253145</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="42" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="44" t="n">
+        <v>1590</v>
+      </c>
+      <c r="D11" s="46" t="n">
+        <v>5054863.660898438</v>
+      </c>
+      <c r="E11" s="46" t="n">
+        <v>2538446.898715996</v>
+      </c>
+      <c r="F11" s="46" t="n">
+        <v>2185805.836182442</v>
+      </c>
+      <c r="G11" s="46" t="n">
+        <v>1573780.202051358</v>
+      </c>
+      <c r="H11" s="46" t="n">
+        <v>-5739735.286235021</v>
+      </c>
+      <c r="I11" s="46" t="n">
+        <v>1596.50748346918</v>
+      </c>
+      <c r="J11" s="48" t="n">
+        <v>0.5021791029403985</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="42" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="44" t="n">
+        <v>2107.734375</v>
+      </c>
+      <c r="D12" s="46" t="n">
+        <v>6700823.83585785</v>
+      </c>
+      <c r="E12" s="46" t="n">
+        <v>3226783.743447408</v>
+      </c>
+      <c r="F12" s="46" t="n">
+        <v>3035775.932988567</v>
+      </c>
+      <c r="G12" s="46" t="n">
+        <v>2185758.671751768</v>
+      </c>
+      <c r="H12" s="46" t="n">
+        <v>-3553976.614483254</v>
+      </c>
+      <c r="I12" s="46" t="n">
+        <v>1530.925235039357</v>
+      </c>
+      <c r="J12" s="48" t="n">
+        <v>0.4815503022449343</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="42" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" s="44" t="n">
+        <v>2559.375</v>
+      </c>
+      <c r="D13" s="46" t="n">
+        <v>8136661.435290528</v>
+      </c>
+      <c r="E13" s="46" t="n">
+        <v>3807773.856105018</v>
+      </c>
+      <c r="F13" s="46" t="n">
+        <v>3796713.15231051</v>
+      </c>
+      <c r="G13" s="46" t="n">
+        <v>2733633.469663567</v>
+      </c>
+      <c r="H13" s="46" t="n">
+        <v>-820343.1448196867</v>
+      </c>
+      <c r="I13" s="46" t="n">
+        <v>1487.774888832241</v>
+      </c>
+      <c r="J13" s="48" t="n">
+        <v>0.4679774237121195</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="42" t="n">
+        <v>7</v>
+      </c>
+      <c r="C14" s="44" t="n">
+        <v>2878.828125</v>
+      </c>
+      <c r="D14" s="46" t="n">
+        <v>9152253.883669738</v>
+      </c>
+      <c r="E14" s="46" t="n">
+        <v>4210013.115550779</v>
+      </c>
+      <c r="F14" s="46" t="n">
+        <v>4343642.005728334</v>
+      </c>
+      <c r="G14" s="46" t="n">
+        <v>3127422.2441244</v>
+      </c>
+      <c r="H14" s="46" t="n">
+        <v>2307079.099304714</v>
+      </c>
+      <c r="I14" s="46" t="n">
+        <v>1462.405163750712</v>
+      </c>
+      <c r="J14" s="48" t="n">
+        <v>0.4599974136494025</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="42" t="n">
+        <v>8</v>
+      </c>
+      <c r="C15" s="44" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D15" s="46" t="n">
+        <v>9537478.60546875</v>
+      </c>
+      <c r="E15" s="46" t="n">
+        <v>4360941.459832817</v>
+      </c>
+      <c r="F15" s="46" t="n">
+        <v>4552742.945635933</v>
+      </c>
+      <c r="G15" s="46" t="n">
+        <v>3277974.920857872</v>
+      </c>
+      <c r="H15" s="46" t="n">
+        <v>5585054.020162586</v>
+      </c>
+      <c r="I15" s="46" t="n">
+        <v>1453.647153277606</v>
+      </c>
+      <c r="J15" s="48" t="n">
+        <v>0.4572425942148139</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>Peak funding need</t>
+        </is>
+      </c>
+      <c r="D17" s="47" t="n">
+        <v>8299327.01208548</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="42" t="inlineStr">
+        <is>
+          <t>Payback</t>
+        </is>
+      </c>
+      <c r="D18" s="43" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="42" t="inlineStr">
+        <is>
+          <t>NPV at 12%</t>
+        </is>
+      </c>
+      <c r="D19" s="47" t="n">
+        <v>-105699.2968567105</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>WHAT THE SNAPSHOT CANNOT SEE</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr"/>
+      <c r="D21" s="8" t="inlineStr"/>
+      <c r="E21" s="8" t="inlineStr"/>
+      <c r="F21" s="8" t="inlineStr"/>
+      <c r="G21" s="8" t="inlineStr"/>
+      <c r="H21" s="8" t="inlineStr"/>
+      <c r="I21" s="8" t="inlineStr"/>
+      <c r="J21" s="8" t="inlineStr"/>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>• The snapshot reports the last row of this table and nothing else: 3,000 customers, 45.7% cost:income, £4.55m of profit. On that evidence the business is comfortably good.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>• The trajectory says it needs £8.3m of funding at its deepest point, takes seven years to repay, and has an NPV at the model's own 12% cost of equity of roughly MINUS £106,000. At that hurdle it is marginal — barely worth building.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>• Both statements are true about the same business. A profitable steady state is not the same thing as a worthwhile investment, and until this tab existed the model could not tell the difference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>• The ramp shape is an assumption and a load-bearing one. Reaching steady state in six years rather than eight changes the answer more than most of the pricing inputs do. It is the first thing to replace with evidence from a real build.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>• Time lives here and nowhere else. Putting years into the base tabs would break the steady-state identities the whole model rests on — the snapshot is the engine, and this is a wrapper around it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v2.1: evidence tab — public sources for three empty cells, and a correction to tab 10
</commit_message>
<xml_diff>
--- a/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
+++ b/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
@@ -23,6 +23,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. Elasticities" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. Backtest" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12. Trajectory" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13. Evidence" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -590,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B52"/>
+  <dimension ref="B1:B54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -607,7 +608,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MODEL VERSION: v2.0 · 22 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
+          <t>MODEL VERSION: v2.1 · 22 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
         </is>
       </c>
     </row>
@@ -618,295 +619,309 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="52" customHeight="1">
+    <row r="5" ht="58" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>• v2.0 (22 Aug 2026) — trajectory. Every other tab describes a steady state; tab 12 describes getting there. Time stays OUT of the base model deliberately — the steady-state identities are what let the whole chain work without a forecast — so the trajectory runs the same model at a series of maturity states and reads the result as a cash flow. Building one regional centre from nothing needs £8.3m of funding at its deepest point, repays in year seven, and has an NPV at the model's own 12% cost of equity of about MINUS £106,000. The snapshot alone reports only the final year and calls the business comfortably good. Both are true: a profitable steady state is not the same thing as a worthwhile investment.</t>
+          <t>• v2.1 (22 Aug 2026) — evidence. Tab 13 fills from public sources three of the cells that shipped empty. Loan application success is 37% (SME Finance Monitor, 18m to Q4 2024) against the model's implicit 100%, so the bank does 2.7 underwriting passes per funded loan — worth £143,644 of operating cost. UK formation rate is 15.0% of the company stock (Companies House, 846,325 incorporations in 2024), which fills the A1 entry point and shows formation alone covers 125% of steady-state replacement at current share. SME current-account switching is 0.44% (CASS 2024), which bounds current-account demand elasticity at about 0.004 and CORRECTS tab 10: v1.8 called the account fee fragile, and the evidence says the customer is near-inert, so raising it industry-wide is comfortably accretive.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="52" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>• v1.9 (22 Aug 2026) — competitive response. Every scenario assumed rivals stand still, which flatters both directions at once: raising a price looks safer than it is, and cutting one looks better than it is. A firm with market share s moving alone faces roughly the industry elasticity divided by s; moving in concert it faces only the industry elasticity. This model's penetration IS market share (16%), so moving alone multiplies the demand response by 6.25x. Tab 10 now inverts every break-even into the industry elasticity the move survives in each regime. The headline lever moves with it: raising the term loan rate survives an industry elasticity of 2.91 in concert but only 0.47 alone — marginal rather than comfortable.</t>
+          <t>• v2.0 (22 Aug 2026) — trajectory. Every other tab describes a steady state; tab 12 describes getting there. Time stays OUT of the base model deliberately — the steady-state identities are what let the whole chain work without a forecast — so the trajectory runs the same model at a series of maturity states and reads the result as a cash flow. Building one regional centre from nothing needs £8.3m of funding at its deepest point, repays in year seven, and has an NPV at the model's own 12% cost of equity of about MINUS £106,000. The snapshot alone reports only the final year and calls the business comfortably good. Both are true: a profitable steady state is not the same thing as a worthwhile investment.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>• v1.8 (22 Aug 2026) — break-even demand elasticity on tab 10. The elasticity table ranked the term loan customer rate as the largest driver of profit at +1.25, which was an artefact: nothing in the model responds to price, so raising any price always looked accretive. Tab 10 now leads with the demand elasticity at which raising each price stops paying. The reordering matters — the card fee breaks even at 0.06 and the current-account fee at 0.13, so both are fragile to almost any customer response, while the loan rate holds to 2.91. The hidden assumption being replaced is zero, which is the least defensible value available.</t>
+          <t>• v1.9 (22 Aug 2026) — competitive response. Every scenario assumed rivals stand still, which flatters both directions at once: raising a price looks safer than it is, and cutting one looks better than it is. A firm with market share s moving alone faces roughly the industry elasticity divided by s; moving in concert it faces only the industry elasticity. This model's penetration IS market share (16%), so moving alone multiplies the demand response by 6.25x. Tab 10 now inverts every break-even into the industry elasticity the move survives in each regime. The headline lever moves with it: raising the term loan rate survives an industry elasticity of 2.91 in concert but only 0.47 alone — marginal rather than comfortable.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>• v1.7 (22 Aug 2026) — operational leverage. Every cost line in the model scaled linearly with its driver, which forces a cost elasticity of exactly 1.0 and makes cost per customer flat at every scale. Allica Bank's own accounts put that elasticity at 0.808 across 2022-23 and 0.622 across 2023-24 — cost rises materially more slowly than the book. Inputs section O adds a cost scale elasticity and the customer count the per-customer rates are calibrated at; the head-office pools, the platform line and change-the-bank now scale by it. Default 1.0 reproduces v1.6 exactly. Tab 11 adds the out-of-sample test that measured it.</t>
+          <t>• v1.8 (22 Aug 2026) — break-even demand elasticity on tab 10. The elasticity table ranked the term loan customer rate as the largest driver of profit at +1.25, which was an artefact: nothing in the model responds to price, so raising any price always looked accretive. Tab 10 now leads with the demand elasticity at which raising each price stops paying. The reordering matters — the card fee breaks even at 0.06 and the current-account fee at 0.13, so both are fragile to almost any customer response, while the loan rate holds to 2.91. The hidden assumption being replaced is zero, which is the least defensible value available.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="52" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>• v1.6 (22 Aug 2026) — validation and drivers. Tab 10 ELASTICITIES: every input bumped +1% and the workbook recalculated, giving the % change in PBT, cost:income, RoE and income. Only one input has an elasticity above 1 on profit — the term loan customer rate, at +1.25; reachable market and penetration are exactly +1.00 (pure scale); nothing else exceeds 0.53. Tab 11 BACKTEST against Allica Bank FY2023 audited accounts: the revenue engine reproduces a real bank's operating income to within 8%, and the cost engine under-predicts by 7x. Diagnosis: head-office cost was modelled purely per customer, which is a scale assumption disguised as a driver. Inputs section N therefore adds a fixed component to each head-office pool, defaulting to 0 so v1.5 results are unchanged.</t>
+          <t>• v1.7 (22 Aug 2026) — operational leverage. Every cost line in the model scaled linearly with its driver, which forces a cost elasticity of exactly 1.0 and makes cost per customer flat at every scale. Allica Bank's own accounts put that elasticity at 0.808 across 2022-23 and 0.622 across 2023-24 — cost rises materially more slowly than the book. Inputs section O adds a cost scale elasticity and the customer count the per-customer rates are calibrated at; the head-office pools, the platform line and change-the-bank now scale by it. Default 1.0 reproduces v1.6 exactly. Tab 11 adds the out-of-sample test that measured it.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="52" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>• v1.5 (22 Aug 2026) — PROCESS LAYER on the Step 2 tabs. Tab 3 gains process columns M-T (process type, yield, attempts, automation, best-in-class intensity and yield, benchmark source, £ gap) and a HEAD-OFFICE PROCESS REGISTER of 22 processes already named in the tab 9 operational model but never costed. Yield inflates ATTEMPTS and never deflates outcomes — that is what stops it double-counting with the CEP layer's demand-side conversion. Head-office costs are carved OUT of the pools, so naming a process moves money from unallocated to attributed and the total never changes. New sheet 3b indexes every process to the numbers it moves, and imputes what each would have to become to hit a target cost:income. Mode OFF (default) = results identical to v1.4.</t>
+          <t>• v1.6 (22 Aug 2026) — validation and drivers. Tab 10 ELASTICITIES: every input bumped +1% and the workbook recalculated, giving the % change in PBT, cost:income, RoE and income. Only one input has an elasticity above 1 on profit — the term loan customer rate, at +1.25; reachable market and penetration are exactly +1.00 (pure scale); nothing else exceeds 0.53. Tab 11 BACKTEST against Allica Bank FY2023 audited accounts: the revenue engine reproduces a real bank's operating income to within 8%, and the cost engine under-predicts by 7x. Diagnosis: head-office cost was modelled purely per customer, which is a scale assumption disguised as a driver. Inputs section N therefore adds a fixed component to each head-office pool, defaulting to 0 so v1.5 results are unchanged.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="52" customHeight="1">
       <c r="B11" s="4" t="inlineStr">
         <is>
+          <t>• v1.5 (22 Aug 2026) — PROCESS LAYER on the Step 2 tabs. Tab 3 gains process columns M-T (process type, yield, attempts, automation, best-in-class intensity and yield, benchmark source, £ gap) and a HEAD-OFFICE PROCESS REGISTER of 22 processes already named in the tab 9 operational model but never costed. Yield inflates ATTEMPTS and never deflates outcomes — that is what stops it double-counting with the CEP layer's demand-side conversion. Head-office costs are carved OUT of the pools, so naming a process moves money from unallocated to attributed and the total never changes. New sheet 3b indexes every process to the numbers it moves, and imputes what each would have to become to hit a target cost:income. Mode OFF (default) = results identical to v1.4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52" customHeight="1">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
           <t>• v1.4 (22 Aug 2026) — CEP DEMAND LAYER. New sheet 1b derives the nine product penetrations and the customer count instead of asserting them: penetration = (lambda*c x L) / (1 + lambda*c x L), where lambda*c = category-entry-point events x presence x conversion and L is the holding life. Little's Law run forwards; no time axis is added and the model stays a steady-state snapshot. Ships deliberately EMPTY — every event/presence/conversion cell is blank and carries the cohort query that fills it, and any unpopulated product falls back to its hardcoded penetration. Mode OFF (default) = results identical to v1.3; CALIBRATE reports the won-event rate implied by today's assumptions and changes nothing.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="B12" s="4" t="inlineStr">
+    <row r="13" ht="40" customHeight="1">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>• v1.3 (21 Aug 2026) — churn replacement is a costed activity end-to-end: new input cac_new (£240 acquisition marketing per new customer won, carved out of the corporate-centre pool — hq_oh £250→£222); driver-linked on tab 4, attributed to the current account (gateway product) on tab 6; 'value of preventing one churn' memo added to tab 6. Raising the churn input now inflates demand-generation cost, not just processing. Central PBT shifts &lt;£1k/unit (carve-out rounding).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
+          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
         <is>
+          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
           <t>• v1.0 (10 Aug 2026) — first published version: 9 tabs + flow register, FTP with liquidity/behavioural terms, fraud/FSCS/change-the-bank lines, segment-pod LMUs, bridge check.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="3" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>What this is</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="39" customHeight="1">
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="39" customHeight="1">
       <c r="B20" s="4" t="inlineStr">
         <is>
+          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="39" customHeight="1">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
           <t>• It follows the Simanis / IVE bottom-up methodology ('Running the Right Numbers'): model the last-mile operating unit, derive every cost from activity drivers (transaction intensity I and customer load L), build whole costs, and check the price/margin covers them including a competitive return on capital.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="3" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>What period this models</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="26" customHeight="1">
-      <c r="B23" s="4" t="inlineStr">
+    <row r="24" ht="26" customHeight="1">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>• One representative operating year at steady state. Balances are annual averages; rates and volumes are annual. There is no time axis, no ramp and no vintage cohorts — the model is a snapshot, not a forecast.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="78" customHeight="1">
-      <c r="B24" s="4" t="inlineStr">
+    <row r="25" ht="78" customHeight="1">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>• The book is stationary but not free to hold flat: customers churn (12% p.a. input) and the model costs their replacement end-to-end — acquisition marketing per new customer won (cac_new, carved from the corporate-centre pool), onboarding hours, KYC per new customer and RM origination effort are all driver-linked (Simanis: at-scale operations include 'replacement of customer churn'). Only residual brand &amp; joint marketing remains pool-costed. The 'value of preventing one churn' memo on tab 6 prices retention: contribution annuity over remaining relationship life + the avoided replacement cost.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="26" customHeight="1">
-      <c r="B25" s="4" t="inlineStr">
+    <row r="26" ht="26" customHeight="1">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>• The capital charge (cost of equity on allocated capital) is the incumbent analogue of Simanis's start-up-cost amortisation: capital earns its required return inside the steady-state P&amp;L.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="52" customHeight="1">
-      <c r="B26" s="4" t="inlineStr">
+    <row r="27" ht="52" customHeight="1">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>• Out of scope by design: transition paths. The cost and cash shape of moving between steady states — digital migration, maturity glide, behaviour-change programmes and their CAC/incentives — belongs in a scenario layer built ON TOP of this base (comparative statics between two runs of this model, plus a separate transition-cost estimate). The base model never carries scenario logic.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="3" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>How the tabs map to the methodology</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="B29" s="4" t="inlineStr">
+    <row r="30" ht="24" customHeight="1">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>• Inputs — every assumption in one place, with sources. Edit blue cells; yellow cells are the biggest levers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="26" customHeight="1">
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="26" customHeight="1">
       <c r="B31" s="4" t="inlineStr">
         <is>
+          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1">
+      <c r="B32" s="4" t="inlineStr">
+        <is>
           <t>• 2. Revenues — unit revenue per product: interest margins measured against internal funds transfer prices (Bank Rate for floating, + premium for term), plus fees.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="39" customHeight="1">
-      <c r="B32" s="4" t="inlineStr">
+    <row r="33" ht="39" customHeight="1">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>• 3. HR &amp; Activity — Step 2: every FTE derived from activity drivers (hours per onboarding, review, renewal…) — nothing is assumed as headcount. From v1.5 this tab is also the PROCESS REGISTER (columns M-T), with the head-office process register below it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="26" customHeight="1">
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>• 1b. Demand &amp; CEPs — the demand layer (v1.4). Penetration is derived, not assumed. Mode cell on Inputs section L: OFF reproduces v1.3, CALIBRATE reports the implied event rates, LIVE derives.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="26" customHeight="1">
       <c r="B34" s="4" t="inlineStr">
         <is>
+          <t>• 1b. Demand &amp; CEPs — the demand layer (v1.4). Penetration is derived, not assumed. Mode cell on Inputs section L: OFF reproduces v1.3, CALIBRATE reports the implied event rates, LIVE derives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="26" customHeight="1">
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>• 13. Evidence — public sources for cells that shipped empty: application success rates, company formation rates and SME switching, each with its tier and what it changes. Includes a correction to tab 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="26" customHeight="1">
+      <c r="B36" s="4" t="inlineStr">
+        <is>
           <t>• 12. Trajectory — the ramp from nothing to steady state: cash flow, peak funding, payback and NPV. Time lives here and nowhere else, as a wrapper around the snapshot rather than inside it.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="39" customHeight="1">
-      <c r="B35" s="4" t="inlineStr">
+    <row r="37" ht="39" customHeight="1">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>• 3b. Process Index — derived view, no assumptions. Every process with its flow, product, owner, the numbers it moves, its cost and its gap to best in class, plus a ranked worst-gap list and the top-down benchmark imputation. Answers 'which process do I improve to move this number?'</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="52" customHeight="1">
-      <c r="B36" s="4" t="inlineStr">
+    <row r="38" ht="52" customHeight="1">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>• 4. Running Costs — Step 2 (cont.): direct running costs plus the share of head-office costs. The attribution memo reads the tab 3 process register and reports the share of the cost base with a named process owner — the model's own assessment of how much of its cost it actually understands. What remains in UNALLOCATED JOINT COSTS is cost with no process to improve.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="26" customHeight="1">
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>• 5. Risk &amp; Capital — Step 3: expected credit losses (PD × LGD), risk-weighted assets, allocated equity, and the required return on it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="91" customHeight="1">
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>• 6. Unit Economics — Steps 4–5: per-product unit costs and revenues on an activity-based costing basis, taken exactly as far as causality runs (the source methodology's own rule: link costs to customers and transactions 'whenever possible'). Costs with real drivers — servicing hours, RM effort per origination, staff-time-driven supervision, per-account and per-facility infrastructure — are attributed to products; genuinely joint costs (brand, exec, finance, platform build) are NOT forced into products but held as an unallocated hurdle that total contribution must clear, with a full-absorption memo showing the source doc's simple-division treatment. Product decisions should run on contribution.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="26" customHeight="1">
       <c r="B39" s="4" t="inlineStr">
         <is>
+          <t>• 5. Risk &amp; Capital — Step 3: expected credit losses (PD × LGD), risk-weighted assets, allocated equity, and the required return on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="91" customHeight="1">
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>• 6. Unit Economics — Steps 4–5: per-product unit costs and revenues on an activity-based costing basis, taken exactly as far as causality runs (the source methodology's own rule: link costs to customers and transactions 'whenever possible'). Costs with real drivers — servicing hours, RM effort per origination, staff-time-driven supervision, per-account and per-facility infrastructure — are attributed to products; genuinely joint costs (brand, exec, finance, platform build) are NOT forced into products but held as an unallocated hurdle that total contribution must clear, with a full-absorption memo showing the source doc's simple-division treatment. Product decisions should run on contribution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="26" customHeight="1">
+      <c r="B41" s="4" t="inlineStr">
+        <is>
           <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="26" customHeight="1">
-      <c r="B40" s="4" t="inlineStr">
+    <row r="42" ht="26" customHeight="1">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>• 8. Org Structure — the whole-bank organisation implied by the model: front-line FTEs from activity drivers × number of centres, head-office FTEs backed out of the per-customer head-office cost allocations.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="52" customHeight="1">
-      <c r="B41" s="4" t="inlineStr">
+    <row r="43" ht="52" customHeight="1">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>• 9. Flow Register — one row per flow on the operational model map: component type (CP/WP/PP/PartP), core/support/enabling, direction, digital/physical medium, the direct/administrative/managerial roles accountable, and the BIAN service domains. Ends with a BIAN completeness checklist. This is where the map, the ARM and BIAN reconcile.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="3" t="inlineStr">
+    <row r="45">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>Colour legend</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="26" customHeight="1">
-      <c r="B44" s="4" t="inlineStr">
+    <row r="46" ht="26" customHeight="1">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>• Blue = hardcoded input (edit these) · Yellow fill = key assumption / sensitivity lever · Black = formula · Green = link to another sheet.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="3" t="inlineStr">
+    <row r="48">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>Reading the results</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="52" customHeight="1">
-      <c r="B47" s="4" t="inlineStr">
+    <row r="49" ht="52" customHeight="1">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>• Deposit products earn the spread between the transfer price and the rate paid; lending earns the customer rate minus the transfer price minus expected losses. Capital-heavy, labour-heavy products (term loans) can show thin or negative economic profit — consistent with the Bank of England's 2026 finding that SME lending earns the lowest product-level returns, driven by impairments and per-borrower servicing costs.</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="39" customHeight="1">
-      <c r="B48" s="4" t="inlineStr">
+    <row r="50" ht="39" customHeight="1">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>• Use the cost-driver table on the P&amp;L tab to find leverage points, then trace them to transaction intensity (I) or customer load (L) assumptions on the Inputs tab — e.g. automating underwriting hours, raising RM portfolio size, or shifting servicing to digital.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="B50" s="3" t="inlineStr">
+    <row r="52">
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>Caveats</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="39" customHeight="1">
-      <c r="B51" s="4" t="inlineStr">
+    <row r="53" ht="39" customHeight="1">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>• Benchmarks are as of August 2026 (Bank Rate 3.75%; BoE effective new SME loan rate ~6.3%; commercial interchange 1.65–1.90%; invoice finance discount base+1–3%). Items marked 'Assumption' are illustrative and should be replaced with your own data.</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="65" customHeight="1">
-      <c r="B52" s="4" t="inlineStr">
+    <row r="54" ht="65" customHeight="1">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>• The FTP now carries an explicit liquidity charge (buffer × drag) and a behavioural credit for stable deposits, shown as memos on the Revenues tab; it is still a single curve, not a full behavioural-maturity model. Fraud &amp; payment losses, the FSCS levy, collateral administration &amp; recoveries, and change-the-bank spend are now modelled explicitly. Operational-risk RWA is proxied at 15% of gross income; head-office and change costs are allocated per customer.</t>
         </is>
@@ -11338,6 +11353,286 @@
       <c r="B26" s="5" t="inlineStr">
         <is>
           <t>• Time lives here and nowhere else. Putting years into the base tabs would break the steady-state identities the whole model rests on — the snapshot is the engine, and this is a wrapper around it.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:F21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="74" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>EVIDENCE — PUBLIC SOURCES FOR CELLS THAT SHIPPED EMPTY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>The demand and process layers ship deliberately empty, each cell carrying the query that would fill it. Most of those queries need an institution's own cohort data. Some do not. This tab holds the ones that can be answered from public sources, with the source named and the evidence tier stated, and says what each one changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="45" t="inlineStr">
+        <is>
+          <t>What</t>
+        </is>
+      </c>
+      <c r="C4" s="45" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="45" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="E4" s="45" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="F4" s="45" t="inlineStr">
+        <is>
+          <t>What it changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1">
+      <c r="B5" s="42" t="inlineStr">
+        <is>
+          <t>Loan application success rate</t>
+        </is>
+      </c>
+      <c r="C5" s="48" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D5" s="70" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>BVA BDRC SME Finance Monitor, 18 months to Q4 2024</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>The model assumed every underwriting activity produces a funded loan — an implicit yield of 100%. At 37% the bank does 2.7 passes per funded loan. Applying it across lending origination raises operating cost £143,644 and cuts profit before tax 3.2%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="B6" s="42" t="inlineStr">
+        <is>
+          <t>…same, BBB 24H1 approvals/applications</t>
+        </is>
+      </c>
+      <c r="C6" s="48" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="D6" s="70" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>British Business Bank: 46,339 applications, 22,352 approved, 24H1</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>The nearer, more conservative reading. Raises operating cost £90,252, cuts profit before tax 2.0%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="B7" s="42" t="inlineStr">
+        <is>
+          <t>…same, pre-pandemic norm</t>
+        </is>
+      </c>
+      <c r="C7" s="48" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D7" s="70" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>SME Finance Monitor — roughly 6 in 10 before 2020</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Use this if modelling a normalised credit environment rather than the current one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="44" customHeight="1">
+      <c r="B8" s="42" t="inlineStr">
+        <is>
+          <t>UK company formation rate</t>
+        </is>
+      </c>
+      <c r="C8" s="48" t="n">
+        <v>0.1503</v>
+      </c>
+      <c r="D8" s="70" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Companies House: 846,325 incorporations in 2024 against 5.63m active companies</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Official statistics — the strongest evidence available to any cell here. Fills the A1 formation entry point on sheet 1b: 2,819 formations a year in an 18,750-business catchment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="44" customHeight="1">
+      <c r="B9" s="42" t="inlineStr">
+        <is>
+          <t>…formation won at current share</t>
+        </is>
+      </c>
+      <c r="C9" s="44" t="n">
+        <v>451</v>
+      </c>
+      <c r="D9" s="70" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>2,819 formations x 16% market share</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>The steady state needs 360 replacements a year. Formation alone, won at nothing better than existing share, covers 125% of that. A bank at this share does not need to win switchers; it needs to not lose the formation moment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
+      <c r="B10" s="42" t="inlineStr">
+        <is>
+          <t>SME current-account switching</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="D10" s="70" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>CASS: 24,000 SME and charity switches in 2024 against ~5.5m businesses</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Lowest in the decade the scheme has run; the ten-year average is 0.60%. This is the single most useful public number for this model — see the derivation below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>DERIVING A DEMAND ELASTICITY FROM INERTIA — AND A CORRECTION TO TAB 10</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr"/>
+      <c r="D12" s="8" t="inlineStr"/>
+      <c r="E12" s="8" t="inlineStr"/>
+      <c r="F12" s="8" t="inlineStr"/>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>• Tab 10 gives the break-even demand elasticity for every price — the responsiveness at which raising it stops paying. It could not say whether real customers are that responsive. For the business current account, public data can.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="39" customHeight="1">
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>• UK SME current-account prices differ by 100%: the majors charge from £8.50 a month, several challengers charge nothing. That gap is permanent, visible and heavily advertised. Against it, 0.44% of SMEs switched in 2024 — and not all of those for price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="39" customHeight="1">
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>• A 100% price difference producing at most 0.44% of annual movement implies an upper-bound elasticity of about 0.004. Allowing a generous ten-fold multiplier for salience — a fee RISE is noticed in a way a standing price gap is not, which is the one robust finding in the FCA's banking trials — still only reaches 0.044.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>• Against a break-even of 0.13, raising the current-account fee industry-wide has roughly three times the headroom it needs. It is comfortably accretive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="39" customHeight="1">
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>• CORRECTION TO TAB 10: v1.8 labelled the current-account fee 'fragile — only a near-inert customer makes this pay'. The evidence says the SME current-account customer IS near-inert. At 0.44% annual switching this is close to the most inert consumer market for which data exists. The fragile reading was wrong and this tab supersedes it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>• Moving alone is the exception and stays genuinely marginal: the break-even falls to 0.021, which is below the salience-adjusted bound of 0.044. Industry-wide, clearly accretive. Unilaterally, a coin toss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="52" customHeight="1">
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>• The bound does NOT transfer to every price. It holds where switching bank is the customer's only escape, which is true of the current account. It does not hold for the card annual fee (cancel the card, keep the bank), the card interest rate (pay the balance down), or loan pricing (brokered and shopped). Those have other margins of adjustment and need their own evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Still needing an institution's own data: process yields outside lending, entry-point incidence for every cross-holding moment, holding lives for five products, and the benchmark columns on tab 3. Those queries are written against each cell and none of them can be answered from public sources.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v2.2: correction — invoice finance penetration was 4.2x too high
UK Finance counts 40,100 businesses on invoice finance or ABL at end-2024 against 5.63m
active companies = 0.71%. The model assumed 3%. Profit before tax falls 22.6%; the
trajectory NPV moves from -£106k to -£1.97m.
</commit_message>
<xml_diff>
--- a/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
+++ b/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B54"/>
+  <dimension ref="B1:B55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -608,7 +608,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MODEL VERSION: v2.1 · 22 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
+          <t>MODEL VERSION: v2.2 · 22 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
         </is>
       </c>
     </row>
@@ -622,306 +622,313 @@
     <row r="5" ht="58" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
+          <t>• v2.2 (22 Aug 2026) — CORRECTION, results change. Nine product penetrations were all labelled 'Assumption'. Tested against published aggregates, three land within a fifth of the survey figure (overdrafts 25% vs 22%, term loans 12% vs 13%, asset finance 8% vs 10%) — real corroboration. Invoice finance did not: the model said 3%, UK Finance counts 40,100 businesses on invoice finance or ABL at end-2024 against 5.63m active companies, which is 0.71%. A hard count, not a survey. Corrected in the base. Profit before tax falls 22.6% and cost:income moves 45.7% to 51.3%, because invoice finance is the highest-value behaviour per adopter in the book and the model was carrying 4.2x too many adopters of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
           <t>• v2.1 (22 Aug 2026) — evidence. Tab 13 fills from public sources three of the cells that shipped empty. Loan application success is 37% (SME Finance Monitor, 18m to Q4 2024) against the model's implicit 100%, so the bank does 2.7 underwriting passes per funded loan — worth £143,644 of operating cost. UK formation rate is 15.0% of the company stock (Companies House, 846,325 incorporations in 2024), which fills the A1 entry point and shows formation alone covers 125% of steady-state replacement at current share. SME current-account switching is 0.44% (CASS 2024), which bounds current-account demand elasticity at about 0.004 and CORRECTS tab 10: v1.8 called the account fee fragile, and the evidence says the customer is near-inert, so raising it industry-wide is comfortably accretive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>• v2.0 (22 Aug 2026) — trajectory. Every other tab describes a steady state; tab 12 describes getting there. Time stays OUT of the base model deliberately — the steady-state identities are what let the whole chain work without a forecast — so the trajectory runs the same model at a series of maturity states and reads the result as a cash flow. Building one regional centre from nothing needs £8.3m of funding at its deepest point, repays in year seven, and has an NPV at the model's own 12% cost of equity of about MINUS £106,000. The snapshot alone reports only the final year and calls the business comfortably good. Both are true: a profitable steady state is not the same thing as a worthwhile investment.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>• v1.9 (22 Aug 2026) — competitive response. Every scenario assumed rivals stand still, which flatters both directions at once: raising a price looks safer than it is, and cutting one looks better than it is. A firm with market share s moving alone faces roughly the industry elasticity divided by s; moving in concert it faces only the industry elasticity. This model's penetration IS market share (16%), so moving alone multiplies the demand response by 6.25x. Tab 10 now inverts every break-even into the industry elasticity the move survives in each regime. The headline lever moves with it: raising the term loan rate survives an industry elasticity of 2.91 in concert but only 0.47 alone — marginal rather than comfortable.</t>
+          <t>• v2.0 (22 Aug 2026) — trajectory. Every other tab describes a steady state; tab 12 describes getting there. Time stays OUT of the base model deliberately — the steady-state identities are what let the whole chain work without a forecast — so the trajectory runs the same model at a series of maturity states and reads the result as a cash flow. Building one regional centre from nothing needs £8.3m of funding at its deepest point, repays in year seven, and has an NPV at the model's own 12% cost of equity of about MINUS £106,000. The snapshot alone reports only the final year and calls the business comfortably good. Both are true: a profitable steady state is not the same thing as a worthwhile investment.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>• v1.8 (22 Aug 2026) — break-even demand elasticity on tab 10. The elasticity table ranked the term loan customer rate as the largest driver of profit at +1.25, which was an artefact: nothing in the model responds to price, so raising any price always looked accretive. Tab 10 now leads with the demand elasticity at which raising each price stops paying. The reordering matters — the card fee breaks even at 0.06 and the current-account fee at 0.13, so both are fragile to almost any customer response, while the loan rate holds to 2.91. The hidden assumption being replaced is zero, which is the least defensible value available.</t>
+          <t>• v1.9 (22 Aug 2026) — competitive response. Every scenario assumed rivals stand still, which flatters both directions at once: raising a price looks safer than it is, and cutting one looks better than it is. A firm with market share s moving alone faces roughly the industry elasticity divided by s; moving in concert it faces only the industry elasticity. This model's penetration IS market share (16%), so moving alone multiplies the demand response by 6.25x. Tab 10 now inverts every break-even into the industry elasticity the move survives in each regime. The headline lever moves with it: raising the term loan rate survives an industry elasticity of 2.91 in concert but only 0.47 alone — marginal rather than comfortable.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="52" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>• v1.7 (22 Aug 2026) — operational leverage. Every cost line in the model scaled linearly with its driver, which forces a cost elasticity of exactly 1.0 and makes cost per customer flat at every scale. Allica Bank's own accounts put that elasticity at 0.808 across 2022-23 and 0.622 across 2023-24 — cost rises materially more slowly than the book. Inputs section O adds a cost scale elasticity and the customer count the per-customer rates are calibrated at; the head-office pools, the platform line and change-the-bank now scale by it. Default 1.0 reproduces v1.6 exactly. Tab 11 adds the out-of-sample test that measured it.</t>
+          <t>• v1.8 (22 Aug 2026) — break-even demand elasticity on tab 10. The elasticity table ranked the term loan customer rate as the largest driver of profit at +1.25, which was an artefact: nothing in the model responds to price, so raising any price always looked accretive. Tab 10 now leads with the demand elasticity at which raising each price stops paying. The reordering matters — the card fee breaks even at 0.06 and the current-account fee at 0.13, so both are fragile to almost any customer response, while the loan rate holds to 2.91. The hidden assumption being replaced is zero, which is the least defensible value available.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="52" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>• v1.6 (22 Aug 2026) — validation and drivers. Tab 10 ELASTICITIES: every input bumped +1% and the workbook recalculated, giving the % change in PBT, cost:income, RoE and income. Only one input has an elasticity above 1 on profit — the term loan customer rate, at +1.25; reachable market and penetration are exactly +1.00 (pure scale); nothing else exceeds 0.53. Tab 11 BACKTEST against Allica Bank FY2023 audited accounts: the revenue engine reproduces a real bank's operating income to within 8%, and the cost engine under-predicts by 7x. Diagnosis: head-office cost was modelled purely per customer, which is a scale assumption disguised as a driver. Inputs section N therefore adds a fixed component to each head-office pool, defaulting to 0 so v1.5 results are unchanged.</t>
+          <t>• v1.7 (22 Aug 2026) — operational leverage. Every cost line in the model scaled linearly with its driver, which forces a cost elasticity of exactly 1.0 and makes cost per customer flat at every scale. Allica Bank's own accounts put that elasticity at 0.808 across 2022-23 and 0.622 across 2023-24 — cost rises materially more slowly than the book. Inputs section O adds a cost scale elasticity and the customer count the per-customer rates are calibrated at; the head-office pools, the platform line and change-the-bank now scale by it. Default 1.0 reproduces v1.6 exactly. Tab 11 adds the out-of-sample test that measured it.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="52" customHeight="1">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>• v1.5 (22 Aug 2026) — PROCESS LAYER on the Step 2 tabs. Tab 3 gains process columns M-T (process type, yield, attempts, automation, best-in-class intensity and yield, benchmark source, £ gap) and a HEAD-OFFICE PROCESS REGISTER of 22 processes already named in the tab 9 operational model but never costed. Yield inflates ATTEMPTS and never deflates outcomes — that is what stops it double-counting with the CEP layer's demand-side conversion. Head-office costs are carved OUT of the pools, so naming a process moves money from unallocated to attributed and the total never changes. New sheet 3b indexes every process to the numbers it moves, and imputes what each would have to become to hit a target cost:income. Mode OFF (default) = results identical to v1.4.</t>
+          <t>• v1.6 (22 Aug 2026) — validation and drivers. Tab 10 ELASTICITIES: every input bumped +1% and the workbook recalculated, giving the % change in PBT, cost:income, RoE and income. Only one input has an elasticity above 1 on profit — the term loan customer rate, at +1.25; reachable market and penetration are exactly +1.00 (pure scale); nothing else exceeds 0.53. Tab 11 BACKTEST against Allica Bank FY2023 audited accounts: the revenue engine reproduces a real bank's operating income to within 8%, and the cost engine under-predicts by 7x. Diagnosis: head-office cost was modelled purely per customer, which is a scale assumption disguised as a driver. Inputs section N therefore adds a fixed component to each head-office pool, defaulting to 0 so v1.5 results are unchanged.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="52" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
+          <t>• v1.5 (22 Aug 2026) — PROCESS LAYER on the Step 2 tabs. Tab 3 gains process columns M-T (process type, yield, attempts, automation, best-in-class intensity and yield, benchmark source, £ gap) and a HEAD-OFFICE PROCESS REGISTER of 22 processes already named in the tab 9 operational model but never costed. Yield inflates ATTEMPTS and never deflates outcomes — that is what stops it double-counting with the CEP layer's demand-side conversion. Head-office costs are carved OUT of the pools, so naming a process moves money from unallocated to attributed and the total never changes. New sheet 3b indexes every process to the numbers it moves, and imputes what each would have to become to hit a target cost:income. Mode OFF (default) = results identical to v1.4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="52" customHeight="1">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
           <t>• v1.4 (22 Aug 2026) — CEP DEMAND LAYER. New sheet 1b derives the nine product penetrations and the customer count instead of asserting them: penetration = (lambda*c x L) / (1 + lambda*c x L), where lambda*c = category-entry-point events x presence x conversion and L is the holding life. Little's Law run forwards; no time axis is added and the model stays a steady-state snapshot. Ships deliberately EMPTY — every event/presence/conversion cell is blank and carries the cohort query that fills it, and any unpopulated product falls back to its hardcoded penetration. Mode OFF (default) = results identical to v1.3; CALIBRATE reports the won-event rate implied by today's assumptions and changes nothing.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="B13" s="4" t="inlineStr">
+    <row r="14" ht="40" customHeight="1">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>• v1.3 (21 Aug 2026) — churn replacement is a costed activity end-to-end: new input cac_new (£240 acquisition marketing per new customer won, carved out of the corporate-centre pool — hq_oh £250→£222); driver-linked on tab 4, attributed to the current account (gateway product) on tab 6; 'value of preventing one churn' memo added to tab 6. Raising the churn input now inflates demand-generation cost, not just processing. Central PBT shifts &lt;£1k/unit (carve-out rounding).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
+          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="B17" s="4" t="inlineStr">
         <is>
+          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
           <t>• v1.0 (10 Aug 2026) — first published version: 9 tabs + flow register, FTP with liquidity/behavioural terms, fraud/FSCS/change-the-bank lines, segment-pod LMUs, bridge check.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="3" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>What this is</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="39" customHeight="1">
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="39" customHeight="1">
       <c r="B21" s="4" t="inlineStr">
         <is>
+          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="39" customHeight="1">
+      <c r="B22" s="4" t="inlineStr">
+        <is>
           <t>• It follows the Simanis / IVE bottom-up methodology ('Running the Right Numbers'): model the last-mile operating unit, derive every cost from activity drivers (transaction intensity I and customer load L), build whole costs, and check the price/margin covers them including a competitive return on capital.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="3" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>What period this models</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="26" customHeight="1">
-      <c r="B24" s="4" t="inlineStr">
+    <row r="25" ht="26" customHeight="1">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>• One representative operating year at steady state. Balances are annual averages; rates and volumes are annual. There is no time axis, no ramp and no vintage cohorts — the model is a snapshot, not a forecast.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="78" customHeight="1">
-      <c r="B25" s="4" t="inlineStr">
+    <row r="26" ht="78" customHeight="1">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>• The book is stationary but not free to hold flat: customers churn (12% p.a. input) and the model costs their replacement end-to-end — acquisition marketing per new customer won (cac_new, carved from the corporate-centre pool), onboarding hours, KYC per new customer and RM origination effort are all driver-linked (Simanis: at-scale operations include 'replacement of customer churn'). Only residual brand &amp; joint marketing remains pool-costed. The 'value of preventing one churn' memo on tab 6 prices retention: contribution annuity over remaining relationship life + the avoided replacement cost.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="26" customHeight="1">
-      <c r="B26" s="4" t="inlineStr">
+    <row r="27" ht="26" customHeight="1">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>• The capital charge (cost of equity on allocated capital) is the incumbent analogue of Simanis's start-up-cost amortisation: capital earns its required return inside the steady-state P&amp;L.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="52" customHeight="1">
-      <c r="B27" s="4" t="inlineStr">
+    <row r="28" ht="52" customHeight="1">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>• Out of scope by design: transition paths. The cost and cash shape of moving between steady states — digital migration, maturity glide, behaviour-change programmes and their CAC/incentives — belongs in a scenario layer built ON TOP of this base (comparative statics between two runs of this model, plus a separate transition-cost estimate). The base model never carries scenario logic.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="3" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>How the tabs map to the methodology</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="B30" s="4" t="inlineStr">
+    <row r="31" ht="24" customHeight="1">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>• Inputs — every assumption in one place, with sources. Edit blue cells; yellow cells are the biggest levers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="26" customHeight="1">
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="26" customHeight="1">
       <c r="B32" s="4" t="inlineStr">
         <is>
+          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1">
+      <c r="B33" s="4" t="inlineStr">
+        <is>
           <t>• 2. Revenues — unit revenue per product: interest margins measured against internal funds transfer prices (Bank Rate for floating, + premium for term), plus fees.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="39" customHeight="1">
-      <c r="B33" s="4" t="inlineStr">
+    <row r="34" ht="39" customHeight="1">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>• 3. HR &amp; Activity — Step 2: every FTE derived from activity drivers (hours per onboarding, review, renewal…) — nothing is assumed as headcount. From v1.5 this tab is also the PROCESS REGISTER (columns M-T), with the head-office process register below it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="26" customHeight="1">
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>• 1b. Demand &amp; CEPs — the demand layer (v1.4). Penetration is derived, not assumed. Mode cell on Inputs section L: OFF reproduces v1.3, CALIBRATE reports the implied event rates, LIVE derives.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="26" customHeight="1">
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>• 13. Evidence — public sources for cells that shipped empty: application success rates, company formation rates and SME switching, each with its tier and what it changes. Includes a correction to tab 10.</t>
+          <t>• 1b. Demand &amp; CEPs — the demand layer (v1.4). Penetration is derived, not assumed. Mode cell on Inputs section L: OFF reproduces v1.3, CALIBRATE reports the implied event rates, LIVE derives.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="26" customHeight="1">
       <c r="B36" s="4" t="inlineStr">
         <is>
+          <t>• 13. Evidence — public sources for cells that shipped empty: application success rates, company formation rates and SME switching, each with its tier and what it changes. Includes a correction to tab 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="26" customHeight="1">
+      <c r="B37" s="4" t="inlineStr">
+        <is>
           <t>• 12. Trajectory — the ramp from nothing to steady state: cash flow, peak funding, payback and NPV. Time lives here and nowhere else, as a wrapper around the snapshot rather than inside it.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="39" customHeight="1">
-      <c r="B37" s="4" t="inlineStr">
+    <row r="38" ht="39" customHeight="1">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>• 3b. Process Index — derived view, no assumptions. Every process with its flow, product, owner, the numbers it moves, its cost and its gap to best in class, plus a ranked worst-gap list and the top-down benchmark imputation. Answers 'which process do I improve to move this number?'</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="52" customHeight="1">
-      <c r="B38" s="4" t="inlineStr">
+    <row r="39" ht="52" customHeight="1">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>• 4. Running Costs — Step 2 (cont.): direct running costs plus the share of head-office costs. The attribution memo reads the tab 3 process register and reports the share of the cost base with a named process owner — the model's own assessment of how much of its cost it actually understands. What remains in UNALLOCATED JOINT COSTS is cost with no process to improve.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="26" customHeight="1">
-      <c r="B39" s="4" t="inlineStr">
+    <row r="40" ht="26" customHeight="1">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>• 5. Risk &amp; Capital — Step 3: expected credit losses (PD × LGD), risk-weighted assets, allocated equity, and the required return on it.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="91" customHeight="1">
-      <c r="B40" s="4" t="inlineStr">
+    <row r="41" ht="91" customHeight="1">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>• 6. Unit Economics — Steps 4–5: per-product unit costs and revenues on an activity-based costing basis, taken exactly as far as causality runs (the source methodology's own rule: link costs to customers and transactions 'whenever possible'). Costs with real drivers — servicing hours, RM effort per origination, staff-time-driven supervision, per-account and per-facility infrastructure — are attributed to products; genuinely joint costs (brand, exec, finance, platform build) are NOT forced into products but held as an unallocated hurdle that total contribution must clear, with a full-absorption memo showing the source doc's simple-division treatment. Product decisions should run on contribution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="26" customHeight="1">
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="26" customHeight="1">
       <c r="B42" s="4" t="inlineStr">
         <is>
+          <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="26" customHeight="1">
+      <c r="B43" s="4" t="inlineStr">
+        <is>
           <t>• 8. Org Structure — the whole-bank organisation implied by the model: front-line FTEs from activity drivers × number of centres, head-office FTEs backed out of the per-customer head-office cost allocations.</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="52" customHeight="1">
-      <c r="B43" s="4" t="inlineStr">
+    <row r="44" ht="52" customHeight="1">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>• 9. Flow Register — one row per flow on the operational model map: component type (CP/WP/PP/PartP), core/support/enabling, direction, digital/physical medium, the direct/administrative/managerial roles accountable, and the BIAN service domains. Ends with a BIAN completeness checklist. This is where the map, the ARM and BIAN reconcile.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="B45" s="3" t="inlineStr">
+    <row r="46">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>Colour legend</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="26" customHeight="1">
-      <c r="B46" s="4" t="inlineStr">
+    <row r="47" ht="26" customHeight="1">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>• Blue = hardcoded input (edit these) · Yellow fill = key assumption / sensitivity lever · Black = formula · Green = link to another sheet.</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="B48" s="3" t="inlineStr">
+    <row r="49">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>Reading the results</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="52" customHeight="1">
-      <c r="B49" s="4" t="inlineStr">
+    <row r="50" ht="52" customHeight="1">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>• Deposit products earn the spread between the transfer price and the rate paid; lending earns the customer rate minus the transfer price minus expected losses. Capital-heavy, labour-heavy products (term loans) can show thin or negative economic profit — consistent with the Bank of England's 2026 finding that SME lending earns the lowest product-level returns, driven by impairments and per-borrower servicing costs.</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="39" customHeight="1">
-      <c r="B50" s="4" t="inlineStr">
+    <row r="51" ht="39" customHeight="1">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>• Use the cost-driver table on the P&amp;L tab to find leverage points, then trace them to transaction intensity (I) or customer load (L) assumptions on the Inputs tab — e.g. automating underwriting hours, raising RM portfolio size, or shifting servicing to digital.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="B52" s="3" t="inlineStr">
+    <row r="53">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>Caveats</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="39" customHeight="1">
-      <c r="B53" s="4" t="inlineStr">
+    <row r="54" ht="39" customHeight="1">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>• Benchmarks are as of August 2026 (Bank Rate 3.75%; BoE effective new SME loan rate ~6.3%; commercial interchange 1.65–1.90%; invoice finance discount base+1–3%). Items marked 'Assumption' are illustrative and should be replaced with your own data.</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="65" customHeight="1">
-      <c r="B54" s="4" t="inlineStr">
+    <row r="55" ht="65" customHeight="1">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>• The FTP now carries an explicit liquidity charge (buffer × drag) and a behavioural credit for stable deposits, shown as memos on the Revenues tab; it is still a single curve, not a full behavioural-maturity model. Fraud &amp; payment losses, the FSCS levy, collateral administration &amp; recoveries, and change-the-bank spend are now modelled explicitly. Operational-risk RWA is proxied at 15% of gross income; head-office and change costs are allocated per customer.</t>
         </is>
@@ -7816,7 +7823,7 @@
     <row r="5">
       <c r="B5" s="42" t="inlineStr">
         <is>
-          <t>Computed at: PBT £4,552,743 · cost:income 45.7% · RoE 21.8%</t>
+          <t>Computed at: PBT £3,521,023 · cost:income 51.3% · RoE 18.3%</t>
         </is>
       </c>
     </row>
@@ -8302,16 +8309,16 @@
         </is>
       </c>
       <c r="E29" s="71" t="n">
-        <v>1.247681048892727</v>
+        <v>1.61327277330784</v>
       </c>
       <c r="F29" s="71" t="n">
-        <v>-0.5920579472668667</v>
+        <v>-0.6707136124121114</v>
       </c>
       <c r="G29" s="71" t="n">
-        <v>1.148369761396499</v>
+        <v>1.505361613400337</v>
       </c>
       <c r="H29" s="71" t="n">
-        <v>0.5955841505629065</v>
+        <v>0.675242556153086</v>
       </c>
     </row>
     <row r="30">
@@ -8329,7 +8336,7 @@
         </is>
       </c>
       <c r="E30" s="71" t="n">
-        <v>1.00000000000003</v>
+        <v>0.9999999999999578</v>
       </c>
       <c r="F30" s="71" t="n">
         <v>0</v>
@@ -8338,7 +8345,7 @@
         <v>0</v>
       </c>
       <c r="H30" s="71" t="n">
-        <v>1.00000000000002</v>
+        <v>0.999999999999992</v>
       </c>
     </row>
     <row r="31">
@@ -8356,7 +8363,7 @@
         </is>
       </c>
       <c r="E31" s="71" t="n">
-        <v>1.00000000000003</v>
+        <v>0.9999999999999578</v>
       </c>
       <c r="F31" s="71" t="n">
         <v>0</v>
@@ -8365,7 +8372,7 @@
         <v>0</v>
       </c>
       <c r="H31" s="71" t="n">
-        <v>1.00000000000002</v>
+        <v>0.999999999999992</v>
       </c>
     </row>
     <row r="32">
@@ -8383,16 +8390,16 @@
         </is>
       </c>
       <c r="E32" s="71" t="n">
-        <v>0.5316502207558557</v>
+        <v>0.6874327592213575</v>
       </c>
       <c r="F32" s="71" t="n">
-        <v>-0.2263724971407025</v>
+        <v>-0.2626076388723727</v>
       </c>
       <c r="G32" s="71" t="n">
-        <v>0.4858715994436417</v>
+        <v>0.6377899386038517</v>
       </c>
       <c r="H32" s="71" t="n">
-        <v>0.2763510458611886</v>
+        <v>0.3133125460550319</v>
       </c>
     </row>
     <row r="33">
@@ -8410,16 +8417,16 @@
         </is>
       </c>
       <c r="E33" s="71" t="n">
-        <v>0.4485219355690576</v>
+        <v>0.5799464755251776</v>
       </c>
       <c r="F33" s="71" t="n">
-        <v>-0.2508408142510311</v>
+        <v>-0.2842949830259432</v>
       </c>
       <c r="G33" s="71" t="n">
-        <v>-0.172627245775743</v>
+        <v>-0.09315289195585527</v>
       </c>
       <c r="H33" s="71" t="n">
-        <v>0.2514716076793886</v>
+        <v>0.2851055237263594</v>
       </c>
     </row>
     <row r="34">
@@ -8437,16 +8444,16 @@
         </is>
       </c>
       <c r="E34" s="71" t="n">
-        <v>0.4269286171458919</v>
+        <v>0.5520259482968808</v>
       </c>
       <c r="F34" s="71" t="n">
-        <v>-0.2009624805300439</v>
+        <v>-0.2283254496988612</v>
       </c>
       <c r="G34" s="71" t="n">
-        <v>0.3928629971036865</v>
+        <v>0.5150956851542485</v>
       </c>
       <c r="H34" s="71" t="n">
-        <v>0.2058338824345483</v>
+        <v>0.2333638274065154</v>
       </c>
     </row>
     <row r="35">
@@ -8464,16 +8471,16 @@
         </is>
       </c>
       <c r="E35" s="71" t="n">
-        <v>0.4168087496628946</v>
+        <v>0.5389407878755174</v>
       </c>
       <c r="F35" s="71" t="n">
-        <v>-0.2178158778235073</v>
+        <v>-0.2509271506335589</v>
       </c>
       <c r="G35" s="71" t="n">
-        <v>-0.2041443250685729</v>
+        <v>-0.1338841620559702</v>
       </c>
       <c r="H35" s="71" t="n">
-        <v>0.2514716076793886</v>
+        <v>0.2851055237263594</v>
       </c>
     </row>
     <row r="36">
@@ -8491,431 +8498,431 @@
         </is>
       </c>
       <c r="E36" s="71" t="n">
-        <v>0.3619938616520847</v>
+        <v>0.468064207295712</v>
       </c>
       <c r="F36" s="71" t="n">
-        <v>-0.1725007356564119</v>
+        <v>-0.1955273153312782</v>
       </c>
       <c r="G36" s="71" t="n">
-        <v>0.3334124986436103</v>
+        <v>0.4370850852513102</v>
       </c>
       <c r="H36" s="71" t="n">
-        <v>0.1727988148833219</v>
+        <v>0.1959103736252198</v>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — average funds in use (advances)</t>
+          <t>Notice &amp; fixed deposits — rate paid</t>
         </is>
       </c>
       <c r="C37" s="63" t="n">
-        <v>150000</v>
+        <v>0.041</v>
       </c>
       <c r="D37" s="14" t="inlineStr">
         <is>
-          <t>£/client</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E37" s="71" t="n">
-        <v>0.3101871844046677</v>
+        <v>-0.3968651022335832</v>
       </c>
       <c r="F37" s="71" t="n">
-        <v>-0.1543074556452041</v>
+        <v>0.166386052133733</v>
       </c>
       <c r="G37" s="71" t="n">
-        <v>0.209829595204097</v>
+        <v>-0.3708096217590231</v>
       </c>
       <c r="H37" s="71" t="n">
-        <v>0.1545459315400012</v>
+        <v>-0.1661096688135927</v>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Notice &amp; fixed deposits — rate paid</t>
+          <t>Head office: technology &amp; central operations</t>
         </is>
       </c>
       <c r="C38" s="63" t="n">
-        <v>0.041</v>
+        <v>450</v>
       </c>
       <c r="D38" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E38" s="71" t="n">
-        <v>-0.3069295380274881</v>
+        <v>-0.3834112609934771</v>
       </c>
       <c r="F38" s="71" t="n">
-        <v>0.1467286786560457</v>
+        <v>0.3128853263417148</v>
       </c>
       <c r="G38" s="71" t="n">
-        <v>-0.2828446455047969</v>
+        <v>-0.3834112609934804</v>
       </c>
       <c r="H38" s="71" t="n">
-        <v>-0.1465137010384164</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — penetration</t>
+          <t>Instant-access savings — rate paid</t>
         </is>
       </c>
       <c r="C39" s="63" t="n">
-        <v>0.03</v>
+        <v>0.033</v>
       </c>
       <c r="D39" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E39" s="71" t="n">
-        <v>0.2968754767403625</v>
+        <v>-0.3407232097226184</v>
       </c>
       <c r="F39" s="71" t="n">
-        <v>-0.1404317212375283</v>
+        <v>0.1428148979391809</v>
       </c>
       <c r="G39" s="71" t="n">
-        <v>0.1965312055379295</v>
+        <v>-0.318341845979591</v>
       </c>
       <c r="H39" s="71" t="n">
-        <v>0.1545459315400012</v>
+        <v>-0.1426112278595273</v>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Head office: technology &amp; central operations</t>
+          <t>Bank of England Bank Rate</t>
         </is>
       </c>
       <c r="C40" s="63" t="n">
-        <v>450</v>
+        <v>0.0375</v>
       </c>
       <c r="D40" s="14" t="inlineStr">
         <is>
-          <t>£/customer/yr</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E40" s="71" t="n">
-        <v>-0.2965245383102628</v>
+        <v>0.2451325388192351</v>
       </c>
       <c r="F40" s="71" t="n">
-        <v>0.3095661825398512</v>
+        <v>-0.1024961613300335</v>
       </c>
       <c r="G40" s="71" t="n">
-        <v>-0.2965245383105712</v>
+        <v>0.2387120231982801</v>
       </c>
       <c r="H40" s="71" t="n">
-        <v>0</v>
+        <v>0.1026013237482584</v>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Instant-access savings — rate paid</t>
+          <t>International payments &amp; FX — penetration</t>
         </is>
       </c>
       <c r="C41" s="63" t="n">
-        <v>0.033</v>
+        <v>0.2</v>
       </c>
       <c r="D41" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E41" s="71" t="n">
-        <v>-0.2635102375261357</v>
+        <v>0.2182541932141037</v>
       </c>
       <c r="F41" s="71" t="n">
-        <v>0.1259457965071908</v>
+        <v>-0.09081039086382579</v>
       </c>
       <c r="G41" s="71" t="n">
-        <v>-0.2428241773307234</v>
+        <v>0.2037664635887323</v>
       </c>
       <c r="H41" s="71" t="n">
-        <v>-0.125787372598882</v>
+        <v>0.09183298763681969</v>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — funded invoices as multiple of advances</t>
+          <t>Asset finance — average balance</t>
         </is>
       </c>
       <c r="C42" s="63" t="n">
-        <v>8</v>
+        <v>80000</v>
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
-          <t>x p.a.</t>
+          <t>£/agreement</t>
         </is>
       </c>
       <c r="E42" s="71" t="n">
-        <v>0.2395547613874036</v>
+        <v>0.2144786405522011</v>
       </c>
       <c r="F42" s="71" t="n">
-        <v>-0.1142215421111091</v>
+        <v>-0.1051256445005265</v>
       </c>
       <c r="G42" s="71" t="n">
-        <v>0.2206618790426836</v>
+        <v>0.04451741174847898</v>
       </c>
       <c r="H42" s="71" t="n">
-        <v>0.1143521569080781</v>
+        <v>0.1052362748127385</v>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — service fee</t>
+          <t>Head office: risk, compliance, financial crime, audit</t>
         </is>
       </c>
       <c r="C43" s="63" t="n">
-        <v>0.01</v>
+        <v>250</v>
       </c>
       <c r="D43" s="14" t="inlineStr">
         <is>
-          <t>% of funded invoices</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E43" s="71" t="n">
-        <v>0.2395547613874036</v>
+        <v>-0.2130062561074872</v>
       </c>
       <c r="F43" s="71" t="n">
-        <v>-0.1142215421111091</v>
+        <v>0.1738251813009527</v>
       </c>
       <c r="G43" s="71" t="n">
-        <v>0.2206618790426836</v>
+        <v>-0.2130062561076665</v>
       </c>
       <c r="H43" s="71" t="n">
-        <v>0.1143521569080781</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>Bank of England Bank Rate</t>
+          <t>Asset finance — penetration</t>
         </is>
       </c>
       <c r="C44" s="63" t="n">
-        <v>0.0375</v>
+        <v>0.08</v>
       </c>
       <c r="D44" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E44" s="71" t="n">
-        <v>0.1990512830997236</v>
+        <v>0.2052216246454376</v>
       </c>
       <c r="F44" s="71" t="n">
-        <v>-0.09492750668173035</v>
+        <v>-0.09757933615100182</v>
       </c>
       <c r="G44" s="71" t="n">
-        <v>0.1931242862657616</v>
+        <v>0.03527609550751072</v>
       </c>
       <c r="H44" s="71" t="n">
-        <v>0.09501770461968793</v>
+        <v>0.1052362748127385</v>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>International payments &amp; FX — penetration</t>
+          <t>Head office: finance, HR, exec, brand &amp; residual (non-acquisition) marketing</t>
         </is>
       </c>
       <c r="C45" s="63" t="n">
-        <v>0.2</v>
+        <v>222</v>
       </c>
       <c r="D45" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E45" s="71" t="n">
-        <v>0.1687945307331029</v>
+        <v>-0.1891495554234487</v>
       </c>
       <c r="F45" s="71" t="n">
-        <v>-0.08000540090128463</v>
+        <v>0.154356760995188</v>
       </c>
       <c r="G45" s="71" t="n">
-        <v>0.1554207840445721</v>
+        <v>-0.1891495554236863</v>
       </c>
       <c r="H45" s="71" t="n">
-        <v>0.08099944447655529</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — average balance</t>
+          <t>Business credit card — penetration</t>
         </is>
       </c>
       <c r="C46" s="63" t="n">
-        <v>80000</v>
+        <v>0.3</v>
       </c>
       <c r="D46" s="14" t="inlineStr">
         <is>
-          <t>£/agreement</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E46" s="71" t="n">
-        <v>0.1658745747382735</v>
+        <v>0.1489064227671268</v>
       </c>
       <c r="F46" s="71" t="n">
-        <v>-0.09273546655296665</v>
+        <v>-0.06216818662197646</v>
       </c>
       <c r="G46" s="71" t="n">
-        <v>0.008961968797843937</v>
+        <v>0.1352333983522107</v>
       </c>
       <c r="H46" s="71" t="n">
-        <v>0.09282154504571802</v>
+        <v>0.06533102015084027</v>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>Head office: risk, compliance, financial crime, audit</t>
+          <t>Equity held against RWAs (CET1 target)</t>
         </is>
       </c>
       <c r="C47" s="63" t="n">
-        <v>250</v>
+        <v>0.14</v>
       </c>
       <c r="D47" s="14" t="inlineStr">
         <is>
-          <t>£/customer/yr</t>
+          <t>% of RWA</t>
         </is>
       </c>
       <c r="E47" s="71" t="n">
-        <v>-0.1647358546168127</v>
+        <v>0.1479233794011383</v>
       </c>
       <c r="F47" s="71" t="n">
-        <v>0.1719812125220667</v>
+        <v>-0.06187568430169751</v>
       </c>
       <c r="G47" s="71" t="n">
-        <v>-0.1647358546170901</v>
+        <v>-0.8436402184144726</v>
       </c>
       <c r="H47" s="71" t="n">
-        <v>0</v>
+        <v>0.06191399400909547</v>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — penetration</t>
+          <t>Overdraft — interest rate (EAR)</t>
         </is>
       </c>
       <c r="C48" s="63" t="n">
-        <v>0.08</v>
+        <v>0.0975</v>
       </c>
       <c r="D48" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E48" s="71" t="n">
-        <v>0.1587153370028682</v>
+        <v>0.141564685857882</v>
       </c>
       <c r="F48" s="71" t="n">
-        <v>-0.08526828474335443</v>
+        <v>-0.05921744646463147</v>
       </c>
       <c r="G48" s="71" t="n">
-        <v>0.001813946205839392</v>
+        <v>0.1322235784995538</v>
       </c>
       <c r="H48" s="71" t="n">
-        <v>0.09282154504571802</v>
+        <v>0.05925253430247758</v>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Head office: finance, HR, exec, brand &amp; residual (non-acquisition) marketing</t>
+          <t>Card — average monthly spend</t>
         </is>
       </c>
       <c r="C49" s="63" t="n">
-        <v>222</v>
+        <v>2500</v>
       </c>
       <c r="D49" s="14" t="inlineStr">
         <is>
-          <t>£/customer/yr</t>
+          <t>£/card/month</t>
         </is>
       </c>
       <c r="E49" s="71" t="n">
-        <v>-0.1462854388997297</v>
+        <v>0.1316430583019145</v>
       </c>
       <c r="F49" s="71" t="n">
-        <v>0.1527193167196385</v>
+        <v>-0.05506944942967034</v>
       </c>
       <c r="G49" s="71" t="n">
-        <v>-0.1462854388999867</v>
+        <v>0.1229574306786514</v>
       </c>
       <c r="H49" s="71" t="n">
-        <v>0</v>
+        <v>0.05509979258210067</v>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>Equity held against RWAs (CET1 target)</t>
+          <t>Card — commercial interchange earned</t>
         </is>
       </c>
       <c r="C50" s="63" t="n">
-        <v>0.14</v>
+        <v>0.017</v>
       </c>
       <c r="D50" s="14" t="inlineStr">
         <is>
-          <t>% of RWA</t>
+          <t>% of spend</t>
         </is>
       </c>
       <c r="E50" s="71" t="n">
-        <v>0.1238711722148994</v>
+        <v>0.1316430583019145</v>
       </c>
       <c r="F50" s="71" t="n">
-        <v>-0.05909531843834973</v>
+        <v>-0.05506944942967034</v>
       </c>
       <c r="G50" s="71" t="n">
-        <v>-0.8674542849359645</v>
+        <v>0.1229574306786514</v>
       </c>
       <c r="H50" s="71" t="n">
-        <v>0.05913026165485447</v>
+        <v>0.05509979258210067</v>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>Business credit card — penetration</t>
+          <t>Term funding premium over Bank Rate</t>
         </is>
       </c>
       <c r="C51" s="63" t="n">
-        <v>0.3</v>
+        <v>0.006</v>
       </c>
       <c r="D51" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E51" s="71" t="n">
-        <v>0.115162001627308</v>
+        <v>-0.129836192795824</v>
       </c>
       <c r="F51" s="71" t="n">
-        <v>-0.05450341134971946</v>
+        <v>0.05437306915937036</v>
       </c>
       <c r="G51" s="71" t="n">
-        <v>0.1025383467743691</v>
+        <v>-0.1212906772764059</v>
       </c>
       <c r="H51" s="71" t="n">
-        <v>0.05762391571351869</v>
+        <v>-0.05434352091919858</v>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — interest rate (EAR)</t>
+          <t>Behavioural term credit for stable non-maturing deposits</t>
         </is>
       </c>
       <c r="C52" s="63" t="n">
-        <v>0.0975</v>
+        <v>0.005</v>
       </c>
       <c r="D52" s="14" t="inlineStr">
         <is>
@@ -8923,283 +8930,283 @@
         </is>
       </c>
       <c r="E52" s="71" t="n">
-        <v>0.1094840120404391</v>
+        <v>0.1290618218646272</v>
       </c>
       <c r="F52" s="71" t="n">
-        <v>-0.05223520978052387</v>
+        <v>-0.05399023928653108</v>
       </c>
       <c r="G52" s="71" t="n">
-        <v>0.1008596961142311</v>
+        <v>0.1205467056942764</v>
       </c>
       <c r="H52" s="71" t="n">
-        <v>0.05226250921193411</v>
+        <v>0.05401940449224688</v>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>Card — average monthly spend</t>
+          <t>FX — average annual conversion volume</t>
         </is>
       </c>
       <c r="C53" s="63" t="n">
-        <v>2500</v>
+        <v>100000</v>
       </c>
       <c r="D53" s="14" t="inlineStr">
         <is>
-          <t>£/card/month</t>
+          <t>£/user/yr</t>
         </is>
       </c>
       <c r="E53" s="71" t="n">
-        <v>0.1018107735896629</v>
+        <v>0.1290618218646272</v>
       </c>
       <c r="F53" s="71" t="n">
-        <v>-0.04857605888322602</v>
+        <v>-0.05399023928653108</v>
       </c>
       <c r="G53" s="71" t="n">
-        <v>0.09379146319211618</v>
+        <v>0.1205467056942764</v>
       </c>
       <c r="H53" s="71" t="n">
-        <v>0.04859966668594098</v>
+        <v>0.05401940449224688</v>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>Card — commercial interchange earned</t>
+          <t>FX — margin on conversion volume</t>
         </is>
       </c>
       <c r="C54" s="63" t="n">
-        <v>0.017</v>
+        <v>0.0075</v>
       </c>
       <c r="D54" s="14" t="inlineStr">
         <is>
-          <t>% of spend</t>
+          <t>% of volume</t>
         </is>
       </c>
       <c r="E54" s="71" t="n">
-        <v>0.1018107735896629</v>
+        <v>0.1290618218646272</v>
       </c>
       <c r="F54" s="71" t="n">
-        <v>-0.04857605888322602</v>
+        <v>-0.05399023928653108</v>
       </c>
       <c r="G54" s="71" t="n">
-        <v>0.09379146319211618</v>
+        <v>0.1205467056942764</v>
       </c>
       <c r="H54" s="71" t="n">
-        <v>0.04859966668594098</v>
+        <v>0.05401940449224688</v>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>Term funding premium over Bank Rate</t>
+          <t>Overdraft — average limit</t>
         </is>
       </c>
       <c r="C55" s="63" t="n">
-        <v>0.006</v>
+        <v>15000</v>
       </c>
       <c r="D55" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/facility</t>
         </is>
       </c>
       <c r="E55" s="71" t="n">
-        <v>-0.1004133708148834</v>
+        <v>0.1230830424521848</v>
       </c>
       <c r="F55" s="71" t="n">
-        <v>0.04795559880866109</v>
+        <v>-0.0590550445253119</v>
       </c>
       <c r="G55" s="71" t="n">
-        <v>-0.09251885130815904</v>
+        <v>0.07584524768646449</v>
       </c>
       <c r="H55" s="71" t="n">
-        <v>-0.04793261243730116</v>
+        <v>0.0590899401158306</v>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>Behavioural term credit for stable non-maturing deposits</t>
+          <t>Overdraft — penetration</t>
         </is>
       </c>
       <c r="C56" s="63" t="n">
-        <v>0.005</v>
+        <v>0.25</v>
       </c>
       <c r="D56" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E56" s="71" t="n">
-        <v>0.09981448391141816</v>
+        <v>0.1051536008356984</v>
       </c>
       <c r="F56" s="71" t="n">
-        <v>-0.04762404074601882</v>
+        <v>-0.04443224426671098</v>
       </c>
       <c r="G56" s="71" t="n">
-        <v>0.09195255933441075</v>
+        <v>0.05792426513148669</v>
       </c>
       <c r="H56" s="71" t="n">
-        <v>0.04764673204503252</v>
+        <v>0.0590899401158306</v>
       </c>
     </row>
     <row r="57">
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>FX — average annual conversion volume</t>
+          <t>Productive hours per FTE per month</t>
         </is>
       </c>
       <c r="C57" s="63" t="n">
-        <v>100000</v>
+        <v>147</v>
       </c>
       <c r="D57" s="14" t="inlineStr">
         <is>
-          <t>£/user/yr</t>
+          <t>hours</t>
         </is>
       </c>
       <c r="E57" s="71" t="n">
-        <v>0.09981448391141816</v>
+        <v>0.1049299343026391</v>
       </c>
       <c r="F57" s="71" t="n">
-        <v>-0.04762404074601882</v>
+        <v>-0.08562877535793163</v>
       </c>
       <c r="G57" s="71" t="n">
-        <v>0.09195255933441075</v>
+        <v>0.1049299343027884</v>
       </c>
       <c r="H57" s="71" t="n">
-        <v>0.04764673204503252</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>FX — margin on conversion volume</t>
+          <t>Customers per relationship manager (L)</t>
         </is>
       </c>
       <c r="C58" s="63" t="n">
-        <v>0.0075</v>
+        <v>120</v>
       </c>
       <c r="D58" s="14" t="inlineStr">
         <is>
-          <t>% of volume</t>
+          <t>customers</t>
         </is>
       </c>
       <c r="E58" s="71" t="n">
-        <v>0.09981448391141816</v>
+        <v>0.1048340737728719</v>
       </c>
       <c r="F58" s="71" t="n">
-        <v>-0.04762404074601882</v>
+        <v>-0.0855505477307521</v>
       </c>
       <c r="G58" s="71" t="n">
-        <v>0.09195255933441075</v>
+        <v>0.1048340737730304</v>
       </c>
       <c r="H58" s="71" t="n">
-        <v>0.04764673204503252</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — average limit</t>
+          <t>Share of customers that are relationship-managed</t>
         </is>
       </c>
       <c r="C59" s="63" t="n">
-        <v>15000</v>
+        <v>0.15</v>
       </c>
       <c r="D59" s="14" t="inlineStr">
         <is>
-          <t>£/facility</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E59" s="71" t="n">
-        <v>0.09519058528012668</v>
+        <v>-0.1046385357465969</v>
       </c>
       <c r="F59" s="71" t="n">
-        <v>-0.05209194641982378</v>
+        <v>0.08539097761546771</v>
       </c>
       <c r="G59" s="71" t="n">
-        <v>0.051574506124141</v>
+        <v>-0.1046385357468233</v>
       </c>
       <c r="H59" s="71" t="n">
-        <v>0.05211909627141639</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>Productive hours per FTE per month</t>
+          <t>BCA — net transaction &amp; cash-handling income</t>
         </is>
       </c>
       <c r="C60" s="63" t="n">
-        <v>147</v>
+        <v>120</v>
       </c>
       <c r="D60" s="14" t="inlineStr">
         <is>
-          <t>hours</t>
+          <t>£/account/yr</t>
         </is>
       </c>
       <c r="E60" s="71" t="n">
-        <v>0.09121190632452875</v>
+        <v>0.1032494574917018</v>
       </c>
       <c r="F60" s="71" t="n">
-        <v>-0.09522355823886089</v>
+        <v>-0.04319685584629245</v>
       </c>
       <c r="G60" s="71" t="n">
-        <v>0.09121190632435788</v>
+        <v>0.0964390048174012</v>
       </c>
       <c r="H60" s="71" t="n">
-        <v>0</v>
+        <v>0.0432155235937975</v>
       </c>
     </row>
     <row r="61">
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — penetration</t>
+          <t>Change-the-bank / transformation spend per customer</t>
         </is>
       </c>
       <c r="C61" s="63" t="n">
-        <v>0.25</v>
+        <v>120</v>
       </c>
       <c r="D61" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E61" s="71" t="n">
-        <v>0.08132422312990931</v>
+        <v>-0.1022430029315939</v>
       </c>
       <c r="F61" s="71" t="n">
-        <v>-0.0376232594615131</v>
+        <v>0.0834360870245049</v>
       </c>
       <c r="G61" s="71" t="n">
-        <v>0.0377141861854879</v>
+        <v>-0.1022430029318107</v>
       </c>
       <c r="H61" s="71" t="n">
-        <v>0.05211909627141639</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Customers per relationship manager (L)</t>
+          <t>Term loans — probability of default</t>
         </is>
       </c>
       <c r="C62" s="63" t="n">
-        <v>120</v>
+        <v>0.018</v>
       </c>
       <c r="D62" s="14" t="inlineStr">
         <is>
-          <t>customers</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E62" s="71" t="n">
-        <v>0.08107710567534358</v>
+        <v>-0.1012205729022779</v>
       </c>
       <c r="F62" s="71" t="n">
-        <v>-0.08464301213748615</v>
+        <v>0</v>
       </c>
       <c r="G62" s="71" t="n">
-        <v>0.08107710567522457</v>
+        <v>-0.1012205729024857</v>
       </c>
       <c r="H62" s="71" t="n">
         <v>0</v>
@@ -9208,11 +9215,11 @@
     <row r="63">
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>Share of customers that are relationship-managed</t>
+          <t>Term loans — loss given default</t>
         </is>
       </c>
       <c r="C63" s="63" t="n">
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
       <c r="D63" s="14" t="inlineStr">
         <is>
@@ -9220,13 +9227,13 @@
         </is>
       </c>
       <c r="E63" s="71" t="n">
-        <v>-0.08092587948856705</v>
+        <v>-0.1012205729022779</v>
       </c>
       <c r="F63" s="71" t="n">
-        <v>0.08448513477060619</v>
+        <v>0</v>
       </c>
       <c r="G63" s="71" t="n">
-        <v>-0.08092587948885854</v>
+        <v>-0.1012205729024857</v>
       </c>
       <c r="H63" s="71" t="n">
         <v>0</v>
@@ -9235,92 +9242,92 @@
     <row r="64">
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>BCA — net transaction &amp; cash-handling income</t>
+          <t>Term loans — arrangement fee</t>
         </is>
       </c>
       <c r="C64" s="63" t="n">
-        <v>120</v>
+        <v>0.015</v>
       </c>
       <c r="D64" s="14" t="inlineStr">
         <is>
-          <t>£/account/yr</t>
+          <t>% of loan</t>
         </is>
       </c>
       <c r="E64" s="71" t="n">
-        <v>0.07985158712913452</v>
+        <v>0.09679636639847039</v>
       </c>
       <c r="F64" s="71" t="n">
-        <v>-0.03810286182134639</v>
+        <v>-0.04049814572625951</v>
       </c>
       <c r="G64" s="71" t="n">
-        <v>0.07356320301076685</v>
+        <v>0.09041195146079069</v>
       </c>
       <c r="H64" s="71" t="n">
-        <v>0.03811738563602602</v>
+        <v>0.04051455336918516</v>
       </c>
     </row>
     <row r="65">
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>Change-the-bank / transformation spend per customer</t>
+          <t>Invoice finance — average funds in use (advances)</t>
         </is>
       </c>
       <c r="C65" s="63" t="n">
-        <v>120</v>
+        <v>150000</v>
       </c>
       <c r="D65" s="14" t="inlineStr">
         <is>
-          <t>£/customer/yr</t>
+          <t>£/client</t>
         </is>
       </c>
       <c r="E65" s="71" t="n">
-        <v>-0.07907321021607008</v>
+        <v>0.09492162631565762</v>
       </c>
       <c r="F65" s="71" t="n">
-        <v>0.08255098201058327</v>
+        <v>-0.04145064460605613</v>
       </c>
       <c r="G65" s="71" t="n">
-        <v>-0.0790732102163739</v>
+        <v>0.0692404302199741</v>
       </c>
       <c r="H65" s="71" t="n">
-        <v>0</v>
+        <v>0.04146783329037527</v>
       </c>
     </row>
     <row r="66">
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>Term loans — probability of default</t>
+          <t>Term loans — risk weight</t>
         </is>
       </c>
       <c r="C66" s="63" t="n">
-        <v>0.018</v>
+        <v>0.7</v>
       </c>
       <c r="D66" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E66" s="71" t="n">
-        <v>-0.07828247811390938</v>
+        <v>0.09393575894340188</v>
       </c>
       <c r="F66" s="71" t="n">
-        <v>0</v>
+        <v>-0.03930178091372589</v>
       </c>
       <c r="G66" s="71" t="n">
-        <v>-0.07828247811415756</v>
+        <v>-0.5376796480568484</v>
       </c>
       <c r="H66" s="71" t="n">
-        <v>0</v>
+        <v>0.03931723328663613</v>
       </c>
     </row>
     <row r="67">
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>Term loans — loss given default</t>
+          <t>Invoice finance — penetration</t>
         </is>
       </c>
       <c r="C67" s="63" t="n">
-        <v>0.25</v>
+        <v>0.0071</v>
       </c>
       <c r="D67" s="14" t="inlineStr">
         <is>
@@ -9328,499 +9335,499 @@
         </is>
       </c>
       <c r="E67" s="71" t="n">
-        <v>-0.07828247811390938</v>
+        <v>0.09084805718049918</v>
       </c>
       <c r="F67" s="71" t="n">
-        <v>0</v>
+        <v>-0.03812775917075606</v>
       </c>
       <c r="G67" s="71" t="n">
-        <v>-0.07828247811415756</v>
+        <v>0.06516790623385817</v>
       </c>
       <c r="H67" s="71" t="n">
-        <v>0</v>
+        <v>0.04146783329037527</v>
       </c>
     </row>
     <row r="68">
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>Term loans — arrangement fee</t>
+          <t>International payments — number per user per year</t>
         </is>
       </c>
       <c r="C68" s="63" t="n">
-        <v>0.015</v>
+        <v>30</v>
       </c>
       <c r="D68" s="14" t="inlineStr">
         <is>
-          <t>% of loan</t>
+          <t>payments</t>
         </is>
       </c>
       <c r="E68" s="71" t="n">
-        <v>0.07486086293356362</v>
+        <v>0.09034327530523904</v>
       </c>
       <c r="F68" s="71" t="n">
-        <v>-0.03572228365829964</v>
+        <v>-0.03779928987864309</v>
       </c>
       <c r="G68" s="71" t="n">
-        <v>0.0689657736584007</v>
+        <v>0.08438484684763596</v>
       </c>
       <c r="H68" s="71" t="n">
-        <v>0.03573504903377439</v>
+        <v>0.03781358314457282</v>
       </c>
     </row>
     <row r="69">
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — discount margin over base</t>
+          <t>International payment fee</t>
         </is>
       </c>
       <c r="C69" s="63" t="n">
-        <v>0.025</v>
+        <v>17.5</v>
       </c>
       <c r="D69" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/payment</t>
         </is>
       </c>
       <c r="E69" s="71" t="n">
-        <v>0.07486086293356362</v>
+        <v>0.09034327530523904</v>
       </c>
       <c r="F69" s="71" t="n">
-        <v>-0.03572228365829964</v>
+        <v>-0.03779928987864309</v>
       </c>
       <c r="G69" s="71" t="n">
-        <v>0.0689657736584007</v>
+        <v>0.08438484684763596</v>
       </c>
       <c r="H69" s="71" t="n">
-        <v>0.03573504903377439</v>
+        <v>0.03781358314457282</v>
       </c>
     </row>
     <row r="70">
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>Term loans — risk weight</t>
+          <t>BCA — monthly account fee</t>
         </is>
       </c>
       <c r="C70" s="63" t="n">
-        <v>0.7</v>
+        <v>8.5</v>
       </c>
       <c r="D70" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/month</t>
         </is>
       </c>
       <c r="E70" s="71" t="n">
-        <v>0.07264851188601439</v>
+        <v>0.08776203886793855</v>
       </c>
       <c r="F70" s="71" t="n">
-        <v>-0.03466695472918382</v>
+        <v>-0.0367197067332557</v>
       </c>
       <c r="G70" s="71" t="n">
-        <v>-0.5108399059911144</v>
+        <v>0.08197399065083791</v>
       </c>
       <c r="H70" s="71" t="n">
-        <v>0.03467897687449064</v>
+        <v>0.03673319505471902</v>
       </c>
     </row>
     <row r="71">
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>International payments — number per user per year</t>
+          <t>Relationship manager — salary</t>
         </is>
       </c>
       <c r="C71" s="63" t="n">
-        <v>30</v>
+        <v>65000</v>
       </c>
       <c r="D71" s="14" t="inlineStr">
         <is>
-          <t>payments</t>
+          <t>£/yr</t>
         </is>
       </c>
       <c r="E71" s="71" t="n">
-        <v>0.06987013873799271</v>
+        <v>-0.08359164263118203</v>
       </c>
       <c r="F71" s="71" t="n">
-        <v>-0.03334159210622355</v>
+        <v>0.0682155195867932</v>
       </c>
       <c r="G71" s="71" t="n">
-        <v>0.06436830819666425</v>
+        <v>-0.08359164263111851</v>
       </c>
       <c r="H71" s="71" t="n">
-        <v>0.03335271243152277</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>International payment fee</t>
+          <t>Instant-access savings — average balance</t>
         </is>
       </c>
       <c r="C72" s="63" t="n">
-        <v>17.5</v>
+        <v>30000</v>
       </c>
       <c r="D72" s="14" t="inlineStr">
         <is>
-          <t>£/payment</t>
+          <t>£/account</t>
         </is>
       </c>
       <c r="E72" s="71" t="n">
-        <v>0.06987013873799271</v>
+        <v>0.07891881788782402</v>
       </c>
       <c r="F72" s="71" t="n">
-        <v>-0.03334159210622355</v>
+        <v>-0.03155780944412719</v>
       </c>
       <c r="G72" s="71" t="n">
-        <v>0.06436830819666425</v>
+        <v>0.07347170588420676</v>
       </c>
       <c r="H72" s="71" t="n">
-        <v>0.03335271243152277</v>
+        <v>0.03457241887503357</v>
       </c>
     </row>
     <row r="73">
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>BCA — monthly account fee</t>
+          <t>Term loans — average life</t>
         </is>
       </c>
       <c r="C73" s="63" t="n">
-        <v>8.5</v>
+        <v>4</v>
       </c>
       <c r="D73" s="14" t="inlineStr">
         <is>
-          <t>£/month</t>
+          <t>years</t>
         </is>
       </c>
       <c r="E73" s="71" t="n">
-        <v>0.06787384905976844</v>
+        <v>-0.07829491028629054</v>
       </c>
       <c r="F73" s="71" t="n">
-        <v>-0.03238928373466862</v>
+        <v>0.02580762668294011</v>
       </c>
       <c r="G73" s="71" t="n">
-        <v>0.06252931190123294</v>
+        <v>-0.07198396348042548</v>
       </c>
       <c r="H73" s="71" t="n">
-        <v>0.03239977779061431</v>
+        <v>-0.0401134191773455</v>
       </c>
     </row>
     <row r="74">
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>Relationship manager — salary</t>
+          <t>BCA — credit interest paid</t>
         </is>
       </c>
       <c r="C74" s="63" t="n">
-        <v>65000</v>
+        <v>0.005</v>
       </c>
       <c r="D74" s="14" t="inlineStr">
         <is>
-          <t>£/yr</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E74" s="71" t="n">
-        <v>-0.06464852694618542</v>
+        <v>-0.07743709311877632</v>
       </c>
       <c r="F74" s="71" t="n">
-        <v>0.06749187708921207</v>
+        <v>0.03242215124722145</v>
       </c>
       <c r="G74" s="71" t="n">
-        <v>-0.06464852694648321</v>
+        <v>-0.07233786615856722</v>
       </c>
       <c r="H74" s="71" t="n">
-        <v>0</v>
+        <v>-0.03241164269534813</v>
       </c>
     </row>
     <row r="75">
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>Instant-access savings — average balance</t>
+          <t>Instant-access savings — penetration</t>
         </is>
       </c>
       <c r="C75" s="63" t="n">
-        <v>30000</v>
+        <v>0.4</v>
       </c>
       <c r="D75" s="14" t="inlineStr">
         <is>
-          <t>£/account</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E75" s="71" t="n">
-        <v>0.06103463413552909</v>
+        <v>0.07661700997629903</v>
       </c>
       <c r="F75" s="71" t="n">
-        <v>-0.02751368315916409</v>
+        <v>-0.02968005287393479</v>
       </c>
       <c r="G75" s="71" t="n">
-        <v>0.05600480950303754</v>
+        <v>0.07117002325613006</v>
       </c>
       <c r="H75" s="71" t="n">
-        <v>0.03049390850881691</v>
+        <v>0.03457241887503357</v>
       </c>
     </row>
     <row r="76">
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t>Term loans — average life</t>
+          <t>Overdraft — average utilisation</t>
         </is>
       </c>
       <c r="C76" s="63" t="n">
-        <v>4</v>
+        <v>0.45</v>
       </c>
       <c r="D76" s="14" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>% of limit</t>
         </is>
       </c>
       <c r="E76" s="71" t="n">
-        <v>-0.0605521133221927</v>
+        <v>0.07468485925308183</v>
       </c>
       <c r="F76" s="71" t="n">
-        <v>0.02122446956929888</v>
+        <v>-0.03881758952731159</v>
       </c>
       <c r="G76" s="71" t="n">
-        <v>-0.05472260563925134</v>
+        <v>0.03065869518523666</v>
       </c>
       <c r="H76" s="71" t="n">
-        <v>-0.03538123666704555</v>
+        <v>0.03883266343130445</v>
       </c>
     </row>
     <row r="77">
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>BCA — credit interest paid</t>
+          <t>Invoice finance — funded invoices as multiple of advances</t>
         </is>
       </c>
       <c r="C77" s="63" t="n">
-        <v>0.005</v>
+        <v>8</v>
       </c>
       <c r="D77" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>x p.a.</t>
         </is>
       </c>
       <c r="E77" s="71" t="n">
-        <v>-0.0598886903468509</v>
+        <v>0.07330711481910879</v>
       </c>
       <c r="F77" s="71" t="n">
-        <v>0.02859621432394117</v>
+        <v>-0.03067361016112366</v>
       </c>
       <c r="G77" s="71" t="n">
-        <v>-0.05517846962304982</v>
+        <v>0.06847304438958647</v>
       </c>
       <c r="H77" s="71" t="n">
-        <v>-0.02858803922701951</v>
+        <v>0.03068302175159092</v>
       </c>
     </row>
     <row r="78">
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t>Instant-access savings — penetration</t>
+          <t>Invoice finance — service fee</t>
         </is>
       </c>
       <c r="C78" s="63" t="n">
-        <v>0.4</v>
+        <v>0.01</v>
       </c>
       <c r="D78" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% of funded invoices</t>
         </is>
       </c>
       <c r="E78" s="71" t="n">
-        <v>0.0592544503026677</v>
+        <v>0.07330711481910879</v>
       </c>
       <c r="F78" s="71" t="n">
-        <v>-0.02565577041929928</v>
+        <v>-0.03067361016112366</v>
       </c>
       <c r="G78" s="71" t="n">
-        <v>0.05422471515567431</v>
+        <v>0.06847304438958647</v>
       </c>
       <c r="H78" s="71" t="n">
-        <v>0.03049390850881691</v>
+        <v>0.03068302175159092</v>
       </c>
     </row>
     <row r="79">
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — average utilisation</t>
+          <t>Credit analyst / underwriter — salary</t>
         </is>
       </c>
       <c r="C79" s="63" t="n">
-        <v>0.45</v>
+        <v>55000</v>
       </c>
       <c r="D79" s="14" t="inlineStr">
         <is>
-          <t>% of limit</t>
+          <t>£/yr</t>
         </is>
       </c>
       <c r="E79" s="71" t="n">
-        <v>0.05776015381344716</v>
+        <v>-0.0568734448830966</v>
       </c>
       <c r="F79" s="71" t="n">
-        <v>-0.03423984406982809</v>
+        <v>0.04641195544512514</v>
       </c>
       <c r="G79" s="71" t="n">
-        <v>0.01710511817772802</v>
+        <v>-0.05687344488291048</v>
       </c>
       <c r="H79" s="71" t="n">
-        <v>0.03425157175458779</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t>Credit analyst / underwriter — salary</t>
+          <t>Liquidity buffer held against deposits (LCR / HQLA)</t>
         </is>
       </c>
       <c r="C80" s="63" t="n">
-        <v>55000</v>
+        <v>0.15</v>
       </c>
       <c r="D80" s="14" t="inlineStr">
         <is>
-          <t>£/yr</t>
+          <t>% of deposits</t>
         </is>
       </c>
       <c r="E80" s="71" t="n">
-        <v>-0.05171141124509487</v>
+        <v>-0.05323800151894711</v>
       </c>
       <c r="F80" s="71" t="n">
-        <v>0.05398576544161963</v>
+        <v>0.02228797078263317</v>
       </c>
       <c r="G80" s="71" t="n">
-        <v>-0.05171141124499209</v>
+        <v>-0.04973148989456535</v>
       </c>
       <c r="H80" s="71" t="n">
-        <v>0</v>
+        <v>-0.02228300435307398</v>
       </c>
     </row>
     <row r="81">
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>Liquidity buffer held against deposits (LCR / HQLA)</t>
+          <t>Yield give-up on the liquidity buffer vs Bank Rate</t>
         </is>
       </c>
       <c r="C81" s="63" t="n">
-        <v>0.15</v>
+        <v>0.01</v>
       </c>
       <c r="D81" s="14" t="inlineStr">
         <is>
-          <t>% of deposits</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E81" s="71" t="n">
-        <v>-0.04117347461329634</v>
+        <v>-0.05323800151894711</v>
       </c>
       <c r="F81" s="71" t="n">
-        <v>0.01965814063393465</v>
+        <v>0.02228797078263317</v>
       </c>
       <c r="G81" s="71" t="n">
-        <v>-0.03793463915464931</v>
+        <v>-0.04973148989456535</v>
       </c>
       <c r="H81" s="71" t="n">
-        <v>-0.01965427696859545</v>
+        <v>-0.02228300435307398</v>
       </c>
     </row>
     <row r="82">
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t>Yield give-up on the liquidity buffer vs Bank Rate</t>
+          <t>Unit-level platform &amp; processing cost</t>
         </is>
       </c>
       <c r="C82" s="63" t="n">
-        <v>0.01</v>
+        <v>60</v>
       </c>
       <c r="D82" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E82" s="71" t="n">
-        <v>-0.04117347461329634</v>
+        <v>-0.05112150146579695</v>
       </c>
       <c r="F82" s="71" t="n">
-        <v>0.01965814063393465</v>
+        <v>0.04171804351234986</v>
       </c>
       <c r="G82" s="71" t="n">
-        <v>-0.03793463915464931</v>
+        <v>-0.05112150146589774</v>
       </c>
       <c r="H82" s="71" t="n">
-        <v>-0.01965427696859545</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t>Unit-level platform &amp; processing cost</t>
+          <t>Overdraft — annual arrangement/renewal fee</t>
         </is>
       </c>
       <c r="C83" s="63" t="n">
-        <v>60</v>
+        <v>0.015</v>
       </c>
       <c r="D83" s="14" t="inlineStr">
         <is>
-          <t>£/customer/yr</t>
+          <t>% of limit</t>
         </is>
       </c>
       <c r="E83" s="71" t="n">
-        <v>-0.03953660510803504</v>
+        <v>0.04839818319938068</v>
       </c>
       <c r="F83" s="71" t="n">
-        <v>0.0412754910054009</v>
+        <v>-0.0202531739430378</v>
       </c>
       <c r="G83" s="71" t="n">
-        <v>-0.03953660510795137</v>
+        <v>0.04520741744945692</v>
       </c>
       <c r="H83" s="71" t="n">
-        <v>0</v>
+        <v>0.02025727668465901</v>
       </c>
     </row>
     <row r="84">
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — annual arrangement/renewal fee</t>
+          <t>Fraud &amp; payment losses (incl. APP reimbursement) per current account</t>
         </is>
       </c>
       <c r="C84" s="63" t="n">
-        <v>0.015</v>
+        <v>45</v>
       </c>
       <c r="D84" s="14" t="inlineStr">
         <is>
-          <t>% of limit</t>
+          <t>£/BCA/yr</t>
         </is>
       </c>
       <c r="E84" s="71" t="n">
-        <v>0.03743043146690454</v>
+        <v>-0.03834112609934771</v>
       </c>
       <c r="F84" s="71" t="n">
-        <v>-0.01786433260297001</v>
+        <v>0.03128853263420828</v>
       </c>
       <c r="G84" s="71" t="n">
-        <v>0.03448390249733824</v>
+        <v>-0.03834112609929025</v>
       </c>
       <c r="H84" s="71" t="n">
-        <v>0.01786752451694579</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t>Fraud &amp; payment losses (incl. APP reimbursement) per current account</t>
+          <t>Asset finance — probability of default</t>
         </is>
       </c>
       <c r="C85" s="63" t="n">
-        <v>45</v>
+        <v>0.022</v>
       </c>
       <c r="D85" s="14" t="inlineStr">
         <is>
-          <t>£/BCA/yr</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E85" s="71" t="n">
-        <v>-0.02965245383102628</v>
+        <v>-0.03694925801944137</v>
       </c>
       <c r="F85" s="71" t="n">
-        <v>0.03095661825405067</v>
+        <v>0</v>
       </c>
       <c r="G85" s="71" t="n">
-        <v>-0.02965245383120229</v>
+        <v>-0.03694925801941038</v>
       </c>
       <c r="H85" s="71" t="n">
         <v>0</v>
@@ -9829,25 +9836,25 @@
     <row r="86">
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — probability of default</t>
+          <t>Asset finance — loss given default</t>
         </is>
       </c>
       <c r="C86" s="63" t="n">
-        <v>0.022</v>
+        <v>0.35</v>
       </c>
       <c r="D86" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E86" s="71" t="n">
-        <v>-0.02857600386260983</v>
+        <v>-0.03694925801944137</v>
       </c>
       <c r="F86" s="71" t="n">
         <v>0</v>
       </c>
       <c r="G86" s="71" t="n">
-        <v>-0.02857600386254362</v>
+        <v>-0.03694925801941038</v>
       </c>
       <c r="H86" s="71" t="n">
         <v>0</v>
@@ -9856,25 +9863,25 @@
     <row r="87">
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — loss given default</t>
+          <t>Management span (staff per manager)</t>
         </is>
       </c>
       <c r="C87" s="63" t="n">
-        <v>0.35</v>
+        <v>8</v>
       </c>
       <c r="D87" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>staff</t>
         </is>
       </c>
       <c r="E87" s="71" t="n">
-        <v>-0.02857600386260983</v>
+        <v>0.03323477624632555</v>
       </c>
       <c r="F87" s="71" t="n">
-        <v>0</v>
+        <v>-0.02712146165108484</v>
       </c>
       <c r="G87" s="71" t="n">
-        <v>-0.02857600386254362</v>
+        <v>0.03323477624586131</v>
       </c>
       <c r="H87" s="71" t="n">
         <v>0</v>
@@ -9883,25 +9890,25 @@
     <row r="88">
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t>Management span (staff per manager)</t>
+          <t>Annual customer churn (replaced at steady state)</t>
         </is>
       </c>
       <c r="C88" s="63" t="n">
-        <v>8</v>
+        <v>0.12</v>
       </c>
       <c r="D88" s="14" t="inlineStr">
         <is>
-          <t>staff</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E88" s="71" t="n">
-        <v>0.02728475739292511</v>
+        <v>-0.03192622160754524</v>
       </c>
       <c r="F88" s="71" t="n">
-        <v>-0.0284847865736678</v>
+        <v>0.02605360687805449</v>
       </c>
       <c r="G88" s="71" t="n">
-        <v>0.02728475739261982</v>
+        <v>-0.03192622160733487</v>
       </c>
       <c r="H88" s="71" t="n">
         <v>0</v>
@@ -9922,13 +9929,13 @@
         </is>
       </c>
       <c r="E89" s="71" t="n">
-        <v>-0.0257511658564655</v>
+        <v>-0.03136675261572086</v>
       </c>
       <c r="F89" s="71" t="n">
-        <v>0.02688374512136233</v>
+        <v>0.02559704846183944</v>
       </c>
       <c r="G89" s="71" t="n">
-        <v>-0.02575116585676012</v>
+        <v>-0.0313667526155505</v>
       </c>
       <c r="H89" s="71" t="n">
         <v>0</v>
@@ -9937,25 +9944,25 @@
     <row r="90">
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t>Annual customer churn (replaced at steady state)</t>
+          <t>Employment on-costs (NI, pension, benefits)</t>
         </is>
       </c>
       <c r="C90" s="63" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="D90" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>% of salary</t>
         </is>
       </c>
       <c r="E90" s="71" t="n">
-        <v>-0.02469126258220576</v>
+        <v>-0.02505108334161372</v>
       </c>
       <c r="F90" s="71" t="n">
-        <v>0.02577722553153486</v>
+        <v>0.02044310426958103</v>
       </c>
       <c r="G90" s="71" t="n">
-        <v>-0.02469126258230462</v>
+        <v>-0.02505108334171299</v>
       </c>
       <c r="H90" s="71" t="n">
         <v>0</v>
@@ -9964,25 +9971,25 @@
     <row r="91">
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t>Employment on-costs (NI, pension, benefits)</t>
+          <t>Churn replacement — acquisition marketing per new customer won</t>
         </is>
       </c>
       <c r="C91" s="63" t="n">
-        <v>0.15</v>
+        <v>240</v>
       </c>
       <c r="D91" s="14" t="inlineStr">
         <is>
-          <t>% of salary</t>
+          <t>£/new customer</t>
         </is>
       </c>
       <c r="E91" s="71" t="n">
-        <v>-0.02057660219051082</v>
+        <v>-0.02361813367720083</v>
       </c>
       <c r="F91" s="71" t="n">
-        <v>0.02148159550679803</v>
+        <v>0.01927373610267698</v>
       </c>
       <c r="G91" s="71" t="n">
-        <v>-0.02057660219063057</v>
+        <v>-0.02361813367739114</v>
       </c>
       <c r="H91" s="71" t="n">
         <v>0</v>
@@ -9991,38 +9998,38 @@
     <row r="92">
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t>Operational-risk RWA multiple of gross income</t>
+          <t>Invoice finance — discount margin over base</t>
         </is>
       </c>
       <c r="C92" s="63" t="n">
-        <v>1.875</v>
+        <v>0.025</v>
       </c>
       <c r="D92" s="14" t="inlineStr">
         <is>
-          <t>x revenue</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E92" s="71" t="n">
-        <v>0.01940217969118421</v>
+        <v>0.02290847338118557</v>
       </c>
       <c r="F92" s="71" t="n">
-        <v>-0.009260828777932256</v>
+        <v>-0.009587525002924749</v>
       </c>
       <c r="G92" s="71" t="n">
-        <v>-0.1370151321223097</v>
+        <v>0.02139853701481027</v>
       </c>
       <c r="H92" s="71" t="n">
-        <v>0.009261686486871161</v>
+        <v>0.009588444297347251</v>
       </c>
     </row>
     <row r="93">
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t>Share of lending balances held by RM-managed customers</t>
+          <t>Asset finance — risk weight</t>
         </is>
       </c>
       <c r="C93" s="63" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="D93" s="14" t="inlineStr">
         <is>
@@ -10030,67 +10037,67 @@
         </is>
       </c>
       <c r="E93" s="71" t="n">
-        <v>0.01833005970171241</v>
+        <v>0.02290243265667439</v>
       </c>
       <c r="F93" s="71" t="n">
-        <v>0</v>
+        <v>-0.009584997115274458</v>
       </c>
       <c r="G93" s="71" t="n">
-        <v>0.0183300597013768</v>
+        <v>-0.1317199514189854</v>
       </c>
       <c r="H93" s="71" t="n">
-        <v>0</v>
+        <v>0.009585915925127142</v>
       </c>
     </row>
     <row r="94">
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t>Stewardship effect: relative PD reduction on RM-covered balances</t>
+          <t>Operational-risk RWA multiple of gross income</t>
         </is>
       </c>
       <c r="C94" s="63" t="n">
-        <v>0.2</v>
+        <v>1.875</v>
       </c>
       <c r="D94" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>x revenue</t>
         </is>
       </c>
       <c r="E94" s="71" t="n">
-        <v>0.01833005970171241</v>
+        <v>0.0220623226696928</v>
       </c>
       <c r="F94" s="71" t="n">
-        <v>0</v>
+        <v>-0.009233431480186292</v>
       </c>
       <c r="G94" s="71" t="n">
-        <v>0.0183300597013768</v>
+        <v>-0.1268953788846724</v>
       </c>
       <c r="H94" s="71" t="n">
-        <v>0</v>
+        <v>0.009234284121481744</v>
       </c>
     </row>
     <row r="95">
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t>Churn replacement — acquisition marketing per new customer won</t>
+          <t>Share of lending balances held by RM-managed customers</t>
         </is>
       </c>
       <c r="C95" s="63" t="n">
-        <v>240</v>
+        <v>0.6</v>
       </c>
       <c r="D95" s="14" t="inlineStr">
         <is>
-          <t>£/new customer</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E95" s="71" t="n">
-        <v>-0.01826591155990401</v>
+        <v>0.02187481379496614</v>
       </c>
       <c r="F95" s="71" t="n">
-        <v>0.01906927684454543</v>
+        <v>0</v>
       </c>
       <c r="G95" s="71" t="n">
-        <v>-0.01826591156004862</v>
+        <v>0.021874813795008</v>
       </c>
       <c r="H95" s="71" t="n">
         <v>0</v>
@@ -10099,11 +10106,11 @@
     <row r="96">
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — risk weight</t>
+          <t>Stewardship effect: relative PD reduction on RM-covered balances</t>
         </is>
       </c>
       <c r="C96" s="63" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="D96" s="14" t="inlineStr">
         <is>
@@ -10111,16 +10118,16 @@
         </is>
       </c>
       <c r="E96" s="71" t="n">
-        <v>0.01771239908840788</v>
+        <v>0.02187481379496614</v>
       </c>
       <c r="F96" s="71" t="n">
-        <v>-0.008454350017280498</v>
+        <v>0</v>
       </c>
       <c r="G96" s="71" t="n">
-        <v>-0.125099206722287</v>
+        <v>0.021874813795008</v>
       </c>
       <c r="H96" s="71" t="n">
-        <v>0.008455064837974957</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -10138,16 +10145,16 @@
         </is>
       </c>
       <c r="E97" s="71" t="n">
-        <v>0.01587050294203331</v>
+        <v>0.02052082967661485</v>
       </c>
       <c r="F97" s="71" t="n">
-        <v>-0.007575256506550518</v>
+        <v>-0.008588347653644276</v>
       </c>
       <c r="G97" s="71" t="n">
-        <v>0.01462142272077909</v>
+        <v>0.01916829711878616</v>
       </c>
       <c r="H97" s="71" t="n">
-        <v>0.007575830395216416</v>
+        <v>0.008589085314331023</v>
       </c>
     </row>
     <row r="98">
@@ -10165,13 +10172,13 @@
         </is>
       </c>
       <c r="E98" s="71" t="n">
-        <v>-0.01564284608034933</v>
+        <v>-0.02022646549070539</v>
       </c>
       <c r="F98" s="71" t="n">
-        <v>0.01633084456626305</v>
+        <v>0.01650594257292187</v>
       </c>
       <c r="G98" s="71" t="n">
-        <v>-0.01564284608081514</v>
+        <v>-0.02022646549081312</v>
       </c>
       <c r="H98" s="71" t="n">
         <v>0</v>
@@ -10192,13 +10199,13 @@
         </is>
       </c>
       <c r="E99" s="71" t="n">
-        <v>-0.01399299296284985</v>
+        <v>-0.01809317740628059</v>
       </c>
       <c r="F99" s="71" t="n">
         <v>0</v>
       </c>
       <c r="G99" s="71" t="n">
-        <v>-0.01399299296281295</v>
+        <v>-0.01809317740626373</v>
       </c>
       <c r="H99" s="71" t="n">
         <v>0</v>
@@ -10219,13 +10226,13 @@
         </is>
       </c>
       <c r="E100" s="71" t="n">
-        <v>-0.01399299296284985</v>
+        <v>-0.01809317740628059</v>
       </c>
       <c r="F100" s="71" t="n">
         <v>0</v>
       </c>
       <c r="G100" s="71" t="n">
-        <v>-0.01399299296281295</v>
+        <v>-0.01809317740626373</v>
       </c>
       <c r="H100" s="71" t="n">
         <v>0</v>
@@ -10246,13 +10253,13 @@
         </is>
       </c>
       <c r="E101" s="71" t="n">
-        <v>-0.01370322847785298</v>
+        <v>-0.0177185070089608</v>
       </c>
       <c r="F101" s="71" t="n">
-        <v>0.01430591934339043</v>
+        <v>0.01445930626422265</v>
       </c>
       <c r="G101" s="71" t="n">
-        <v>-0.0137032284779602</v>
+        <v>-0.01771850700938827</v>
       </c>
       <c r="H101" s="71" t="n">
         <v>0</v>
@@ -10261,25 +10268,25 @@
     <row r="102">
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — probability of default</t>
+          <t>BCA servicing (queries, payments support)</t>
         </is>
       </c>
       <c r="C102" s="63" t="n">
-        <v>0.026</v>
+        <v>0.6</v>
       </c>
       <c r="D102" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>hrs/account/yr</t>
         </is>
       </c>
       <c r="E102" s="71" t="n">
-        <v>-0.01356896287307272</v>
+        <v>-0.01726355933582919</v>
       </c>
       <c r="F102" s="71" t="n">
-        <v>0</v>
+        <v>0.01408804316967071</v>
       </c>
       <c r="G102" s="71" t="n">
-        <v>-0.01356896287333288</v>
+        <v>-0.01726355933577883</v>
       </c>
       <c r="H102" s="71" t="n">
         <v>0</v>
@@ -10288,25 +10295,25 @@
     <row r="103">
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — loss given default</t>
+          <t>Premises &amp; facilities per unit FTE</t>
         </is>
       </c>
       <c r="C103" s="63" t="n">
-        <v>0.2</v>
+        <v>6000</v>
       </c>
       <c r="D103" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/FTE/yr</t>
         </is>
       </c>
       <c r="E103" s="71" t="n">
-        <v>-0.01356896287307272</v>
+        <v>-0.0165027854462771</v>
       </c>
       <c r="F103" s="71" t="n">
-        <v>0</v>
+        <v>0.01346720854414594</v>
       </c>
       <c r="G103" s="71" t="n">
-        <v>-0.01356896287333288</v>
+        <v>-0.01650278544651348</v>
       </c>
       <c r="H103" s="71" t="n">
         <v>0</v>
@@ -10315,25 +10322,25 @@
     <row r="104">
       <c r="B104" s="10" t="inlineStr">
         <is>
-          <t>Premises &amp; facilities per unit FTE</t>
+          <t>Overdraft annual review &amp; renewal</t>
         </is>
       </c>
       <c r="C104" s="63" t="n">
-        <v>6000</v>
+        <v>1.5</v>
       </c>
       <c r="D104" s="14" t="inlineStr">
         <is>
-          <t>£/FTE/yr</t>
+          <t>hrs/facility/yr</t>
         </is>
       </c>
       <c r="E104" s="71" t="n">
-        <v>-0.01354829332592148</v>
+        <v>-0.01582009554374381</v>
       </c>
       <c r="F104" s="71" t="n">
-        <v>0.01414416988493427</v>
+        <v>0.01291009487869291</v>
       </c>
       <c r="G104" s="71" t="n">
-        <v>-0.01354829332627234</v>
+        <v>-0.01582009554390931</v>
       </c>
       <c r="H104" s="71" t="n">
         <v>0</v>
@@ -10342,25 +10349,25 @@
     <row r="105">
       <c r="B105" s="10" t="inlineStr">
         <is>
-          <t>BCA servicing (queries, payments support)</t>
+          <t>Term loan annual review</t>
         </is>
       </c>
       <c r="C105" s="63" t="n">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="D105" s="14" t="inlineStr">
         <is>
-          <t>hrs/account/yr</t>
+          <t>hrs/loan/yr</t>
         </is>
       </c>
       <c r="E105" s="71" t="n">
-        <v>-0.01335137874766737</v>
+        <v>-0.01518729172200041</v>
       </c>
       <c r="F105" s="71" t="n">
-        <v>0.01393859467455354</v>
+        <v>0.01239369108365343</v>
       </c>
       <c r="G105" s="71" t="n">
-        <v>-0.01335137874769045</v>
+        <v>-0.01518729172225025</v>
       </c>
       <c r="H105" s="71" t="n">
         <v>0</v>
@@ -10369,55 +10376,55 @@
     <row r="106">
       <c r="B106" s="10" t="inlineStr">
         <is>
-          <t>Overdraft annual review &amp; renewal</t>
+          <t>Card — share of cards revolving a balance</t>
         </is>
       </c>
       <c r="C106" s="63" t="n">
-        <v>1.5</v>
+        <v>0.25</v>
       </c>
       <c r="D106" s="14" t="inlineStr">
         <is>
-          <t>hrs/facility/yr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E106" s="71" t="n">
-        <v>-0.01223502542667563</v>
+        <v>0.01282939010311848</v>
       </c>
       <c r="F106" s="71" t="n">
-        <v>0.01277314227084876</v>
+        <v>-0.00677352684355925</v>
       </c>
       <c r="G106" s="71" t="n">
-        <v>-0.01223502542703396</v>
+        <v>0.008393731325598055</v>
       </c>
       <c r="H106" s="71" t="n">
-        <v>0</v>
+        <v>0.00677398568124732</v>
       </c>
     </row>
     <row r="107">
       <c r="B107" s="10" t="inlineStr">
         <is>
-          <t>Term loan annual review</t>
+          <t>Card — average revolving balance (revolvers)</t>
         </is>
       </c>
       <c r="C107" s="63" t="n">
-        <v>3</v>
+        <v>2000</v>
       </c>
       <c r="D107" s="14" t="inlineStr">
         <is>
-          <t>hrs/loan/yr</t>
+          <t>£/card</t>
         </is>
       </c>
       <c r="E107" s="71" t="n">
-        <v>-0.01174562440962334</v>
+        <v>0.01282939010311848</v>
       </c>
       <c r="F107" s="71" t="n">
-        <v>0.01226221658007843</v>
+        <v>-0.00677352684355925</v>
       </c>
       <c r="G107" s="71" t="n">
-        <v>-0.01174562440975294</v>
+        <v>0.008393731325598055</v>
       </c>
       <c r="H107" s="71" t="n">
-        <v>0</v>
+        <v>0.00677398568124732</v>
       </c>
     </row>
     <row r="108">
@@ -10435,13 +10442,13 @@
         </is>
       </c>
       <c r="E108" s="71" t="n">
-        <v>-0.009785309764238673</v>
+        <v>-0.01265257161278474</v>
       </c>
       <c r="F108" s="71" t="n">
-        <v>0.01021568402375696</v>
+        <v>0.0103252157693554</v>
       </c>
       <c r="G108" s="71" t="n">
-        <v>-0.009785309764105748</v>
+        <v>-0.0126525716125313</v>
       </c>
       <c r="H108" s="71" t="n">
         <v>0</v>
@@ -10462,13 +10469,13 @@
         </is>
       </c>
       <c r="E109" s="71" t="n">
-        <v>-0.009785309764238673</v>
+        <v>-0.01265257161278474</v>
       </c>
       <c r="F109" s="71" t="n">
-        <v>0.01021568402375696</v>
+        <v>0.0103252157693554</v>
       </c>
       <c r="G109" s="71" t="n">
-        <v>-0.009785309764105748</v>
+        <v>-0.0126525716125313</v>
       </c>
       <c r="H109" s="71" t="n">
         <v>0</v>
@@ -10477,55 +10484,55 @@
     <row r="110">
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — risk weight</t>
+          <t>Overdraft — risk weight</t>
         </is>
       </c>
       <c r="C110" s="63" t="n">
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
       <c r="D110" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% of drawn</t>
         </is>
       </c>
       <c r="E110" s="71" t="n">
-        <v>0.009340522956773279</v>
+        <v>0.00566130690060681</v>
       </c>
       <c r="F110" s="71" t="n">
-        <v>-0.00445852680457372</v>
+        <v>-0.002369509251789935</v>
       </c>
       <c r="G110" s="71" t="n">
-        <v>-0.06601483744602295</v>
+        <v>-0.03259810445684302</v>
       </c>
       <c r="H110" s="71" t="n">
-        <v>0.004458725598148796</v>
+        <v>0.002369565398971374</v>
       </c>
     </row>
     <row r="111">
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — risk weight</t>
+          <t>Invoice finance — risk weight</t>
         </is>
       </c>
       <c r="C111" s="63" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="D111" s="14" t="inlineStr">
         <is>
-          <t>% of drawn</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E111" s="71" t="n">
-        <v>0.004378370135987474</v>
+        <v>0.002858330950708488</v>
       </c>
       <c r="F111" s="71" t="n">
-        <v>-0.002089983942857775</v>
+        <v>-0.001196352928703285</v>
       </c>
       <c r="G111" s="71" t="n">
-        <v>-0.03095684670595658</v>
+        <v>-0.01646153881572723</v>
       </c>
       <c r="H111" s="71" t="n">
-        <v>0.002090027624132248</v>
+        <v>0.001196367241437099</v>
       </c>
     </row>
     <row r="112">
@@ -10549,7 +10556,7 @@
         <v>0</v>
       </c>
       <c r="G112" s="71" t="n">
-        <v>-0.388888888889195</v>
+        <v>-0.3888888888889994</v>
       </c>
       <c r="H112" s="71" t="n">
         <v>0</v>
@@ -11052,25 +11059,25 @@
         <v>301.171875</v>
       </c>
       <c r="D8" s="46" t="n">
-        <v>957473.4381271362</v>
+        <v>844520.2381530761</v>
       </c>
       <c r="E8" s="46" t="n">
-        <v>621931.4444624339</v>
+        <v>617287.2083901584</v>
       </c>
       <c r="F8" s="46" t="n">
-        <v>272918.9040553273</v>
+        <v>169343.9283410428</v>
       </c>
       <c r="G8" s="46" t="n">
-        <v>-5803498.389080164</v>
+        <v>-5878072.37159445</v>
       </c>
       <c r="H8" s="46" t="n">
-        <v>-5803498.389080164</v>
+        <v>-5878072.37159445</v>
       </c>
       <c r="I8" s="46" t="n">
-        <v>2065.038259174878</v>
+        <v>2049.617708792225</v>
       </c>
       <c r="J8" s="48" t="n">
-        <v>0.6495547758264308</v>
+        <v>0.7309324045805401</v>
       </c>
     </row>
     <row r="9">
@@ -11081,25 +11088,25 @@
         <v>620.625</v>
       </c>
       <c r="D9" s="46" t="n">
-        <v>1973065.886506348</v>
+        <v>1740303.183369141</v>
       </c>
       <c r="E9" s="46" t="n">
-        <v>1143780.437777619</v>
+        <v>1134210.058696385</v>
       </c>
       <c r="F9" s="46" t="n">
-        <v>700238.0236037285</v>
+        <v>486801.0308477557</v>
       </c>
       <c r="G9" s="46" t="n">
-        <v>-2495828.623005316</v>
+        <v>-2649503.257789616</v>
       </c>
       <c r="H9" s="46" t="n">
-        <v>-8299327.01208548</v>
+        <v>-8527575.629384065</v>
       </c>
       <c r="I9" s="46" t="n">
-        <v>1842.949345865247</v>
+        <v>1827.528795482594</v>
       </c>
       <c r="J9" s="48" t="n">
-        <v>0.579697031710826</v>
+        <v>0.6517313014969096</v>
       </c>
     </row>
     <row r="10">
@@ -11110,25 +11117,25 @@
         <v>1072.265625</v>
       </c>
       <c r="D10" s="46" t="n">
-        <v>3408903.485939026</v>
+        <v>3006754.933502197</v>
       </c>
       <c r="E10" s="46" t="n">
-        <v>1816763.121417706</v>
+        <v>1800228.195323807</v>
       </c>
       <c r="F10" s="46" t="n">
-        <v>1369182.671943195</v>
+        <v>1000423.517162765</v>
       </c>
       <c r="G10" s="46" t="n">
-        <v>985811.5237991003</v>
+        <v>720304.9323571911</v>
       </c>
       <c r="H10" s="46" t="n">
-        <v>-7313515.48828638</v>
+        <v>-7807270.697026874</v>
       </c>
       <c r="I10" s="46" t="n">
-        <v>1694.321891012506</v>
+        <v>1678.901340629852</v>
       </c>
       <c r="J10" s="48" t="n">
-        <v>0.5329464823253145</v>
+        <v>0.5987279426284813</v>
       </c>
     </row>
     <row r="11">
@@ -11139,25 +11146,25 @@
         <v>1590</v>
       </c>
       <c r="D11" s="46" t="n">
-        <v>5054863.660898438</v>
+        <v>4458541.08609375</v>
       </c>
       <c r="E11" s="46" t="n">
-        <v>2538446.898715996</v>
+        <v>2513928.223607578</v>
       </c>
       <c r="F11" s="46" t="n">
-        <v>2185805.836182442</v>
+        <v>1638994.446886172</v>
       </c>
       <c r="G11" s="46" t="n">
-        <v>1573780.202051358</v>
+        <v>1180076.001758044</v>
       </c>
       <c r="H11" s="46" t="n">
-        <v>-5739735.286235021</v>
+        <v>-6627194.69526883</v>
       </c>
       <c r="I11" s="46" t="n">
-        <v>1596.50748346918</v>
+        <v>1581.086933086527</v>
       </c>
       <c r="J11" s="48" t="n">
-        <v>0.5021791029403985</v>
+        <v>0.5638454765951477</v>
       </c>
     </row>
     <row r="12">
@@ -11168,25 +11175,25 @@
         <v>2107.734375</v>
       </c>
       <c r="D12" s="46" t="n">
-        <v>6700823.83585785</v>
+        <v>5910327.238685302</v>
       </c>
       <c r="E12" s="46" t="n">
-        <v>3226783.743447408</v>
+        <v>3194281.319324471</v>
       </c>
       <c r="F12" s="46" t="n">
-        <v>3035775.932988567</v>
+        <v>2310912.309176456</v>
       </c>
       <c r="G12" s="46" t="n">
-        <v>2185758.671751768</v>
+        <v>1663856.862607048</v>
       </c>
       <c r="H12" s="46" t="n">
-        <v>-3553976.614483254</v>
+        <v>-4963337.832661781</v>
       </c>
       <c r="I12" s="46" t="n">
-        <v>1530.925235039357</v>
+        <v>1515.504684656705</v>
       </c>
       <c r="J12" s="48" t="n">
-        <v>0.4815503022449343</v>
+        <v>0.5404576075613385</v>
       </c>
     </row>
     <row r="13">
@@ -11197,25 +11204,25 @@
         <v>2559.375</v>
       </c>
       <c r="D13" s="46" t="n">
-        <v>8136661.435290528</v>
+        <v>7176778.98881836</v>
       </c>
       <c r="E13" s="46" t="n">
-        <v>3807773.856105018</v>
+        <v>3768306.884969415</v>
       </c>
       <c r="F13" s="46" t="n">
-        <v>3796713.15231051</v>
+        <v>2916527.366473945</v>
       </c>
       <c r="G13" s="46" t="n">
-        <v>2733633.469663567</v>
+        <v>2099899.70386124</v>
       </c>
       <c r="H13" s="46" t="n">
-        <v>-820343.1448196867</v>
+        <v>-2863438.128800541</v>
       </c>
       <c r="I13" s="46" t="n">
-        <v>1487.774888832241</v>
+        <v>1472.354338449588</v>
       </c>
       <c r="J13" s="48" t="n">
-        <v>0.4679774237121195</v>
+        <v>0.5250693787339072</v>
       </c>
     </row>
     <row r="14">
@@ -11226,25 +11233,25 @@
         <v>2878.828125</v>
       </c>
       <c r="D14" s="46" t="n">
-        <v>9152253.883669738</v>
+        <v>8072561.934034424</v>
       </c>
       <c r="E14" s="46" t="n">
-        <v>4210013.115550779</v>
+        <v>4165620.001406218</v>
       </c>
       <c r="F14" s="46" t="n">
-        <v>4343642.005728334</v>
+        <v>3353594.202850081</v>
       </c>
       <c r="G14" s="46" t="n">
-        <v>3127422.2441244</v>
+        <v>2414587.826052058</v>
       </c>
       <c r="H14" s="46" t="n">
-        <v>2307079.099304714</v>
+        <v>-448850.3027484827</v>
       </c>
       <c r="I14" s="46" t="n">
-        <v>1462.405163750712</v>
+        <v>1446.984613368058</v>
       </c>
       <c r="J14" s="48" t="n">
-        <v>0.4599974136494025</v>
+        <v>0.516022055382902</v>
       </c>
     </row>
     <row r="15">
@@ -11255,25 +11262,25 @@
         <v>3000</v>
       </c>
       <c r="D15" s="46" t="n">
-        <v>9537478.60546875</v>
+        <v>8412341.671875</v>
       </c>
       <c r="E15" s="46" t="n">
-        <v>4360941.459832817</v>
+        <v>4314679.808684858</v>
       </c>
       <c r="F15" s="46" t="n">
-        <v>4552742.945635933</v>
+        <v>3521023.343190143</v>
       </c>
       <c r="G15" s="46" t="n">
-        <v>3277974.920857872</v>
+        <v>2535136.807096903</v>
       </c>
       <c r="H15" s="46" t="n">
-        <v>5585054.020162586</v>
+        <v>2086286.50434842</v>
       </c>
       <c r="I15" s="46" t="n">
-        <v>1453.647153277606</v>
+        <v>1438.226602894953</v>
       </c>
       <c r="J15" s="48" t="n">
-        <v>0.4572425942148139</v>
+        <v>0.5128987833566171</v>
       </c>
     </row>
     <row r="17">
@@ -11283,7 +11290,7 @@
         </is>
       </c>
       <c r="D17" s="47" t="n">
-        <v>8299327.01208548</v>
+        <v>8527575.629384065</v>
       </c>
     </row>
     <row r="18">
@@ -11293,7 +11300,7 @@
         </is>
       </c>
       <c r="D18" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
@@ -11303,7 +11310,7 @@
         </is>
       </c>
       <c r="D19" s="47" t="n">
-        <v>-105699.2968567105</v>
+        <v>-1973660.467868997</v>
       </c>
     </row>
     <row r="21">
@@ -11367,7 +11374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F21"/>
+  <dimension ref="B1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -11572,7 +11579,7 @@
     <row r="12">
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>DERIVING A DEMAND ELASTICITY FROM INERTIA — AND A CORRECTION TO TAB 10</t>
+          <t>TESTING THE NINE PRODUCT PENETRATIONS AGAINST PUBLISHED AGGREGATES</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr"/>
@@ -11580,57 +11587,200 @@
       <c r="E12" s="8" t="inlineStr"/>
       <c r="F12" s="8" t="inlineStr"/>
     </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="B13" s="5" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="45" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C13" s="45" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="D13" s="45" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="E13" s="45" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="F13" s="45" t="inlineStr">
+        <is>
+          <t>Source and basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="B14" s="42" t="inlineStr">
+        <is>
+          <t>Business overdrafts</t>
+        </is>
+      </c>
+      <c r="C14" s="48" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D14" s="48" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E14" s="72" t="n">
+        <v>1.136363636363636</v>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>SME Finance Monitor 2024 — 22% of SMEs use an overdraft. Survey.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="B15" s="42" t="inlineStr">
+        <is>
+          <t>Term loans / mortgages</t>
+        </is>
+      </c>
+      <c r="C15" s="48" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="D15" s="48" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E15" s="72" t="n">
+        <v>0.923076923076923</v>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>SME Finance Monitor 2024 — 13% use a bank loan or commercial mortgage. Survey.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="B16" s="42" t="inlineStr">
+        <is>
+          <t>Asset finance</t>
+        </is>
+      </c>
+      <c r="C16" s="48" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D16" s="48" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E16" s="72" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>SME Finance Monitor 2024 — 10% use leasing or hire purchase. Survey.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>Invoice finance (CORRECTED)</t>
+        </is>
+      </c>
+      <c r="C17" s="48" t="n">
+        <v>0.0071</v>
+      </c>
+      <c r="D17" s="48" t="n">
+        <v>0.0071</v>
+      </c>
+      <c r="E17" s="72" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>UK Finance — 40,100 businesses on invoice finance or ABL at end-2024 against 5.63m active companies. Hard count. Model said 3.00% through v2.1; corrected in v2.2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="39" customHeight="1">
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>• Three of four land within a fifth of the published figure. For a set of cells every one of which was labelled 'Assumption', that is real corroboration, and the differences sit inside the wobble between 'share of SMEs surveyed' and 'share of a bank's customers'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>• Invoice finance did not. 4.2x is beyond any definitional difference, and the published figure is a hard count rather than a survey estimate, so the model was corrected rather than caveated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="52" customHeight="1">
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>• The cost of that one unchecked cell: profit before tax overstated by 22.6%, cost:income understated by 5.6 points. Invoice finance is the highest-value behaviour per adopter in the whole book, so an assumption that drifted high on adopter count flattered the model's most attractive product — which is the direction an unchecked assumption always drifts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>DERIVING A DEMAND ELASTICITY FROM INERTIA — AND A CORRECTION TO TAB 10</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr"/>
+      <c r="D23" s="8" t="inlineStr"/>
+      <c r="E23" s="8" t="inlineStr"/>
+      <c r="F23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>• Tab 10 gives the break-even demand elasticity for every price — the responsiveness at which raising it stops paying. It could not say whether real customers are that responsive. For the business current account, public data can.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="39" customHeight="1">
-      <c r="B14" s="5" t="inlineStr">
+    <row r="25" ht="39" customHeight="1">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>• UK SME current-account prices differ by 100%: the majors charge from £8.50 a month, several challengers charge nothing. That gap is permanent, visible and heavily advertised. Against it, 0.44% of SMEs switched in 2024 — and not all of those for price.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="39" customHeight="1">
-      <c r="B15" s="5" t="inlineStr">
+    <row r="26" ht="39" customHeight="1">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>• A 100% price difference producing at most 0.44% of annual movement implies an upper-bound elasticity of about 0.004. Allowing a generous ten-fold multiplier for salience — a fee RISE is noticed in a way a standing price gap is not, which is the one robust finding in the FCA's banking trials — still only reaches 0.044.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="26" customHeight="1">
-      <c r="B16" s="5" t="inlineStr">
+    <row r="27" ht="26" customHeight="1">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>• Against a break-even of 0.13, raising the current-account fee industry-wide has roughly three times the headroom it needs. It is comfortably accretive.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="39" customHeight="1">
-      <c r="B17" s="5" t="inlineStr">
+    <row r="28" ht="39" customHeight="1">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>• CORRECTION TO TAB 10: v1.8 labelled the current-account fee 'fragile — only a near-inert customer makes this pay'. The evidence says the SME current-account customer IS near-inert. At 0.44% annual switching this is close to the most inert consumer market for which data exists. The fragile reading was wrong and this tab supersedes it.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="26" customHeight="1">
-      <c r="B18" s="5" t="inlineStr">
+    <row r="29" ht="26" customHeight="1">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>• Moving alone is the exception and stays genuinely marginal: the break-even falls to 0.021, which is below the salience-adjusted bound of 0.044. Industry-wide, clearly accretive. Unilaterally, a coin toss.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="52" customHeight="1">
-      <c r="B19" s="5" t="inlineStr">
+    <row r="30" ht="52" customHeight="1">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>• The bound does NOT transfer to every price. It holds where switching bank is the customer's only escape, which is true of the current account. It does not hold for the card annual fee (cancel the card, keep the bank), the card interest rate (pay the balance down), or loan pricing (brokered and shopped). Those have other margins of adjustment and need their own evidence.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="B21" s="5" t="inlineStr">
+    <row r="32" ht="30" customHeight="1">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>Still needing an institution's own data: process yields outside lending, entry-point incidence for every cross-holding moment, holding lives for five products, and the benchmark columns on tab 3. Those queries are written against each cell and none of them can be answered from public sources.</t>
         </is>
@@ -12788,14 +12938,14 @@
           <t>Invoice finance — penetration</t>
         </is>
       </c>
-      <c r="C45" s="17" t="n">
-        <v>0.03</v>
+      <c r="C45" s="23" t="n">
+        <v>0.0071</v>
       </c>
       <c r="D45" s="18" t="n">
-        <v>0.03</v>
+        <v>0.0071</v>
       </c>
       <c r="E45" s="18" t="n">
-        <v>0.03</v>
+        <v>0.0071</v>
       </c>
       <c r="F45" s="19">
         <f>CHOOSE('Inputs'!$C$4,D45,C45,E45)</f>
@@ -12808,7 +12958,7 @@
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>Assumption</t>
+          <t>CORRECTED in v2.2. Was 0.03 (Assumption) through v2.1. UK Finance reports 40,100 businesses on invoice finance or asset-based lending at end-2024 against 5.63m active companies (Companies House) = 0.71%. A hard count, not a survey estimate, so the 4.2x gap is beyond any definitional difference. Correcting it cuts modelled profit before tax 22.6%: invoice finance is the highest-value behaviour per adopter in the book, so overstating adopters flattered the model's most attractive product.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v2.2.1: generic wording in two source notes; results unchanged
</commit_message>
<xml_diff>
--- a/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
+++ b/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B55"/>
+  <dimension ref="B1:B56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -608,7 +608,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MODEL VERSION: v2.2 · 22 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
+          <t>MODEL VERSION: v2.2.1 · 22 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
         </is>
       </c>
     </row>
@@ -619,316 +619,323 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1">
+    <row r="5" ht="40" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>• v2.2 (22 Aug 2026) — CORRECTION, results change. Nine product penetrations were all labelled 'Assumption'. Tested against published aggregates, three land within a fifth of the survey figure (overdrafts 25% vs 22%, term loans 12% vs 13%, asset finance 8% vs 10%) — real corroboration. Invoice finance did not: the model said 3%, UK Finance counts 40,100 businesses on invoice finance or ABL at end-2024 against 5.63m active companies, which is 0.71%. A hard count, not a survey. Corrected in the base. Profit before tax falls 22.6% and cost:income moves 45.7% to 51.3%, because invoice finance is the highest-value behaviour per adopter in the book and the model was carrying 4.2x too many adopters of it.</t>
+          <t>• v2.2.1 (22 Aug 2026) — editorial only: named UK banks removed from two source notes on the Inputs tab (market-share context and the standard business tariff), which now read generically. The figures, their sources and every result are unchanged from v2.2. Named institutions remain where they are the subject of published analysis rather than a pricing reference — the cost:income benchmarks and the Allica backtest on tab 11.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="58" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
+          <t>• v2.2 (22 Aug 2026) — CORRECTION, results change. Nine product penetrations were all labelled 'Assumption'. Tested against published aggregates, three land within a fifth of the survey figure (overdrafts 25% vs 22%, term loans 12% vs 13%, asset finance 8% vs 10%) — real corroboration. Invoice finance did not: the model said 3%, UK Finance counts 40,100 businesses on invoice finance or ABL at end-2024 against 5.63m active companies, which is 0.71%. A hard count, not a survey. Corrected in the base. Profit before tax falls 22.6% and cost:income moves 45.7% to 51.3%, because invoice finance is the highest-value behaviour per adopter in the book and the model was carrying 4.2x too many adopters of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
           <t>• v2.1 (22 Aug 2026) — evidence. Tab 13 fills from public sources three of the cells that shipped empty. Loan application success is 37% (SME Finance Monitor, 18m to Q4 2024) against the model's implicit 100%, so the bank does 2.7 underwriting passes per funded loan — worth £143,644 of operating cost. UK formation rate is 15.0% of the company stock (Companies House, 846,325 incorporations in 2024), which fills the A1 entry point and shows formation alone covers 125% of steady-state replacement at current share. SME current-account switching is 0.44% (CASS 2024), which bounds current-account demand elasticity at about 0.004 and CORRECTS tab 10: v1.8 called the account fee fragile, and the evidence says the customer is near-inert, so raising it industry-wide is comfortably accretive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="52" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>• v2.0 (22 Aug 2026) — trajectory. Every other tab describes a steady state; tab 12 describes getting there. Time stays OUT of the base model deliberately — the steady-state identities are what let the whole chain work without a forecast — so the trajectory runs the same model at a series of maturity states and reads the result as a cash flow. Building one regional centre from nothing needs £8.3m of funding at its deepest point, repays in year seven, and has an NPV at the model's own 12% cost of equity of about MINUS £106,000. The snapshot alone reports only the final year and calls the business comfortably good. Both are true: a profitable steady state is not the same thing as a worthwhile investment.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>• v1.9 (22 Aug 2026) — competitive response. Every scenario assumed rivals stand still, which flatters both directions at once: raising a price looks safer than it is, and cutting one looks better than it is. A firm with market share s moving alone faces roughly the industry elasticity divided by s; moving in concert it faces only the industry elasticity. This model's penetration IS market share (16%), so moving alone multiplies the demand response by 6.25x. Tab 10 now inverts every break-even into the industry elasticity the move survives in each regime. The headline lever moves with it: raising the term loan rate survives an industry elasticity of 2.91 in concert but only 0.47 alone — marginal rather than comfortable.</t>
+          <t>• v2.0 (22 Aug 2026) — trajectory. Every other tab describes a steady state; tab 12 describes getting there. Time stays OUT of the base model deliberately — the steady-state identities are what let the whole chain work without a forecast — so the trajectory runs the same model at a series of maturity states and reads the result as a cash flow. Building one regional centre from nothing needs £8.3m of funding at its deepest point, repays in year seven, and has an NPV at the model's own 12% cost of equity of about MINUS £106,000. The snapshot alone reports only the final year and calls the business comfortably good. Both are true: a profitable steady state is not the same thing as a worthwhile investment.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="52" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>• v1.8 (22 Aug 2026) — break-even demand elasticity on tab 10. The elasticity table ranked the term loan customer rate as the largest driver of profit at +1.25, which was an artefact: nothing in the model responds to price, so raising any price always looked accretive. Tab 10 now leads with the demand elasticity at which raising each price stops paying. The reordering matters — the card fee breaks even at 0.06 and the current-account fee at 0.13, so both are fragile to almost any customer response, while the loan rate holds to 2.91. The hidden assumption being replaced is zero, which is the least defensible value available.</t>
+          <t>• v1.9 (22 Aug 2026) — competitive response. Every scenario assumed rivals stand still, which flatters both directions at once: raising a price looks safer than it is, and cutting one looks better than it is. A firm with market share s moving alone faces roughly the industry elasticity divided by s; moving in concert it faces only the industry elasticity. This model's penetration IS market share (16%), so moving alone multiplies the demand response by 6.25x. Tab 10 now inverts every break-even into the industry elasticity the move survives in each regime. The headline lever moves with it: raising the term loan rate survives an industry elasticity of 2.91 in concert but only 0.47 alone — marginal rather than comfortable.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="52" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>• v1.7 (22 Aug 2026) — operational leverage. Every cost line in the model scaled linearly with its driver, which forces a cost elasticity of exactly 1.0 and makes cost per customer flat at every scale. Allica Bank's own accounts put that elasticity at 0.808 across 2022-23 and 0.622 across 2023-24 — cost rises materially more slowly than the book. Inputs section O adds a cost scale elasticity and the customer count the per-customer rates are calibrated at; the head-office pools, the platform line and change-the-bank now scale by it. Default 1.0 reproduces v1.6 exactly. Tab 11 adds the out-of-sample test that measured it.</t>
+          <t>• v1.8 (22 Aug 2026) — break-even demand elasticity on tab 10. The elasticity table ranked the term loan customer rate as the largest driver of profit at +1.25, which was an artefact: nothing in the model responds to price, so raising any price always looked accretive. Tab 10 now leads with the demand elasticity at which raising each price stops paying. The reordering matters — the card fee breaks even at 0.06 and the current-account fee at 0.13, so both are fragile to almost any customer response, while the loan rate holds to 2.91. The hidden assumption being replaced is zero, which is the least defensible value available.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="52" customHeight="1">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>• v1.6 (22 Aug 2026) — validation and drivers. Tab 10 ELASTICITIES: every input bumped +1% and the workbook recalculated, giving the % change in PBT, cost:income, RoE and income. Only one input has an elasticity above 1 on profit — the term loan customer rate, at +1.25; reachable market and penetration are exactly +1.00 (pure scale); nothing else exceeds 0.53. Tab 11 BACKTEST against Allica Bank FY2023 audited accounts: the revenue engine reproduces a real bank's operating income to within 8%, and the cost engine under-predicts by 7x. Diagnosis: head-office cost was modelled purely per customer, which is a scale assumption disguised as a driver. Inputs section N therefore adds a fixed component to each head-office pool, defaulting to 0 so v1.5 results are unchanged.</t>
+          <t>• v1.7 (22 Aug 2026) — operational leverage. Every cost line in the model scaled linearly with its driver, which forces a cost elasticity of exactly 1.0 and makes cost per customer flat at every scale. Allica Bank's own accounts put that elasticity at 0.808 across 2022-23 and 0.622 across 2023-24 — cost rises materially more slowly than the book. Inputs section O adds a cost scale elasticity and the customer count the per-customer rates are calibrated at; the head-office pools, the platform line and change-the-bank now scale by it. Default 1.0 reproduces v1.6 exactly. Tab 11 adds the out-of-sample test that measured it.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="52" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>• v1.5 (22 Aug 2026) — PROCESS LAYER on the Step 2 tabs. Tab 3 gains process columns M-T (process type, yield, attempts, automation, best-in-class intensity and yield, benchmark source, £ gap) and a HEAD-OFFICE PROCESS REGISTER of 22 processes already named in the tab 9 operational model but never costed. Yield inflates ATTEMPTS and never deflates outcomes — that is what stops it double-counting with the CEP layer's demand-side conversion. Head-office costs are carved OUT of the pools, so naming a process moves money from unallocated to attributed and the total never changes. New sheet 3b indexes every process to the numbers it moves, and imputes what each would have to become to hit a target cost:income. Mode OFF (default) = results identical to v1.4.</t>
+          <t>• v1.6 (22 Aug 2026) — validation and drivers. Tab 10 ELASTICITIES: every input bumped +1% and the workbook recalculated, giving the % change in PBT, cost:income, RoE and income. Only one input has an elasticity above 1 on profit — the term loan customer rate, at +1.25; reachable market and penetration are exactly +1.00 (pure scale); nothing else exceeds 0.53. Tab 11 BACKTEST against Allica Bank FY2023 audited accounts: the revenue engine reproduces a real bank's operating income to within 8%, and the cost engine under-predicts by 7x. Diagnosis: head-office cost was modelled purely per customer, which is a scale assumption disguised as a driver. Inputs section N therefore adds a fixed component to each head-office pool, defaulting to 0 so v1.5 results are unchanged.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="52" customHeight="1">
       <c r="B13" s="4" t="inlineStr">
         <is>
+          <t>• v1.5 (22 Aug 2026) — PROCESS LAYER on the Step 2 tabs. Tab 3 gains process columns M-T (process type, yield, attempts, automation, best-in-class intensity and yield, benchmark source, £ gap) and a HEAD-OFFICE PROCESS REGISTER of 22 processes already named in the tab 9 operational model but never costed. Yield inflates ATTEMPTS and never deflates outcomes — that is what stops it double-counting with the CEP layer's demand-side conversion. Head-office costs are carved OUT of the pools, so naming a process moves money from unallocated to attributed and the total never changes. New sheet 3b indexes every process to the numbers it moves, and imputes what each would have to become to hit a target cost:income. Mode OFF (default) = results identical to v1.4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="52" customHeight="1">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
           <t>• v1.4 (22 Aug 2026) — CEP DEMAND LAYER. New sheet 1b derives the nine product penetrations and the customer count instead of asserting them: penetration = (lambda*c x L) / (1 + lambda*c x L), where lambda*c = category-entry-point events x presence x conversion and L is the holding life. Little's Law run forwards; no time axis is added and the model stays a steady-state snapshot. Ships deliberately EMPTY — every event/presence/conversion cell is blank and carries the cohort query that fills it, and any unpopulated product falls back to its hardcoded penetration. Mode OFF (default) = results identical to v1.3; CALIBRATE reports the won-event rate implied by today's assumptions and changes nothing.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="B14" s="4" t="inlineStr">
+    <row r="15" ht="40" customHeight="1">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>• v1.3 (21 Aug 2026) — churn replacement is a costed activity end-to-end: new input cac_new (£240 acquisition marketing per new customer won, carved out of the corporate-centre pool — hq_oh £250→£222); driver-linked on tab 4, attributed to the current account (gateway product) on tab 6; 'value of preventing one churn' memo added to tab 6. Raising the churn input now inflates demand-generation cost, not just processing. Central PBT shifts &lt;£1k/unit (carve-out rounding).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
+          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
         <is>
+          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
           <t>• v1.0 (10 Aug 2026) — first published version: 9 tabs + flow register, FTP with liquidity/behavioural terms, fraud/FSCS/change-the-bank lines, segment-pod LMUs, bridge check.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="3" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>What this is</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="39" customHeight="1">
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="39" customHeight="1">
       <c r="B22" s="4" t="inlineStr">
         <is>
+          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="39" customHeight="1">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
           <t>• It follows the Simanis / IVE bottom-up methodology ('Running the Right Numbers'): model the last-mile operating unit, derive every cost from activity drivers (transaction intensity I and customer load L), build whole costs, and check the price/margin covers them including a competitive return on capital.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="3" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>What period this models</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="26" customHeight="1">
-      <c r="B25" s="4" t="inlineStr">
+    <row r="26" ht="26" customHeight="1">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>• One representative operating year at steady state. Balances are annual averages; rates and volumes are annual. There is no time axis, no ramp and no vintage cohorts — the model is a snapshot, not a forecast.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="78" customHeight="1">
-      <c r="B26" s="4" t="inlineStr">
+    <row r="27" ht="78" customHeight="1">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>• The book is stationary but not free to hold flat: customers churn (12% p.a. input) and the model costs their replacement end-to-end — acquisition marketing per new customer won (cac_new, carved from the corporate-centre pool), onboarding hours, KYC per new customer and RM origination effort are all driver-linked (Simanis: at-scale operations include 'replacement of customer churn'). Only residual brand &amp; joint marketing remains pool-costed. The 'value of preventing one churn' memo on tab 6 prices retention: contribution annuity over remaining relationship life + the avoided replacement cost.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="26" customHeight="1">
-      <c r="B27" s="4" t="inlineStr">
+    <row r="28" ht="26" customHeight="1">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>• The capital charge (cost of equity on allocated capital) is the incumbent analogue of Simanis's start-up-cost amortisation: capital earns its required return inside the steady-state P&amp;L.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="52" customHeight="1">
-      <c r="B28" s="4" t="inlineStr">
+    <row r="29" ht="52" customHeight="1">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>• Out of scope by design: transition paths. The cost and cash shape of moving between steady states — digital migration, maturity glide, behaviour-change programmes and their CAC/incentives — belongs in a scenario layer built ON TOP of this base (comparative statics between two runs of this model, plus a separate transition-cost estimate). The base model never carries scenario logic.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="3" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>How the tabs map to the methodology</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="24" customHeight="1">
-      <c r="B31" s="4" t="inlineStr">
+    <row r="32" ht="24" customHeight="1">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>• Inputs — every assumption in one place, with sources. Edit blue cells; yellow cells are the biggest levers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="26" customHeight="1">
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="26" customHeight="1">
       <c r="B33" s="4" t="inlineStr">
         <is>
+          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
+      <c r="B34" s="4" t="inlineStr">
+        <is>
           <t>• 2. Revenues — unit revenue per product: interest margins measured against internal funds transfer prices (Bank Rate for floating, + premium for term), plus fees.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="39" customHeight="1">
-      <c r="B34" s="4" t="inlineStr">
+    <row r="35" ht="39" customHeight="1">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>• 3. HR &amp; Activity — Step 2: every FTE derived from activity drivers (hours per onboarding, review, renewal…) — nothing is assumed as headcount. From v1.5 this tab is also the PROCESS REGISTER (columns M-T), with the head-office process register below it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="26" customHeight="1">
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>• 1b. Demand &amp; CEPs — the demand layer (v1.4). Penetration is derived, not assumed. Mode cell on Inputs section L: OFF reproduces v1.3, CALIBRATE reports the implied event rates, LIVE derives.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="26" customHeight="1">
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>• 13. Evidence — public sources for cells that shipped empty: application success rates, company formation rates and SME switching, each with its tier and what it changes. Includes a correction to tab 10.</t>
+          <t>• 1b. Demand &amp; CEPs — the demand layer (v1.4). Penetration is derived, not assumed. Mode cell on Inputs section L: OFF reproduces v1.3, CALIBRATE reports the implied event rates, LIVE derives.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="26" customHeight="1">
       <c r="B37" s="4" t="inlineStr">
         <is>
+          <t>• 13. Evidence — public sources for cells that shipped empty: application success rates, company formation rates and SME switching, each with its tier and what it changes. Includes a correction to tab 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="26" customHeight="1">
+      <c r="B38" s="4" t="inlineStr">
+        <is>
           <t>• 12. Trajectory — the ramp from nothing to steady state: cash flow, peak funding, payback and NPV. Time lives here and nowhere else, as a wrapper around the snapshot rather than inside it.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="39" customHeight="1">
-      <c r="B38" s="4" t="inlineStr">
+    <row r="39" ht="39" customHeight="1">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>• 3b. Process Index — derived view, no assumptions. Every process with its flow, product, owner, the numbers it moves, its cost and its gap to best in class, plus a ranked worst-gap list and the top-down benchmark imputation. Answers 'which process do I improve to move this number?'</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="52" customHeight="1">
-      <c r="B39" s="4" t="inlineStr">
+    <row r="40" ht="52" customHeight="1">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>• 4. Running Costs — Step 2 (cont.): direct running costs plus the share of head-office costs. The attribution memo reads the tab 3 process register and reports the share of the cost base with a named process owner — the model's own assessment of how much of its cost it actually understands. What remains in UNALLOCATED JOINT COSTS is cost with no process to improve.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="26" customHeight="1">
-      <c r="B40" s="4" t="inlineStr">
+    <row r="41" ht="26" customHeight="1">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>• 5. Risk &amp; Capital — Step 3: expected credit losses (PD × LGD), risk-weighted assets, allocated equity, and the required return on it.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="91" customHeight="1">
-      <c r="B41" s="4" t="inlineStr">
+    <row r="42" ht="91" customHeight="1">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>• 6. Unit Economics — Steps 4–5: per-product unit costs and revenues on an activity-based costing basis, taken exactly as far as causality runs (the source methodology's own rule: link costs to customers and transactions 'whenever possible'). Costs with real drivers — servicing hours, RM effort per origination, staff-time-driven supervision, per-account and per-facility infrastructure — are attributed to products; genuinely joint costs (brand, exec, finance, platform build) are NOT forced into products but held as an unallocated hurdle that total contribution must clear, with a full-absorption memo showing the source doc's simple-division treatment. Product decisions should run on contribution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="26" customHeight="1">
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="26" customHeight="1">
       <c r="B43" s="4" t="inlineStr">
         <is>
+          <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="26" customHeight="1">
+      <c r="B44" s="4" t="inlineStr">
+        <is>
           <t>• 8. Org Structure — the whole-bank organisation implied by the model: front-line FTEs from activity drivers × number of centres, head-office FTEs backed out of the per-customer head-office cost allocations.</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="52" customHeight="1">
-      <c r="B44" s="4" t="inlineStr">
+    <row r="45" ht="52" customHeight="1">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>• 9. Flow Register — one row per flow on the operational model map: component type (CP/WP/PP/PartP), core/support/enabling, direction, digital/physical medium, the direct/administrative/managerial roles accountable, and the BIAN service domains. Ends with a BIAN completeness checklist. This is where the map, the ARM and BIAN reconcile.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="3" t="inlineStr">
+    <row r="47">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>Colour legend</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="26" customHeight="1">
-      <c r="B47" s="4" t="inlineStr">
+    <row r="48" ht="26" customHeight="1">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>• Blue = hardcoded input (edit these) · Yellow fill = key assumption / sensitivity lever · Black = formula · Green = link to another sheet.</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="B49" s="3" t="inlineStr">
+    <row r="50">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Reading the results</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="52" customHeight="1">
-      <c r="B50" s="4" t="inlineStr">
+    <row r="51" ht="52" customHeight="1">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>• Deposit products earn the spread between the transfer price and the rate paid; lending earns the customer rate minus the transfer price minus expected losses. Capital-heavy, labour-heavy products (term loans) can show thin or negative economic profit — consistent with the Bank of England's 2026 finding that SME lending earns the lowest product-level returns, driven by impairments and per-borrower servicing costs.</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="39" customHeight="1">
-      <c r="B51" s="4" t="inlineStr">
+    <row r="52" ht="39" customHeight="1">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t>• Use the cost-driver table on the P&amp;L tab to find leverage points, then trace them to transaction intensity (I) or customer load (L) assumptions on the Inputs tab — e.g. automating underwriting hours, raising RM portfolio size, or shifting servicing to digital.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="B53" s="3" t="inlineStr">
+    <row r="54">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>Caveats</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="39" customHeight="1">
-      <c r="B54" s="4" t="inlineStr">
+    <row r="55" ht="39" customHeight="1">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>• Benchmarks are as of August 2026 (Bank Rate 3.75%; BoE effective new SME loan rate ~6.3%; commercial interchange 1.65–1.90%; invoice finance discount base+1–3%). Items marked 'Assumption' are illustrative and should be replaced with your own data.</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="65" customHeight="1">
-      <c r="B55" s="4" t="inlineStr">
+    <row r="56" ht="65" customHeight="1">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>• The FTP now carries an explicit liquidity charge (buffer × drag) and a behavioural credit for stable deposits, shown as memos on the Revenues tab; it is still a single curve, not a full behavioural-maturity model. Fraud &amp; payment losses, the FSCS levy, collateral administration &amp; recoveries, and change-the-bank spend are now modelled explicitly. Operational-risk RWA is proxied at 15% of gross income; head-office and change costs are allocated per customer.</t>
         </is>
@@ -12281,7 +12288,7 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>Set so 300 centres × 3,000 customers = 900,000 BCA customers — a ~16% national SME market share, i.e. big-4 incumbent territory (Barclays/Lloyds each serve ~1m+ business customers)</t>
+          <t>Set so 300 centres × 3,000 customers = 900,000 BCA customers — a ~16% national SME market share, i.e. big-4 incumbent territory (the largest UK banks each serve ~1m+ business customers)</t>
         </is>
       </c>
     </row>
@@ -13365,7 +13372,7 @@
       </c>
       <c r="H59" s="5" t="inlineStr">
         <is>
-          <t>Barclays standard business tariff from £8.50/mo post free period; NatWest £5–10 (anna.money comparison, 2026)</t>
+          <t>Major UK banks charge from £8.50/mo on standard business tariffs after the free period, with a £5–10 range across the group (anna.money comparison, 2026)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v2.3: service-churn break-even on tab 10; two more penetrations tested on tab 13
</commit_message>
<xml_diff>
--- a/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
+++ b/UK_SME_Bank_Bottom_Up_Unit_Economics.xlsx
@@ -32,14 +32,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="£#,##0"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="£#,##0.00"/>
     <numFmt numFmtId="168" formatCode="0.00000"/>
     <numFmt numFmtId="169" formatCode="+0.00;-0.00;0.00"/>
-    <numFmt numFmtId="170" formatCode="0.00\x"/>
+    <numFmt numFmtId="170" formatCode="0.000"/>
+    <numFmt numFmtId="171" formatCode="0.00\x"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -138,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -225,7 +226,8 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="169" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -591,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B56"/>
+  <dimension ref="B1:B57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -608,7 +610,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MODEL VERSION: v2.2.1 · 22 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
+          <t>MODEL VERSION: v2.3 · 22 August 2026 — check github.com/tmth-studio/sme-bank-models for the latest; the version history below tells you what changed since your download.</t>
         </is>
       </c>
     </row>
@@ -619,323 +621,330 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="40" customHeight="1">
+    <row r="5" ht="58" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
+          <t>• v2.3 (22 Aug 2026) — the service free lunch, priced. Nothing in the model connected service to retention, so servicing hours could be cut to zero and profit only rose. Tab 10 now prices the trade: one percentage point of extra churn costs £354,736 a year, while halving ALL customer servicing saves £40,270. Break-even is a 0.114 point rise in churn — a 0.9% relative increase. Cut service in half and lose more than 0.9% of the customers who would have stayed, and you are worse off. Tab 13 adds two more penetrations tested and NOT corrected: FX users (model 20% vs 12% of SMEs exporting, but importers belong in the model's construct) and business cards (model 30% vs ~18% using cards as finance, but the model measures cards held).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
           <t>• v2.2.1 (22 Aug 2026) — editorial only: named UK banks removed from two source notes on the Inputs tab (market-share context and the standard business tariff), which now read generically. The figures, their sources and every result are unchanged from v2.2. Named institutions remain where they are the subject of published analysis rather than a pricing reference — the cost:income benchmarks and the Allica backtest on tab 11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>• v2.2 (22 Aug 2026) — CORRECTION, results change. Nine product penetrations were all labelled 'Assumption'. Tested against published aggregates, three land within a fifth of the survey figure (overdrafts 25% vs 22%, term loans 12% vs 13%, asset finance 8% vs 10%) — real corroboration. Invoice finance did not: the model said 3%, UK Finance counts 40,100 businesses on invoice finance or ABL at end-2024 against 5.63m active companies, which is 0.71%. A hard count, not a survey. Corrected in the base. Profit before tax falls 22.6% and cost:income moves 45.7% to 51.3%, because invoice finance is the highest-value behaviour per adopter in the book and the model was carrying 4.2x too many adopters of it.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
+          <t>• v2.2 (22 Aug 2026) — CORRECTION, results change. Nine product penetrations were all labelled 'Assumption'. Tested against published aggregates, three land within a fifth of the survey figure (overdrafts 25% vs 22%, term loans 12% vs 13%, asset finance 8% vs 10%) — real corroboration. Invoice finance did not: the model said 3%, UK Finance counts 40,100 businesses on invoice finance or ABL at end-2024 against 5.63m active companies, which is 0.71%. A hard count, not a survey. Corrected in the base. Profit before tax falls 22.6% and cost:income moves 45.7% to 51.3%, because invoice finance is the highest-value behaviour per adopter in the book and the model was carrying 4.2x too many adopters of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
           <t>• v2.1 (22 Aug 2026) — evidence. Tab 13 fills from public sources three of the cells that shipped empty. Loan application success is 37% (SME Finance Monitor, 18m to Q4 2024) against the model's implicit 100%, so the bank does 2.7 underwriting passes per funded loan — worth £143,644 of operating cost. UK formation rate is 15.0% of the company stock (Companies House, 846,325 incorporations in 2024), which fills the A1 entry point and shows formation alone covers 125% of steady-state replacement at current share. SME current-account switching is 0.44% (CASS 2024), which bounds current-account demand elasticity at about 0.004 and CORRECTS tab 10: v1.8 called the account fee fragile, and the evidence says the customer is near-inert, so raising it industry-wide is comfortably accretive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="52" customHeight="1">
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>• v2.0 (22 Aug 2026) — trajectory. Every other tab describes a steady state; tab 12 describes getting there. Time stays OUT of the base model deliberately — the steady-state identities are what let the whole chain work without a forecast — so the trajectory runs the same model at a series of maturity states and reads the result as a cash flow. Building one regional centre from nothing needs £8.3m of funding at its deepest point, repays in year seven, and has an NPV at the model's own 12% cost of equity of about MINUS £106,000. The snapshot alone reports only the final year and calls the business comfortably good. Both are true: a profitable steady state is not the same thing as a worthwhile investment.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="52" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>• v1.9 (22 Aug 2026) — competitive response. Every scenario assumed rivals stand still, which flatters both directions at once: raising a price looks safer than it is, and cutting one looks better than it is. A firm with market share s moving alone faces roughly the industry elasticity divided by s; moving in concert it faces only the industry elasticity. This model's penetration IS market share (16%), so moving alone multiplies the demand response by 6.25x. Tab 10 now inverts every break-even into the industry elasticity the move survives in each regime. The headline lever moves with it: raising the term loan rate survives an industry elasticity of 2.91 in concert but only 0.47 alone — marginal rather than comfortable.</t>
+          <t>• v2.0 (22 Aug 2026) — trajectory. Every other tab describes a steady state; tab 12 describes getting there. Time stays OUT of the base model deliberately — the steady-state identities are what let the whole chain work without a forecast — so the trajectory runs the same model at a series of maturity states and reads the result as a cash flow. Building one regional centre from nothing needs £8.3m of funding at its deepest point, repays in year seven, and has an NPV at the model's own 12% cost of equity of about MINUS £106,000. The snapshot alone reports only the final year and calls the business comfortably good. Both are true: a profitable steady state is not the same thing as a worthwhile investment.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="52" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>• v1.8 (22 Aug 2026) — break-even demand elasticity on tab 10. The elasticity table ranked the term loan customer rate as the largest driver of profit at +1.25, which was an artefact: nothing in the model responds to price, so raising any price always looked accretive. Tab 10 now leads with the demand elasticity at which raising each price stops paying. The reordering matters — the card fee breaks even at 0.06 and the current-account fee at 0.13, so both are fragile to almost any customer response, while the loan rate holds to 2.91. The hidden assumption being replaced is zero, which is the least defensible value available.</t>
+          <t>• v1.9 (22 Aug 2026) — competitive response. Every scenario assumed rivals stand still, which flatters both directions at once: raising a price looks safer than it is, and cutting one looks better than it is. A firm with market share s moving alone faces roughly the industry elasticity divided by s; moving in concert it faces only the industry elasticity. This model's penetration IS market share (16%), so moving alone multiplies the demand response by 6.25x. Tab 10 now inverts every break-even into the industry elasticity the move survives in each regime. The headline lever moves with it: raising the term loan rate survives an industry elasticity of 2.91 in concert but only 0.47 alone — marginal rather than comfortable.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="52" customHeight="1">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>• v1.7 (22 Aug 2026) — operational leverage. Every cost line in the model scaled linearly with its driver, which forces a cost elasticity of exactly 1.0 and makes cost per customer flat at every scale. Allica Bank's own accounts put that elasticity at 0.808 across 2022-23 and 0.622 across 2023-24 — cost rises materially more slowly than the book. Inputs section O adds a cost scale elasticity and the customer count the per-customer rates are calibrated at; the head-office pools, the platform line and change-the-bank now scale by it. Default 1.0 reproduces v1.6 exactly. Tab 11 adds the out-of-sample test that measured it.</t>
+          <t>• v1.8 (22 Aug 2026) — break-even demand elasticity on tab 10. The elasticity table ranked the term loan customer rate as the largest driver of profit at +1.25, which was an artefact: nothing in the model responds to price, so raising any price always looked accretive. Tab 10 now leads with the demand elasticity at which raising each price stops paying. The reordering matters — the card fee breaks even at 0.06 and the current-account fee at 0.13, so both are fragile to almost any customer response, while the loan rate holds to 2.91. The hidden assumption being replaced is zero, which is the least defensible value available.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="52" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>• v1.6 (22 Aug 2026) — validation and drivers. Tab 10 ELASTICITIES: every input bumped +1% and the workbook recalculated, giving the % change in PBT, cost:income, RoE and income. Only one input has an elasticity above 1 on profit — the term loan customer rate, at +1.25; reachable market and penetration are exactly +1.00 (pure scale); nothing else exceeds 0.53. Tab 11 BACKTEST against Allica Bank FY2023 audited accounts: the revenue engine reproduces a real bank's operating income to within 8%, and the cost engine under-predicts by 7x. Diagnosis: head-office cost was modelled purely per customer, which is a scale assumption disguised as a driver. Inputs section N therefore adds a fixed component to each head-office pool, defaulting to 0 so v1.5 results are unchanged.</t>
+          <t>• v1.7 (22 Aug 2026) — operational leverage. Every cost line in the model scaled linearly with its driver, which forces a cost elasticity of exactly 1.0 and makes cost per customer flat at every scale. Allica Bank's own accounts put that elasticity at 0.808 across 2022-23 and 0.622 across 2023-24 — cost rises materially more slowly than the book. Inputs section O adds a cost scale elasticity and the customer count the per-customer rates are calibrated at; the head-office pools, the platform line and change-the-bank now scale by it. Default 1.0 reproduces v1.6 exactly. Tab 11 adds the out-of-sample test that measured it.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="52" customHeight="1">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>• v1.5 (22 Aug 2026) — PROCESS LAYER on the Step 2 tabs. Tab 3 gains process columns M-T (process type, yield, attempts, automation, best-in-class intensity and yield, benchmark source, £ gap) and a HEAD-OFFICE PROCESS REGISTER of 22 processes already named in the tab 9 operational model but never costed. Yield inflates ATTEMPTS and never deflates outcomes — that is what stops it double-counting with the CEP layer's demand-side conversion. Head-office costs are carved OUT of the pools, so naming a process moves money from unallocated to attributed and the total never changes. New sheet 3b indexes every process to the numbers it moves, and imputes what each would have to become to hit a target cost:income. Mode OFF (default) = results identical to v1.4.</t>
+          <t>• v1.6 (22 Aug 2026) — validation and drivers. Tab 10 ELASTICITIES: every input bumped +1% and the workbook recalculated, giving the % change in PBT, cost:income, RoE and income. Only one input has an elasticity above 1 on profit — the term loan customer rate, at +1.25; reachable market and penetration are exactly +1.00 (pure scale); nothing else exceeds 0.53. Tab 11 BACKTEST against Allica Bank FY2023 audited accounts: the revenue engine reproduces a real bank's operating income to within 8%, and the cost engine under-predicts by 7x. Diagnosis: head-office cost was modelled purely per customer, which is a scale assumption disguised as a driver. Inputs section N therefore adds a fixed component to each head-office pool, defaulting to 0 so v1.5 results are unchanged.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="52" customHeight="1">
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>• v1.5 (22 Aug 2026) — PROCESS LAYER on the Step 2 tabs. Tab 3 gains process columns M-T (process type, yield, attempts, automation, best-in-class intensity and yield, benchmark source, £ gap) and a HEAD-OFFICE PROCESS REGISTER of 22 processes already named in the tab 9 operational model but never costed. Yield inflates ATTEMPTS and never deflates outcomes — that is what stops it double-counting with the CEP layer's demand-side conversion. Head-office costs are carved OUT of the pools, so naming a process moves money from unallocated to attributed and the total never changes. New sheet 3b indexes every process to the numbers it moves, and imputes what each would have to become to hit a target cost:income. Mode OFF (default) = results identical to v1.4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
           <t>• v1.4 (22 Aug 2026) — CEP DEMAND LAYER. New sheet 1b derives the nine product penetrations and the customer count instead of asserting them: penetration = (lambda*c x L) / (1 + lambda*c x L), where lambda*c = category-entry-point events x presence x conversion and L is the holding life. Little's Law run forwards; no time axis is added and the model stays a steady-state snapshot. Ships deliberately EMPTY — every event/presence/conversion cell is blank and carries the cohort query that fills it, and any unpopulated product falls back to its hardcoded penetration. Mode OFF (default) = results identical to v1.3; CALIBRATE reports the won-event rate implied by today's assumptions and changes nothing.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="B15" s="4" t="inlineStr">
+    <row r="16" ht="40" customHeight="1">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>• v1.3 (21 Aug 2026) — churn replacement is a costed activity end-to-end: new input cac_new (£240 acquisition marketing per new customer won, carved out of the corporate-centre pool — hq_oh £250→£222); driver-linked on tab 4, attributed to the current account (gateway product) on tab 6; 'value of preventing one churn' memo added to tab 6. Raising the churn input now inflates demand-generation cost, not just processing. Central PBT shifts &lt;£1k/unit (carve-out rounding).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
+          <t>• v1.2.1 (21 Aug 2026) — documentation only: added 'What period this models' to this Guide (steady-state annual snapshot, stationary book, churn replacement costed, transitions out of scope). No formula or input changes — results identical to v1.2.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+          <t>• v1.2 (12 Aug 2026) — ranges, not points: every input carries Pessimistic/Central/Optimistic (direction-aware) with one scenario toggle driving the ACTIVE column; bands seeded only where benchmark evidence exists (BoE loan rates, Jefferies CoE, peer CET1, BoE SME PD, best-buy savings). Central results identical to v1.1.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="B19" s="4" t="inlineStr">
         <is>
+          <t>• v1.1 (12 Aug 2026) — scenario-building granularity: Channel tag (digital-amenable/judgement) on every activity row (tab 3); per-product RM-held share inputs + RM/digital unit split columns (tab 1). Economics unchanged — tie-out and all product margins identical to v1.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="B20" s="4" t="inlineStr">
+        <is>
           <t>• v1.0 (10 Aug 2026) — first published version: 9 tabs + flow register, FTP with liquidity/behavioural terms, fraud/FSCS/change-the-bank lines, segment-pod LMUs, bridge check.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="3" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>What this is</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="39" customHeight="1">
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="39" customHeight="1">
       <c r="B23" s="4" t="inlineStr">
         <is>
+          <t>• A bottom-up financial model of one regional business centre of an established UK SME bank at steady state, built to show unit costs and unit revenues across the full product suite: current accounts, instant savings, notice &amp; fixed deposits, overdrafts, term loans, asset finance, invoice finance, credit cards, and payments &amp; FX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="39" customHeight="1">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
           <t>• It follows the Simanis / IVE bottom-up methodology ('Running the Right Numbers'): model the last-mile operating unit, derive every cost from activity drivers (transaction intensity I and customer load L), build whole costs, and check the price/margin covers them including a competitive return on capital.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="3" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>What period this models</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="26" customHeight="1">
-      <c r="B26" s="4" t="inlineStr">
+    <row r="27" ht="26" customHeight="1">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>• One representative operating year at steady state. Balances are annual averages; rates and volumes are annual. There is no time axis, no ramp and no vintage cohorts — the model is a snapshot, not a forecast.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="78" customHeight="1">
-      <c r="B27" s="4" t="inlineStr">
+    <row r="28" ht="78" customHeight="1">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>• The book is stationary but not free to hold flat: customers churn (12% p.a. input) and the model costs their replacement end-to-end — acquisition marketing per new customer won (cac_new, carved from the corporate-centre pool), onboarding hours, KYC per new customer and RM origination effort are all driver-linked (Simanis: at-scale operations include 'replacement of customer churn'). Only residual brand &amp; joint marketing remains pool-costed. The 'value of preventing one churn' memo on tab 6 prices retention: contribution annuity over remaining relationship life + the avoided replacement cost.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="26" customHeight="1">
-      <c r="B28" s="4" t="inlineStr">
+    <row r="29" ht="26" customHeight="1">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>• The capital charge (cost of equity on allocated capital) is the incumbent analogue of Simanis's start-up-cost amortisation: capital earns its required return inside the steady-state P&amp;L.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="52" customHeight="1">
-      <c r="B29" s="4" t="inlineStr">
+    <row r="30" ht="52" customHeight="1">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>• Out of scope by design: transition paths. The cost and cash shape of moving between steady states — digital migration, maturity glide, behaviour-change programmes and their CAC/incentives — belongs in a scenario layer built ON TOP of this base (comparative statics between two runs of this model, plus a separate transition-cost estimate). The base model never carries scenario logic.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="3" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>How the tabs map to the methodology</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="24" customHeight="1">
-      <c r="B32" s="4" t="inlineStr">
+    <row r="33" ht="24" customHeight="1">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>• Inputs — every assumption in one place, with sources. Edit blue cells; yellow cells are the biggest levers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="26" customHeight="1">
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="26" customHeight="1">
       <c r="B34" s="4" t="inlineStr">
         <is>
+          <t>• 1. Customers — Step 1: bound the operating unit. Reachable market (R) × penetration (P) → customers → product volumes and balances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="26" customHeight="1">
+      <c r="B35" s="4" t="inlineStr">
+        <is>
           <t>• 2. Revenues — unit revenue per product: interest margins measured against internal funds transfer prices (Bank Rate for floating, + premium for term), plus fees.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="39" customHeight="1">
-      <c r="B35" s="4" t="inlineStr">
+    <row r="36" ht="39" customHeight="1">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>• 3. HR &amp; Activity — Step 2: every FTE derived from activity drivers (hours per onboarding, review, renewal…) — nothing is assumed as headcount. From v1.5 this tab is also the PROCESS REGISTER (columns M-T), with the head-office process register below it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="26" customHeight="1">
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>• 1b. Demand &amp; CEPs — the demand layer (v1.4). Penetration is derived, not assumed. Mode cell on Inputs section L: OFF reproduces v1.3, CALIBRATE reports the implied event rates, LIVE derives.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="26" customHeight="1">
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>• 13. Evidence — public sources for cells that shipped empty: application success rates, company formation rates and SME switching, each with its tier and what it changes. Includes a correction to tab 10.</t>
+          <t>• 1b. Demand &amp; CEPs — the demand layer (v1.4). Penetration is derived, not assumed. Mode cell on Inputs section L: OFF reproduces v1.3, CALIBRATE reports the implied event rates, LIVE derives.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="26" customHeight="1">
       <c r="B38" s="4" t="inlineStr">
         <is>
+          <t>• 13. Evidence — public sources for cells that shipped empty: application success rates, company formation rates and SME switching, each with its tier and what it changes. Includes a correction to tab 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="26" customHeight="1">
+      <c r="B39" s="4" t="inlineStr">
+        <is>
           <t>• 12. Trajectory — the ramp from nothing to steady state: cash flow, peak funding, payback and NPV. Time lives here and nowhere else, as a wrapper around the snapshot rather than inside it.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="39" customHeight="1">
-      <c r="B39" s="4" t="inlineStr">
+    <row r="40" ht="39" customHeight="1">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>• 3b. Process Index — derived view, no assumptions. Every process with its flow, product, owner, the numbers it moves, its cost and its gap to best in class, plus a ranked worst-gap list and the top-down benchmark imputation. Answers 'which process do I improve to move this number?'</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="52" customHeight="1">
-      <c r="B40" s="4" t="inlineStr">
+    <row r="41" ht="52" customHeight="1">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>• 4. Running Costs — Step 2 (cont.): direct running costs plus the share of head-office costs. The attribution memo reads the tab 3 process register and reports the share of the cost base with a named process owner — the model's own assessment of how much of its cost it actually understands. What remains in UNALLOCATED JOINT COSTS is cost with no process to improve.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="26" customHeight="1">
-      <c r="B41" s="4" t="inlineStr">
+    <row r="42" ht="26" customHeight="1">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>• 5. Risk &amp; Capital — Step 3: expected credit losses (PD × LGD), risk-weighted assets, allocated equity, and the required return on it.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="91" customHeight="1">
-      <c r="B42" s="4" t="inlineStr">
+    <row r="43" ht="91" customHeight="1">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>• 6. Unit Economics — Steps 4–5: per-product unit costs and revenues on an activity-based costing basis, taken exactly as far as causality runs (the source methodology's own rule: link costs to customers and transactions 'whenever possible'). Costs with real drivers — servicing hours, RM effort per origination, staff-time-driven supervision, per-account and per-facility infrastructure — are attributed to products; genuinely joint costs (brand, exec, finance, platform build) are NOT forced into products but held as an unallocated hurdle that total contribution must clear, with a full-absorption memo showing the source doc's simple-division treatment. Product decisions should run on contribution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="26" customHeight="1">
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="26" customHeight="1">
       <c r="B44" s="4" t="inlineStr">
         <is>
+          <t>• 7. P&amp;L — the whole-cost P&amp;L of the operating unit at steady state, key ratios vs industry benchmarks, and the Simanis cost-driver table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="26" customHeight="1">
+      <c r="B45" s="4" t="inlineStr">
+        <is>
           <t>• 8. Org Structure — the whole-bank organisation implied by the model: front-line FTEs from activity drivers × number of centres, head-office FTEs backed out of the per-customer head-office cost allocations.</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="52" customHeight="1">
-      <c r="B45" s="4" t="inlineStr">
+    <row r="46" ht="52" customHeight="1">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>• 9. Flow Register — one row per flow on the operational model map: component type (CP/WP/PP/PartP), core/support/enabling, direction, digital/physical medium, the direct/administrative/managerial roles accountable, and the BIAN service domains. Ends with a BIAN completeness checklist. This is where the map, the ARM and BIAN reconcile.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="B47" s="3" t="inlineStr">
+    <row r="48">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>Colour legend</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="26" customHeight="1">
-      <c r="B48" s="4" t="inlineStr">
+    <row r="49" ht="26" customHeight="1">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>• Blue = hardcoded input (edit these) · Yellow fill = key assumption / sensitivity lever · Black = formula · Green = link to another sheet.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="B50" s="3" t="inlineStr">
+    <row r="51">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>Reading the results</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="52" customHeight="1">
-      <c r="B51" s="4" t="inlineStr">
+    <row r="52" ht="52" customHeight="1">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t>• Deposit products earn the spread between the transfer price and the rate paid; lending earns the customer rate minus the transfer price minus expected losses. Capital-heavy, labour-heavy products (term loans) can show thin or negative economic profit — consistent with the Bank of England's 2026 finding that SME lending earns the lowest product-level returns, driven by impairments and per-borrower servicing costs.</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="39" customHeight="1">
-      <c r="B52" s="4" t="inlineStr">
+    <row r="53" ht="39" customHeight="1">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>• Use the cost-driver table on the P&amp;L tab to find leverage points, then trace them to transaction intensity (I) or customer load (L) assumptions on the Inputs tab — e.g. automating underwriting hours, raising RM portfolio size, or shifting servicing to digital.</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="B54" s="3" t="inlineStr">
+    <row r="55">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>Caveats</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="39" customHeight="1">
-      <c r="B55" s="4" t="inlineStr">
+    <row r="56" ht="39" customHeight="1">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>• Benchmarks are as of August 2026 (Bank Rate 3.75%; BoE effective new SME loan rate ~6.3%; commercial interchange 1.65–1.90%; invoice finance discount base+1–3%). Items marked 'Assumption' are illustrative and should be replaced with your own data.</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="65" customHeight="1">
-      <c r="B56" s="4" t="inlineStr">
+    <row r="57" ht="65" customHeight="1">
+      <c r="B57" s="4" t="inlineStr">
         <is>
           <t>• The FTP now carries an explicit liquidity charge (buffer × drag) and a behavioural credit for stable deposits, shown as memos on the Revenues tab; it is still a single curve, not a full behavioural-maturity model. Fraud &amp; payment losses, the FSCS levy, collateral administration &amp; recoveries, and change-the-bank spend are now modelled explicitly. Operational-risk RWA is proxied at 15% of gross income; head-office and change costs are allocated per customer.</t>
         </is>
@@ -7793,7 +7802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H112"/>
+  <dimension ref="B1:H125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -8257,679 +8266,435 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="62" customHeight="1">
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>A cut is the mirror image: cut alone and share moves, so the cut can pay; cut and get matched and volume responds only at the industry elasticity, because nobody's relative price changed — you keep your share and give away the margin. For the term loan rate the band between 0.47 and 2.91 is where the answer depends entirely on whether rivals follow. The same move creates value in one regime and destroys it in the other, and no amount of internal analysis resolves that. SME banking is concentrated with observable prices, which is the textbook setting for high match rates: the prior should be that rivals follow.</t>
+    <row r="26">
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>CUTTING SERVICE — the other free lunch</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr"/>
+      <c r="D26" s="8" t="inlineStr"/>
+      <c r="E26" s="8" t="inlineStr"/>
+      <c r="F26" s="8" t="inlineStr"/>
+      <c r="G26" s="8" t="inlineStr"/>
+      <c r="H26" s="8" t="inlineStr"/>
+    </row>
+    <row r="27" ht="44" customHeight="1">
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Nothing in this model connects service to whether customers stay. Servicing hours can be cut to zero and profit only rises. Every process-layer improvement — lower intensity, higher automation — therefore drops straight to the bottom line untaxed. That matters more than the pricing case, because cutting servicing is exactly what a cost programme proposes.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="45" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="C28" s="45" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="D28" s="45" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="E28" s="45" t="inlineStr">
-        <is>
-          <t>e(PBT)</t>
-        </is>
-      </c>
-      <c r="F28" s="45" t="inlineStr">
-        <is>
-          <t>e(Cost:income)</t>
-        </is>
-      </c>
-      <c r="G28" s="45" t="inlineStr">
-        <is>
-          <t>e(RoE)</t>
-        </is>
-      </c>
-      <c r="H28" s="45" t="inlineStr">
-        <is>
-          <t>e(Income)</t>
-        </is>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Contribution per customer per year</t>
+        </is>
+      </c>
+      <c r="E28" s="46" t="n">
+        <v>1365.887287730048</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Term loans — customer rate</t>
-        </is>
-      </c>
-      <c r="C29" s="63" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="D29" s="14" t="inlineStr">
-        <is>
-          <t>% p.a.</t>
-        </is>
-      </c>
-      <c r="E29" s="71" t="n">
-        <v>1.61327277330784</v>
-      </c>
-      <c r="F29" s="71" t="n">
-        <v>-0.6707136124121114</v>
-      </c>
-      <c r="G29" s="71" t="n">
-        <v>1.505361613400337</v>
-      </c>
-      <c r="H29" s="71" t="n">
-        <v>0.675242556153086</v>
+          <t>Expected remaining relationship life (years)</t>
+        </is>
+      </c>
+      <c r="E29" s="51" t="n">
+        <v>8.333333333333334</v>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Reachable SMEs in region (R)</t>
-        </is>
-      </c>
-      <c r="C30" s="63" t="n">
-        <v>18750</v>
-      </c>
-      <c r="D30" s="14" t="inlineStr">
-        <is>
-          <t>businesses</t>
-        </is>
-      </c>
-      <c r="E30" s="71" t="n">
-        <v>0.9999999999999578</v>
-      </c>
-      <c r="F30" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="71" t="n">
-        <v>0.999999999999992</v>
+          <t>Replacement cost of one lost customer</t>
+        </is>
+      </c>
+      <c r="E30" s="46" t="n">
+        <v>442.1541950113379</v>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>Steady-state penetration (P)</t>
-        </is>
-      </c>
-      <c r="C31" s="63" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="D31" s="14" t="inlineStr">
-        <is>
-          <t>% of reachable</t>
-        </is>
-      </c>
-      <c r="E31" s="71" t="n">
-        <v>0.9999999999999578</v>
-      </c>
-      <c r="F31" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="71" t="n">
-        <v>0.999999999999992</v>
+      <c r="B31" s="42" t="inlineStr">
+        <is>
+          <t>VALUE OF PREVENTING ONE CHURN</t>
+        </is>
+      </c>
+      <c r="E31" s="46" t="n">
+        <v>11824.5482594284</v>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>Business current account — penetration</t>
-        </is>
-      </c>
-      <c r="C32" s="63" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" s="14" t="inlineStr">
-        <is>
-          <t>% of customers</t>
-        </is>
-      </c>
-      <c r="E32" s="71" t="n">
-        <v>0.6874327592213575</v>
-      </c>
-      <c r="F32" s="71" t="n">
-        <v>-0.2626076388723727</v>
-      </c>
-      <c r="G32" s="71" t="n">
-        <v>0.6377899386038517</v>
-      </c>
-      <c r="H32" s="71" t="n">
-        <v>0.3133125460550319</v>
+          <t>Cost of one percentage point of extra churn</t>
+        </is>
+      </c>
+      <c r="E32" s="46" t="n">
+        <v>354736.447782852</v>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Term loans — average balance</t>
-        </is>
-      </c>
-      <c r="C33" s="63" t="n">
-        <v>250000</v>
-      </c>
-      <c r="D33" s="14" t="inlineStr">
-        <is>
-          <t>£/loan</t>
-        </is>
-      </c>
-      <c r="E33" s="71" t="n">
-        <v>0.5799464755251776</v>
-      </c>
-      <c r="F33" s="71" t="n">
-        <v>-0.2842949830259432</v>
-      </c>
-      <c r="G33" s="71" t="n">
-        <v>-0.09315289195585527</v>
-      </c>
-      <c r="H33" s="71" t="n">
-        <v>0.2851055237263594</v>
+          <t>Saving from halving all customer servicing</t>
+        </is>
+      </c>
+      <c r="E33" s="46" t="n">
+        <v>40270.32445790805</v>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="10" t="inlineStr">
-        <is>
-          <t>BCA — average credit balance</t>
-        </is>
-      </c>
-      <c r="C34" s="63" t="n">
-        <v>18000</v>
-      </c>
-      <c r="D34" s="14" t="inlineStr">
-        <is>
-          <t>£/account</t>
-        </is>
-      </c>
-      <c r="E34" s="71" t="n">
-        <v>0.5520259482968808</v>
-      </c>
-      <c r="F34" s="71" t="n">
-        <v>-0.2283254496988612</v>
-      </c>
-      <c r="G34" s="71" t="n">
-        <v>0.5150956851542485</v>
-      </c>
-      <c r="H34" s="71" t="n">
-        <v>0.2333638274065154</v>
+      <c r="B34" s="42" t="inlineStr">
+        <is>
+          <t>BREAK-EVEN churn increase (percentage points)</t>
+        </is>
+      </c>
+      <c r="E34" s="72" t="n">
+        <v>0.1135218123471741</v>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Term loans / commercial mortgages — penetration</t>
-        </is>
-      </c>
-      <c r="C35" s="63" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="D35" s="14" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E35" s="71" t="n">
-        <v>0.5389407878755174</v>
-      </c>
-      <c r="F35" s="71" t="n">
-        <v>-0.2509271506335589</v>
-      </c>
-      <c r="G35" s="71" t="n">
-        <v>-0.1338841620559702</v>
-      </c>
-      <c r="H35" s="71" t="n">
-        <v>0.2851055237263594</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>Asset finance — customer yield</t>
-        </is>
-      </c>
-      <c r="C36" s="63" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-      <c r="D36" s="14" t="inlineStr">
-        <is>
-          <t>% p.a.</t>
-        </is>
-      </c>
-      <c r="E36" s="71" t="n">
-        <v>0.468064207295712</v>
-      </c>
-      <c r="F36" s="71" t="n">
-        <v>-0.1955273153312782</v>
-      </c>
-      <c r="G36" s="71" t="n">
-        <v>0.4370850852513102</v>
-      </c>
-      <c r="H36" s="71" t="n">
-        <v>0.1959103736252198</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t>Notice &amp; fixed deposits — rate paid</t>
-        </is>
-      </c>
-      <c r="C37" s="63" t="n">
-        <v>0.041</v>
-      </c>
-      <c r="D37" s="14" t="inlineStr">
-        <is>
-          <t>% p.a.</t>
-        </is>
-      </c>
-      <c r="E37" s="71" t="n">
-        <v>-0.3968651022335832</v>
-      </c>
-      <c r="F37" s="71" t="n">
-        <v>0.166386052133733</v>
-      </c>
-      <c r="G37" s="71" t="n">
-        <v>-0.3708096217590231</v>
-      </c>
-      <c r="H37" s="71" t="n">
-        <v>-0.1661096688135927</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t>Head office: technology &amp; central operations</t>
-        </is>
-      </c>
-      <c r="C38" s="63" t="n">
-        <v>450</v>
-      </c>
-      <c r="D38" s="14" t="inlineStr">
-        <is>
-          <t>£/customer/yr</t>
-        </is>
-      </c>
-      <c r="E38" s="71" t="n">
-        <v>-0.3834112609934771</v>
-      </c>
-      <c r="F38" s="71" t="n">
-        <v>0.3128853263417148</v>
-      </c>
-      <c r="G38" s="71" t="n">
-        <v>-0.3834112609934804</v>
-      </c>
-      <c r="H38" s="71" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="10" t="inlineStr">
-        <is>
-          <t>Instant-access savings — rate paid</t>
-        </is>
-      </c>
-      <c r="C39" s="63" t="n">
-        <v>0.033</v>
-      </c>
-      <c r="D39" s="14" t="inlineStr">
-        <is>
-          <t>% p.a.</t>
-        </is>
-      </c>
-      <c r="E39" s="71" t="n">
-        <v>-0.3407232097226184</v>
-      </c>
-      <c r="F39" s="71" t="n">
-        <v>0.1428148979391809</v>
-      </c>
-      <c r="G39" s="71" t="n">
-        <v>-0.318341845979591</v>
-      </c>
-      <c r="H39" s="71" t="n">
-        <v>-0.1426112278595273</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="10" t="inlineStr">
-        <is>
-          <t>Bank of England Bank Rate</t>
-        </is>
-      </c>
-      <c r="C40" s="63" t="n">
-        <v>0.0375</v>
-      </c>
-      <c r="D40" s="14" t="inlineStr">
-        <is>
-          <t>% p.a.</t>
-        </is>
-      </c>
-      <c r="E40" s="71" t="n">
-        <v>0.2451325388192351</v>
-      </c>
-      <c r="F40" s="71" t="n">
-        <v>-0.1024961613300335</v>
-      </c>
-      <c r="G40" s="71" t="n">
-        <v>0.2387120231982801</v>
-      </c>
-      <c r="H40" s="71" t="n">
-        <v>0.1026013237482584</v>
+          <t>…as a relative increase on 12% base churn</t>
+        </is>
+      </c>
+      <c r="E35" s="48" t="n">
+        <v>0.009460151028931173</v>
+      </c>
+    </row>
+    <row r="37" ht="44" customHeight="1">
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Read it plainly: halve customer service, and if more than 0.9% of the customers who would have stayed decide to leave, you are worse off. The model was previously silent on that trade and reported the saving as pure profit. It still cannot tell you the true service-churn elasticity — but it can say exactly how small it has to be for the cut to be worth making, and 0.9% is a demanding bar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="62" customHeight="1">
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>A cut is the mirror image: cut alone and share moves, so the cut can pay; cut and get matched and volume responds only at the industry elasticity, because nobody's relative price changed — you keep your share and give away the margin. For the term loan rate the band between 0.47 and 2.91 is where the answer depends entirely on whether rivals follow. The same move creates value in one regime and destroys it in the other, and no amount of internal analysis resolves that. SME banking is concentrated with observable prices, which is the textbook setting for high match rates: the prior should be that rivals follow.</t>
+        </is>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t>International payments &amp; FX — penetration</t>
-        </is>
-      </c>
-      <c r="C41" s="63" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D41" s="14" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E41" s="71" t="n">
-        <v>0.2182541932141037</v>
-      </c>
-      <c r="F41" s="71" t="n">
-        <v>-0.09081039086382579</v>
-      </c>
-      <c r="G41" s="71" t="n">
-        <v>0.2037664635887323</v>
-      </c>
-      <c r="H41" s="71" t="n">
-        <v>0.09183298763681969</v>
+      <c r="B41" s="45" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="C41" s="45" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D41" s="45" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E41" s="45" t="inlineStr">
+        <is>
+          <t>e(PBT)</t>
+        </is>
+      </c>
+      <c r="F41" s="45" t="inlineStr">
+        <is>
+          <t>e(Cost:income)</t>
+        </is>
+      </c>
+      <c r="G41" s="45" t="inlineStr">
+        <is>
+          <t>e(RoE)</t>
+        </is>
+      </c>
+      <c r="H41" s="45" t="inlineStr">
+        <is>
+          <t>e(Income)</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — average balance</t>
+          <t>Term loans — customer rate</t>
         </is>
       </c>
       <c r="C42" s="63" t="n">
-        <v>80000</v>
+        <v>0.0625</v>
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
-          <t>£/agreement</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E42" s="71" t="n">
-        <v>0.2144786405522011</v>
+        <v>1.61327277330784</v>
       </c>
       <c r="F42" s="71" t="n">
-        <v>-0.1051256445005265</v>
+        <v>-0.6707136124121114</v>
       </c>
       <c r="G42" s="71" t="n">
-        <v>0.04451741174847898</v>
+        <v>1.505361613400337</v>
       </c>
       <c r="H42" s="71" t="n">
-        <v>0.1052362748127385</v>
+        <v>0.675242556153086</v>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>Head office: risk, compliance, financial crime, audit</t>
+          <t>Reachable SMEs in region (R)</t>
         </is>
       </c>
       <c r="C43" s="63" t="n">
-        <v>250</v>
+        <v>18750</v>
       </c>
       <c r="D43" s="14" t="inlineStr">
         <is>
-          <t>£/customer/yr</t>
+          <t>businesses</t>
         </is>
       </c>
       <c r="E43" s="71" t="n">
-        <v>-0.2130062561074872</v>
+        <v>0.9999999999999578</v>
       </c>
       <c r="F43" s="71" t="n">
-        <v>0.1738251813009527</v>
+        <v>0</v>
       </c>
       <c r="G43" s="71" t="n">
-        <v>-0.2130062561076665</v>
+        <v>0</v>
       </c>
       <c r="H43" s="71" t="n">
-        <v>0</v>
+        <v>0.999999999999992</v>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — penetration</t>
+          <t>Steady-state penetration (P)</t>
         </is>
       </c>
       <c r="C44" s="63" t="n">
-        <v>0.08</v>
+        <v>0.16</v>
       </c>
       <c r="D44" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% of reachable</t>
         </is>
       </c>
       <c r="E44" s="71" t="n">
-        <v>0.2052216246454376</v>
+        <v>0.9999999999999578</v>
       </c>
       <c r="F44" s="71" t="n">
-        <v>-0.09757933615100182</v>
+        <v>0</v>
       </c>
       <c r="G44" s="71" t="n">
-        <v>0.03527609550751072</v>
+        <v>0</v>
       </c>
       <c r="H44" s="71" t="n">
-        <v>0.1052362748127385</v>
+        <v>0.999999999999992</v>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>Head office: finance, HR, exec, brand &amp; residual (non-acquisition) marketing</t>
+          <t>Business current account — penetration</t>
         </is>
       </c>
       <c r="C45" s="63" t="n">
-        <v>222</v>
+        <v>1</v>
       </c>
       <c r="D45" s="14" t="inlineStr">
         <is>
-          <t>£/customer/yr</t>
+          <t>% of customers</t>
         </is>
       </c>
       <c r="E45" s="71" t="n">
-        <v>-0.1891495554234487</v>
+        <v>0.6874327592213575</v>
       </c>
       <c r="F45" s="71" t="n">
-        <v>0.154356760995188</v>
+        <v>-0.2626076388723727</v>
       </c>
       <c r="G45" s="71" t="n">
-        <v>-0.1891495554236863</v>
+        <v>0.6377899386038517</v>
       </c>
       <c r="H45" s="71" t="n">
-        <v>0</v>
+        <v>0.3133125460550319</v>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>Business credit card — penetration</t>
+          <t>Term loans — average balance</t>
         </is>
       </c>
       <c r="C46" s="63" t="n">
-        <v>0.3</v>
+        <v>250000</v>
       </c>
       <c r="D46" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/loan</t>
         </is>
       </c>
       <c r="E46" s="71" t="n">
-        <v>0.1489064227671268</v>
+        <v>0.5799464755251776</v>
       </c>
       <c r="F46" s="71" t="n">
-        <v>-0.06216818662197646</v>
+        <v>-0.2842949830259432</v>
       </c>
       <c r="G46" s="71" t="n">
-        <v>0.1352333983522107</v>
+        <v>-0.09315289195585527</v>
       </c>
       <c r="H46" s="71" t="n">
-        <v>0.06533102015084027</v>
+        <v>0.2851055237263594</v>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>Equity held against RWAs (CET1 target)</t>
+          <t>BCA — average credit balance</t>
         </is>
       </c>
       <c r="C47" s="63" t="n">
-        <v>0.14</v>
+        <v>18000</v>
       </c>
       <c r="D47" s="14" t="inlineStr">
         <is>
-          <t>% of RWA</t>
+          <t>£/account</t>
         </is>
       </c>
       <c r="E47" s="71" t="n">
-        <v>0.1479233794011383</v>
+        <v>0.5520259482968808</v>
       </c>
       <c r="F47" s="71" t="n">
-        <v>-0.06187568430169751</v>
+        <v>-0.2283254496988612</v>
       </c>
       <c r="G47" s="71" t="n">
-        <v>-0.8436402184144726</v>
+        <v>0.5150956851542485</v>
       </c>
       <c r="H47" s="71" t="n">
-        <v>0.06191399400909547</v>
+        <v>0.2333638274065154</v>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — interest rate (EAR)</t>
+          <t>Term loans / commercial mortgages — penetration</t>
         </is>
       </c>
       <c r="C48" s="63" t="n">
-        <v>0.0975</v>
+        <v>0.12</v>
       </c>
       <c r="D48" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E48" s="71" t="n">
-        <v>0.141564685857882</v>
+        <v>0.5389407878755174</v>
       </c>
       <c r="F48" s="71" t="n">
-        <v>-0.05921744646463147</v>
+        <v>-0.2509271506335589</v>
       </c>
       <c r="G48" s="71" t="n">
-        <v>0.1322235784995538</v>
+        <v>-0.1338841620559702</v>
       </c>
       <c r="H48" s="71" t="n">
-        <v>0.05925253430247758</v>
+        <v>0.2851055237263594</v>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Card — average monthly spend</t>
+          <t>Asset finance — customer yield</t>
         </is>
       </c>
       <c r="C49" s="63" t="n">
-        <v>2500</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="D49" s="14" t="inlineStr">
         <is>
-          <t>£/card/month</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E49" s="71" t="n">
-        <v>0.1316430583019145</v>
+        <v>0.468064207295712</v>
       </c>
       <c r="F49" s="71" t="n">
-        <v>-0.05506944942967034</v>
+        <v>-0.1955273153312782</v>
       </c>
       <c r="G49" s="71" t="n">
-        <v>0.1229574306786514</v>
+        <v>0.4370850852513102</v>
       </c>
       <c r="H49" s="71" t="n">
-        <v>0.05509979258210067</v>
+        <v>0.1959103736252198</v>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>Card — commercial interchange earned</t>
+          <t>Notice &amp; fixed deposits — rate paid</t>
         </is>
       </c>
       <c r="C50" s="63" t="n">
-        <v>0.017</v>
+        <v>0.041</v>
       </c>
       <c r="D50" s="14" t="inlineStr">
         <is>
-          <t>% of spend</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E50" s="71" t="n">
-        <v>0.1316430583019145</v>
+        <v>-0.3968651022335832</v>
       </c>
       <c r="F50" s="71" t="n">
-        <v>-0.05506944942967034</v>
+        <v>0.166386052133733</v>
       </c>
       <c r="G50" s="71" t="n">
-        <v>0.1229574306786514</v>
+        <v>-0.3708096217590231</v>
       </c>
       <c r="H50" s="71" t="n">
-        <v>0.05509979258210067</v>
+        <v>-0.1661096688135927</v>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>Term funding premium over Bank Rate</t>
+          <t>Head office: technology &amp; central operations</t>
         </is>
       </c>
       <c r="C51" s="63" t="n">
-        <v>0.006</v>
+        <v>450</v>
       </c>
       <c r="D51" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E51" s="71" t="n">
-        <v>-0.129836192795824</v>
+        <v>-0.3834112609934771</v>
       </c>
       <c r="F51" s="71" t="n">
-        <v>0.05437306915937036</v>
+        <v>0.3128853263417148</v>
       </c>
       <c r="G51" s="71" t="n">
-        <v>-0.1212906772764059</v>
+        <v>-0.3834112609934804</v>
       </c>
       <c r="H51" s="71" t="n">
-        <v>-0.05434352091919858</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>Behavioural term credit for stable non-maturing deposits</t>
+          <t>Instant-access savings — rate paid</t>
         </is>
       </c>
       <c r="C52" s="63" t="n">
-        <v>0.005</v>
+        <v>0.033</v>
       </c>
       <c r="D52" s="14" t="inlineStr">
         <is>
@@ -8937,175 +8702,175 @@
         </is>
       </c>
       <c r="E52" s="71" t="n">
-        <v>0.1290618218646272</v>
+        <v>-0.3407232097226184</v>
       </c>
       <c r="F52" s="71" t="n">
-        <v>-0.05399023928653108</v>
+        <v>0.1428148979391809</v>
       </c>
       <c r="G52" s="71" t="n">
-        <v>0.1205467056942764</v>
+        <v>-0.318341845979591</v>
       </c>
       <c r="H52" s="71" t="n">
-        <v>0.05401940449224688</v>
+        <v>-0.1426112278595273</v>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>FX — average annual conversion volume</t>
+          <t>Bank of England Bank Rate</t>
         </is>
       </c>
       <c r="C53" s="63" t="n">
-        <v>100000</v>
+        <v>0.0375</v>
       </c>
       <c r="D53" s="14" t="inlineStr">
         <is>
-          <t>£/user/yr</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E53" s="71" t="n">
-        <v>0.1290618218646272</v>
+        <v>0.2451325388192351</v>
       </c>
       <c r="F53" s="71" t="n">
-        <v>-0.05399023928653108</v>
+        <v>-0.1024961613300335</v>
       </c>
       <c r="G53" s="71" t="n">
-        <v>0.1205467056942764</v>
+        <v>0.2387120231982801</v>
       </c>
       <c r="H53" s="71" t="n">
-        <v>0.05401940449224688</v>
+        <v>0.1026013237482584</v>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>FX — margin on conversion volume</t>
+          <t>International payments &amp; FX — penetration</t>
         </is>
       </c>
       <c r="C54" s="63" t="n">
-        <v>0.0075</v>
+        <v>0.2</v>
       </c>
       <c r="D54" s="14" t="inlineStr">
         <is>
-          <t>% of volume</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E54" s="71" t="n">
-        <v>0.1290618218646272</v>
+        <v>0.2182541932141037</v>
       </c>
       <c r="F54" s="71" t="n">
-        <v>-0.05399023928653108</v>
+        <v>-0.09081039086382579</v>
       </c>
       <c r="G54" s="71" t="n">
-        <v>0.1205467056942764</v>
+        <v>0.2037664635887323</v>
       </c>
       <c r="H54" s="71" t="n">
-        <v>0.05401940449224688</v>
+        <v>0.09183298763681969</v>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — average limit</t>
+          <t>Asset finance — average balance</t>
         </is>
       </c>
       <c r="C55" s="63" t="n">
-        <v>15000</v>
+        <v>80000</v>
       </c>
       <c r="D55" s="14" t="inlineStr">
         <is>
-          <t>£/facility</t>
+          <t>£/agreement</t>
         </is>
       </c>
       <c r="E55" s="71" t="n">
-        <v>0.1230830424521848</v>
+        <v>0.2144786405522011</v>
       </c>
       <c r="F55" s="71" t="n">
-        <v>-0.0590550445253119</v>
+        <v>-0.1051256445005265</v>
       </c>
       <c r="G55" s="71" t="n">
-        <v>0.07584524768646449</v>
+        <v>0.04451741174847898</v>
       </c>
       <c r="H55" s="71" t="n">
-        <v>0.0590899401158306</v>
+        <v>0.1052362748127385</v>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — penetration</t>
+          <t>Head office: risk, compliance, financial crime, audit</t>
         </is>
       </c>
       <c r="C56" s="63" t="n">
-        <v>0.25</v>
+        <v>250</v>
       </c>
       <c r="D56" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E56" s="71" t="n">
-        <v>0.1051536008356984</v>
+        <v>-0.2130062561074872</v>
       </c>
       <c r="F56" s="71" t="n">
-        <v>-0.04443224426671098</v>
+        <v>0.1738251813009527</v>
       </c>
       <c r="G56" s="71" t="n">
-        <v>0.05792426513148669</v>
+        <v>-0.2130062561076665</v>
       </c>
       <c r="H56" s="71" t="n">
-        <v>0.0590899401158306</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>Productive hours per FTE per month</t>
+          <t>Asset finance — penetration</t>
         </is>
       </c>
       <c r="C57" s="63" t="n">
-        <v>147</v>
+        <v>0.08</v>
       </c>
       <c r="D57" s="14" t="inlineStr">
         <is>
-          <t>hours</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E57" s="71" t="n">
-        <v>0.1049299343026391</v>
+        <v>0.2052216246454376</v>
       </c>
       <c r="F57" s="71" t="n">
-        <v>-0.08562877535793163</v>
+        <v>-0.09757933615100182</v>
       </c>
       <c r="G57" s="71" t="n">
-        <v>0.1049299343027884</v>
+        <v>0.03527609550751072</v>
       </c>
       <c r="H57" s="71" t="n">
-        <v>0</v>
+        <v>0.1052362748127385</v>
       </c>
     </row>
     <row r="58">
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>Customers per relationship manager (L)</t>
+          <t>Head office: finance, HR, exec, brand &amp; residual (non-acquisition) marketing</t>
         </is>
       </c>
       <c r="C58" s="63" t="n">
-        <v>120</v>
+        <v>222</v>
       </c>
       <c r="D58" s="14" t="inlineStr">
         <is>
-          <t>customers</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E58" s="71" t="n">
-        <v>0.1048340737728719</v>
+        <v>-0.1891495554234487</v>
       </c>
       <c r="F58" s="71" t="n">
-        <v>-0.0855505477307521</v>
+        <v>0.154356760995188</v>
       </c>
       <c r="G58" s="71" t="n">
-        <v>0.1048340737730304</v>
+        <v>-0.1891495554236863</v>
       </c>
       <c r="H58" s="71" t="n">
         <v>0</v>
@@ -9114,11 +8879,11 @@
     <row r="59">
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>Share of customers that are relationship-managed</t>
+          <t>Business credit card — penetration</t>
         </is>
       </c>
       <c r="C59" s="63" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="D59" s="14" t="inlineStr">
         <is>
@@ -9126,337 +8891,337 @@
         </is>
       </c>
       <c r="E59" s="71" t="n">
-        <v>-0.1046385357465969</v>
+        <v>0.1489064227671268</v>
       </c>
       <c r="F59" s="71" t="n">
-        <v>0.08539097761546771</v>
+        <v>-0.06216818662197646</v>
       </c>
       <c r="G59" s="71" t="n">
-        <v>-0.1046385357468233</v>
+        <v>0.1352333983522107</v>
       </c>
       <c r="H59" s="71" t="n">
-        <v>0</v>
+        <v>0.06533102015084027</v>
       </c>
     </row>
     <row r="60">
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>BCA — net transaction &amp; cash-handling income</t>
+          <t>Equity held against RWAs (CET1 target)</t>
         </is>
       </c>
       <c r="C60" s="63" t="n">
-        <v>120</v>
+        <v>0.14</v>
       </c>
       <c r="D60" s="14" t="inlineStr">
         <is>
-          <t>£/account/yr</t>
+          <t>% of RWA</t>
         </is>
       </c>
       <c r="E60" s="71" t="n">
-        <v>0.1032494574917018</v>
+        <v>0.1479233794011383</v>
       </c>
       <c r="F60" s="71" t="n">
-        <v>-0.04319685584629245</v>
+        <v>-0.06187568430169751</v>
       </c>
       <c r="G60" s="71" t="n">
-        <v>0.0964390048174012</v>
+        <v>-0.8436402184144726</v>
       </c>
       <c r="H60" s="71" t="n">
-        <v>0.0432155235937975</v>
+        <v>0.06191399400909547</v>
       </c>
     </row>
     <row r="61">
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>Change-the-bank / transformation spend per customer</t>
+          <t>Overdraft — interest rate (EAR)</t>
         </is>
       </c>
       <c r="C61" s="63" t="n">
-        <v>120</v>
+        <v>0.0975</v>
       </c>
       <c r="D61" s="14" t="inlineStr">
         <is>
-          <t>£/customer/yr</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E61" s="71" t="n">
-        <v>-0.1022430029315939</v>
+        <v>0.141564685857882</v>
       </c>
       <c r="F61" s="71" t="n">
-        <v>0.0834360870245049</v>
+        <v>-0.05921744646463147</v>
       </c>
       <c r="G61" s="71" t="n">
-        <v>-0.1022430029318107</v>
+        <v>0.1322235784995538</v>
       </c>
       <c r="H61" s="71" t="n">
-        <v>0</v>
+        <v>0.05925253430247758</v>
       </c>
     </row>
     <row r="62">
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Term loans — probability of default</t>
+          <t>Card — average monthly spend</t>
         </is>
       </c>
       <c r="C62" s="63" t="n">
-        <v>0.018</v>
+        <v>2500</v>
       </c>
       <c r="D62" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/card/month</t>
         </is>
       </c>
       <c r="E62" s="71" t="n">
-        <v>-0.1012205729022779</v>
+        <v>0.1316430583019145</v>
       </c>
       <c r="F62" s="71" t="n">
-        <v>0</v>
+        <v>-0.05506944942967034</v>
       </c>
       <c r="G62" s="71" t="n">
-        <v>-0.1012205729024857</v>
+        <v>0.1229574306786514</v>
       </c>
       <c r="H62" s="71" t="n">
-        <v>0</v>
+        <v>0.05509979258210067</v>
       </c>
     </row>
     <row r="63">
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>Term loans — loss given default</t>
+          <t>Card — commercial interchange earned</t>
         </is>
       </c>
       <c r="C63" s="63" t="n">
-        <v>0.25</v>
+        <v>0.017</v>
       </c>
       <c r="D63" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% of spend</t>
         </is>
       </c>
       <c r="E63" s="71" t="n">
-        <v>-0.1012205729022779</v>
+        <v>0.1316430583019145</v>
       </c>
       <c r="F63" s="71" t="n">
-        <v>0</v>
+        <v>-0.05506944942967034</v>
       </c>
       <c r="G63" s="71" t="n">
-        <v>-0.1012205729024857</v>
+        <v>0.1229574306786514</v>
       </c>
       <c r="H63" s="71" t="n">
-        <v>0</v>
+        <v>0.05509979258210067</v>
       </c>
     </row>
     <row r="64">
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>Term loans — arrangement fee</t>
+          <t>Term funding premium over Bank Rate</t>
         </is>
       </c>
       <c r="C64" s="63" t="n">
-        <v>0.015</v>
+        <v>0.006</v>
       </c>
       <c r="D64" s="14" t="inlineStr">
         <is>
-          <t>% of loan</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E64" s="71" t="n">
-        <v>0.09679636639847039</v>
+        <v>-0.129836192795824</v>
       </c>
       <c r="F64" s="71" t="n">
-        <v>-0.04049814572625951</v>
+        <v>0.05437306915937036</v>
       </c>
       <c r="G64" s="71" t="n">
-        <v>0.09041195146079069</v>
+        <v>-0.1212906772764059</v>
       </c>
       <c r="H64" s="71" t="n">
-        <v>0.04051455336918516</v>
+        <v>-0.05434352091919858</v>
       </c>
     </row>
     <row r="65">
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — average funds in use (advances)</t>
+          <t>Behavioural term credit for stable non-maturing deposits</t>
         </is>
       </c>
       <c r="C65" s="63" t="n">
-        <v>150000</v>
+        <v>0.005</v>
       </c>
       <c r="D65" s="14" t="inlineStr">
         <is>
-          <t>£/client</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E65" s="71" t="n">
-        <v>0.09492162631565762</v>
+        <v>0.1290618218646272</v>
       </c>
       <c r="F65" s="71" t="n">
-        <v>-0.04145064460605613</v>
+        <v>-0.05399023928653108</v>
       </c>
       <c r="G65" s="71" t="n">
-        <v>0.0692404302199741</v>
+        <v>0.1205467056942764</v>
       </c>
       <c r="H65" s="71" t="n">
-        <v>0.04146783329037527</v>
+        <v>0.05401940449224688</v>
       </c>
     </row>
     <row r="66">
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>Term loans — risk weight</t>
+          <t>FX — average annual conversion volume</t>
         </is>
       </c>
       <c r="C66" s="63" t="n">
-        <v>0.7</v>
+        <v>100000</v>
       </c>
       <c r="D66" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/user/yr</t>
         </is>
       </c>
       <c r="E66" s="71" t="n">
-        <v>0.09393575894340188</v>
+        <v>0.1290618218646272</v>
       </c>
       <c r="F66" s="71" t="n">
-        <v>-0.03930178091372589</v>
+        <v>-0.05399023928653108</v>
       </c>
       <c r="G66" s="71" t="n">
-        <v>-0.5376796480568484</v>
+        <v>0.1205467056942764</v>
       </c>
       <c r="H66" s="71" t="n">
-        <v>0.03931723328663613</v>
+        <v>0.05401940449224688</v>
       </c>
     </row>
     <row r="67">
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — penetration</t>
+          <t>FX — margin on conversion volume</t>
         </is>
       </c>
       <c r="C67" s="63" t="n">
-        <v>0.0071</v>
+        <v>0.0075</v>
       </c>
       <c r="D67" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% of volume</t>
         </is>
       </c>
       <c r="E67" s="71" t="n">
-        <v>0.09084805718049918</v>
+        <v>0.1290618218646272</v>
       </c>
       <c r="F67" s="71" t="n">
-        <v>-0.03812775917075606</v>
+        <v>-0.05399023928653108</v>
       </c>
       <c r="G67" s="71" t="n">
-        <v>0.06516790623385817</v>
+        <v>0.1205467056942764</v>
       </c>
       <c r="H67" s="71" t="n">
-        <v>0.04146783329037527</v>
+        <v>0.05401940449224688</v>
       </c>
     </row>
     <row r="68">
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>International payments — number per user per year</t>
+          <t>Overdraft — average limit</t>
         </is>
       </c>
       <c r="C68" s="63" t="n">
-        <v>30</v>
+        <v>15000</v>
       </c>
       <c r="D68" s="14" t="inlineStr">
         <is>
-          <t>payments</t>
+          <t>£/facility</t>
         </is>
       </c>
       <c r="E68" s="71" t="n">
-        <v>0.09034327530523904</v>
+        <v>0.1230830424521848</v>
       </c>
       <c r="F68" s="71" t="n">
-        <v>-0.03779928987864309</v>
+        <v>-0.0590550445253119</v>
       </c>
       <c r="G68" s="71" t="n">
-        <v>0.08438484684763596</v>
+        <v>0.07584524768646449</v>
       </c>
       <c r="H68" s="71" t="n">
-        <v>0.03781358314457282</v>
+        <v>0.0590899401158306</v>
       </c>
     </row>
     <row r="69">
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>International payment fee</t>
+          <t>Overdraft — penetration</t>
         </is>
       </c>
       <c r="C69" s="63" t="n">
-        <v>17.5</v>
+        <v>0.25</v>
       </c>
       <c r="D69" s="14" t="inlineStr">
         <is>
-          <t>£/payment</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E69" s="71" t="n">
-        <v>0.09034327530523904</v>
+        <v>0.1051536008356984</v>
       </c>
       <c r="F69" s="71" t="n">
-        <v>-0.03779928987864309</v>
+        <v>-0.04443224426671098</v>
       </c>
       <c r="G69" s="71" t="n">
-        <v>0.08438484684763596</v>
+        <v>0.05792426513148669</v>
       </c>
       <c r="H69" s="71" t="n">
-        <v>0.03781358314457282</v>
+        <v>0.0590899401158306</v>
       </c>
     </row>
     <row r="70">
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>BCA — monthly account fee</t>
+          <t>Productive hours per FTE per month</t>
         </is>
       </c>
       <c r="C70" s="63" t="n">
-        <v>8.5</v>
+        <v>147</v>
       </c>
       <c r="D70" s="14" t="inlineStr">
         <is>
-          <t>£/month</t>
+          <t>hours</t>
         </is>
       </c>
       <c r="E70" s="71" t="n">
-        <v>0.08776203886793855</v>
+        <v>0.1049299343026391</v>
       </c>
       <c r="F70" s="71" t="n">
-        <v>-0.0367197067332557</v>
+        <v>-0.08562877535793163</v>
       </c>
       <c r="G70" s="71" t="n">
-        <v>0.08197399065083791</v>
+        <v>0.1049299343027884</v>
       </c>
       <c r="H70" s="71" t="n">
-        <v>0.03673319505471902</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>Relationship manager — salary</t>
+          <t>Customers per relationship manager (L)</t>
         </is>
       </c>
       <c r="C71" s="63" t="n">
-        <v>65000</v>
+        <v>120</v>
       </c>
       <c r="D71" s="14" t="inlineStr">
         <is>
-          <t>£/yr</t>
+          <t>customers</t>
         </is>
       </c>
       <c r="E71" s="71" t="n">
-        <v>-0.08359164263118203</v>
+        <v>0.1048340737728719</v>
       </c>
       <c r="F71" s="71" t="n">
-        <v>0.0682155195867932</v>
+        <v>-0.0855505477307521</v>
       </c>
       <c r="G71" s="71" t="n">
-        <v>-0.08359164263111851</v>
+        <v>0.1048340737730304</v>
       </c>
       <c r="H71" s="71" t="n">
         <v>0</v>
@@ -9465,349 +9230,349 @@
     <row r="72">
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>Instant-access savings — average balance</t>
+          <t>Share of customers that are relationship-managed</t>
         </is>
       </c>
       <c r="C72" s="63" t="n">
-        <v>30000</v>
+        <v>0.15</v>
       </c>
       <c r="D72" s="14" t="inlineStr">
         <is>
-          <t>£/account</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E72" s="71" t="n">
-        <v>0.07891881788782402</v>
+        <v>-0.1046385357465969</v>
       </c>
       <c r="F72" s="71" t="n">
-        <v>-0.03155780944412719</v>
+        <v>0.08539097761546771</v>
       </c>
       <c r="G72" s="71" t="n">
-        <v>0.07347170588420676</v>
+        <v>-0.1046385357468233</v>
       </c>
       <c r="H72" s="71" t="n">
-        <v>0.03457241887503357</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>Term loans — average life</t>
+          <t>BCA — net transaction &amp; cash-handling income</t>
         </is>
       </c>
       <c r="C73" s="63" t="n">
-        <v>4</v>
+        <v>120</v>
       </c>
       <c r="D73" s="14" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>£/account/yr</t>
         </is>
       </c>
       <c r="E73" s="71" t="n">
-        <v>-0.07829491028629054</v>
+        <v>0.1032494574917018</v>
       </c>
       <c r="F73" s="71" t="n">
-        <v>0.02580762668294011</v>
+        <v>-0.04319685584629245</v>
       </c>
       <c r="G73" s="71" t="n">
-        <v>-0.07198396348042548</v>
+        <v>0.0964390048174012</v>
       </c>
       <c r="H73" s="71" t="n">
-        <v>-0.0401134191773455</v>
+        <v>0.0432155235937975</v>
       </c>
     </row>
     <row r="74">
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>BCA — credit interest paid</t>
+          <t>Change-the-bank / transformation spend per customer</t>
         </is>
       </c>
       <c r="C74" s="63" t="n">
-        <v>0.005</v>
+        <v>120</v>
       </c>
       <c r="D74" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E74" s="71" t="n">
-        <v>-0.07743709311877632</v>
+        <v>-0.1022430029315939</v>
       </c>
       <c r="F74" s="71" t="n">
-        <v>0.03242215124722145</v>
+        <v>0.0834360870245049</v>
       </c>
       <c r="G74" s="71" t="n">
-        <v>-0.07233786615856722</v>
+        <v>-0.1022430029318107</v>
       </c>
       <c r="H74" s="71" t="n">
-        <v>-0.03241164269534813</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>Instant-access savings — penetration</t>
+          <t>Term loans — probability of default</t>
         </is>
       </c>
       <c r="C75" s="63" t="n">
-        <v>0.4</v>
+        <v>0.018</v>
       </c>
       <c r="D75" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E75" s="71" t="n">
-        <v>0.07661700997629903</v>
+        <v>-0.1012205729022779</v>
       </c>
       <c r="F75" s="71" t="n">
-        <v>-0.02968005287393479</v>
+        <v>0</v>
       </c>
       <c r="G75" s="71" t="n">
-        <v>0.07117002325613006</v>
+        <v>-0.1012205729024857</v>
       </c>
       <c r="H75" s="71" t="n">
-        <v>0.03457241887503357</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — average utilisation</t>
+          <t>Term loans — loss given default</t>
         </is>
       </c>
       <c r="C76" s="63" t="n">
-        <v>0.45</v>
+        <v>0.25</v>
       </c>
       <c r="D76" s="14" t="inlineStr">
         <is>
-          <t>% of limit</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E76" s="71" t="n">
-        <v>0.07468485925308183</v>
+        <v>-0.1012205729022779</v>
       </c>
       <c r="F76" s="71" t="n">
-        <v>-0.03881758952731159</v>
+        <v>0</v>
       </c>
       <c r="G76" s="71" t="n">
-        <v>0.03065869518523666</v>
+        <v>-0.1012205729024857</v>
       </c>
       <c r="H76" s="71" t="n">
-        <v>0.03883266343130445</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — funded invoices as multiple of advances</t>
+          <t>Term loans — arrangement fee</t>
         </is>
       </c>
       <c r="C77" s="63" t="n">
-        <v>8</v>
+        <v>0.015</v>
       </c>
       <c r="D77" s="14" t="inlineStr">
         <is>
-          <t>x p.a.</t>
+          <t>% of loan</t>
         </is>
       </c>
       <c r="E77" s="71" t="n">
-        <v>0.07330711481910879</v>
+        <v>0.09679636639847039</v>
       </c>
       <c r="F77" s="71" t="n">
-        <v>-0.03067361016112366</v>
+        <v>-0.04049814572625951</v>
       </c>
       <c r="G77" s="71" t="n">
-        <v>0.06847304438958647</v>
+        <v>0.09041195146079069</v>
       </c>
       <c r="H77" s="71" t="n">
-        <v>0.03068302175159092</v>
+        <v>0.04051455336918516</v>
       </c>
     </row>
     <row r="78">
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — service fee</t>
+          <t>Invoice finance — average funds in use (advances)</t>
         </is>
       </c>
       <c r="C78" s="63" t="n">
-        <v>0.01</v>
+        <v>150000</v>
       </c>
       <c r="D78" s="14" t="inlineStr">
         <is>
-          <t>% of funded invoices</t>
+          <t>£/client</t>
         </is>
       </c>
       <c r="E78" s="71" t="n">
-        <v>0.07330711481910879</v>
+        <v>0.09492162631565762</v>
       </c>
       <c r="F78" s="71" t="n">
-        <v>-0.03067361016112366</v>
+        <v>-0.04145064460605613</v>
       </c>
       <c r="G78" s="71" t="n">
-        <v>0.06847304438958647</v>
+        <v>0.0692404302199741</v>
       </c>
       <c r="H78" s="71" t="n">
-        <v>0.03068302175159092</v>
+        <v>0.04146783329037527</v>
       </c>
     </row>
     <row r="79">
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t>Credit analyst / underwriter — salary</t>
+          <t>Term loans — risk weight</t>
         </is>
       </c>
       <c r="C79" s="63" t="n">
-        <v>55000</v>
+        <v>0.7</v>
       </c>
       <c r="D79" s="14" t="inlineStr">
         <is>
-          <t>£/yr</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E79" s="71" t="n">
-        <v>-0.0568734448830966</v>
+        <v>0.09393575894340188</v>
       </c>
       <c r="F79" s="71" t="n">
-        <v>0.04641195544512514</v>
+        <v>-0.03930178091372589</v>
       </c>
       <c r="G79" s="71" t="n">
-        <v>-0.05687344488291048</v>
+        <v>-0.5376796480568484</v>
       </c>
       <c r="H79" s="71" t="n">
-        <v>0</v>
+        <v>0.03931723328663613</v>
       </c>
     </row>
     <row r="80">
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t>Liquidity buffer held against deposits (LCR / HQLA)</t>
+          <t>Invoice finance — penetration</t>
         </is>
       </c>
       <c r="C80" s="63" t="n">
-        <v>0.15</v>
+        <v>0.0071</v>
       </c>
       <c r="D80" s="14" t="inlineStr">
         <is>
-          <t>% of deposits</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E80" s="71" t="n">
-        <v>-0.05323800151894711</v>
+        <v>0.09084805718049918</v>
       </c>
       <c r="F80" s="71" t="n">
-        <v>0.02228797078263317</v>
+        <v>-0.03812775917075606</v>
       </c>
       <c r="G80" s="71" t="n">
-        <v>-0.04973148989456535</v>
+        <v>0.06516790623385817</v>
       </c>
       <c r="H80" s="71" t="n">
-        <v>-0.02228300435307398</v>
+        <v>0.04146783329037527</v>
       </c>
     </row>
     <row r="81">
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>Yield give-up on the liquidity buffer vs Bank Rate</t>
+          <t>International payments — number per user per year</t>
         </is>
       </c>
       <c r="C81" s="63" t="n">
-        <v>0.01</v>
+        <v>30</v>
       </c>
       <c r="D81" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>payments</t>
         </is>
       </c>
       <c r="E81" s="71" t="n">
-        <v>-0.05323800151894711</v>
+        <v>0.09034327530523904</v>
       </c>
       <c r="F81" s="71" t="n">
-        <v>0.02228797078263317</v>
+        <v>-0.03779928987864309</v>
       </c>
       <c r="G81" s="71" t="n">
-        <v>-0.04973148989456535</v>
+        <v>0.08438484684763596</v>
       </c>
       <c r="H81" s="71" t="n">
-        <v>-0.02228300435307398</v>
+        <v>0.03781358314457282</v>
       </c>
     </row>
     <row r="82">
       <c r="B82" s="10" t="inlineStr">
         <is>
-          <t>Unit-level platform &amp; processing cost</t>
+          <t>International payment fee</t>
         </is>
       </c>
       <c r="C82" s="63" t="n">
-        <v>60</v>
+        <v>17.5</v>
       </c>
       <c r="D82" s="14" t="inlineStr">
         <is>
-          <t>£/customer/yr</t>
+          <t>£/payment</t>
         </is>
       </c>
       <c r="E82" s="71" t="n">
-        <v>-0.05112150146579695</v>
+        <v>0.09034327530523904</v>
       </c>
       <c r="F82" s="71" t="n">
-        <v>0.04171804351234986</v>
+        <v>-0.03779928987864309</v>
       </c>
       <c r="G82" s="71" t="n">
-        <v>-0.05112150146589774</v>
+        <v>0.08438484684763596</v>
       </c>
       <c r="H82" s="71" t="n">
-        <v>0</v>
+        <v>0.03781358314457282</v>
       </c>
     </row>
     <row r="83">
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — annual arrangement/renewal fee</t>
+          <t>BCA — monthly account fee</t>
         </is>
       </c>
       <c r="C83" s="63" t="n">
-        <v>0.015</v>
+        <v>8.5</v>
       </c>
       <c r="D83" s="14" t="inlineStr">
         <is>
-          <t>% of limit</t>
+          <t>£/month</t>
         </is>
       </c>
       <c r="E83" s="71" t="n">
-        <v>0.04839818319938068</v>
+        <v>0.08776203886793855</v>
       </c>
       <c r="F83" s="71" t="n">
-        <v>-0.0202531739430378</v>
+        <v>-0.0367197067332557</v>
       </c>
       <c r="G83" s="71" t="n">
-        <v>0.04520741744945692</v>
+        <v>0.08197399065083791</v>
       </c>
       <c r="H83" s="71" t="n">
-        <v>0.02025727668465901</v>
+        <v>0.03673319505471902</v>
       </c>
     </row>
     <row r="84">
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t>Fraud &amp; payment losses (incl. APP reimbursement) per current account</t>
+          <t>Relationship manager — salary</t>
         </is>
       </c>
       <c r="C84" s="63" t="n">
-        <v>45</v>
+        <v>65000</v>
       </c>
       <c r="D84" s="14" t="inlineStr">
         <is>
-          <t>£/BCA/yr</t>
+          <t>£/yr</t>
         </is>
       </c>
       <c r="E84" s="71" t="n">
-        <v>-0.03834112609934771</v>
+        <v>-0.08359164263118203</v>
       </c>
       <c r="F84" s="71" t="n">
-        <v>0.03128853263420828</v>
+        <v>0.0682155195867932</v>
       </c>
       <c r="G84" s="71" t="n">
-        <v>-0.03834112609929025</v>
+        <v>-0.08359164263111851</v>
       </c>
       <c r="H84" s="71" t="n">
         <v>0</v>
@@ -9816,295 +9581,295 @@
     <row r="85">
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — probability of default</t>
+          <t>Instant-access savings — average balance</t>
         </is>
       </c>
       <c r="C85" s="63" t="n">
-        <v>0.022</v>
+        <v>30000</v>
       </c>
       <c r="D85" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/account</t>
         </is>
       </c>
       <c r="E85" s="71" t="n">
-        <v>-0.03694925801944137</v>
+        <v>0.07891881788782402</v>
       </c>
       <c r="F85" s="71" t="n">
-        <v>0</v>
+        <v>-0.03155780944412719</v>
       </c>
       <c r="G85" s="71" t="n">
-        <v>-0.03694925801941038</v>
+        <v>0.07347170588420676</v>
       </c>
       <c r="H85" s="71" t="n">
-        <v>0</v>
+        <v>0.03457241887503357</v>
       </c>
     </row>
     <row r="86">
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — loss given default</t>
+          <t>Term loans — average life</t>
         </is>
       </c>
       <c r="C86" s="63" t="n">
-        <v>0.35</v>
+        <v>4</v>
       </c>
       <c r="D86" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>years</t>
         </is>
       </c>
       <c r="E86" s="71" t="n">
-        <v>-0.03694925801944137</v>
+        <v>-0.07829491028629054</v>
       </c>
       <c r="F86" s="71" t="n">
-        <v>0</v>
+        <v>0.02580762668294011</v>
       </c>
       <c r="G86" s="71" t="n">
-        <v>-0.03694925801941038</v>
+        <v>-0.07198396348042548</v>
       </c>
       <c r="H86" s="71" t="n">
-        <v>0</v>
+        <v>-0.0401134191773455</v>
       </c>
     </row>
     <row r="87">
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t>Management span (staff per manager)</t>
+          <t>BCA — credit interest paid</t>
         </is>
       </c>
       <c r="C87" s="63" t="n">
-        <v>8</v>
+        <v>0.005</v>
       </c>
       <c r="D87" s="14" t="inlineStr">
         <is>
-          <t>staff</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E87" s="71" t="n">
-        <v>0.03323477624632555</v>
+        <v>-0.07743709311877632</v>
       </c>
       <c r="F87" s="71" t="n">
-        <v>-0.02712146165108484</v>
+        <v>0.03242215124722145</v>
       </c>
       <c r="G87" s="71" t="n">
-        <v>0.03323477624586131</v>
+        <v>-0.07233786615856722</v>
       </c>
       <c r="H87" s="71" t="n">
-        <v>0</v>
+        <v>-0.03241164269534813</v>
       </c>
     </row>
     <row r="88">
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t>Annual customer churn (replaced at steady state)</t>
+          <t>Instant-access savings — penetration</t>
         </is>
       </c>
       <c r="C88" s="63" t="n">
-        <v>0.12</v>
+        <v>0.4</v>
       </c>
       <c r="D88" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E88" s="71" t="n">
-        <v>-0.03192622160754524</v>
+        <v>0.07661700997629903</v>
       </c>
       <c r="F88" s="71" t="n">
-        <v>0.02605360687805449</v>
+        <v>-0.02968005287393479</v>
       </c>
       <c r="G88" s="71" t="n">
-        <v>-0.03192622160733487</v>
+        <v>0.07117002325613006</v>
       </c>
       <c r="H88" s="71" t="n">
-        <v>0</v>
+        <v>0.03457241887503357</v>
       </c>
     </row>
     <row r="89">
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t>Team manager — salary</t>
+          <t>Overdraft — average utilisation</t>
         </is>
       </c>
       <c r="C89" s="63" t="n">
-        <v>85000</v>
+        <v>0.45</v>
       </c>
       <c r="D89" s="14" t="inlineStr">
         <is>
-          <t>£/yr</t>
+          <t>% of limit</t>
         </is>
       </c>
       <c r="E89" s="71" t="n">
-        <v>-0.03136675261572086</v>
+        <v>0.07468485925308183</v>
       </c>
       <c r="F89" s="71" t="n">
-        <v>0.02559704846183944</v>
+        <v>-0.03881758952731159</v>
       </c>
       <c r="G89" s="71" t="n">
-        <v>-0.0313667526155505</v>
+        <v>0.03065869518523666</v>
       </c>
       <c r="H89" s="71" t="n">
-        <v>0</v>
+        <v>0.03883266343130445</v>
       </c>
     </row>
     <row r="90">
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t>Employment on-costs (NI, pension, benefits)</t>
+          <t>Invoice finance — funded invoices as multiple of advances</t>
         </is>
       </c>
       <c r="C90" s="63" t="n">
-        <v>0.15</v>
+        <v>8</v>
       </c>
       <c r="D90" s="14" t="inlineStr">
         <is>
-          <t>% of salary</t>
+          <t>x p.a.</t>
         </is>
       </c>
       <c r="E90" s="71" t="n">
-        <v>-0.02505108334161372</v>
+        <v>0.07330711481910879</v>
       </c>
       <c r="F90" s="71" t="n">
-        <v>0.02044310426958103</v>
+        <v>-0.03067361016112366</v>
       </c>
       <c r="G90" s="71" t="n">
-        <v>-0.02505108334171299</v>
+        <v>0.06847304438958647</v>
       </c>
       <c r="H90" s="71" t="n">
-        <v>0</v>
+        <v>0.03068302175159092</v>
       </c>
     </row>
     <row r="91">
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t>Churn replacement — acquisition marketing per new customer won</t>
+          <t>Invoice finance — service fee</t>
         </is>
       </c>
       <c r="C91" s="63" t="n">
-        <v>240</v>
+        <v>0.01</v>
       </c>
       <c r="D91" s="14" t="inlineStr">
         <is>
-          <t>£/new customer</t>
+          <t>% of funded invoices</t>
         </is>
       </c>
       <c r="E91" s="71" t="n">
-        <v>-0.02361813367720083</v>
+        <v>0.07330711481910879</v>
       </c>
       <c r="F91" s="71" t="n">
-        <v>0.01927373610267698</v>
+        <v>-0.03067361016112366</v>
       </c>
       <c r="G91" s="71" t="n">
-        <v>-0.02361813367739114</v>
+        <v>0.06847304438958647</v>
       </c>
       <c r="H91" s="71" t="n">
-        <v>0</v>
+        <v>0.03068302175159092</v>
       </c>
     </row>
     <row r="92">
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — discount margin over base</t>
+          <t>Credit analyst / underwriter — salary</t>
         </is>
       </c>
       <c r="C92" s="63" t="n">
-        <v>0.025</v>
+        <v>55000</v>
       </c>
       <c r="D92" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/yr</t>
         </is>
       </c>
       <c r="E92" s="71" t="n">
-        <v>0.02290847338118557</v>
+        <v>-0.0568734448830966</v>
       </c>
       <c r="F92" s="71" t="n">
-        <v>-0.009587525002924749</v>
+        <v>0.04641195544512514</v>
       </c>
       <c r="G92" s="71" t="n">
-        <v>0.02139853701481027</v>
+        <v>-0.05687344488291048</v>
       </c>
       <c r="H92" s="71" t="n">
-        <v>0.009588444297347251</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93">
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t>Asset finance — risk weight</t>
+          <t>Liquidity buffer held against deposits (LCR / HQLA)</t>
         </is>
       </c>
       <c r="C93" s="63" t="n">
-        <v>0.8</v>
+        <v>0.15</v>
       </c>
       <c r="D93" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% of deposits</t>
         </is>
       </c>
       <c r="E93" s="71" t="n">
-        <v>0.02290243265667439</v>
+        <v>-0.05323800151894711</v>
       </c>
       <c r="F93" s="71" t="n">
-        <v>-0.009584997115274458</v>
+        <v>0.02228797078263317</v>
       </c>
       <c r="G93" s="71" t="n">
-        <v>-0.1317199514189854</v>
+        <v>-0.04973148989456535</v>
       </c>
       <c r="H93" s="71" t="n">
-        <v>0.009585915925127142</v>
+        <v>-0.02228300435307398</v>
       </c>
     </row>
     <row r="94">
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t>Operational-risk RWA multiple of gross income</t>
+          <t>Yield give-up on the liquidity buffer vs Bank Rate</t>
         </is>
       </c>
       <c r="C94" s="63" t="n">
-        <v>1.875</v>
+        <v>0.01</v>
       </c>
       <c r="D94" s="14" t="inlineStr">
         <is>
-          <t>x revenue</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E94" s="71" t="n">
-        <v>0.0220623226696928</v>
+        <v>-0.05323800151894711</v>
       </c>
       <c r="F94" s="71" t="n">
-        <v>-0.009233431480186292</v>
+        <v>0.02228797078263317</v>
       </c>
       <c r="G94" s="71" t="n">
-        <v>-0.1268953788846724</v>
+        <v>-0.04973148989456535</v>
       </c>
       <c r="H94" s="71" t="n">
-        <v>0.009234284121481744</v>
+        <v>-0.02228300435307398</v>
       </c>
     </row>
     <row r="95">
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t>Share of lending balances held by RM-managed customers</t>
+          <t>Unit-level platform &amp; processing cost</t>
         </is>
       </c>
       <c r="C95" s="63" t="n">
-        <v>0.6</v>
+        <v>60</v>
       </c>
       <c r="D95" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/customer/yr</t>
         </is>
       </c>
       <c r="E95" s="71" t="n">
-        <v>0.02187481379496614</v>
+        <v>-0.05112150146579695</v>
       </c>
       <c r="F95" s="71" t="n">
-        <v>0</v>
+        <v>0.04171804351234986</v>
       </c>
       <c r="G95" s="71" t="n">
-        <v>0.021874813795008</v>
+        <v>-0.05112150146589774</v>
       </c>
       <c r="H95" s="71" t="n">
         <v>0</v>
@@ -10113,79 +9878,79 @@
     <row r="96">
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t>Stewardship effect: relative PD reduction on RM-covered balances</t>
+          <t>Overdraft — annual arrangement/renewal fee</t>
         </is>
       </c>
       <c r="C96" s="63" t="n">
-        <v>0.2</v>
+        <v>0.015</v>
       </c>
       <c r="D96" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% of limit</t>
         </is>
       </c>
       <c r="E96" s="71" t="n">
-        <v>0.02187481379496614</v>
+        <v>0.04839818319938068</v>
       </c>
       <c r="F96" s="71" t="n">
-        <v>0</v>
+        <v>-0.0202531739430378</v>
       </c>
       <c r="G96" s="71" t="n">
-        <v>0.021874813795008</v>
+        <v>0.04520741744945692</v>
       </c>
       <c r="H96" s="71" t="n">
-        <v>0</v>
+        <v>0.02025727668465901</v>
       </c>
     </row>
     <row r="97">
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t>Card — interest rate on revolving balances</t>
+          <t>Fraud &amp; payment losses (incl. APP reimbursement) per current account</t>
         </is>
       </c>
       <c r="C97" s="63" t="n">
-        <v>0.159</v>
+        <v>45</v>
       </c>
       <c r="D97" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>£/BCA/yr</t>
         </is>
       </c>
       <c r="E97" s="71" t="n">
-        <v>0.02052082967661485</v>
+        <v>-0.03834112609934771</v>
       </c>
       <c r="F97" s="71" t="n">
-        <v>-0.008588347653644276</v>
+        <v>0.03128853263420828</v>
       </c>
       <c r="G97" s="71" t="n">
-        <v>0.01916829711878616</v>
+        <v>-0.03834112609929025</v>
       </c>
       <c r="H97" s="71" t="n">
-        <v>0.008589085314331023</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t>Service &amp; operations staff — salary</t>
+          <t>Asset finance — probability of default</t>
         </is>
       </c>
       <c r="C98" s="63" t="n">
-        <v>32000</v>
+        <v>0.022</v>
       </c>
       <c r="D98" s="14" t="inlineStr">
         <is>
-          <t>£/yr</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E98" s="71" t="n">
-        <v>-0.02022646549070539</v>
+        <v>-0.03694925801944137</v>
       </c>
       <c r="F98" s="71" t="n">
-        <v>0.01650594257292187</v>
+        <v>0</v>
       </c>
       <c r="G98" s="71" t="n">
-        <v>-0.02022646549081312</v>
+        <v>-0.03694925801941038</v>
       </c>
       <c r="H98" s="71" t="n">
         <v>0</v>
@@ -10194,25 +9959,25 @@
     <row r="99">
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — probability of default</t>
+          <t>Asset finance — loss given default</t>
         </is>
       </c>
       <c r="C99" s="63" t="n">
-        <v>0.026</v>
+        <v>0.35</v>
       </c>
       <c r="D99" s="14" t="inlineStr">
         <is>
-          <t>% p.a.</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E99" s="71" t="n">
-        <v>-0.01809317740628059</v>
+        <v>-0.03694925801944137</v>
       </c>
       <c r="F99" s="71" t="n">
         <v>0</v>
       </c>
       <c r="G99" s="71" t="n">
-        <v>-0.01809317740626373</v>
+        <v>-0.03694925801941038</v>
       </c>
       <c r="H99" s="71" t="n">
         <v>0</v>
@@ -10221,25 +9986,25 @@
     <row r="100">
       <c r="B100" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — loss given default</t>
+          <t>Management span (staff per manager)</t>
         </is>
       </c>
       <c r="C100" s="63" t="n">
-        <v>0.55</v>
+        <v>8</v>
       </c>
       <c r="D100" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>staff</t>
         </is>
       </c>
       <c r="E100" s="71" t="n">
-        <v>-0.01809317740628059</v>
+        <v>0.03323477624632555</v>
       </c>
       <c r="F100" s="71" t="n">
-        <v>0</v>
+        <v>-0.02712146165108484</v>
       </c>
       <c r="G100" s="71" t="n">
-        <v>-0.01809317740626373</v>
+        <v>0.03323477624586131</v>
       </c>
       <c r="H100" s="71" t="n">
         <v>0</v>
@@ -10248,25 +10013,25 @@
     <row r="101">
       <c r="B101" s="10" t="inlineStr">
         <is>
-          <t>Term loan underwriting &amp; completion</t>
+          <t>Annual customer churn (replaced at steady state)</t>
         </is>
       </c>
       <c r="C101" s="63" t="n">
-        <v>14</v>
+        <v>0.12</v>
       </c>
       <c r="D101" s="14" t="inlineStr">
         <is>
-          <t>hrs/new loan</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E101" s="71" t="n">
-        <v>-0.0177185070089608</v>
+        <v>-0.03192622160754524</v>
       </c>
       <c r="F101" s="71" t="n">
-        <v>0.01445930626422265</v>
+        <v>0.02605360687805449</v>
       </c>
       <c r="G101" s="71" t="n">
-        <v>-0.01771850700938827</v>
+        <v>-0.03192622160733487</v>
       </c>
       <c r="H101" s="71" t="n">
         <v>0</v>
@@ -10275,25 +10040,25 @@
     <row r="102">
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t>BCA servicing (queries, payments support)</t>
+          <t>Team manager — salary</t>
         </is>
       </c>
       <c r="C102" s="63" t="n">
-        <v>0.6</v>
+        <v>85000</v>
       </c>
       <c r="D102" s="14" t="inlineStr">
         <is>
-          <t>hrs/account/yr</t>
+          <t>£/yr</t>
         </is>
       </c>
       <c r="E102" s="71" t="n">
-        <v>-0.01726355933582919</v>
+        <v>-0.03136675261572086</v>
       </c>
       <c r="F102" s="71" t="n">
-        <v>0.01408804316967071</v>
+        <v>0.02559704846183944</v>
       </c>
       <c r="G102" s="71" t="n">
-        <v>-0.01726355933577883</v>
+        <v>-0.0313667526155505</v>
       </c>
       <c r="H102" s="71" t="n">
         <v>0</v>
@@ -10302,25 +10067,25 @@
     <row r="103">
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t>Premises &amp; facilities per unit FTE</t>
+          <t>Employment on-costs (NI, pension, benefits)</t>
         </is>
       </c>
       <c r="C103" s="63" t="n">
-        <v>6000</v>
+        <v>0.15</v>
       </c>
       <c r="D103" s="14" t="inlineStr">
         <is>
-          <t>£/FTE/yr</t>
+          <t>% of salary</t>
         </is>
       </c>
       <c r="E103" s="71" t="n">
-        <v>-0.0165027854462771</v>
+        <v>-0.02505108334161372</v>
       </c>
       <c r="F103" s="71" t="n">
-        <v>0.01346720854414594</v>
+        <v>0.02044310426958103</v>
       </c>
       <c r="G103" s="71" t="n">
-        <v>-0.01650278544651348</v>
+        <v>-0.02505108334171299</v>
       </c>
       <c r="H103" s="71" t="n">
         <v>0</v>
@@ -10329,25 +10094,25 @@
     <row r="104">
       <c r="B104" s="10" t="inlineStr">
         <is>
-          <t>Overdraft annual review &amp; renewal</t>
+          <t>Churn replacement — acquisition marketing per new customer won</t>
         </is>
       </c>
       <c r="C104" s="63" t="n">
-        <v>1.5</v>
+        <v>240</v>
       </c>
       <c r="D104" s="14" t="inlineStr">
         <is>
-          <t>hrs/facility/yr</t>
+          <t>£/new customer</t>
         </is>
       </c>
       <c r="E104" s="71" t="n">
-        <v>-0.01582009554374381</v>
+        <v>-0.02361813367720083</v>
       </c>
       <c r="F104" s="71" t="n">
-        <v>0.01291009487869291</v>
+        <v>0.01927373610267698</v>
       </c>
       <c r="G104" s="71" t="n">
-        <v>-0.01582009554390931</v>
+        <v>-0.02361813367739114</v>
       </c>
       <c r="H104" s="71" t="n">
         <v>0</v>
@@ -10356,38 +10121,38 @@
     <row r="105">
       <c r="B105" s="10" t="inlineStr">
         <is>
-          <t>Term loan annual review</t>
+          <t>Invoice finance — discount margin over base</t>
         </is>
       </c>
       <c r="C105" s="63" t="n">
-        <v>3</v>
+        <v>0.025</v>
       </c>
       <c r="D105" s="14" t="inlineStr">
         <is>
-          <t>hrs/loan/yr</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E105" s="71" t="n">
-        <v>-0.01518729172200041</v>
+        <v>0.02290847338118557</v>
       </c>
       <c r="F105" s="71" t="n">
-        <v>0.01239369108365343</v>
+        <v>-0.009587525002924749</v>
       </c>
       <c r="G105" s="71" t="n">
-        <v>-0.01518729172225025</v>
+        <v>0.02139853701481027</v>
       </c>
       <c r="H105" s="71" t="n">
-        <v>0</v>
+        <v>0.009588444297347251</v>
       </c>
     </row>
     <row r="106">
       <c r="B106" s="10" t="inlineStr">
         <is>
-          <t>Card — share of cards revolving a balance</t>
+          <t>Asset finance — risk weight</t>
         </is>
       </c>
       <c r="C106" s="63" t="n">
-        <v>0.25</v>
+        <v>0.8</v>
       </c>
       <c r="D106" s="14" t="inlineStr">
         <is>
@@ -10395,67 +10160,67 @@
         </is>
       </c>
       <c r="E106" s="71" t="n">
-        <v>0.01282939010311848</v>
+        <v>0.02290243265667439</v>
       </c>
       <c r="F106" s="71" t="n">
-        <v>-0.00677352684355925</v>
+        <v>-0.009584997115274458</v>
       </c>
       <c r="G106" s="71" t="n">
-        <v>0.008393731325598055</v>
+        <v>-0.1317199514189854</v>
       </c>
       <c r="H106" s="71" t="n">
-        <v>0.00677398568124732</v>
+        <v>0.009585915925127142</v>
       </c>
     </row>
     <row r="107">
       <c r="B107" s="10" t="inlineStr">
         <is>
-          <t>Card — average revolving balance (revolvers)</t>
+          <t>Operational-risk RWA multiple of gross income</t>
         </is>
       </c>
       <c r="C107" s="63" t="n">
-        <v>2000</v>
+        <v>1.875</v>
       </c>
       <c r="D107" s="14" t="inlineStr">
         <is>
-          <t>£/card</t>
+          <t>x revenue</t>
         </is>
       </c>
       <c r="E107" s="71" t="n">
-        <v>0.01282939010311848</v>
+        <v>0.0220623226696928</v>
       </c>
       <c r="F107" s="71" t="n">
-        <v>-0.00677352684355925</v>
+        <v>-0.009233431480186292</v>
       </c>
       <c r="G107" s="71" t="n">
-        <v>0.008393731325598055</v>
+        <v>-0.1268953788846724</v>
       </c>
       <c r="H107" s="71" t="n">
-        <v>0.00677398568124732</v>
+        <v>0.009234284121481744</v>
       </c>
     </row>
     <row r="108">
       <c r="B108" s="10" t="inlineStr">
         <is>
-          <t>FSCS deposit-protection levy</t>
+          <t>Share of lending balances held by RM-managed customers</t>
         </is>
       </c>
       <c r="C108" s="63" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.6</v>
       </c>
       <c r="D108" s="14" t="inlineStr">
         <is>
-          <t>% of protected deposits</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E108" s="71" t="n">
-        <v>-0.01265257161278474</v>
+        <v>0.02187481379496614</v>
       </c>
       <c r="F108" s="71" t="n">
-        <v>0.0103252157693554</v>
+        <v>0</v>
       </c>
       <c r="G108" s="71" t="n">
-        <v>-0.0126525716125313</v>
+        <v>0.021874813795008</v>
       </c>
       <c r="H108" s="71" t="n">
         <v>0</v>
@@ -10464,11 +10229,11 @@
     <row r="109">
       <c r="B109" s="10" t="inlineStr">
         <is>
-          <t>Share of deposit balances that are FSCS-protected</t>
+          <t>Stewardship effect: relative PD reduction on RM-covered balances</t>
         </is>
       </c>
       <c r="C109" s="63" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="D109" s="14" t="inlineStr">
         <is>
@@ -10476,13 +10241,13 @@
         </is>
       </c>
       <c r="E109" s="71" t="n">
-        <v>-0.01265257161278474</v>
+        <v>0.02187481379496614</v>
       </c>
       <c r="F109" s="71" t="n">
-        <v>0.0103252157693554</v>
+        <v>0</v>
       </c>
       <c r="G109" s="71" t="n">
-        <v>-0.0126525716125313</v>
+        <v>0.021874813795008</v>
       </c>
       <c r="H109" s="71" t="n">
         <v>0</v>
@@ -10491,81 +10256,432 @@
     <row r="110">
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t>Overdraft — risk weight</t>
+          <t>Card — interest rate on revolving balances</t>
         </is>
       </c>
       <c r="C110" s="63" t="n">
-        <v>0.75</v>
+        <v>0.159</v>
       </c>
       <c r="D110" s="14" t="inlineStr">
         <is>
-          <t>% of drawn</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E110" s="71" t="n">
-        <v>0.00566130690060681</v>
+        <v>0.02052082967661485</v>
       </c>
       <c r="F110" s="71" t="n">
-        <v>-0.002369509251789935</v>
+        <v>-0.008588347653644276</v>
       </c>
       <c r="G110" s="71" t="n">
-        <v>-0.03259810445684302</v>
+        <v>0.01916829711878616</v>
       </c>
       <c r="H110" s="71" t="n">
-        <v>0.002369565398971374</v>
+        <v>0.008589085314331023</v>
       </c>
     </row>
     <row r="111">
       <c r="B111" s="10" t="inlineStr">
         <is>
-          <t>Invoice finance — risk weight</t>
+          <t>Service &amp; operations staff — salary</t>
         </is>
       </c>
       <c r="C111" s="63" t="n">
-        <v>0.6</v>
+        <v>32000</v>
       </c>
       <c r="D111" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>£/yr</t>
         </is>
       </c>
       <c r="E111" s="71" t="n">
-        <v>0.002858330950708488</v>
+        <v>-0.02022646549070539</v>
       </c>
       <c r="F111" s="71" t="n">
-        <v>-0.001196352928703285</v>
+        <v>0.01650594257292187</v>
       </c>
       <c r="G111" s="71" t="n">
-        <v>-0.01646153881572723</v>
+        <v>-0.02022646549081312</v>
       </c>
       <c r="H111" s="71" t="n">
-        <v>0.001196367241437099</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112">
       <c r="B112" s="10" t="inlineStr">
         <is>
-          <t>Tax rate (corporation tax + bank surcharge)</t>
+          <t>Overdraft — probability of default</t>
         </is>
       </c>
       <c r="C112" s="63" t="n">
-        <v>0.28</v>
+        <v>0.026</v>
       </c>
       <c r="D112" s="14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>% p.a.</t>
         </is>
       </c>
       <c r="E112" s="71" t="n">
-        <v>0</v>
+        <v>-0.01809317740628059</v>
       </c>
       <c r="F112" s="71" t="n">
         <v>0</v>
       </c>
       <c r="G112" s="71" t="n">
+        <v>-0.01809317740626373</v>
+      </c>
+      <c r="H112" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" s="10" t="inlineStr">
+        <is>
+          <t>Overdraft — loss given default</t>
+        </is>
+      </c>
+      <c r="C113" s="63" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D113" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E113" s="71" t="n">
+        <v>-0.01809317740628059</v>
+      </c>
+      <c r="F113" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G113" s="71" t="n">
+        <v>-0.01809317740626373</v>
+      </c>
+      <c r="H113" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="10" t="inlineStr">
+        <is>
+          <t>Term loan underwriting &amp; completion</t>
+        </is>
+      </c>
+      <c r="C114" s="63" t="n">
+        <v>14</v>
+      </c>
+      <c r="D114" s="14" t="inlineStr">
+        <is>
+          <t>hrs/new loan</t>
+        </is>
+      </c>
+      <c r="E114" s="71" t="n">
+        <v>-0.0177185070089608</v>
+      </c>
+      <c r="F114" s="71" t="n">
+        <v>0.01445930626422265</v>
+      </c>
+      <c r="G114" s="71" t="n">
+        <v>-0.01771850700938827</v>
+      </c>
+      <c r="H114" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="10" t="inlineStr">
+        <is>
+          <t>BCA servicing (queries, payments support)</t>
+        </is>
+      </c>
+      <c r="C115" s="63" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D115" s="14" t="inlineStr">
+        <is>
+          <t>hrs/account/yr</t>
+        </is>
+      </c>
+      <c r="E115" s="71" t="n">
+        <v>-0.01726355933582919</v>
+      </c>
+      <c r="F115" s="71" t="n">
+        <v>0.01408804316967071</v>
+      </c>
+      <c r="G115" s="71" t="n">
+        <v>-0.01726355933577883</v>
+      </c>
+      <c r="H115" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" s="10" t="inlineStr">
+        <is>
+          <t>Premises &amp; facilities per unit FTE</t>
+        </is>
+      </c>
+      <c r="C116" s="63" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D116" s="14" t="inlineStr">
+        <is>
+          <t>£/FTE/yr</t>
+        </is>
+      </c>
+      <c r="E116" s="71" t="n">
+        <v>-0.0165027854462771</v>
+      </c>
+      <c r="F116" s="71" t="n">
+        <v>0.01346720854414594</v>
+      </c>
+      <c r="G116" s="71" t="n">
+        <v>-0.01650278544651348</v>
+      </c>
+      <c r="H116" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="B117" s="10" t="inlineStr">
+        <is>
+          <t>Overdraft annual review &amp; renewal</t>
+        </is>
+      </c>
+      <c r="C117" s="63" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D117" s="14" t="inlineStr">
+        <is>
+          <t>hrs/facility/yr</t>
+        </is>
+      </c>
+      <c r="E117" s="71" t="n">
+        <v>-0.01582009554374381</v>
+      </c>
+      <c r="F117" s="71" t="n">
+        <v>0.01291009487869291</v>
+      </c>
+      <c r="G117" s="71" t="n">
+        <v>-0.01582009554390931</v>
+      </c>
+      <c r="H117" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" s="10" t="inlineStr">
+        <is>
+          <t>Term loan annual review</t>
+        </is>
+      </c>
+      <c r="C118" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="D118" s="14" t="inlineStr">
+        <is>
+          <t>hrs/loan/yr</t>
+        </is>
+      </c>
+      <c r="E118" s="71" t="n">
+        <v>-0.01518729172200041</v>
+      </c>
+      <c r="F118" s="71" t="n">
+        <v>0.01239369108365343</v>
+      </c>
+      <c r="G118" s="71" t="n">
+        <v>-0.01518729172225025</v>
+      </c>
+      <c r="H118" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="B119" s="10" t="inlineStr">
+        <is>
+          <t>Card — share of cards revolving a balance</t>
+        </is>
+      </c>
+      <c r="C119" s="63" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D119" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E119" s="71" t="n">
+        <v>0.01282939010311848</v>
+      </c>
+      <c r="F119" s="71" t="n">
+        <v>-0.00677352684355925</v>
+      </c>
+      <c r="G119" s="71" t="n">
+        <v>0.008393731325598055</v>
+      </c>
+      <c r="H119" s="71" t="n">
+        <v>0.00677398568124732</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="B120" s="10" t="inlineStr">
+        <is>
+          <t>Card — average revolving balance (revolvers)</t>
+        </is>
+      </c>
+      <c r="C120" s="63" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D120" s="14" t="inlineStr">
+        <is>
+          <t>£/card</t>
+        </is>
+      </c>
+      <c r="E120" s="71" t="n">
+        <v>0.01282939010311848</v>
+      </c>
+      <c r="F120" s="71" t="n">
+        <v>-0.00677352684355925</v>
+      </c>
+      <c r="G120" s="71" t="n">
+        <v>0.008393731325598055</v>
+      </c>
+      <c r="H120" s="71" t="n">
+        <v>0.00677398568124732</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="B121" s="10" t="inlineStr">
+        <is>
+          <t>FSCS deposit-protection levy</t>
+        </is>
+      </c>
+      <c r="C121" s="63" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="D121" s="14" t="inlineStr">
+        <is>
+          <t>% of protected deposits</t>
+        </is>
+      </c>
+      <c r="E121" s="71" t="n">
+        <v>-0.01265257161278474</v>
+      </c>
+      <c r="F121" s="71" t="n">
+        <v>0.0103252157693554</v>
+      </c>
+      <c r="G121" s="71" t="n">
+        <v>-0.0126525716125313</v>
+      </c>
+      <c r="H121" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="B122" s="10" t="inlineStr">
+        <is>
+          <t>Share of deposit balances that are FSCS-protected</t>
+        </is>
+      </c>
+      <c r="C122" s="63" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D122" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E122" s="71" t="n">
+        <v>-0.01265257161278474</v>
+      </c>
+      <c r="F122" s="71" t="n">
+        <v>0.0103252157693554</v>
+      </c>
+      <c r="G122" s="71" t="n">
+        <v>-0.0126525716125313</v>
+      </c>
+      <c r="H122" s="71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" s="10" t="inlineStr">
+        <is>
+          <t>Overdraft — risk weight</t>
+        </is>
+      </c>
+      <c r="C123" s="63" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D123" s="14" t="inlineStr">
+        <is>
+          <t>% of drawn</t>
+        </is>
+      </c>
+      <c r="E123" s="71" t="n">
+        <v>0.00566130690060681</v>
+      </c>
+      <c r="F123" s="71" t="n">
+        <v>-0.002369509251789935</v>
+      </c>
+      <c r="G123" s="71" t="n">
+        <v>-0.03259810445684302</v>
+      </c>
+      <c r="H123" s="71" t="n">
+        <v>0.002369565398971374</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="B124" s="10" t="inlineStr">
+        <is>
+          <t>Invoice finance — risk weight</t>
+        </is>
+      </c>
+      <c r="C124" s="63" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D124" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E124" s="71" t="n">
+        <v>0.002858330950708488</v>
+      </c>
+      <c r="F124" s="71" t="n">
+        <v>-0.001196352928703285</v>
+      </c>
+      <c r="G124" s="71" t="n">
+        <v>-0.01646153881572723</v>
+      </c>
+      <c r="H124" s="71" t="n">
+        <v>0.001196367241437099</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="B125" s="10" t="inlineStr">
+        <is>
+          <t>Tax rate (corporation tax + bank surcharge)</t>
+        </is>
+      </c>
+      <c r="C125" s="63" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="D125" s="14" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E125" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="F125" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G125" s="71" t="n">
         <v>-0.3888888888889994</v>
       </c>
-      <c r="H112" s="71" t="n">
+      <c r="H125" s="71" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10647,7 +10763,7 @@
       <c r="D6" s="46" t="n">
         <v>86808000</v>
       </c>
-      <c r="E6" s="72" t="n">
+      <c r="E6" s="73" t="n">
         <v>1.077256393419961</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -10668,7 +10784,7 @@
       <c r="D7" s="46" t="n">
         <v>56438000</v>
       </c>
-      <c r="E7" s="72" t="n">
+      <c r="E7" s="73" t="n">
         <v>0.1446567738048832</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -10689,7 +10805,7 @@
       <c r="D8" s="46" t="n">
         <v>16091000</v>
       </c>
-      <c r="E8" s="72" t="n">
+      <c r="E8" s="73" t="n">
         <v>4.762930458020011</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -10710,7 +10826,7 @@
       <c r="D9" s="44" t="n">
         <v>496</v>
       </c>
-      <c r="E9" s="72" t="n">
+      <c r="E9" s="73" t="n">
         <v>0.09072580645161291</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -10731,7 +10847,7 @@
       <c r="D10" s="48" t="n">
         <v>0.65</v>
       </c>
-      <c r="E10" s="72" t="n">
+      <c r="E10" s="73" t="n">
         <v>0.1343076923076923</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -11381,7 +11497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F32"/>
+  <dimension ref="B1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -11633,7 +11749,7 @@
       <c r="D14" s="48" t="n">
         <v>0.22</v>
       </c>
-      <c r="E14" s="72" t="n">
+      <c r="E14" s="73" t="n">
         <v>1.136363636363636</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -11654,7 +11770,7 @@
       <c r="D15" s="48" t="n">
         <v>0.13</v>
       </c>
-      <c r="E15" s="72" t="n">
+      <c r="E15" s="73" t="n">
         <v>0.923076923076923</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -11675,7 +11791,7 @@
       <c r="D16" s="48" t="n">
         <v>0.1</v>
       </c>
-      <c r="E16" s="72" t="n">
+      <c r="E16" s="73" t="n">
         <v>0.7999999999999999</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -11696,7 +11812,7 @@
       <c r="D17" s="48" t="n">
         <v>0.0071</v>
       </c>
-      <c r="E17" s="72" t="n">
+      <c r="E17" s="73" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -11726,68 +11842,117 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="7" t="inlineStr">
+    <row r="22" ht="44" customHeight="1">
+      <c r="B22" s="42" t="inlineStr">
+        <is>
+          <t>Payments &amp; FX users</t>
+        </is>
+      </c>
+      <c r="C22" s="48" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D22" s="48" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E22" s="73" t="n">
+        <v>1.666666666666667</v>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>ONS Annual Business Survey 2024 — 12.0% of SMEs were exporters. NOT correction-grade: the model's construct is 'uses international payments or FX', which legitimately includes importers, a larger group than exporters. Corroborated at the top of the plausible range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="44" customHeight="1">
+      <c r="B23" s="42" t="inlineStr">
+        <is>
+          <t>Business credit cards</t>
+        </is>
+      </c>
+      <c r="C23" s="48" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D23" s="48" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="E23" s="73" t="n">
+        <v>1.666666666666667</v>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>SME Finance Monitor — roughly one in five SMEs hold a business credit card (17% Q2 2025, 12% Q1 2023). NOT correction-grade: the survey measures cards used AS FINANCE, while the model measures cards HELD and carries a separate 25% revolving share. The constructs differ by more than the gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="44" customHeight="1">
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>The bar for correcting a cell rather than corroborating it: a HARD COUNT of the same construct. UK Finance's 40,100 invoice finance clients and Companies House incorporations are hard counts, so they corrected the model. Survey percentages and near-miss constructs are corroboration — three of them agreed with the model to within a fifth, which is the more common and less dramatic outcome of checking your assumptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>DERIVING A DEMAND ELASTICITY FROM INERTIA — AND A CORRECTION TO TAB 10</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr"/>
-      <c r="D23" s="8" t="inlineStr"/>
-      <c r="E23" s="8" t="inlineStr"/>
-      <c r="F23" s="8" t="inlineStr"/>
-    </row>
-    <row r="24" ht="26" customHeight="1">
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>• Tab 10 gives the break-even demand elasticity for every price — the responsiveness at which raising it stops paying. It could not say whether real customers are that responsive. For the business current account, public data can.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="39" customHeight="1">
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>• UK SME current-account prices differ by 100%: the majors charge from £8.50 a month, several challengers charge nothing. That gap is permanent, visible and heavily advertised. Against it, 0.44% of SMEs switched in 2024 — and not all of those for price.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="39" customHeight="1">
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>• A 100% price difference producing at most 0.44% of annual movement implies an upper-bound elasticity of about 0.004. Allowing a generous ten-fold multiplier for salience — a fee RISE is noticed in a way a standing price gap is not, which is the one robust finding in the FCA's banking trials — still only reaches 0.044.</t>
-        </is>
-      </c>
+      <c r="C26" s="8" t="inlineStr"/>
+      <c r="D26" s="8" t="inlineStr"/>
+      <c r="E26" s="8" t="inlineStr"/>
+      <c r="F26" s="8" t="inlineStr"/>
     </row>
     <row r="27" ht="26" customHeight="1">
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>• Against a break-even of 0.13, raising the current-account fee industry-wide has roughly three times the headroom it needs. It is comfortably accretive.</t>
+          <t>• Tab 10 gives the break-even demand elasticity for every price — the responsiveness at which raising it stops paying. It could not say whether real customers are that responsive. For the business current account, public data can.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="39" customHeight="1">
       <c r="B28" s="5" t="inlineStr">
         <is>
+          <t>• UK SME current-account prices differ by 100%: the majors charge from £8.50 a month, several challengers charge nothing. That gap is permanent, visible and heavily advertised. Against it, 0.44% of SMEs switched in 2024 — and not all of those for price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="39" customHeight="1">
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>• A 100% price difference producing at most 0.44% of annual movement implies an upper-bound elasticity of about 0.004. Allowing a generous ten-fold multiplier for salience — a fee RISE is noticed in a way a standing price gap is not, which is the one robust finding in the FCA's banking trials — still only reaches 0.044.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1">
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>• Against a break-even of 0.13, raising the current-account fee industry-wide has roughly three times the headroom it needs. It is comfortably accretive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="39" customHeight="1">
+      <c r="B31" s="5" t="inlineStr">
+        <is>
           <t>• CORRECTION TO TAB 10: v1.8 labelled the current-account fee 'fragile — only a near-inert customer makes this pay'. The evidence says the SME current-account customer IS near-inert. At 0.44% annual switching this is close to the most inert consumer market for which data exists. The fragile reading was wrong and this tab supersedes it.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="26" customHeight="1">
-      <c r="B29" s="5" t="inlineStr">
+    <row r="32" ht="26" customHeight="1">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>• Moving alone is the exception and stays genuinely marginal: the break-even falls to 0.021, which is below the salience-adjusted bound of 0.044. Industry-wide, clearly accretive. Unilaterally, a coin toss.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="52" customHeight="1">
-      <c r="B30" s="5" t="inlineStr">
+    <row r="33" ht="52" customHeight="1">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>• The bound does NOT transfer to every price. It holds where switching bank is the customer's only escape, which is true of the current account. It does not hold for the card annual fee (cancel the card, keep the bank), the card interest rate (pay the balance down), or loan pricing (brokered and shopped). Those have other margins of adjustment and need their own evidence.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="B32" s="5" t="inlineStr">
+    <row r="35" ht="30" customHeight="1">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>Still needing an institution's own data: process yields outside lending, entry-point incidence for every cross-holding moment, holding lives for five products, and the benchmark columns on tab 3. Those queries are written against each cell and none of them can be answered from public sources.</t>
         </is>

</xml_diff>